<commit_message>
Record the 13/09/2026 guichet unique filing (stone activity) and what is left to declare
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xqm9tFtdvLdJdkiWw2VVp6
</commit_message>
<xml_diff>
--- a/minyala/clients-potentiels.xlsx
+++ b/minyala/clients-potentiels.xlsx
@@ -90,12 +90,12 @@
     <t xml:space="preserve">Spa / hammam</t>
   </si>
   <si>
+    <t xml:space="preserve">Maître d'œuvre</t>
+  </si>
+  <si>
     <t xml:space="preserve">Jardinerie / matériaux paysage</t>
   </si>
   <si>
-    <t xml:space="preserve">Maître d'œuvre</t>
-  </si>
-  <si>
     <t xml:space="preserve">Hôtel / restaurant</t>
   </si>
   <si>
@@ -105,15 +105,15 @@
     <t xml:space="preserve">Promoteur</t>
   </si>
   <si>
+    <t xml:space="preserve">Salle de bains</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entreprise bâtiment</t>
+  </si>
+  <si>
     <t xml:space="preserve">Travaux publics / VRD</t>
   </si>
   <si>
-    <t xml:space="preserve">Salle de bains</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Entreprise bâtiment</t>
-  </si>
-  <si>
     <t xml:space="preserve">Canaux de vente — vérification au 13/10/2026</t>
   </si>
   <si>
@@ -225,7 +225,7 @@
     <t xml:space="preserve">•</t>
   </si>
   <si>
-    <t xml:space="preserve">Activité : le registre indique un entrepreneur individuel en 85.51Z (enseignement sports et loisirs). Ajouter l'achat-revente de pierre.</t>
+    <t xml:space="preserve">Activité : vente de pierre déclarée au guichet unique le 13/09/2026 (formalité Y00280607979), pas encore visible au registre le 13/10/2026 : vérifier son statut et répondre à toute demande de régularisation. Déclarer aussi le dépôt de Gennevilliers et le nom de domaine pierredegypte.online.</t>
   </si>
   <si>
     <t xml:space="preserve">TVA : si franchise de TVA, remplacer « HT / TTC » par « TVA non applicable, art. 293 B du CGI » partout (prix public et tarif pro).</t>
@@ -5143,7 +5143,7 @@
         <v>20</v>
       </c>
       <c r="B23" s="0" t="n">
-        <f aca="false">COUNTIF('Tous les clients'!D2:D250,"Jardinerie / matériaux paysage")</f>
+        <f aca="false">COUNTIF('Tous les clients'!D2:D250,"Maître d'œuvre")</f>
         <v>3</v>
       </c>
     </row>
@@ -5152,7 +5152,7 @@
         <v>21</v>
       </c>
       <c r="B24" s="0" t="n">
-        <f aca="false">COUNTIF('Tous les clients'!D2:D250,"Maître d'œuvre")</f>
+        <f aca="false">COUNTIF('Tous les clients'!D2:D250,"Jardinerie / matériaux paysage")</f>
         <v>3</v>
       </c>
     </row>
@@ -5188,7 +5188,7 @@
         <v>25</v>
       </c>
       <c r="B28" s="0" t="n">
-        <f aca="false">COUNTIF('Tous les clients'!D2:D250,"Travaux publics / VRD")</f>
+        <f aca="false">COUNTIF('Tous les clients'!D2:D250,"Salle de bains")</f>
         <v>1</v>
       </c>
     </row>
@@ -5197,7 +5197,7 @@
         <v>26</v>
       </c>
       <c r="B29" s="0" t="n">
-        <f aca="false">COUNTIF('Tous les clients'!D2:D250,"Salle de bains")</f>
+        <f aca="false">COUNTIF('Tous les clients'!D2:D250,"Entreprise bâtiment")</f>
         <v>1</v>
       </c>
     </row>
@@ -5206,7 +5206,7 @@
         <v>27</v>
       </c>
       <c r="B30" s="0" t="n">
-        <f aca="false">COUNTIF('Tous les clients'!D2:D250,"Entreprise bâtiment")</f>
+        <f aca="false">COUNTIF('Tous les clients'!D2:D250,"Travaux publics / VRD")</f>
         <v>1</v>
       </c>
     </row>
@@ -5511,7 +5511,7 @@
         <v>1</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E2" s="5" t="s">
         <v>88</v>
@@ -7159,7 +7159,7 @@
         <v>1</v>
       </c>
       <c r="D40" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E40" s="5" t="s">
         <v>271</v>
@@ -7891,7 +7891,7 @@
         <v>2</v>
       </c>
       <c r="D57" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E57" s="5" t="s">
         <v>347</v>
@@ -7933,7 +7933,7 @@
         <v>2</v>
       </c>
       <c r="D58" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E58" s="5" t="s">
         <v>351</v>
@@ -8021,7 +8021,7 @@
         <v>2</v>
       </c>
       <c r="D60" s="5" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E60" s="5" t="s">
         <v>360</v>
@@ -11793,7 +11793,7 @@
         <v>3</v>
       </c>
       <c r="D148" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E148" s="5" t="s">
         <v>731</v>
@@ -12131,7 +12131,7 @@
         <v>3</v>
       </c>
       <c r="D156" s="5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E156" s="5" t="s">
         <v>762</v>
@@ -12901,7 +12901,7 @@
         <v>3</v>
       </c>
       <c r="D174" s="5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E174" s="5" t="s">
         <v>833</v>
@@ -13415,7 +13415,7 @@
         <v>3</v>
       </c>
       <c r="D186" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E186" s="5" t="s">
         <v>883</v>

</xml_diff>

<commit_message>
Two new StoneContact travertine leads (Teodosiu, Cristina): substitution-check reply (two questions, no volume, no price) and tracker rows with one-channel rule
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xqm9tFtdvLdJdkiWw2VVp6
</commit_message>
<xml_diff>
--- a/minyala/clients-potentiels.xlsx
+++ b/minyala/clients-potentiels.xlsx
@@ -17662,45 +17662,45 @@
       </c>
     </row>
     <row r="254" ht="15" customHeight="1" s="13">
-      <c r="A254" t="n">
+      <c r="A254" s="12" t="n">
         <v>254</v>
       </c>
-      <c r="B254" t="inlineStr">
+      <c r="B254" s="12" t="inlineStr">
         <is>
           <t>Acheteur export (RFQ)</t>
         </is>
       </c>
-      <c r="C254" t="n">
+      <c r="C254" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="D254" t="inlineStr">
+      <c r="D254" s="12" t="inlineStr">
         <is>
           <t>Négoce / revendeur</t>
         </is>
       </c>
-      <c r="E254" t="inlineStr">
+      <c r="E254" s="12" t="inlineStr">
         <is>
           <t>FABIAN (demande StoneContact)</t>
         </is>
       </c>
-      <c r="F254" t="inlineStr">
+      <c r="F254" s="12" t="inlineStr">
         <is>
           <t>France</t>
         </is>
       </c>
-      <c r="G254" t="inlineStr">
+      <c r="G254" s="12" t="inlineStr">
         <is>
           <t>France</t>
         </is>
       </c>
-      <c r="H254" t="inlineStr">
+      <c r="H254" s="12" t="inlineStr">
         <is>
           <t>Demande d'environ 500 m² de dalles en 55×85 cm reçue via StoneContact : format non disponible (stock en 30×60×2 cm), contre-proposition à envoyer.</t>
         </is>
       </c>
-      <c r="I254" t="inlineStr"/>
-      <c r="J254" t="inlineStr"/>
-      <c r="K254" t="inlineStr">
+      <c r="I254" s="12" t="inlineStr"/>
+      <c r="J254" s="12" t="inlineStr"/>
+      <c r="K254" s="12" t="inlineStr">
         <is>
           <t>StoneContact (détails derrière abonnement)</t>
         </is>
@@ -17710,29 +17710,149 @@
           <t>À contacter</t>
         </is>
       </c>
-      <c r="M254" t="inlineStr"/>
-      <c r="N254" t="inlineStr">
+      <c r="M254" s="12" t="inlineStr"/>
+      <c r="N254" s="12" t="inlineStr">
         <is>
           <t>Répondre via StoneContact avec la contre-proposition préparée (reponses-pistes-2026-10.md) — Une seule voie de contact par piste ; répondre avec le message préparé (minyala/reponses-pistes-2026-10.md) et noter la date ici</t>
         </is>
       </c>
-      <c r="O254" t="inlineStr">
+      <c r="O254" s="12" t="inlineStr">
         <is>
           <t>[15/10] Conditions pro uniquement sur devis écrit après SIRET/coordonnées d'entreprise ; ne pas payer l'abonnement avant d'avoir vu les détails gratuits de la demande.</t>
         </is>
       </c>
-      <c r="P254" t="inlineStr">
+      <c r="P254" s="12" t="inlineStr">
         <is>
           <t>StoneContact</t>
         </is>
       </c>
-      <c r="Q254" t="inlineStr"/>
+      <c r="Q254" s="12" t="inlineStr"/>
     </row>
     <row r="255" ht="15" customHeight="1" s="13">
-      <c r="L255" s="12" t="n"/>
+      <c r="A255" t="n">
+        <v>255</v>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>Acheteur export (RFQ)</t>
+        </is>
+      </c>
+      <c r="C255" t="n">
+        <v>2</v>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>À qualifier</t>
+        </is>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>Teodosiu (demande StoneContact — travertin)</t>
+        </is>
+      </c>
+      <c r="F255" t="inlineStr">
+        <is>
+          <t>À préciser</t>
+        </is>
+      </c>
+      <c r="G255" t="inlineStr">
+        <is>
+          <t>À préciser</t>
+        </is>
+      </c>
+      <c r="H255" t="inlineStr">
+        <is>
+          <t>Cherche du travertin : MINYALA en substitution possible.</t>
+        </is>
+      </c>
+      <c r="K255" t="inlineStr">
+        <is>
+          <t>StoneContact</t>
+        </is>
+      </c>
+      <c r="L255" s="12" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="N255" t="inlineStr">
+        <is>
+          <t>Répondre via StoneContact avec le message « alternative travertin » (reponses-pistes-2026-10.md) ; noter la date ici</t>
+        </is>
+      </c>
+      <c r="O255" t="inlineStr">
+        <is>
+          <t>[16/10] Demande de TRAVERTIN sur StoneContact — nous n'en vendons pas : alternative MINYALA (30×60×2) à proposer. Première réponse = 2 questions (recherche en cours ? alternative acceptable ?), aucun volume ni tarif. Aucune coordonnée vérifiée ; une seule voie de contact : StoneContact.</t>
+        </is>
+      </c>
+      <c r="P255" t="inlineStr">
+        <is>
+          <t>StoneContact</t>
+        </is>
+      </c>
     </row>
     <row r="256" ht="15" customHeight="1" s="13">
-      <c r="L256" s="12" t="n"/>
+      <c r="A256" t="n">
+        <v>256</v>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>Acheteur export (RFQ)</t>
+        </is>
+      </c>
+      <c r="C256" t="n">
+        <v>2</v>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>À qualifier</t>
+        </is>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>Cristina (demande StoneContact — travertin)</t>
+        </is>
+      </c>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>À préciser</t>
+        </is>
+      </c>
+      <c r="G256" t="inlineStr">
+        <is>
+          <t>À préciser</t>
+        </is>
+      </c>
+      <c r="H256" t="inlineStr">
+        <is>
+          <t>Cherche du travertin : MINYALA en substitution possible.</t>
+        </is>
+      </c>
+      <c r="K256" t="inlineStr">
+        <is>
+          <t>StoneContact</t>
+        </is>
+      </c>
+      <c r="L256" s="12" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="N256" t="inlineStr">
+        <is>
+          <t>Répondre via StoneContact avec le message « alternative travertin » (reponses-pistes-2026-10.md) ; noter la date ici</t>
+        </is>
+      </c>
+      <c r="O256" t="inlineStr">
+        <is>
+          <t>[16/10] Demande de TRAVERTIN sur StoneContact — nous n'en vendons pas : alternative MINYALA (30×60×2) à proposer. Première réponse = 2 questions (recherche en cours ? alternative acceptable ?), aucun volume ni tarif. Aucune coordonnée vérifiée ; une seule voie de contact : StoneContact.</t>
+        </is>
+      </c>
+      <c r="P256" t="inlineStr">
+        <is>
+          <t>StoneContact</t>
+        </is>
+      </c>
     </row>
     <row r="257" ht="15" customHeight="1" s="13">
       <c r="L257" s="12" t="n"/>

</xml_diff>

<commit_message>
Log the 3 real sends of 15/10 found in Gmail (Pillaud, Torchio, Belles Piscines): new send registry with RFC Message-IDs, tracker statuses to Contacté 15/10, no reply as of 16/10
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xqm9tFtdvLdJdkiWw2VVp6
</commit_message>
<xml_diff>
--- a/minyala/clients-potentiels.xlsx
+++ b/minyala/clients-potentiels.xlsx
@@ -1872,14 +1872,22 @@
       </c>
       <c r="L10" s="21" t="inlineStr">
         <is>
-          <t>À contacter</t>
-        </is>
-      </c>
-      <c r="M10" s="21" t="n"/>
-      <c r="N10" s="21" t="n"/>
+          <t>Contacté</t>
+        </is>
+      </c>
+      <c r="M10" s="21" t="inlineStr">
+        <is>
+          <t>15/10/2026</t>
+        </is>
+      </c>
+      <c r="N10" s="21" t="inlineStr">
+        <is>
+          <t>Attendre la réponse ; pas de relance avant le 22/10</t>
+        </is>
+      </c>
       <c r="O10" s="21" t="inlineStr">
         <is>
-          <t>[13/10] Page agence de Caen du site Pillaud.</t>
+          <t>[13/10] Page agence de Caen du site Pillaud. | [15/10] Message A (version courte) envoyé depuis Gmail (constaté dans les éléments envoyés, voir registre-envois-2026-10-15.csv) ; remise non confirmée, aucune réponse au 16/10.</t>
         </is>
       </c>
       <c r="P10" s="15" t="inlineStr">
@@ -2141,14 +2149,22 @@
       </c>
       <c r="L14" s="21" t="inlineStr">
         <is>
-          <t>À contacter</t>
-        </is>
-      </c>
-      <c r="M14" s="21" t="n"/>
-      <c r="N14" s="21" t="n"/>
+          <t>Contacté</t>
+        </is>
+      </c>
+      <c r="M14" s="21" t="inlineStr">
+        <is>
+          <t>15/10/2026</t>
+        </is>
+      </c>
+      <c r="N14" s="21" t="inlineStr">
+        <is>
+          <t>Attendre la réponse ; pas de relance avant le 22/10</t>
+        </is>
+      </c>
       <c r="O14" s="21" t="inlineStr">
         <is>
-          <t>[13/10] Affiché en forme anti-spam « info[@]torchio.fr » sur les mentions légales du site.</t>
+          <t>[13/10] Affiché en forme anti-spam « info[@]torchio.fr » sur les mentions légales du site. | [15/10] Message A (version courte) envoyé depuis Gmail (constaté dans les éléments envoyés, voir registre-envois-2026-10-15.csv) ; remise non confirmée, aucune réponse au 16/10.</t>
         </is>
       </c>
       <c r="P14" s="15" t="inlineStr">
@@ -2382,14 +2398,22 @@
       </c>
       <c r="L17" s="21" t="inlineStr">
         <is>
-          <t>À contacter</t>
-        </is>
-      </c>
-      <c r="M17" s="21" t="n"/>
-      <c r="N17" s="21" t="n"/>
+          <t>Contacté</t>
+        </is>
+      </c>
+      <c r="M17" s="21" t="inlineStr">
+        <is>
+          <t>15/10/2026</t>
+        </is>
+      </c>
+      <c r="N17" s="21" t="inlineStr">
+        <is>
+          <t>Attendre la réponse ; pas de relance avant le 22/10</t>
+        </is>
+      </c>
       <c r="O17" s="21" t="inlineStr">
         <is>
-          <t>[13/10] Lien « Envoyer un e-mail » de la page Notre agence (Coignières).</t>
+          <t>[13/10] Lien « Envoyer un e-mail » de la page Notre agence (Coignières). | [15/10] Message A (version courte) envoyé depuis Gmail (constaté dans les éléments envoyés, voir registre-envois-2026-10-15.csv) ; remise non confirmée, aucune réponse au 16/10.</t>
         </is>
       </c>
       <c r="P17" s="15" t="inlineStr">
@@ -17729,43 +17753,43 @@
       <c r="Q254" s="12" t="inlineStr"/>
     </row>
     <row r="255" ht="15" customHeight="1" s="13">
-      <c r="A255" t="n">
+      <c r="A255" s="12" t="n">
         <v>255</v>
       </c>
-      <c r="B255" t="inlineStr">
+      <c r="B255" s="12" t="inlineStr">
         <is>
           <t>Acheteur export (RFQ)</t>
         </is>
       </c>
-      <c r="C255" t="n">
+      <c r="C255" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="D255" t="inlineStr">
+      <c r="D255" s="12" t="inlineStr">
         <is>
           <t>À qualifier</t>
         </is>
       </c>
-      <c r="E255" t="inlineStr">
+      <c r="E255" s="12" t="inlineStr">
         <is>
           <t>Teodosiu (demande StoneContact — travertin)</t>
         </is>
       </c>
-      <c r="F255" t="inlineStr">
+      <c r="F255" s="12" t="inlineStr">
         <is>
           <t>À préciser</t>
         </is>
       </c>
-      <c r="G255" t="inlineStr">
+      <c r="G255" s="12" t="inlineStr">
         <is>
           <t>À préciser</t>
         </is>
       </c>
-      <c r="H255" t="inlineStr">
+      <c r="H255" s="12" t="inlineStr">
         <is>
           <t>Cherche du travertin : MINYALA en substitution possible.</t>
         </is>
       </c>
-      <c r="K255" t="inlineStr">
+      <c r="K255" s="12" t="inlineStr">
         <is>
           <t>StoneContact</t>
         </is>
@@ -17775,60 +17799,60 @@
           <t>À contacter</t>
         </is>
       </c>
-      <c r="N255" t="inlineStr">
+      <c r="N255" s="12" t="inlineStr">
         <is>
           <t>Répondre via StoneContact avec le message « alternative travertin » (reponses-pistes-2026-10.md) ; noter la date ici</t>
         </is>
       </c>
-      <c r="O255" t="inlineStr">
+      <c r="O255" s="12" t="inlineStr">
         <is>
           <t>[16/10] Demande de TRAVERTIN sur StoneContact — nous n'en vendons pas : alternative MINYALA (30×60×2) à proposer. Première réponse = 2 questions (recherche en cours ? alternative acceptable ?), aucun volume ni tarif. Aucune coordonnée vérifiée ; une seule voie de contact : StoneContact.</t>
         </is>
       </c>
-      <c r="P255" t="inlineStr">
+      <c r="P255" s="12" t="inlineStr">
         <is>
           <t>StoneContact</t>
         </is>
       </c>
     </row>
     <row r="256" ht="15" customHeight="1" s="13">
-      <c r="A256" t="n">
+      <c r="A256" s="12" t="n">
         <v>256</v>
       </c>
-      <c r="B256" t="inlineStr">
+      <c r="B256" s="12" t="inlineStr">
         <is>
           <t>Acheteur export (RFQ)</t>
         </is>
       </c>
-      <c r="C256" t="n">
+      <c r="C256" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="D256" t="inlineStr">
+      <c r="D256" s="12" t="inlineStr">
         <is>
           <t>À qualifier</t>
         </is>
       </c>
-      <c r="E256" t="inlineStr">
+      <c r="E256" s="12" t="inlineStr">
         <is>
           <t>Cristina (demande StoneContact — travertin)</t>
         </is>
       </c>
-      <c r="F256" t="inlineStr">
+      <c r="F256" s="12" t="inlineStr">
         <is>
           <t>À préciser</t>
         </is>
       </c>
-      <c r="G256" t="inlineStr">
+      <c r="G256" s="12" t="inlineStr">
         <is>
           <t>À préciser</t>
         </is>
       </c>
-      <c r="H256" t="inlineStr">
+      <c r="H256" s="12" t="inlineStr">
         <is>
           <t>Cherche du travertin : MINYALA en substitution possible.</t>
         </is>
       </c>
-      <c r="K256" t="inlineStr">
+      <c r="K256" s="12" t="inlineStr">
         <is>
           <t>StoneContact</t>
         </is>
@@ -17838,17 +17862,17 @@
           <t>À contacter</t>
         </is>
       </c>
-      <c r="N256" t="inlineStr">
+      <c r="N256" s="12" t="inlineStr">
         <is>
           <t>Répondre via StoneContact avec le message « alternative travertin » (reponses-pistes-2026-10.md) ; noter la date ici</t>
         </is>
       </c>
-      <c r="O256" t="inlineStr">
+      <c r="O256" s="12" t="inlineStr">
         <is>
           <t>[16/10] Demande de TRAVERTIN sur StoneContact — nous n'en vendons pas : alternative MINYALA (30×60×2) à proposer. Première réponse = 2 questions (recherche en cours ? alternative acceptable ?), aucun volume ni tarif. Aucune coordonnée vérifiée ; une seule voie de contact : StoneContact.</t>
         </is>
       </c>
-      <c r="P256" t="inlineStr">
+      <c r="P256" s="12" t="inlineStr">
         <is>
           <t>StoneContact</t>
         </is>

</xml_diff>

<commit_message>
Send batch 1 of remaining lot 1 (Le Comptoir du Sol, Midi Carrelage, Décomarbre) from Gmail at 10:38 UTC: registry with RFC Message-IDs, trackers to Contacté 16/10
First real contact for these three (previous Hotmail attempts were rejected outbound, never delivered). Batch 2 (La Halle aux Pierres, Natou Pierre, Paco) scheduled ~3h later to respect spaced-batch rule.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xqm9tFtdvLdJdkiWw2VVp6
</commit_message>
<xml_diff>
--- a/minyala/clients-potentiels.xlsx
+++ b/minyala/clients-potentiels.xlsx
@@ -1482,18 +1482,22 @@
       </c>
       <c r="L5" s="21" t="inlineStr">
         <is>
-          <t>À contacter</t>
-        </is>
-      </c>
-      <c r="M5" s="21" t="n"/>
+          <t>Contacté</t>
+        </is>
+      </c>
+      <c r="M5" s="21" t="inlineStr">
+        <is>
+          <t>16/10/2026</t>
+        </is>
+      </c>
       <c r="N5" s="21" t="inlineStr">
         <is>
-          <t>Prochain contact depuis la boîte Gmail (pas Hotmail), après fusion du suivi</t>
+          <t>Attendre la réponse ; pas de relance avant le 23/10</t>
         </is>
       </c>
       <c r="O5" s="21" t="inlineStr">
         <is>
-          <t>Rapprochement du 13/10 (autre assistant) : dernier envoi rejeté (échec de remise) — à confirmer, puis trouver une autre adresse. | [13/10] Tentative depuis Hotmail rejetée EN SORTIE (5.7.520 : contenu classé spam par Microsoft) — message non remis ; l'adresse n'est pas forcément invalide. Prochain contact depuis la boîte Gmail, nouveau modèle, jamais depuis Hotmail.</t>
+          <t>Rapprochement du 13/10 (autre assistant) : dernier envoi rejeté (échec de remise) — à confirmer, puis trouver une autre adresse. | [13/10] Tentative depuis Hotmail rejetée EN SORTIE (5.7.520 : contenu classé spam par Microsoft) — message non remis ; l'adresse n'est pas forcément invalide. Prochain contact depuis la boîte Gmail, nouveau modèle, jamais depuis Hotmail. | [16/10] Message A (version courte) envoyé depuis Gmail à 10h38 UTC (registre-envois-2026-10-16.csv) ; adresse précédemment visée par un rejet 5.7.520 côté Hotmail (jamais remise) : ceci est le premier contact réel. Remise non confirmée.</t>
         </is>
       </c>
       <c r="P5" s="15" t="inlineStr">
@@ -1644,18 +1648,22 @@
       </c>
       <c r="L7" s="21" t="inlineStr">
         <is>
-          <t>À contacter</t>
-        </is>
-      </c>
-      <c r="M7" s="21" t="n"/>
+          <t>Contacté</t>
+        </is>
+      </c>
+      <c r="M7" s="21" t="inlineStr">
+        <is>
+          <t>16/10/2026</t>
+        </is>
+      </c>
       <c r="N7" s="21" t="inlineStr">
         <is>
-          <t>Prochain contact depuis la boîte Gmail (pas Hotmail), après fusion du suivi</t>
+          <t>Attendre la réponse ; pas de relance avant le 23/10</t>
         </is>
       </c>
       <c r="O7" s="21" t="inlineStr">
         <is>
-          <t>[13/10] Tentative depuis Hotmail rejetée EN SORTIE (5.7.520 : contenu classé spam par Microsoft) — message non remis ; l'adresse n'est pas forcément invalide. Prochain contact depuis la boîte Gmail, nouveau modèle, jamais depuis Hotmail.</t>
+          <t>[13/10] Tentative depuis Hotmail rejetée EN SORTIE (5.7.520 : contenu classé spam par Microsoft) — message non remis ; l'adresse n'est pas forcément invalide. Prochain contact depuis la boîte Gmail, nouveau modèle, jamais depuis Hotmail. | [16/10] Message A (version courte) envoyé depuis Gmail à 10h38 UTC (registre-envois-2026-10-16.csv) ; adresse précédemment visée par un rejet 5.7.520 côté Hotmail (jamais remise) : ceci est le premier contact réel. Remise non confirmée.</t>
         </is>
       </c>
       <c r="P7" s="15" t="inlineStr">
@@ -2825,18 +2833,22 @@
       </c>
       <c r="L23" s="21" t="inlineStr">
         <is>
-          <t>À contacter</t>
-        </is>
-      </c>
-      <c r="M23" s="21" t="n"/>
+          <t>Contacté</t>
+        </is>
+      </c>
+      <c r="M23" s="21" t="inlineStr">
+        <is>
+          <t>16/10/2026</t>
+        </is>
+      </c>
       <c r="N23" s="21" t="inlineStr">
         <is>
-          <t>Prochain contact depuis la boîte Gmail (pas Hotmail), après fusion du suivi</t>
+          <t>Attendre la réponse ; pas de relance avant le 23/10</t>
         </is>
       </c>
       <c r="O23" s="21" t="inlineStr">
         <is>
-          <t>[13/10] Tentative depuis Hotmail rejetée EN SORTIE (5.7.520 : contenu classé spam par Microsoft) — message non remis ; l'adresse n'est pas forcément invalide. Prochain contact depuis la boîte Gmail, nouveau modèle, jamais depuis Hotmail.</t>
+          <t>[13/10] Tentative depuis Hotmail rejetée EN SORTIE (5.7.520 : contenu classé spam par Microsoft) — message non remis ; l'adresse n'est pas forcément invalide. Prochain contact depuis la boîte Gmail, nouveau modèle, jamais depuis Hotmail. | [16/10] Message A (version courte) envoyé depuis Gmail à 10h38 UTC (registre-envois-2026-10-16.csv) ; adresse précédemment visée par un rejet 5.7.520 côté Hotmail (jamais remise) : ceci est le premier contact réel. Remise non confirmée.</t>
         </is>
       </c>
       <c r="P23" s="15" t="inlineStr">

</xml_diff>

<commit_message>
Fill official contact e-mails for 9 of the 12 remaining P1 prospects (own-site sources cited; 3 form-only noted with phone); next send batches now stocked
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xqm9tFtdvLdJdkiWw2VVp6
</commit_message>
<xml_diff>
--- a/minyala/clients-potentiels.xlsx
+++ b/minyala/clients-potentiels.xlsx
@@ -1340,7 +1340,7 @@
       <c r="N3" s="21" t="n"/>
       <c r="O3" s="21" t="inlineStr">
         <is>
-          <t>[13/10] Aucun e-mail publié : formulaire de la fiche magasin BigMat Évreux uniquement.</t>
+          <t>[13/10] Aucun e-mail publié : formulaire de la fiche magasin BigMat Évreux uniquement. | [16/10] Pas d'e-mail publié (fiche officielle magasins.bigmat.fr : formulaire seul). Tél. 02 32 31 20 17. Contact par formulaire ou téléphone.</t>
         </is>
       </c>
       <c r="P3" s="15" t="inlineStr">
@@ -1819,7 +1819,11 @@
       </c>
       <c r="M9" s="21" t="n"/>
       <c r="N9" s="21" t="n"/>
-      <c r="O9" s="21" t="n"/>
+      <c r="O9" s="21" t="inlineStr">
+        <is>
+          <t>[16/10] Aucun e-mail publié (formulaire avec choix d'agence uniquement, mentions légales comprises). Tél. agence de Caen : 02 31 68 69 68.</t>
+        </is>
+      </c>
       <c r="P9" s="15" t="inlineStr">
         <is>
           <t>3e liste (12/10)</t>
@@ -1968,10 +1972,19 @@
       </c>
       <c r="M11" s="21" t="n"/>
       <c r="N11" s="21" t="n"/>
-      <c r="O11" s="21" t="n"/>
+      <c r="O11" s="21" t="inlineStr">
+        <is>
+          <t>[16/10] E-mail de l'éditeur sur sedelka.fr/mentions-legales (dpo@ réservé aux données personnelles).</t>
+        </is>
+      </c>
       <c r="P11" s="15" t="inlineStr">
         <is>
           <t>3e liste (12/10)</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>contact@sedelka.fr</t>
         </is>
       </c>
     </row>
@@ -2030,10 +2043,19 @@
       </c>
       <c r="M12" s="21" t="n"/>
       <c r="N12" s="21" t="n"/>
-      <c r="O12" s="21" t="n"/>
+      <c r="O12" s="21" t="inlineStr">
+        <is>
+          <t>[16/10] E-mail « Espace Pro » de la fiche agence Évreux sur solmur.fr (tél. 02 32 62 94 80). Ne PAS utiliser espace.pro.bihorel@ (pied de page = siège Bihorel).</t>
+        </is>
+      </c>
       <c r="P12" s="15" t="inlineStr">
         <is>
           <t>3e liste (12/10)</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>espace.pro.evreux@solmur.fr</t>
         </is>
       </c>
     </row>
@@ -2096,10 +2118,19 @@
       </c>
       <c r="M13" s="21" t="n"/>
       <c r="N13" s="21" t="n"/>
-      <c r="O13" s="21" t="n"/>
+      <c r="O13" s="21" t="inlineStr">
+        <is>
+          <t>[16/10] Seule adresse affichée sur le site officiel (page contact) — semi-nominative sur hotmail.com, pas de générique. À utiliser telle quelle.</t>
+        </is>
+      </c>
       <c r="P13" s="15" t="inlineStr">
         <is>
           <t>3e liste (12/10)</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>anthony.tendance@hotmail.com</t>
         </is>
       </c>
     </row>
@@ -2490,7 +2521,11 @@
       </c>
       <c r="M18" s="21" t="n"/>
       <c r="N18" s="21" t="n"/>
-      <c r="O18" s="21" t="n"/>
+      <c r="O18" s="21" t="inlineStr">
+        <is>
+          <t>[16/10] Pas d'e-mail publié (fiche officielle magasins.bigmat.fr : formulaire seul). Tél. 01 30 90 71 75. Contact par formulaire ou téléphone.</t>
+        </is>
+      </c>
       <c r="P18" s="15" t="inlineStr">
         <is>
           <t>3e liste (12/10)</t>
@@ -2706,10 +2741,19 @@
       </c>
       <c r="M21" s="21" t="n"/>
       <c r="N21" s="21" t="n"/>
-      <c r="O21" s="21" t="n"/>
+      <c r="O21" s="21" t="inlineStr">
+        <is>
+          <t>[16/10] E-mail du pied de page/page contact du site officiel pedrazzini.fr (showroom Voisenon confirmé).</t>
+        </is>
+      </c>
       <c r="P21" s="15" t="inlineStr">
         <is>
           <t>1re liste (08/10)</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>contact@pedrazzini.fr</t>
         </is>
       </c>
     </row>
@@ -2772,10 +2816,19 @@
       </c>
       <c r="M22" s="21" t="n"/>
       <c r="N22" s="21" t="n"/>
-      <c r="O22" s="21" t="n"/>
+      <c r="O22" s="21" t="inlineStr">
+        <is>
+          <t>[16/10] E-mail du magasin de Sarcelles sur ceramico.fr (accueil, bloc « Magasin 1 &amp; Dépôt — Sarcelles »). Ne PAS utiliser commercial@ceramico.fr (magasin du Perreux).</t>
+        </is>
+      </c>
       <c r="P22" s="15" t="inlineStr">
         <is>
           <t>3e liste (12/10)</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>info@ceramico.fr</t>
         </is>
       </c>
     </row>
@@ -3652,10 +3705,19 @@
       </c>
       <c r="M33" s="21" t="n"/>
       <c r="N33" s="21" t="n"/>
-      <c r="O33" s="21" t="n"/>
+      <c r="O33" s="21" t="inlineStr">
+        <is>
+          <t>[16/10] E-mail général du pied de page (mpt-marbrier.fr/contact) ; domaine de l'adresse ≠ domaine du site, tel qu'affiché par le site officiel.</t>
+        </is>
+      </c>
       <c r="P33" s="15" t="inlineStr">
         <is>
           <t>3e liste (12/10)</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>accueil@marbrierpierretaille.fr</t>
         </is>
       </c>
     </row>
@@ -4180,10 +4242,19 @@
       </c>
       <c r="M40" s="21" t="n"/>
       <c r="N40" s="21" t="n"/>
-      <c r="O40" s="21" t="n"/>
+      <c r="O40" s="21" t="inlineStr">
+        <is>
+          <t>[16/10] Unique e-mail du site officiel pierres-nat.com (page contact, en-tête, pied de page ; adresse Linas confirmée).</t>
+        </is>
+      </c>
       <c r="P40" s="15" t="inlineStr">
         <is>
           <t>3e liste (12/10)</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>pierres.nat@gmail.com</t>
         </is>
       </c>
     </row>
@@ -4317,10 +4388,19 @@
       </c>
       <c r="M42" s="21" t="n"/>
       <c r="N42" s="21" t="n"/>
-      <c r="O42" s="21" t="n"/>
+      <c r="O42" s="21" t="inlineStr">
+        <is>
+          <t>[16/10] Adresse générique RABONI IDF lue sur lestudioraboni.fr/mentions-legales — pas propre au showroom de Boulogne (sa page contact = formulaire seul, tél. 01 46 09 54 80). raboni.fr protégé anti-bot.</t>
+        </is>
+      </c>
       <c r="P42" s="15" t="inlineStr">
         <is>
           <t>3e liste (12/10)</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>contact@raboni.fr</t>
         </is>
       </c>
     </row>
@@ -4468,12 +4548,17 @@
       <c r="N44" s="21" t="n"/>
       <c r="O44" s="21" t="inlineStr">
         <is>
-          <t>[13/10] Aucun e-mail propre à SNNMC publié : formulaire sur la fiche France Matériaux, ou téléphone.</t>
+          <t>[13/10] Aucun e-mail propre à SNNMC publié : formulaire sur la fiche France Matériaux, ou téléphone. | [16/10] E-mail du site officiel materiaux-batiment.fr (accueil + page contact, itemprop=email). Site parfois en 503 : réessayer. Ne PAS utiliser contact@france-materiaux.fr (réseau, pas SNNMC).</t>
         </is>
       </c>
       <c r="P44" s="15" t="inlineStr">
         <is>
           <t>2e liste (12/10)</t>
+        </is>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>contact@materiaux-batiment.fr</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Send batch 2 of 16/10 (La Halle aux Pierres, Natou Pierre, Paco) at 13:42 UTC: registry rows with RFC Message-IDs, trackers to Contacté 16/10; no replies/STOP/bounces before sending
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xqm9tFtdvLdJdkiWw2VVp6
</commit_message>
<xml_diff>
--- a/minyala/clients-potentiels.xlsx
+++ b/minyala/clients-potentiels.xlsx
@@ -1982,7 +1982,7 @@
           <t>3e liste (12/10)</t>
         </is>
       </c>
-      <c r="Q11" t="inlineStr">
+      <c r="Q11" s="12" t="inlineStr">
         <is>
           <t>contact@sedelka.fr</t>
         </is>
@@ -2053,7 +2053,7 @@
           <t>3e liste (12/10)</t>
         </is>
       </c>
-      <c r="Q12" t="inlineStr">
+      <c r="Q12" s="12" t="inlineStr">
         <is>
           <t>espace.pro.evreux@solmur.fr</t>
         </is>
@@ -2128,7 +2128,7 @@
           <t>3e liste (12/10)</t>
         </is>
       </c>
-      <c r="Q13" t="inlineStr">
+      <c r="Q13" s="12" t="inlineStr">
         <is>
           <t>anthony.tendance@hotmail.com</t>
         </is>
@@ -2751,7 +2751,7 @@
           <t>1re liste (08/10)</t>
         </is>
       </c>
-      <c r="Q21" t="inlineStr">
+      <c r="Q21" s="12" t="inlineStr">
         <is>
           <t>contact@pedrazzini.fr</t>
         </is>
@@ -2826,7 +2826,7 @@
           <t>3e liste (12/10)</t>
         </is>
       </c>
-      <c r="Q22" t="inlineStr">
+      <c r="Q22" s="12" t="inlineStr">
         <is>
           <t>info@ceramico.fr</t>
         </is>
@@ -3293,18 +3293,22 @@
       </c>
       <c r="L28" s="21" t="inlineStr">
         <is>
-          <t>À contacter</t>
-        </is>
-      </c>
-      <c r="M28" s="21" t="n"/>
+          <t>Contacté</t>
+        </is>
+      </c>
+      <c r="M28" s="21" t="inlineStr">
+        <is>
+          <t>16/10/2026</t>
+        </is>
+      </c>
       <c r="N28" s="21" t="inlineStr">
         <is>
-          <t>Prochain contact depuis la boîte Gmail (pas Hotmail), après fusion du suivi</t>
+          <t>Attendre la réponse ; pas de relance avant le 23/10</t>
         </is>
       </c>
       <c r="O28" s="21" t="inlineStr">
         <is>
-          <t>Rapprochement du 13/10 (autre assistant) : dernier envoi rejeté (échec de remise) — à confirmer, puis trouver une autre adresse. | [13/10] Tentative depuis Hotmail rejetée EN SORTIE (5.7.520 : contenu classé spam par Microsoft) — message non remis ; l'adresse n'est pas forcément invalide. Prochain contact depuis la boîte Gmail, nouveau modèle, jamais depuis Hotmail.</t>
+          <t>Rapprochement du 13/10 (autre assistant) : dernier envoi rejeté (échec de remise) — à confirmer, puis trouver une autre adresse. | [13/10] Tentative depuis Hotmail rejetée EN SORTIE (5.7.520 : contenu classé spam par Microsoft) — message non remis ; l'adresse n'est pas forcément invalide. Prochain contact depuis la boîte Gmail, nouveau modèle, jamais depuis Hotmail. | [16/10] Message A (version courte) envoyé depuis Gmail à 13h42 UTC (registre-envois-2026-10-16.csv) ; adresse précédemment visée par un rejet 5.7.520 côté Hotmail (jamais remise) : premier contact réel. Remise non confirmée.</t>
         </is>
       </c>
       <c r="P28" s="15" t="inlineStr">
@@ -3715,7 +3719,7 @@
           <t>3e liste (12/10)</t>
         </is>
       </c>
-      <c r="Q33" t="inlineStr">
+      <c r="Q33" s="12" t="inlineStr">
         <is>
           <t>accueil@marbrierpierretaille.fr</t>
         </is>
@@ -3767,18 +3771,22 @@
       </c>
       <c r="L34" s="21" t="inlineStr">
         <is>
-          <t>À contacter</t>
-        </is>
-      </c>
-      <c r="M34" s="21" t="n"/>
+          <t>Contacté</t>
+        </is>
+      </c>
+      <c r="M34" s="21" t="inlineStr">
+        <is>
+          <t>16/10/2026</t>
+        </is>
+      </c>
       <c r="N34" s="21" t="inlineStr">
         <is>
-          <t>Prochain contact depuis la boîte Gmail (pas Hotmail), après fusion du suivi</t>
+          <t>Attendre la réponse ; pas de relance avant le 23/10</t>
         </is>
       </c>
       <c r="O34" s="21" t="inlineStr">
         <is>
-          <t>Rapprochement du 13/10 (autre assistant) : dernier envoi rejeté (échec de remise) — à confirmer, puis trouver une autre adresse. | [13/10] Tentative depuis Hotmail rejetée EN SORTIE (5.7.520 : contenu classé spam par Microsoft) — message non remis ; l'adresse n'est pas forcément invalide. Prochain contact depuis la boîte Gmail, nouveau modèle, jamais depuis Hotmail.</t>
+          <t>Rapprochement du 13/10 (autre assistant) : dernier envoi rejeté (échec de remise) — à confirmer, puis trouver une autre adresse. | [13/10] Tentative depuis Hotmail rejetée EN SORTIE (5.7.520 : contenu classé spam par Microsoft) — message non remis ; l'adresse n'est pas forcément invalide. Prochain contact depuis la boîte Gmail, nouveau modèle, jamais depuis Hotmail. | [16/10] Message A (version courte) envoyé depuis Gmail à 13h42 UTC (registre-envois-2026-10-16.csv) ; adresse précédemment visée par un rejet 5.7.520 côté Hotmail (jamais remise) : premier contact réel. Remise non confirmée.</t>
         </is>
       </c>
       <c r="P34" s="15" t="inlineStr">
@@ -3921,18 +3929,22 @@
       </c>
       <c r="L36" s="21" t="inlineStr">
         <is>
-          <t>À contacter</t>
-        </is>
-      </c>
-      <c r="M36" s="21" t="n"/>
+          <t>Contacté</t>
+        </is>
+      </c>
+      <c r="M36" s="21" t="inlineStr">
+        <is>
+          <t>16/10/2026</t>
+        </is>
+      </c>
       <c r="N36" s="21" t="inlineStr">
         <is>
-          <t>Prochain contact depuis la boîte Gmail (pas Hotmail), après fusion du suivi</t>
+          <t>Attendre la réponse ; pas de relance avant le 23/10</t>
         </is>
       </c>
       <c r="O36" s="21" t="inlineStr">
         <is>
-          <t>Rapprochement du 13/10 (autre assistant) : dernier envoi rejeté (échec de remise) — à confirmer, puis trouver une autre adresse. | [13/10] Tentative depuis Hotmail rejetée EN SORTIE (5.7.520 : contenu classé spam par Microsoft) — message non remis ; l'adresse n'est pas forcément invalide. Prochain contact depuis la boîte Gmail, nouveau modèle, jamais depuis Hotmail.</t>
+          <t>Rapprochement du 13/10 (autre assistant) : dernier envoi rejeté (échec de remise) — à confirmer, puis trouver une autre adresse. | [13/10] Tentative depuis Hotmail rejetée EN SORTIE (5.7.520 : contenu classé spam par Microsoft) — message non remis ; l'adresse n'est pas forcément invalide. Prochain contact depuis la boîte Gmail, nouveau modèle, jamais depuis Hotmail. | [16/10] Message A (version courte) envoyé depuis Gmail à 13h42 UTC (registre-envois-2026-10-16.csv) ; adresse précédemment visée par un rejet 5.7.520 côté Hotmail (jamais remise) : premier contact réel. Remise non confirmée.</t>
         </is>
       </c>
       <c r="P36" s="15" t="inlineStr">
@@ -4252,7 +4264,7 @@
           <t>3e liste (12/10)</t>
         </is>
       </c>
-      <c r="Q40" t="inlineStr">
+      <c r="Q40" s="12" t="inlineStr">
         <is>
           <t>pierres.nat@gmail.com</t>
         </is>
@@ -4398,7 +4410,7 @@
           <t>3e liste (12/10)</t>
         </is>
       </c>
-      <c r="Q42" t="inlineStr">
+      <c r="Q42" s="12" t="inlineStr">
         <is>
           <t>contact@raboni.fr</t>
         </is>
@@ -4556,7 +4568,7 @@
           <t>2e liste (12/10)</t>
         </is>
       </c>
-      <c r="Q44" t="inlineStr">
+      <c r="Q44" s="12" t="inlineStr">
         <is>
           <t>contact@materiaux-batiment.fr</t>
         </is>

</xml_diff>

<commit_message>
Send lot 3 sub-batch 1 (Pedrazzini, Ceramico, MPT, Pierres Nat', Raboni) at 08:47 UTC: registry with RFC Message-IDs, trackers to Contacté 17/10; pre-checks green, no replies/bounces on the 9 prior sends
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xqm9tFtdvLdJdkiWw2VVp6
</commit_message>
<xml_diff>
--- a/minyala/clients-potentiels.xlsx
+++ b/minyala/clients-potentiels.xlsx
@@ -2736,14 +2736,22 @@
       </c>
       <c r="L21" s="21" t="inlineStr">
         <is>
-          <t>À contacter</t>
-        </is>
-      </c>
-      <c r="M21" s="21" t="n"/>
-      <c r="N21" s="21" t="n"/>
+          <t>Contacté</t>
+        </is>
+      </c>
+      <c r="M21" s="21" t="inlineStr">
+        <is>
+          <t>17/10/2026</t>
+        </is>
+      </c>
+      <c r="N21" s="21" t="inlineStr">
+        <is>
+          <t>Attendre la réponse ; pas de relance avant le 24/10</t>
+        </is>
+      </c>
       <c r="O21" s="21" t="inlineStr">
         <is>
-          <t>[16/10] E-mail du pied de page/page contact du site officiel pedrazzini.fr (showroom Voisenon confirmé).</t>
+          <t>[16/10] E-mail du pied de page/page contact du site officiel pedrazzini.fr (showroom Voisenon confirmé). | [17/10] Message A (version courte) envoyé depuis Gmail à 08h47 UTC (registre-envois-2026-10-17.csv) ; remise non confirmée.</t>
         </is>
       </c>
       <c r="P21" s="15" t="inlineStr">
@@ -2811,14 +2819,22 @@
       </c>
       <c r="L22" s="21" t="inlineStr">
         <is>
-          <t>À contacter</t>
-        </is>
-      </c>
-      <c r="M22" s="21" t="n"/>
-      <c r="N22" s="21" t="n"/>
+          <t>Contacté</t>
+        </is>
+      </c>
+      <c r="M22" s="21" t="inlineStr">
+        <is>
+          <t>17/10/2026</t>
+        </is>
+      </c>
+      <c r="N22" s="21" t="inlineStr">
+        <is>
+          <t>Attendre la réponse ; pas de relance avant le 24/10</t>
+        </is>
+      </c>
       <c r="O22" s="21" t="inlineStr">
         <is>
-          <t>[16/10] E-mail du magasin de Sarcelles sur ceramico.fr (accueil, bloc « Magasin 1 &amp; Dépôt — Sarcelles »). Ne PAS utiliser commercial@ceramico.fr (magasin du Perreux).</t>
+          <t>[16/10] E-mail du magasin de Sarcelles sur ceramico.fr (accueil, bloc « Magasin 1 &amp; Dépôt — Sarcelles »). Ne PAS utiliser commercial@ceramico.fr (magasin du Perreux). | [17/10] Message A (version courte) envoyé depuis Gmail à 08h47 UTC (registre-envois-2026-10-17.csv) ; remise non confirmée.</t>
         </is>
       </c>
       <c r="P22" s="15" t="inlineStr">
@@ -3704,14 +3720,22 @@
       </c>
       <c r="L33" s="21" t="inlineStr">
         <is>
-          <t>À contacter</t>
-        </is>
-      </c>
-      <c r="M33" s="21" t="n"/>
-      <c r="N33" s="21" t="n"/>
+          <t>Contacté</t>
+        </is>
+      </c>
+      <c r="M33" s="21" t="inlineStr">
+        <is>
+          <t>17/10/2026</t>
+        </is>
+      </c>
+      <c r="N33" s="21" t="inlineStr">
+        <is>
+          <t>Attendre la réponse ; pas de relance avant le 24/10</t>
+        </is>
+      </c>
       <c r="O33" s="21" t="inlineStr">
         <is>
-          <t>[16/10] E-mail général du pied de page (mpt-marbrier.fr/contact) ; domaine de l'adresse ≠ domaine du site, tel qu'affiché par le site officiel.</t>
+          <t>[16/10] E-mail général du pied de page (mpt-marbrier.fr/contact) ; domaine de l'adresse ≠ domaine du site, tel qu'affiché par le site officiel. | [17/10] Message A (version courte) envoyé depuis Gmail à 08h47 UTC (registre-envois-2026-10-17.csv) ; remise non confirmée.</t>
         </is>
       </c>
       <c r="P33" s="15" t="inlineStr">
@@ -4249,14 +4273,22 @@
       </c>
       <c r="L40" s="21" t="inlineStr">
         <is>
-          <t>À contacter</t>
-        </is>
-      </c>
-      <c r="M40" s="21" t="n"/>
-      <c r="N40" s="21" t="n"/>
+          <t>Contacté</t>
+        </is>
+      </c>
+      <c r="M40" s="21" t="inlineStr">
+        <is>
+          <t>17/10/2026</t>
+        </is>
+      </c>
+      <c r="N40" s="21" t="inlineStr">
+        <is>
+          <t>Attendre la réponse ; pas de relance avant le 24/10</t>
+        </is>
+      </c>
       <c r="O40" s="21" t="inlineStr">
         <is>
-          <t>[16/10] Unique e-mail du site officiel pierres-nat.com (page contact, en-tête, pied de page ; adresse Linas confirmée).</t>
+          <t>[16/10] Unique e-mail du site officiel pierres-nat.com (page contact, en-tête, pied de page ; adresse Linas confirmée). | [17/10] Message A (version courte) envoyé depuis Gmail à 08h47 UTC (registre-envois-2026-10-17.csv) ; remise non confirmée.</t>
         </is>
       </c>
       <c r="P40" s="15" t="inlineStr">
@@ -4395,14 +4427,22 @@
       </c>
       <c r="L42" s="21" t="inlineStr">
         <is>
-          <t>À contacter</t>
-        </is>
-      </c>
-      <c r="M42" s="21" t="n"/>
-      <c r="N42" s="21" t="n"/>
+          <t>Contacté</t>
+        </is>
+      </c>
+      <c r="M42" s="21" t="inlineStr">
+        <is>
+          <t>17/10/2026</t>
+        </is>
+      </c>
+      <c r="N42" s="21" t="inlineStr">
+        <is>
+          <t>Attendre la réponse ; pas de relance avant le 24/10</t>
+        </is>
+      </c>
       <c r="O42" s="21" t="inlineStr">
         <is>
-          <t>[16/10] Adresse générique RABONI IDF lue sur lestudioraboni.fr/mentions-legales — pas propre au showroom de Boulogne (sa page contact = formulaire seul, tél. 01 46 09 54 80). raboni.fr protégé anti-bot.</t>
+          <t>[16/10] Adresse générique RABONI IDF lue sur lestudioraboni.fr/mentions-legales — pas propre au showroom de Boulogne (sa page contact = formulaire seul, tél. 01 46 09 54 80). raboni.fr protégé anti-bot. | [17/10] Message A (version courte) envoyé depuis Gmail à 08h47 UTC (registre-envois-2026-10-17.csv) ; remise non confirmée.</t>
         </is>
       </c>
       <c r="P42" s="15" t="inlineStr">

</xml_diff>

<commit_message>
Ajout 4e liste importateurs (17/10) : 9 cibles vérifiées sur sites officiels
- 7 envoyables P1 : NR Distribution (nrd@, page Grossiste pierre d'Égypte/Sinaï),
  FrancePierre (page GALALA/SINAI PEARL ; domaine au registre-rejets 12/10 jamais livré,
  premier contact légitime), Créa Stone (aucune mention Égypte — Message A standard),
  ELK International (2 500+ conteneurs, pierre d'Égypte au catalogue), Stones Partner
  (conteneurs, Égypte pays partenaire), Européenne de Négoce (UNIQUEMENT cette adresse),
  Azur Pierre Agencement (arrivages réguliers calcaire égyptien en gros)
- La Maison du Pavé : doublon EdN — ne pas contacter
- La Pierre & le Marbre (Aubagne) : aucun e-mail publié — formulaire/tél uniquement
- CSV ré-exporté (garde tarif pro OK), N° dédupliqués

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xqm9tFtdvLdJdkiWw2VVp6
</commit_message>
<xml_diff>
--- a/minyala/clients-potentiels.xlsx
+++ b/minyala/clients-potentiels.xlsx
@@ -18028,31 +18028,671 @@
       </c>
     </row>
     <row r="257" ht="15" customHeight="1" s="13">
-      <c r="L257" s="12" t="n"/>
+      <c r="A257" s="12" t="n">
+        <v>257</v>
+      </c>
+      <c r="B257" s="12" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C257" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D257" s="12" t="inlineStr">
+        <is>
+          <t>Importateur / grossiste</t>
+        </is>
+      </c>
+      <c r="E257" s="12" t="inlineStr">
+        <is>
+          <t>NR Distribution (SARL Natural Rock Distribution)</t>
+        </is>
+      </c>
+      <c r="F257" s="12" t="inlineStr">
+        <is>
+          <t>Avignon (84140)</t>
+        </is>
+      </c>
+      <c r="G257" s="12" t="inlineStr">
+        <is>
+          <t>PACA / Sud-Est</t>
+        </is>
+      </c>
+      <c r="H257" s="12" t="inlineStr">
+        <is>
+          <t>Importateur-grossiste de travertin et pierres naturelles, livre les revendeurs pros dans toute la France depuis son parc d'Avignon ; page dédiée « Grossiste pierre d'Égypte » (pierre extraite au Sinaï) — meilleure adéquation du lot.</t>
+        </is>
+      </c>
+      <c r="I257" s="12" t="inlineStr">
+        <is>
+          <t>https://www.nr-distribution.fr/</t>
+        </is>
+      </c>
+      <c r="K257" s="12" t="inlineStr">
+        <is>
+          <t>Site officiel (vérifié 17/10)</t>
+        </is>
+      </c>
+      <c r="L257" s="12" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="N257" s="12" t="inlineStr">
+        <is>
+          <t>Envoi programmé lundi 19/10 (Message A + ligne importateur, ≤10/jour, contrôles standard avant envoi)</t>
+        </is>
+      </c>
+      <c r="O257" s="12" t="inlineStr">
+        <is>
+          <t>[17/10] E-mail lu sur les mentions légales (https://www.nr-distribution.fr/mentions-legales/) — la page contact n'a qu'un formulaire, sans e-mail ni téléphone. Page Égypte : nr-distribution.fr/nos-prestations/grossiste-pierre-degypte-en-normandie/. Vérifié sur site officiel le 17/10.</t>
+        </is>
+      </c>
+      <c r="P257" s="12" t="inlineStr">
+        <is>
+          <t>4e liste — importateurs (17/10)</t>
+        </is>
+      </c>
+      <c r="Q257" s="12" t="inlineStr">
+        <is>
+          <t>nrd@nr-distribution.fr</t>
+        </is>
+      </c>
     </row>
     <row r="258" ht="15" customHeight="1" s="13">
-      <c r="L258" s="12" t="n"/>
+      <c r="A258" s="12" t="n">
+        <v>258</v>
+      </c>
+      <c r="B258" s="12" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C258" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D258" s="12" t="inlineStr">
+        <is>
+          <t>Importateur / grossiste</t>
+        </is>
+      </c>
+      <c r="E258" s="12" t="inlineStr">
+        <is>
+          <t>FrancePierre</t>
+        </is>
+      </c>
+      <c r="F258" s="12" t="inlineStr">
+        <is>
+          <t>Paris (75007) — showrooms Nîmes, Béziers, Périgueux</t>
+        </is>
+      </c>
+      <c r="G258" s="12" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="H258" s="12" t="inlineStr">
+        <is>
+          <t>Page dédiée pierre d'Égypte (variétés GALALA et SINAI PEARL) ; se présente en « fabricant de pierre naturelle — vente directe » plutôt que grossiste.</t>
+        </is>
+      </c>
+      <c r="I258" s="12" t="inlineStr">
+        <is>
+          <t>https://www.francepierre.fr/</t>
+        </is>
+      </c>
+      <c r="K258" s="12" t="inlineStr">
+        <is>
+          <t>Site officiel (vérifié 17/10)</t>
+        </is>
+      </c>
+      <c r="L258" s="12" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="N258" s="12" t="inlineStr">
+        <is>
+          <t>Envoi programmé lundi 19/10 (Message A + ligne importateur, ≤10/jour, contrôles standard avant envoi)</t>
+        </is>
+      </c>
+      <c r="O258" s="12" t="inlineStr">
+        <is>
+          <t>[17/10] E-mail confirmé sur l'accueil, le pied de page et la page Égypte (francepierre.fr/pierres-d-ailleurs/pierre-d-egypte/). Domaine francepierre.fr au registre-rejets du 12/10 (5.7.520 — jamais livré) : premier contact légitime. Positionnement « sur mesure, sans volume » — accroche lot fin de stock adaptée.</t>
+        </is>
+      </c>
+      <c r="P258" s="12" t="inlineStr">
+        <is>
+          <t>4e liste — importateurs (17/10)</t>
+        </is>
+      </c>
+      <c r="Q258" s="12" t="inlineStr">
+        <is>
+          <t>contact@francepierre.fr</t>
+        </is>
+      </c>
     </row>
     <row r="259" ht="15" customHeight="1" s="13">
-      <c r="L259" s="12" t="n"/>
+      <c r="A259" s="12" t="n">
+        <v>259</v>
+      </c>
+      <c r="B259" s="12" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C259" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D259" s="12" t="inlineStr">
+        <is>
+          <t>Négoce / revendeur</t>
+        </is>
+      </c>
+      <c r="E259" s="12" t="inlineStr">
+        <is>
+          <t>Créa Stone (CREA STONE)</t>
+        </is>
+      </c>
+      <c r="F259" s="12" t="inlineStr">
+        <is>
+          <t>Feillens (01570) ; siège Brignoles (83170)</t>
+        </is>
+      </c>
+      <c r="G259" s="12" t="inlineStr">
+        <is>
+          <t>Ain / Var</t>
+        </is>
+      </c>
+      <c r="H259" s="12" t="inlineStr">
+        <is>
+          <t>« Fournisseur et grossiste de pierre naturelle » (site dallage-pierre.com ; crea-stone.com y redirige).</t>
+        </is>
+      </c>
+      <c r="I259" s="12" t="inlineStr">
+        <is>
+          <t>https://dallage-pierre.com/</t>
+        </is>
+      </c>
+      <c r="J259" s="12" t="inlineStr">
+        <is>
+          <t>04 12 16 05 26</t>
+        </is>
+      </c>
+      <c r="K259" s="12" t="inlineStr">
+        <is>
+          <t>Site officiel (vérifié 17/10)</t>
+        </is>
+      </c>
+      <c r="L259" s="12" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="N259" s="12" t="inlineStr">
+        <is>
+          <t>Envoi programmé lundi 19/10 (Message A + ligne importateur, ≤10/jour, contrôles standard avant envoi)</t>
+        </is>
+      </c>
+      <c r="O259" s="12" t="inlineStr">
+        <is>
+          <t>[17/10] E-mail confirmé au pied de page de dallage-pierre.com. AUCUNE mention de l'Égypte sur le site (cite le marbre de Turquie) — ne pas le présenter comme importateur de calcaire égyptien : Message A standard uniquement, sans ligne importateur.</t>
+        </is>
+      </c>
+      <c r="P259" s="12" t="inlineStr">
+        <is>
+          <t>4e liste — importateurs (17/10)</t>
+        </is>
+      </c>
+      <c r="Q259" s="12" t="inlineStr">
+        <is>
+          <t>info@crea-stone.com</t>
+        </is>
+      </c>
     </row>
     <row r="260" ht="15" customHeight="1" s="13">
-      <c r="L260" s="12" t="n"/>
+      <c r="A260" s="12" t="n">
+        <v>260</v>
+      </c>
+      <c r="B260" s="12" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C260" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D260" s="12" t="inlineStr">
+        <is>
+          <t>Importateur / grossiste</t>
+        </is>
+      </c>
+      <c r="E260" s="12" t="inlineStr">
+        <is>
+          <t>ELK International</t>
+        </is>
+      </c>
+      <c r="F260" s="12" t="inlineStr">
+        <is>
+          <t>La Roche-Jaudy (22450)</t>
+        </is>
+      </c>
+      <c r="G260" s="12" t="inlineStr">
+        <is>
+          <t>Bretagne</t>
+        </is>
+      </c>
+      <c r="H260" s="12" t="inlineStr">
+        <is>
+          <t>« Importateur direct de pierre naturelle » (2 500+ conteneurs importés, approvisionnement direct en carrière/usine) ; « PIERRE D'EGYPTE » figure au catalogue.</t>
+        </is>
+      </c>
+      <c r="I260" s="12" t="inlineStr">
+        <is>
+          <t>https://www.elk-international.com</t>
+        </is>
+      </c>
+      <c r="K260" s="12" t="inlineStr">
+        <is>
+          <t>Site officiel (vérifié 17/10)</t>
+        </is>
+      </c>
+      <c r="L260" s="12" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="N260" s="12" t="inlineStr">
+        <is>
+          <t>Envoi programmé lundi 19/10 (Message A + ligne importateur, ≤10/jour, contrôles standard avant envoi)</t>
+        </is>
+      </c>
+      <c r="O260" s="12" t="inlineStr">
+        <is>
+          <t>[17/10] E-mail lu sur la page d'accueil du site officiel. Gamme : grès, granit, ardoise, porphyre, calcaire, travertin. Vérifié sur site officiel le 17/10.</t>
+        </is>
+      </c>
+      <c r="P260" s="12" t="inlineStr">
+        <is>
+          <t>4e liste — importateurs (17/10)</t>
+        </is>
+      </c>
+      <c r="Q260" s="12" t="inlineStr">
+        <is>
+          <t>contact@elk-international.com</t>
+        </is>
+      </c>
     </row>
     <row r="261" ht="15" customHeight="1" s="13">
-      <c r="L261" s="12" t="n"/>
+      <c r="A261" s="12" t="n">
+        <v>261</v>
+      </c>
+      <c r="B261" s="12" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C261" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D261" s="12" t="inlineStr">
+        <is>
+          <t>Importateur / grossiste</t>
+        </is>
+      </c>
+      <c r="E261" s="12" t="inlineStr">
+        <is>
+          <t>Stones Partner</t>
+        </is>
+      </c>
+      <c r="F261" s="12" t="inlineStr">
+        <is>
+          <t>Mouazé (35250)</t>
+        </is>
+      </c>
+      <c r="G261" s="12" t="inlineStr">
+        <is>
+          <t>Bretagne</t>
+        </is>
+      </c>
+      <c r="H261" s="12" t="inlineStr">
+        <is>
+          <t>Importateur B2B pour distributeurs de matériaux d'aménagement, « commander en container ou en commande groupée » ; l'Égypte figure parmi ses « Pays Partner ».</t>
+        </is>
+      </c>
+      <c r="I261" s="12" t="inlineStr">
+        <is>
+          <t>https://www.stonespartner.com</t>
+        </is>
+      </c>
+      <c r="J261" s="12" t="inlineStr">
+        <is>
+          <t>02 99 54 97 50</t>
+        </is>
+      </c>
+      <c r="K261" s="12" t="inlineStr">
+        <is>
+          <t>Site officiel (vérifié 17/10)</t>
+        </is>
+      </c>
+      <c r="L261" s="12" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="N261" s="12" t="inlineStr">
+        <is>
+          <t>Envoi programmé lundi 19/10 (Message A + ligne importateur, ≤10/jour, contrôles standard avant envoi)</t>
+        </is>
+      </c>
+      <c r="O261" s="12" t="inlineStr">
+        <is>
+          <t>[17/10] E-mail lu sur le site officiel. Gammes : travertin, grès, tandur, ardoise, parements. Vérifié sur site officiel le 17/10.</t>
+        </is>
+      </c>
+      <c r="P261" s="12" t="inlineStr">
+        <is>
+          <t>4e liste — importateurs (17/10)</t>
+        </is>
+      </c>
+      <c r="Q261" s="12" t="inlineStr">
+        <is>
+          <t>contact@stonespartner.com</t>
+        </is>
+      </c>
     </row>
     <row r="262" ht="15" customHeight="1" s="13">
-      <c r="L262" s="12" t="n"/>
+      <c r="A262" s="12" t="n">
+        <v>262</v>
+      </c>
+      <c r="B262" s="12" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C262" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D262" s="12" t="inlineStr">
+        <is>
+          <t>Importateur / grossiste</t>
+        </is>
+      </c>
+      <c r="E262" s="12" t="inlineStr">
+        <is>
+          <t>Européenne de Négoce</t>
+        </is>
+      </c>
+      <c r="F262" s="12" t="inlineStr">
+        <is>
+          <t>Pontarmé (60520)</t>
+        </is>
+      </c>
+      <c r="G262" s="12" t="inlineStr">
+        <is>
+          <t>Hauts-de-France</t>
+        </is>
+      </c>
+      <c r="H262" s="12" t="inlineStr">
+        <is>
+          <t>« Distributeur et importateur de pierres naturelles » (pavés, bordures, dallages ; catégorie pavés calcaire) avec parc de stockage à Pontarmé (~12 000 m² selon Opalis — le chiffre de 40 000 m² n'est pas confirmé).</t>
+        </is>
+      </c>
+      <c r="I262" s="12" t="inlineStr">
+        <is>
+          <t>https://www.europeennedenegoce.fr</t>
+        </is>
+      </c>
+      <c r="K262" s="12" t="inlineStr">
+        <is>
+          <t>Site officiel (vérifié 17/10)</t>
+        </is>
+      </c>
+      <c r="L262" s="12" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="N262" s="12" t="inlineStr">
+        <is>
+          <t>Envoi programmé lundi 19/10 (Message A + ligne importateur, ≤10/jour, contrôles standard avant envoi)</t>
+        </is>
+      </c>
+      <c r="O262" s="12" t="inlineStr">
+        <is>
+          <t>[17/10] E-mail lu en clair sur europeennedenegoce.fr. Contacter UNIQUEMENT europeennedenegoce@orange.fr — La Maison du Pavé (lamaisondupave.fr) est la MÊME entreprise (même adresse à Pontarmé, confirmé sur les deux sites) : jamais les deux adresses.</t>
+        </is>
+      </c>
+      <c r="P262" s="12" t="inlineStr">
+        <is>
+          <t>4e liste — importateurs (17/10)</t>
+        </is>
+      </c>
+      <c r="Q262" s="12" t="inlineStr">
+        <is>
+          <t>europeennedenegoce@orange.fr</t>
+        </is>
+      </c>
     </row>
     <row r="263" ht="15" customHeight="1" s="13">
-      <c r="L263" s="12" t="n"/>
+      <c r="A263" s="12" t="n">
+        <v>263</v>
+      </c>
+      <c r="B263" s="12" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C263" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D263" s="12" t="inlineStr">
+        <is>
+          <t>Importateur / grossiste</t>
+        </is>
+      </c>
+      <c r="E263" s="12" t="inlineStr">
+        <is>
+          <t>Azur Pierre Agencement</t>
+        </is>
+      </c>
+      <c r="F263" s="12" t="inlineStr">
+        <is>
+          <t>Grasse (06130)</t>
+        </is>
+      </c>
+      <c r="G263" s="12" t="inlineStr">
+        <is>
+          <t>PACA</t>
+        </is>
+      </c>
+      <c r="H263" s="12" t="inlineStr">
+        <is>
+          <t>Importateur-grossiste approvisionné « directement depuis les carrières partenaires » : « arrivages réguliers de pierres calcaires d'Égypte … en gros », « dalles calcaires égyptiennes en grand format » — très bonne adéquation.</t>
+        </is>
+      </c>
+      <c r="I263" s="12" t="inlineStr">
+        <is>
+          <t>https://www.azurpierre.com</t>
+        </is>
+      </c>
+      <c r="J263" s="12" t="inlineStr">
+        <is>
+          <t>04 69 00 16 12</t>
+        </is>
+      </c>
+      <c r="K263" s="12" t="inlineStr">
+        <is>
+          <t>Site officiel (vérifié 17/10)</t>
+        </is>
+      </c>
+      <c r="L263" s="12" t="inlineStr">
+        <is>
+          <t>À contacter</t>
+        </is>
+      </c>
+      <c r="N263" s="12" t="inlineStr">
+        <is>
+          <t>Envoi programmé lundi 19/10 (Message A + ligne importateur, ≤10/jour, contrôles standard avant envoi)</t>
+        </is>
+      </c>
+      <c r="O263" s="12" t="inlineStr">
+        <is>
+          <t>[17/10] E-mail lu sur la page contact (azurpierre.com/contact) et au pied de page. Téléphone du site = celui fourni (04 69 00 16 12). Vérifié sur site officiel le 17/10.</t>
+        </is>
+      </c>
+      <c r="P263" s="12" t="inlineStr">
+        <is>
+          <t>4e liste — importateurs (17/10)</t>
+        </is>
+      </c>
+      <c r="Q263" s="12" t="inlineStr">
+        <is>
+          <t>info@azurpierre.com</t>
+        </is>
+      </c>
     </row>
     <row r="264" ht="15" customHeight="1" s="13">
-      <c r="L264" s="12" t="n"/>
+      <c r="A264" s="12" t="n">
+        <v>264</v>
+      </c>
+      <c r="B264" s="12" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C264" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="D264" s="12" t="inlineStr">
+        <is>
+          <t>Doublon (e-commerce EdN)</t>
+        </is>
+      </c>
+      <c r="E264" s="12" t="inlineStr">
+        <is>
+          <t>La Maison du Pavé</t>
+        </is>
+      </c>
+      <c r="F264" s="12" t="inlineStr">
+        <is>
+          <t>Pontarmé (60520) — même adresse qu'Européenne de Négoce</t>
+        </is>
+      </c>
+      <c r="G264" s="12" t="inlineStr">
+        <is>
+          <t>Hauts-de-France</t>
+        </is>
+      </c>
+      <c r="H264" s="12" t="inlineStr">
+        <is>
+          <t>Boutique e-commerce de l'Européenne de Négoce (pavés, dallages, margelles, bordures).</t>
+        </is>
+      </c>
+      <c r="I264" s="12" t="inlineStr">
+        <is>
+          <t>https://www.lamaisondupave.fr</t>
+        </is>
+      </c>
+      <c r="K264" s="12" t="inlineStr">
+        <is>
+          <t>Site officiel (vérifié 17/10)</t>
+        </is>
+      </c>
+      <c r="L264" s="12" t="inlineStr">
+        <is>
+          <t>Doublon — ne pas contacter</t>
+        </is>
+      </c>
+      <c r="N264" s="12" t="inlineStr">
+        <is>
+          <t>Aucune — passer par Européenne de Négoce uniquement</t>
+        </is>
+      </c>
+      <c r="O264" s="12" t="inlineStr">
+        <is>
+          <t>[17/10] MÊME entreprise que l'Européenne de Négoce (confirmé sur les deux sites : « Qui sommes-nous ? », pied de page, même adresse 5003F Route de Paris). NE PAS CONTACTER — doublon. (Adresse contact@lamaisondupave.fr décodée de la protection anti-spam : ne pas l'utiliser.)</t>
+        </is>
+      </c>
+      <c r="P264" s="12" t="inlineStr">
+        <is>
+          <t>4e liste — importateurs (17/10)</t>
+        </is>
+      </c>
     </row>
     <row r="265" ht="15" customHeight="1" s="13">
-      <c r="L265" s="12" t="n"/>
+      <c r="A265" s="12" t="n">
+        <v>265</v>
+      </c>
+      <c r="B265" s="12" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C265" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D265" s="12" t="inlineStr">
+        <is>
+          <t>Importateur / grossiste</t>
+        </is>
+      </c>
+      <c r="E265" s="12" t="inlineStr">
+        <is>
+          <t>La Pierre &amp; le Marbre</t>
+        </is>
+      </c>
+      <c r="F265" s="12" t="inlineStr">
+        <is>
+          <t>Aubagne (13400)</t>
+        </is>
+      </c>
+      <c r="G265" s="12" t="inlineStr">
+        <is>
+          <t>PACA</t>
+        </is>
+      </c>
+      <c r="H265" s="12" t="inlineStr">
+        <is>
+          <t>Importateur-grossiste de marbre, pierre naturelle, granit près de Marseille ; pages prestations dédiées « Achat et vente de pierre d'Égypte, pierre du Sinaï » — la pierre d'Égypte est explicitement au catalogue.</t>
+        </is>
+      </c>
+      <c r="I265" s="12" t="inlineStr">
+        <is>
+          <t>https://lapierreetlemarbre.com</t>
+        </is>
+      </c>
+      <c r="J265" s="12" t="inlineStr">
+        <is>
+          <t>04 42 70 12 44</t>
+        </is>
+      </c>
+      <c r="K265" s="12" t="inlineStr">
+        <is>
+          <t>Site officiel (vérifié 17/10)</t>
+        </is>
+      </c>
+      <c r="L265" s="12" t="inlineStr">
+        <is>
+          <t>À contacter (formulaire/tél)</t>
+        </is>
+      </c>
+      <c r="N265" s="12" t="inlineStr">
+        <is>
+          <t>Contacter via le formulaire https://lapierreetlemarbre.com/contact/ ou par téléphone — AUCUN e-mail publié, ne pas deviner d'adresse</t>
+        </is>
+      </c>
+      <c r="O265" s="12" t="inlineStr">
+        <is>
+          <t>[17/10] Aucune adresse e-mail publiée (page contact = formulaire seul ; mentions légales vides ; vérifié aussi sur l'accueil et les pages prestations). Tél 04 42 70 12 44, fax 04 42 70 12 45.</t>
+        </is>
+      </c>
+      <c r="P265" s="12" t="inlineStr">
+        <is>
+          <t>4e liste — importateurs (17/10)</t>
+        </is>
+      </c>
     </row>
     <row r="266" ht="15" customHeight="1" s="13">
       <c r="L266" s="12" t="n"/>

</xml_diff>

<commit_message>
Lot 3 sous-lot 2 envoyé (17/10 11:06 UTC) : Sedelka, SNNMC, Solmur Évreux, Tendance Carrelage Rouen
- 4 envois Message A version courte, Message-ID RFC au registre du 17/10
- Statuts « Contacté » 17/10 dans les deux classeurs, relance pas avant le 24/10
- Scan Gmail avant envoi : aucune réponse humaine, aucun STOP, aucun rebond
- Découverte : Décomarbre (16/10) et Pillaud Caen (15/10) derrière Mailinblack —
  envois RETENUS par le filtre anti-robot, validation expéditeur manuelle requise
  (action propriétaire) ; noté dans les classeurs
- Quota du jour : 9/10

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xqm9tFtdvLdJdkiWw2VVp6
</commit_message>
<xml_diff>
--- a/minyala/clients-potentiels.xlsx
+++ b/minyala/clients-potentiels.xlsx
@@ -1899,7 +1899,7 @@
       </c>
       <c r="O10" s="21" t="inlineStr">
         <is>
-          <t>[13/10] Page agence de Caen du site Pillaud. | [15/10] Message A (version courte) envoyé depuis Gmail (constaté dans les éléments envoyés, voir registre-envois-2026-10-15.csv) ; remise non confirmée, aucune réponse au 16/10.</t>
+          <t>[13/10] Page agence de Caen du site Pillaud. | [15/10] Message A (version courte) envoyé depuis Gmail (constaté dans les éléments envoyés, voir registre-envois-2026-10-15.csv) ; remise non confirmée, aucune réponse au 16/10. [17/10] Mailinblack : l'envoi du 15/10 est RETENU par le filtre anti-robot du destinataire (invitations reçues 15/10) — message non remis tant que l'expéditeur n'est pas validé manuellement (action côté propriétaire).</t>
         </is>
       </c>
       <c r="P10" s="15" t="inlineStr">
@@ -1967,14 +1967,22 @@
       </c>
       <c r="L11" s="21" t="inlineStr">
         <is>
-          <t>À contacter</t>
-        </is>
-      </c>
-      <c r="M11" s="21" t="n"/>
-      <c r="N11" s="21" t="n"/>
+          <t>Contacté</t>
+        </is>
+      </c>
+      <c r="M11" s="21" t="inlineStr">
+        <is>
+          <t>17/10/2026</t>
+        </is>
+      </c>
+      <c r="N11" s="21" t="inlineStr">
+        <is>
+          <t>Attendre la réponse ; pas de relance avant le 24/10</t>
+        </is>
+      </c>
       <c r="O11" s="21" t="inlineStr">
         <is>
-          <t>[16/10] E-mail de l'éditeur sur sedelka.fr/mentions-legales (dpo@ réservé aux données personnelles).</t>
+          <t>[16/10] E-mail de l'éditeur sur sedelka.fr/mentions-legales (dpo@ réservé aux données personnelles). E-mail de prospection MINYALA (Message A version courte) du 17/10 — sous-lot 2.</t>
         </is>
       </c>
       <c r="P11" s="15" t="inlineStr">
@@ -2038,14 +2046,22 @@
       </c>
       <c r="L12" s="21" t="inlineStr">
         <is>
-          <t>À contacter</t>
-        </is>
-      </c>
-      <c r="M12" s="21" t="n"/>
-      <c r="N12" s="21" t="n"/>
+          <t>Contacté</t>
+        </is>
+      </c>
+      <c r="M12" s="21" t="inlineStr">
+        <is>
+          <t>17/10/2026</t>
+        </is>
+      </c>
+      <c r="N12" s="21" t="inlineStr">
+        <is>
+          <t>Attendre la réponse ; pas de relance avant le 24/10</t>
+        </is>
+      </c>
       <c r="O12" s="21" t="inlineStr">
         <is>
-          <t>[16/10] E-mail « Espace Pro » de la fiche agence Évreux sur solmur.fr (tél. 02 32 62 94 80). Ne PAS utiliser espace.pro.bihorel@ (pied de page = siège Bihorel).</t>
+          <t>[16/10] E-mail « Espace Pro » de la fiche agence Évreux sur solmur.fr (tél. 02 32 62 94 80). Ne PAS utiliser espace.pro.bihorel@ (pied de page = siège Bihorel). E-mail de prospection MINYALA (Message A version courte) du 17/10 — sous-lot 2.</t>
         </is>
       </c>
       <c r="P12" s="15" t="inlineStr">
@@ -2113,14 +2129,22 @@
       </c>
       <c r="L13" s="21" t="inlineStr">
         <is>
-          <t>À contacter</t>
-        </is>
-      </c>
-      <c r="M13" s="21" t="n"/>
-      <c r="N13" s="21" t="n"/>
+          <t>Contacté</t>
+        </is>
+      </c>
+      <c r="M13" s="21" t="inlineStr">
+        <is>
+          <t>17/10/2026</t>
+        </is>
+      </c>
+      <c r="N13" s="21" t="inlineStr">
+        <is>
+          <t>Attendre la réponse ; pas de relance avant le 24/10</t>
+        </is>
+      </c>
       <c r="O13" s="21" t="inlineStr">
         <is>
-          <t>[16/10] Seule adresse affichée sur le site officiel (page contact) — semi-nominative sur hotmail.com, pas de générique. À utiliser telle quelle.</t>
+          <t>[16/10] Seule adresse affichée sur le site officiel (page contact) — semi-nominative sur hotmail.com, pas de générique. À utiliser telle quelle. E-mail de prospection MINYALA (Message A version courte) du 17/10 — sous-lot 2.</t>
         </is>
       </c>
       <c r="P13" s="15" t="inlineStr">
@@ -2917,7 +2941,7 @@
       </c>
       <c r="O23" s="21" t="inlineStr">
         <is>
-          <t>[13/10] Tentative depuis Hotmail rejetée EN SORTIE (5.7.520 : contenu classé spam par Microsoft) — message non remis ; l'adresse n'est pas forcément invalide. Prochain contact depuis la boîte Gmail, nouveau modèle, jamais depuis Hotmail. | [16/10] Message A (version courte) envoyé depuis Gmail à 10h38 UTC (registre-envois-2026-10-16.csv) ; adresse précédemment visée par un rejet 5.7.520 côté Hotmail (jamais remise) : ceci est le premier contact réel. Remise non confirmée.</t>
+          <t>[13/10] Tentative depuis Hotmail rejetée EN SORTIE (5.7.520 : contenu classé spam par Microsoft) — message non remis ; l'adresse n'est pas forcément invalide. Prochain contact depuis la boîte Gmail, nouveau modèle, jamais depuis Hotmail. | [16/10] Message A (version courte) envoyé depuis Gmail à 10h38 UTC (registre-envois-2026-10-16.csv) ; adresse précédemment visée par un rejet 5.7.520 côté Hotmail (jamais remise) : ceci est le premier contact réel. Remise non confirmée. [17/10] Mailinblack : l'envoi du 16/10 est RETENU par le filtre anti-robot du destinataire (invitation reçue 16/10 10:38 UTC) — message non remis tant que l'expéditeur n'est pas validé manuellement (action côté propriétaire).</t>
         </is>
       </c>
       <c r="P23" s="15" t="inlineStr">
@@ -4593,14 +4617,22 @@
       </c>
       <c r="L44" s="21" t="inlineStr">
         <is>
-          <t>À contacter</t>
-        </is>
-      </c>
-      <c r="M44" s="21" t="n"/>
-      <c r="N44" s="21" t="n"/>
+          <t>Contacté</t>
+        </is>
+      </c>
+      <c r="M44" s="21" t="inlineStr">
+        <is>
+          <t>17/10/2026</t>
+        </is>
+      </c>
+      <c r="N44" s="21" t="inlineStr">
+        <is>
+          <t>Attendre la réponse ; pas de relance avant le 24/10</t>
+        </is>
+      </c>
       <c r="O44" s="21" t="inlineStr">
         <is>
-          <t>[13/10] Aucun e-mail propre à SNNMC publié : formulaire sur la fiche France Matériaux, ou téléphone. | [16/10] E-mail du site officiel materiaux-batiment.fr (accueil + page contact, itemprop=email). Site parfois en 503 : réessayer. Ne PAS utiliser contact@france-materiaux.fr (réseau, pas SNNMC).</t>
+          <t>[13/10] Aucun e-mail propre à SNNMC publié : formulaire sur la fiche France Matériaux, ou téléphone. | [16/10] E-mail du site officiel materiaux-batiment.fr (accueil + page contact, itemprop=email). Site parfois en 503 : réessayer. Ne PAS utiliser contact@france-materiaux.fr (réseau, pas SNNMC). E-mail de prospection MINYALA (Message A version courte) du 17/10 — sous-lot 2.</t>
         </is>
       </c>
       <c r="P44" s="15" t="inlineStr">

</xml_diff>

<commit_message>
Lot importateurs envoyé (24/10 10:33 UTC, Gmail direct) : 6 cibles ; EdN retirée (négociation en cours)
- 6 envois Message A + ligne importateur (Créa Stone sans la ligne), Message-ID RFC
  au registre du 24/10 — via connecteur Gmail direct (Zapier toujours bloqué)
- Européenne de Négoce RETIRÉE du lot : négociation déjà en cours depuis le 19/10
  sur le fil Hotmail du propriétaire (1 500 m² à 25,90 €/m² livré Pontarmé ;
  photos du lot envoyées le 22/10) — statut « En négociation », ne pas prospecter
- Scan Gmail : aucun bounce, aucun STOP ; Décomarbre/Pillaud toujours sous Mailinblack
- Statuts « Contacté 24/10 », relance pas avant le 31/10 ; CSV ré-exporté (garde OK)

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xqm9tFtdvLdJdkiWw2VVp6
</commit_message>
<xml_diff>
--- a/minyala/clients-potentiels.xlsx
+++ b/minyala/clients-potentiels.xlsx
@@ -18108,17 +18108,22 @@
       </c>
       <c r="L257" s="12" t="inlineStr">
         <is>
-          <t>À contacter</t>
+          <t>Contacté</t>
+        </is>
+      </c>
+      <c r="M257" t="inlineStr">
+        <is>
+          <t>24/10/2026</t>
         </is>
       </c>
       <c r="N257" s="12" t="inlineStr">
         <is>
-          <t>Envoi programmé lundi 19/10 (Message A + ligne importateur, ≤10/jour, contrôles standard avant envoi)</t>
+          <t>Attendre la réponse ; pas de relance avant le 31/10</t>
         </is>
       </c>
       <c r="O257" s="12" t="inlineStr">
         <is>
-          <t>[17/10] E-mail lu sur les mentions légales (https://www.nr-distribution.fr/mentions-legales/) — la page contact n'a qu'un formulaire, sans e-mail ni téléphone. Page Égypte : nr-distribution.fr/nos-prestations/grossiste-pierre-degypte-en-normandie/. Vérifié sur site officiel le 17/10.</t>
+          <t>[17/10] E-mail lu sur les mentions légales (https://www.nr-distribution.fr/mentions-legales/) — la page contact n'a qu'un formulaire, sans e-mail ni téléphone. Page Égypte : nr-distribution.fr/nos-prestations/grossiste-pierre-degypte-en-normandie/. Vérifié sur site officiel le 17/10. E-mail de prospection MINYALA (Message A + ligne importateur ; Créa Stone sans la ligne) du 24/10 — connecteur Gmail direct.</t>
         </is>
       </c>
       <c r="P257" s="12" t="inlineStr">
@@ -18181,17 +18186,22 @@
       </c>
       <c r="L258" s="12" t="inlineStr">
         <is>
-          <t>À contacter</t>
+          <t>Contacté</t>
+        </is>
+      </c>
+      <c r="M258" t="inlineStr">
+        <is>
+          <t>24/10/2026</t>
         </is>
       </c>
       <c r="N258" s="12" t="inlineStr">
         <is>
-          <t>Envoi programmé lundi 19/10 (Message A + ligne importateur, ≤10/jour, contrôles standard avant envoi)</t>
+          <t>Attendre la réponse ; pas de relance avant le 31/10</t>
         </is>
       </c>
       <c r="O258" s="12" t="inlineStr">
         <is>
-          <t>[17/10] E-mail confirmé sur l'accueil, le pied de page et la page Égypte (francepierre.fr/pierres-d-ailleurs/pierre-d-egypte/). Domaine francepierre.fr au registre-rejets du 12/10 (5.7.520 — jamais livré) : premier contact légitime. Positionnement « sur mesure, sans volume » — accroche lot fin de stock adaptée.</t>
+          <t>[17/10] E-mail confirmé sur l'accueil, le pied de page et la page Égypte (francepierre.fr/pierres-d-ailleurs/pierre-d-egypte/). Domaine francepierre.fr au registre-rejets du 12/10 (5.7.520 — jamais livré) : premier contact légitime. Positionnement « sur mesure, sans volume » — accroche lot fin de stock adaptée. E-mail de prospection MINYALA (Message A + ligne importateur ; Créa Stone sans la ligne) du 24/10 — connecteur Gmail direct.</t>
         </is>
       </c>
       <c r="P258" s="12" t="inlineStr">
@@ -18259,17 +18269,22 @@
       </c>
       <c r="L259" s="12" t="inlineStr">
         <is>
-          <t>À contacter</t>
+          <t>Contacté</t>
+        </is>
+      </c>
+      <c r="M259" t="inlineStr">
+        <is>
+          <t>24/10/2026</t>
         </is>
       </c>
       <c r="N259" s="12" t="inlineStr">
         <is>
-          <t>Envoi programmé lundi 19/10 (Message A + ligne importateur, ≤10/jour, contrôles standard avant envoi)</t>
+          <t>Attendre la réponse ; pas de relance avant le 31/10</t>
         </is>
       </c>
       <c r="O259" s="12" t="inlineStr">
         <is>
-          <t>[17/10] E-mail confirmé au pied de page de dallage-pierre.com. AUCUNE mention de l'Égypte sur le site (cite le marbre de Turquie) — ne pas le présenter comme importateur de calcaire égyptien : Message A standard uniquement, sans ligne importateur.</t>
+          <t>[17/10] E-mail confirmé au pied de page de dallage-pierre.com. AUCUNE mention de l'Égypte sur le site (cite le marbre de Turquie) — ne pas le présenter comme importateur de calcaire égyptien : Message A standard uniquement, sans ligne importateur. E-mail de prospection MINYALA (Message A + ligne importateur ; Créa Stone sans la ligne) du 24/10 — connecteur Gmail direct.</t>
         </is>
       </c>
       <c r="P259" s="12" t="inlineStr">
@@ -18332,17 +18347,22 @@
       </c>
       <c r="L260" s="12" t="inlineStr">
         <is>
-          <t>À contacter</t>
+          <t>Contacté</t>
+        </is>
+      </c>
+      <c r="M260" t="inlineStr">
+        <is>
+          <t>24/10/2026</t>
         </is>
       </c>
       <c r="N260" s="12" t="inlineStr">
         <is>
-          <t>Envoi programmé lundi 19/10 (Message A + ligne importateur, ≤10/jour, contrôles standard avant envoi)</t>
+          <t>Attendre la réponse ; pas de relance avant le 31/10</t>
         </is>
       </c>
       <c r="O260" s="12" t="inlineStr">
         <is>
-          <t>[17/10] E-mail lu sur la page d'accueil du site officiel. Gamme : grès, granit, ardoise, porphyre, calcaire, travertin. Vérifié sur site officiel le 17/10.</t>
+          <t>[17/10] E-mail lu sur la page d'accueil du site officiel. Gamme : grès, granit, ardoise, porphyre, calcaire, travertin. Vérifié sur site officiel le 17/10. E-mail de prospection MINYALA (Message A + ligne importateur ; Créa Stone sans la ligne) du 24/10 — connecteur Gmail direct.</t>
         </is>
       </c>
       <c r="P260" s="12" t="inlineStr">
@@ -18410,17 +18430,22 @@
       </c>
       <c r="L261" s="12" t="inlineStr">
         <is>
-          <t>À contacter</t>
+          <t>Contacté</t>
+        </is>
+      </c>
+      <c r="M261" t="inlineStr">
+        <is>
+          <t>24/10/2026</t>
         </is>
       </c>
       <c r="N261" s="12" t="inlineStr">
         <is>
-          <t>Envoi programmé lundi 19/10 (Message A + ligne importateur, ≤10/jour, contrôles standard avant envoi)</t>
+          <t>Attendre la réponse ; pas de relance avant le 31/10</t>
         </is>
       </c>
       <c r="O261" s="12" t="inlineStr">
         <is>
-          <t>[17/10] E-mail lu sur le site officiel. Gammes : travertin, grès, tandur, ardoise, parements. Vérifié sur site officiel le 17/10.</t>
+          <t>[17/10] E-mail lu sur le site officiel. Gammes : travertin, grès, tandur, ardoise, parements. Vérifié sur site officiel le 17/10. E-mail de prospection MINYALA (Message A + ligne importateur ; Créa Stone sans la ligne) du 24/10 — connecteur Gmail direct.</t>
         </is>
       </c>
       <c r="P261" s="12" t="inlineStr">
@@ -18483,17 +18508,22 @@
       </c>
       <c r="L262" s="12" t="inlineStr">
         <is>
-          <t>À contacter</t>
+          <t>En négociation — canal propriétaire (Hotmail)</t>
+        </is>
+      </c>
+      <c r="M262" t="inlineStr">
+        <is>
+          <t>19/10/2026</t>
         </is>
       </c>
       <c r="N262" s="12" t="inlineStr">
         <is>
-          <t>Envoi programmé lundi 19/10 (Message A + ligne importateur, ≤10/jour, contrôles standard avant envoi)</t>
+          <t>NE PAS prospecter — négociation en cours menée par Joseph depuis joseph.hanna@hotmail.fr (fil « MINYALA - À l'attention du service achats »)</t>
         </is>
       </c>
       <c r="O262" s="12" t="inlineStr">
         <is>
-          <t>[17/10] E-mail lu en clair sur europeennedenegoce.fr. Contacter UNIQUEMENT europeennedenegoce@orange.fr — La Maison du Pavé (lamaisondupave.fr) est la MÊME entreprise (même adresse à Pontarmé, confirmé sur les deux sites) : jamais les deux adresses.</t>
+          <t>[17/10] E-mail lu en clair sur europeennedenegoce.fr. Contacter UNIQUEMENT europeennedenegoce@orange.fr — La Maison du Pavé (lamaisondupave.fr) est la MÊME entreprise (même adresse à Pontarmé, confirmé sur les deux sites) : jamais les deux adresses. [24/10] Négociation DÉJÀ EN COURS, découverte dans Gmail (cc info@pierredegypte.online) : 19/10 proposition du propriétaire 1 500 m² à 25,90 €/m² livraison Pontarmé incluse, prix ferme ; 19/10 justification vs 35 €/m² public (2 cm vs 1,2 cm) ; 22/10 PHOTOS du lot envoyées (prises le jour même) avec invitation à faire une offre. Une seule voie de contact : le fil Hotmail du propriétaire. Retiré du lot d'envoi du 24/10.</t>
         </is>
       </c>
       <c r="P262" s="12" t="inlineStr">
@@ -18561,17 +18591,22 @@
       </c>
       <c r="L263" s="12" t="inlineStr">
         <is>
-          <t>À contacter</t>
+          <t>Contacté</t>
+        </is>
+      </c>
+      <c r="M263" t="inlineStr">
+        <is>
+          <t>24/10/2026</t>
         </is>
       </c>
       <c r="N263" s="12" t="inlineStr">
         <is>
-          <t>Envoi programmé lundi 19/10 (Message A + ligne importateur, ≤10/jour, contrôles standard avant envoi)</t>
+          <t>Attendre la réponse ; pas de relance avant le 31/10</t>
         </is>
       </c>
       <c r="O263" s="12" t="inlineStr">
         <is>
-          <t>[17/10] E-mail lu sur la page contact (azurpierre.com/contact) et au pied de page. Téléphone du site = celui fourni (04 69 00 16 12). Vérifié sur site officiel le 17/10.</t>
+          <t>[17/10] E-mail lu sur la page contact (azurpierre.com/contact) et au pied de page. Téléphone du site = celui fourni (04 69 00 16 12). Vérifié sur site officiel le 17/10. E-mail de prospection MINYALA (Message A + ligne importateur ; Créa Stone sans la ligne) du 24/10 — connecteur Gmail direct.</t>
         </is>
       </c>
       <c r="P263" s="12" t="inlineStr">

</xml_diff>

<commit_message>
FrancePierre : réponse du 24/10 et négociation en cours (14 € HT/m² × 500 m² proposé) — statut « En négociation »
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xqm9tFtdvLdJdkiWw2VVp6
</commit_message>
<xml_diff>
--- a/minyala/clients-potentiels.xlsx
+++ b/minyala/clients-potentiels.xlsx
@@ -18111,7 +18111,7 @@
           <t>Contacté</t>
         </is>
       </c>
-      <c r="M257" t="inlineStr">
+      <c r="M257" s="12" t="inlineStr">
         <is>
           <t>24/10/2026</t>
         </is>
@@ -18186,22 +18186,22 @@
       </c>
       <c r="L258" s="12" t="inlineStr">
         <is>
-          <t>Contacté</t>
-        </is>
-      </c>
-      <c r="M258" t="inlineStr">
+          <t>En négociation</t>
+        </is>
+      </c>
+      <c r="M258" s="12" t="inlineStr">
         <is>
           <t>24/10/2026</t>
         </is>
       </c>
       <c r="N258" s="12" t="inlineStr">
         <is>
-          <t>Attendre la réponse ; pas de relance avant le 31/10</t>
+          <t>Relancer ou appeler Laurent Plainchamp (06 79 17 55 43) si silence — dernier mot à nous le 24/10 11:31 UTC</t>
         </is>
       </c>
       <c r="O258" s="12" t="inlineStr">
         <is>
-          <t>[17/10] E-mail confirmé sur l'accueil, le pied de page et la page Égypte (francepierre.fr/pierres-d-ailleurs/pierre-d-egypte/). Domaine francepierre.fr au registre-rejets du 12/10 (5.7.520 — jamais livré) : premier contact légitime. Positionnement « sur mesure, sans volume » — accroche lot fin de stock adaptée. E-mail de prospection MINYALA (Message A + ligne importateur ; Créa Stone sans la ligne) du 24/10 — connecteur Gmail direct.</t>
+          <t>[17/10] E-mail confirmé sur l'accueil, le pied de page et la page Égypte (francepierre.fr/pierres-d-ailleurs/pierre-d-egypte/). Domaine francepierre.fr au registre-rejets du 12/10 (5.7.520 — jamais livré) : premier contact légitime. Positionnement « sur mesure, sans volume » — accroche lot fin de stock adaptée. E-mail de prospection MINYALA (Message A + ligne importateur ; Créa Stone sans la ligne) du 24/10 — connecteur Gmail direct. [25/10] RÉPONSE le 24/10 (1 min après l'envoi !) — Laurent PLAINCHAMP, 06 79 17 55 43, francepierrecontact@gmail.com : « En dallage pourquoi pas » ; achète les dallages à 14 € HT. Négociation menée par le propriétaire depuis la boîte le 24/10 : offre faite 14 € HT/m² × 500 m² = 7 000 € HT, enlèvement par leurs soins, 30 % d'acompte ; FP « Non, nous pensions avoir mieux » ; tenue du 14 € (11:31 UTC). Dernier mot à nous — relance/appel conseillé si silence. NE PAS re-prospecter : négociation en cours.</t>
         </is>
       </c>
       <c r="P258" s="12" t="inlineStr">
@@ -18272,7 +18272,7 @@
           <t>Contacté</t>
         </is>
       </c>
-      <c r="M259" t="inlineStr">
+      <c r="M259" s="12" t="inlineStr">
         <is>
           <t>24/10/2026</t>
         </is>
@@ -18350,7 +18350,7 @@
           <t>Contacté</t>
         </is>
       </c>
-      <c r="M260" t="inlineStr">
+      <c r="M260" s="12" t="inlineStr">
         <is>
           <t>24/10/2026</t>
         </is>
@@ -18433,7 +18433,7 @@
           <t>Contacté</t>
         </is>
       </c>
-      <c r="M261" t="inlineStr">
+      <c r="M261" s="12" t="inlineStr">
         <is>
           <t>24/10/2026</t>
         </is>
@@ -18511,7 +18511,7 @@
           <t>En négociation — canal propriétaire (Hotmail)</t>
         </is>
       </c>
-      <c r="M262" t="inlineStr">
+      <c r="M262" s="12" t="inlineStr">
         <is>
           <t>19/10/2026</t>
         </is>
@@ -18594,7 +18594,7 @@
           <t>Contacté</t>
         </is>
       </c>
-      <c r="M263" t="inlineStr">
+      <c r="M263" s="12" t="inlineStr">
         <is>
           <t>24/10/2026</t>
         </is>

</xml_diff>

<commit_message>
Mailinblack validé le 25/10 (Décomarbre, Pillaud) : messages remis, relance pas avant le 01/11
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xqm9tFtdvLdJdkiWw2VVp6
</commit_message>
<xml_diff>
--- a/minyala/clients-potentiels.xlsx
+++ b/minyala/clients-potentiels.xlsx
@@ -1894,12 +1894,12 @@
       </c>
       <c r="N10" s="21" t="inlineStr">
         <is>
-          <t>Attendre la réponse ; pas de relance avant le 22/10</t>
+          <t>Attendre la réponse ; pas de relance avant le 01/11 (message remis le 25/10 après validation Mailinblack)</t>
         </is>
       </c>
       <c r="O10" s="21" t="inlineStr">
         <is>
-          <t>[13/10] Page agence de Caen du site Pillaud. | [15/10] Message A (version courte) envoyé depuis Gmail (constaté dans les éléments envoyés, voir registre-envois-2026-10-15.csv) ; remise non confirmée, aucune réponse au 16/10. [17/10] Mailinblack : l'envoi du 15/10 est RETENU par le filtre anti-robot du destinataire (invitations reçues 15/10) — message non remis tant que l'expéditeur n'est pas validé manuellement (action côté propriétaire).</t>
+          <t>[13/10] Page agence de Caen du site Pillaud. | [15/10] Message A (version courte) envoyé depuis Gmail (constaté dans les éléments envoyés, voir registre-envois-2026-10-15.csv) ; remise non confirmée, aucune réponse au 16/10. [17/10] Mailinblack : l'envoi du 15/10 est RETENU par le filtre anti-robot du destinataire (invitations reçues 15/10) — message non remis tant que l'expéditeur n'est pas validé manuellement (action côté propriétaire). [25/10] Mailinblack VALIDÉ par le propriétaire le 25/10 — le message initial est maintenant remis en boîte de réception. Horloge de réponse repartie du 25/10 : pas de relance avant le 01/11.</t>
         </is>
       </c>
       <c r="P10" s="15" t="inlineStr">
@@ -2936,12 +2936,12 @@
       </c>
       <c r="N23" s="21" t="inlineStr">
         <is>
-          <t>Attendre la réponse ; pas de relance avant le 23/10</t>
+          <t>Attendre la réponse ; pas de relance avant le 01/11 (message remis le 25/10 après validation Mailinblack)</t>
         </is>
       </c>
       <c r="O23" s="21" t="inlineStr">
         <is>
-          <t>[13/10] Tentative depuis Hotmail rejetée EN SORTIE (5.7.520 : contenu classé spam par Microsoft) — message non remis ; l'adresse n'est pas forcément invalide. Prochain contact depuis la boîte Gmail, nouveau modèle, jamais depuis Hotmail. | [16/10] Message A (version courte) envoyé depuis Gmail à 10h38 UTC (registre-envois-2026-10-16.csv) ; adresse précédemment visée par un rejet 5.7.520 côté Hotmail (jamais remise) : ceci est le premier contact réel. Remise non confirmée. [17/10] Mailinblack : l'envoi du 16/10 est RETENU par le filtre anti-robot du destinataire (invitation reçue 16/10 10:38 UTC) — message non remis tant que l'expéditeur n'est pas validé manuellement (action côté propriétaire).</t>
+          <t>[13/10] Tentative depuis Hotmail rejetée EN SORTIE (5.7.520 : contenu classé spam par Microsoft) — message non remis ; l'adresse n'est pas forcément invalide. Prochain contact depuis la boîte Gmail, nouveau modèle, jamais depuis Hotmail. | [16/10] Message A (version courte) envoyé depuis Gmail à 10h38 UTC (registre-envois-2026-10-16.csv) ; adresse précédemment visée par un rejet 5.7.520 côté Hotmail (jamais remise) : ceci est le premier contact réel. Remise non confirmée. [17/10] Mailinblack : l'envoi du 16/10 est RETENU par le filtre anti-robot du destinataire (invitation reçue 16/10 10:38 UTC) — message non remis tant que l'expéditeur n'est pas validé manuellement (action côté propriétaire). [25/10] Mailinblack VALIDÉ par le propriétaire le 25/10 — le message initial est maintenant remis en boîte de réception. Horloge de réponse repartie du 25/10 : pas de relance avant le 01/11.</t>
         </is>
       </c>
       <c r="P23" s="15" t="inlineStr">

</xml_diff>

<commit_message>
Rectifications propriétaire 25/10 : EdN = refus du 19/10 (réouverture tentée, pas une négociation) ; FrancePierre = négociation ouverte sans accord ferme ; preuves Mailinblack datées
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xqm9tFtdvLdJdkiWw2VVp6
</commit_message>
<xml_diff>
--- a/minyala/clients-potentiels.xlsx
+++ b/minyala/clients-potentiels.xlsx
@@ -1899,7 +1899,7 @@
       </c>
       <c r="O10" s="21" t="inlineStr">
         <is>
-          <t>[13/10] Page agence de Caen du site Pillaud. | [15/10] Message A (version courte) envoyé depuis Gmail (constaté dans les éléments envoyés, voir registre-envois-2026-10-15.csv) ; remise non confirmée, aucune réponse au 16/10. [17/10] Mailinblack : l'envoi du 15/10 est RETENU par le filtre anti-robot du destinataire (invitations reçues 15/10) — message non remis tant que l'expéditeur n'est pas validé manuellement (action côté propriétaire). [25/10] Mailinblack VALIDÉ par le propriétaire le 25/10 — le message initial est maintenant remis en boîte de réception. Horloge de réponse repartie du 25/10 : pas de relance avant le 01/11.</t>
+          <t>[13/10] Page agence de Caen du site Pillaud. | [15/10] Message A (version courte) envoyé depuis Gmail (constaté dans les éléments envoyés, voir registre-envois-2026-10-15.csv) ; remise non confirmée, aucune réponse au 16/10. [17/10] Mailinblack : l'envoi du 15/10 est RETENU par le filtre anti-robot du destinataire (invitations reçues 15/10) — message non remis tant que l'expéditeur n'est pas validé manuellement (action côté propriétaire). [25/10] Mailinblack VALIDÉ par le propriétaire le 25/10 — le message initial est maintenant remis en boîte de réception. Horloge de réponse repartie du 25/10 : pas de relance avant le 01/11. Preuve de retenue : invitations Mailinblack du 15/10 10:52/11:07 UTC, Gmail ids 1a13f3269baf04e3 et 1a13f3ed5f4dd439.</t>
         </is>
       </c>
       <c r="P10" s="15" t="inlineStr">
@@ -2941,7 +2941,7 @@
       </c>
       <c r="O23" s="21" t="inlineStr">
         <is>
-          <t>[13/10] Tentative depuis Hotmail rejetée EN SORTIE (5.7.520 : contenu classé spam par Microsoft) — message non remis ; l'adresse n'est pas forcément invalide. Prochain contact depuis la boîte Gmail, nouveau modèle, jamais depuis Hotmail. | [16/10] Message A (version courte) envoyé depuis Gmail à 10h38 UTC (registre-envois-2026-10-16.csv) ; adresse précédemment visée par un rejet 5.7.520 côté Hotmail (jamais remise) : ceci est le premier contact réel. Remise non confirmée. [17/10] Mailinblack : l'envoi du 16/10 est RETENU par le filtre anti-robot du destinataire (invitation reçue 16/10 10:38 UTC) — message non remis tant que l'expéditeur n'est pas validé manuellement (action côté propriétaire). [25/10] Mailinblack VALIDÉ par le propriétaire le 25/10 — le message initial est maintenant remis en boîte de réception. Horloge de réponse repartie du 25/10 : pas de relance avant le 01/11.</t>
+          <t>[13/10] Tentative depuis Hotmail rejetée EN SORTIE (5.7.520 : contenu classé spam par Microsoft) — message non remis ; l'adresse n'est pas forcément invalide. Prochain contact depuis la boîte Gmail, nouveau modèle, jamais depuis Hotmail. | [16/10] Message A (version courte) envoyé depuis Gmail à 10h38 UTC (registre-envois-2026-10-16.csv) ; adresse précédemment visée par un rejet 5.7.520 côté Hotmail (jamais remise) : ceci est le premier contact réel. Remise non confirmée. [17/10] Mailinblack : l'envoi du 16/10 est RETENU par le filtre anti-robot du destinataire (invitation reçue 16/10 10:38 UTC) — message non remis tant que l'expéditeur n'est pas validé manuellement (action côté propriétaire). [25/10] Mailinblack VALIDÉ par le propriétaire le 25/10 — le message initial est maintenant remis en boîte de réception. Horloge de réponse repartie du 25/10 : pas de relance avant le 01/11. Preuve de retenue : invitation Mailinblack du 16/10 10:38 UTC, Gmail id 1a1444aca3b8edcd.</t>
         </is>
       </c>
       <c r="P23" s="15" t="inlineStr">
@@ -18201,7 +18201,7 @@
       </c>
       <c r="O258" s="12" t="inlineStr">
         <is>
-          <t>[17/10] E-mail confirmé sur l'accueil, le pied de page et la page Égypte (francepierre.fr/pierres-d-ailleurs/pierre-d-egypte/). Domaine francepierre.fr au registre-rejets du 12/10 (5.7.520 — jamais livré) : premier contact légitime. Positionnement « sur mesure, sans volume » — accroche lot fin de stock adaptée. E-mail de prospection MINYALA (Message A + ligne importateur ; Créa Stone sans la ligne) du 24/10 — connecteur Gmail direct. [25/10] RÉPONSE le 24/10 (1 min après l'envoi !) — Laurent PLAINCHAMP, 06 79 17 55 43, francepierrecontact@gmail.com : « En dallage pourquoi pas » ; achète les dallages à 14 € HT. Négociation menée par le propriétaire depuis la boîte le 24/10 : offre faite 14 € HT/m² × 500 m² = 7 000 € HT, enlèvement par leurs soins, 30 % d'acompte ; FP « Non, nous pensions avoir mieux » ; tenue du 14 € (11:31 UTC). Dernier mot à nous — relance/appel conseillé si silence. NE PAS re-prospecter : négociation en cours.</t>
+          <t>[17/10] E-mail confirmé sur l'accueil, le pied de page et la page Égypte (francepierre.fr/pierres-d-ailleurs/pierre-d-egypte/). Domaine francepierre.fr au registre-rejets du 12/10 (5.7.520 — jamais livré) : premier contact légitime. Positionnement « sur mesure, sans volume » — accroche lot fin de stock adaptée. E-mail de prospection MINYALA (Message A + ligne importateur ; Créa Stone sans la ligne) du 24/10 — connecteur Gmail direct. [25/10] RÉPONSE le 24/10 (1 min après l'envoi !) — Laurent PLAINCHAMP, 06 79 17 55 43, francepierrecontact@gmail.com : « En dallage pourquoi pas » ; achète les dallages à 14 € HT. Négociation menée par le propriétaire depuis la boîte le 24/10 : offre faite 14 € HT/m² × 500 m² = 7 000 € HT, enlèvement par leurs soins, 30 % d'acompte ; FP « Non, nous pensions avoir mieux » ; tenue du 14 € (11:31 UTC). Dernier mot à nous — relance/appel conseillé si silence. NE PAS re-prospecter : négociation en cours. [25/10, rectif propriétaire] Négociation OUVERTE seulement : aucun accord ferme, aucun acompte confirmé — la dernière réponse de FP est « Non, nous pensions avoir mieux ».</t>
         </is>
       </c>
       <c r="P258" s="12" t="inlineStr">
@@ -18508,7 +18508,7 @@
       </c>
       <c r="L262" s="12" t="inlineStr">
         <is>
-          <t>En négociation — canal propriétaire (Hotmail)</t>
+          <t>Refus le 19/10 — réouverture tentée (photos 22/10), en attente</t>
         </is>
       </c>
       <c r="M262" s="12" t="inlineStr">
@@ -18518,12 +18518,12 @@
       </c>
       <c r="N262" s="12" t="inlineStr">
         <is>
-          <t>NE PAS prospecter — négociation en cours menée par Joseph depuis joseph.hanna@hotmail.fr (fil « MINYALA - À l'attention du service achats »)</t>
+          <t>Ne reclasser « En négociation » QUE sur réponse de réouverture d'EdN (fil Hotmail du propriétaire) ; sinon statuer « Sans réponse — clos » après ~10 jours</t>
         </is>
       </c>
       <c r="O262" s="12" t="inlineStr">
         <is>
-          <t>[17/10] E-mail lu en clair sur europeennedenegoce.fr. Contacter UNIQUEMENT europeennedenegoce@orange.fr — La Maison du Pavé (lamaisondupave.fr) est la MÊME entreprise (même adresse à Pontarmé, confirmé sur les deux sites) : jamais les deux adresses. [24/10] Négociation DÉJÀ EN COURS, découverte dans Gmail (cc info@pierredegypte.online) : 19/10 proposition du propriétaire 1 500 m² à 25,90 €/m² livraison Pontarmé incluse, prix ferme ; 19/10 justification vs 35 €/m² public (2 cm vs 1,2 cm) ; 22/10 PHOTOS du lot envoyées (prises le jour même) avec invitation à faire une offre. Une seule voie de contact : le fil Hotmail du propriétaire. Retiré du lot d'envoi du 24/10.</t>
+          <t>[17/10] E-mail lu en clair sur europeennedenegoce.fr. Contacter UNIQUEMENT europeennedenegoce@orange.fr — La Maison du Pavé (lamaisondupave.fr) est la MÊME entreprise (même adresse à Pontarmé, confirmé sur les deux sites) : jamais les deux adresses. [24/10] Négociation DÉJÀ EN COURS, découverte dans Gmail (cc info@pierredegypte.online) : 19/10 proposition du propriétaire 1 500 m² à 25,90 €/m² livraison Pontarmé incluse, prix ferme ; 19/10 justification vs 35 €/m² public (2 cm vs 1,2 cm) ; 22/10 PHOTOS du lot envoyées (prises le jour même) avec invitation à faire une offre. Une seule voie de contact : le fil Hotmail du propriétaire. Retiré du lot d'envoi du 24/10. [25/10, rectif propriétaire] La dernière réponse EXPLICITE d'EdN est un REFUS le 19/10. L'envoi des photos du 22/10 est une tentative de réouverture, pas une négociation en cours : attendre une réponse de réouverture avant tout reclassement.</t>
         </is>
       </c>
       <c r="P262" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Ajout prospect « Entreprise Koita » (demande propriétaire 26/10) — coordonnées à confirmer avant tout envoi
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xqm9tFtdvLdJdkiWw2VVp6
</commit_message>
<xml_diff>
--- a/minyala/clients-potentiels.xlsx
+++ b/minyala/clients-potentiels.xlsx
@@ -18762,7 +18762,67 @@
       </c>
     </row>
     <row r="266" ht="15" customHeight="1" s="13">
-      <c r="L266" s="12" t="n"/>
+      <c r="A266" t="n">
+        <v>266</v>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C266" t="n">
+        <v>2</v>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>À qualifier</t>
+        </is>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>Entreprise Koita</t>
+        </is>
+      </c>
+      <c r="F266" t="inlineStr">
+        <is>
+          <t>À préciser</t>
+        </is>
+      </c>
+      <c r="G266" t="inlineStr">
+        <is>
+          <t>À préciser</t>
+        </is>
+      </c>
+      <c r="H266" t="inlineStr">
+        <is>
+          <t>Ajout direct du propriétaire — activité à qualifier.</t>
+        </is>
+      </c>
+      <c r="K266" t="inlineStr">
+        <is>
+          <t>Propriétaire (26/10)</t>
+        </is>
+      </c>
+      <c r="L266" s="12" t="inlineStr">
+        <is>
+          <t>À contacter (coordonnées manquantes)</t>
+        </is>
+      </c>
+      <c r="N266" t="inlineStr">
+        <is>
+          <t>Obtenir du propriétaire (ou vérifier sur site officiel) : activité, ville, e-mail — puis Message A avec les contrôles standard</t>
+        </is>
+      </c>
+      <c r="O266" t="inlineStr">
+        <is>
+          <t>[26/10] Ajout demandé par le propriétaire (« entreprise Koita »). Coordonnées, ville et activité à préciser — aucune adresse e-mail connue : NE PAS envoyer tant que l'e-mail n'est pas confirmé (risque d'homonymie).</t>
+        </is>
+      </c>
+      <c r="P266" t="inlineStr">
+        <is>
+          <t>Ajout propriétaire (26/10)</t>
+        </is>
+      </c>
     </row>
     <row r="267" ht="15" customHeight="1" s="13">
       <c r="L267" s="12" t="n"/>

</xml_diff>

<commit_message>
KOITA RENOVATION identifiée (Clamart 92, SIREN 921 863 296) : fiche complétée, priorité 1, canaux tél/Instagram/intro Waldy — pas d'e-mail publié
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xqm9tFtdvLdJdkiWw2VVp6
</commit_message>
<xml_diff>
--- a/minyala/clients-potentiels.xlsx
+++ b/minyala/clients-potentiels.xlsx
@@ -18762,63 +18762,68 @@
       </c>
     </row>
     <row r="266" ht="15" customHeight="1" s="13">
-      <c r="A266" t="n">
+      <c r="A266" s="12" t="n">
         <v>266</v>
       </c>
-      <c r="B266" t="inlineStr">
+      <c r="B266" s="12" t="inlineStr">
         <is>
           <t>Pro France</t>
         </is>
       </c>
-      <c r="C266" t="n">
-        <v>2</v>
-      </c>
-      <c r="D266" t="inlineStr">
-        <is>
-          <t>À qualifier</t>
-        </is>
-      </c>
-      <c r="E266" t="inlineStr">
-        <is>
-          <t>Entreprise Koita</t>
-        </is>
-      </c>
-      <c r="F266" t="inlineStr">
-        <is>
-          <t>À préciser</t>
-        </is>
-      </c>
-      <c r="G266" t="inlineStr">
-        <is>
-          <t>À préciser</t>
-        </is>
-      </c>
-      <c r="H266" t="inlineStr">
-        <is>
-          <t>Ajout direct du propriétaire — activité à qualifier.</t>
-        </is>
-      </c>
-      <c r="K266" t="inlineStr">
+      <c r="C266" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D266" s="12" t="inlineStr">
+        <is>
+          <t>Rénovation / plomberie-chauffage</t>
+        </is>
+      </c>
+      <c r="E266" s="12" t="inlineStr">
+        <is>
+          <t>KOITA RENOVATION (Entreprise Koita)</t>
+        </is>
+      </c>
+      <c r="F266" s="12" t="inlineStr">
+        <is>
+          <t>Clamart (92140)</t>
+        </is>
+      </c>
+      <c r="G266" s="12" t="inlineStr">
+        <is>
+          <t>Île-de-France</t>
+        </is>
+      </c>
+      <c r="H266" s="12" t="inlineStr">
+        <is>
+          <t>Rénovation générale / plomberie / chauffage en Île-de-France — chantiers salle de bains et sols visibles sur son Instagram (236 K abonnés, compte vérifié) : acheteur potentiel de dallage pour ses chantiers, et relais d'audience possible.</t>
+        </is>
+      </c>
+      <c r="J266" t="inlineStr">
+        <is>
+          <t>06 12 38 05 34</t>
+        </is>
+      </c>
+      <c r="K266" s="12" t="inlineStr">
         <is>
           <t>Propriétaire (26/10)</t>
         </is>
       </c>
       <c r="L266" s="12" t="inlineStr">
         <is>
-          <t>À contacter (coordonnées manquantes)</t>
-        </is>
-      </c>
-      <c r="N266" t="inlineStr">
-        <is>
-          <t>Obtenir du propriétaire (ou vérifier sur site officiel) : activité, ville, e-mail — puis Message A avec les contrôles standard</t>
-        </is>
-      </c>
-      <c r="O266" t="inlineStr">
-        <is>
-          <t>[26/10] Ajout demandé par le propriétaire (« entreprise Koita »). Coordonnées, ville et activité à préciser — aucune adresse e-mail connue : NE PAS envoyer tant que l'e-mail n'est pas confirmé (risque d'homonymie).</t>
-        </is>
-      </c>
-      <c r="P266" t="inlineStr">
+          <t>À contacter (tél/Instagram — pas d’e-mail)</t>
+        </is>
+      </c>
+      <c r="N266" s="12" t="inlineStr">
+        <is>
+          <t>Choisir le canal (appel 06 12 38 05 34, DM Instagram, ou intro par Waldy) — action propriétaire ; pas d'e-mail connu</t>
+        </is>
+      </c>
+      <c r="O266" s="12" t="inlineStr">
+        <is>
+          <t>[26/10] Identifiée : KOITA RENOVATION, SAS au capital de 7 000 €, 7 rue du Nivernais 92140 CLAMART (même département que le dépôt !), SIREN 921 863 296, président Abodalahy Koita, créée le 18/10/2022 (source : fiche légale via recherche web + profil Instagram @entreprise_koita fourni par le propriétaire). AUCUN e-mail ni site web publiés. Canaux possibles : tél 06 12 38 05 34 (bio Instagram), DM Instagram, ou INTRO CHALEUREUSE via Waldy (waldy_nz suit le compte). UNE SEULE VOIE : choix du propriétaire ; pas d'e-mail possible à ce stade.</t>
+        </is>
+      </c>
+      <c r="P266" s="12" t="inlineStr">
         <is>
           <t>Ajout propriétaire (26/10)</t>
         </is>

</xml_diff>

<commit_message>
5e liste (relais 26/10) : 14 nouveaux prospects + 2 fiches enrichies (Granits et Matériaux, Marbres et Tendances) + mémo marchés publics Rennes — AUCUN ENVOI
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xqm9tFtdvLdJdkiWw2VVp6
</commit_message>
<xml_diff>
--- a/minyala/clients-potentiels.xlsx
+++ b/minyala/clients-potentiels.xlsx
@@ -6148,7 +6148,7 @@
       </c>
       <c r="J68" s="15" t="inlineStr">
         <is>
-          <t>02 35 75 64 07</t>
+          <t>06 60 18 31 14</t>
         </is>
       </c>
       <c r="K68" s="20" t="inlineStr">
@@ -6162,11 +6162,24 @@
         </is>
       </c>
       <c r="M68" s="21" t="n"/>
-      <c r="N68" s="21" t="n"/>
-      <c r="O68" s="21" t="n"/>
+      <c r="N68" s="21" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi</t>
+        </is>
+      </c>
+      <c r="O68" s="21" t="inlineStr">
+        <is>
+          <t>[26/10] E-mail apporté par le relais tiers : christophe.devaux@granits-materiaux.fr. Showroom marbrerie Le Houlme (76), proche Vernon — proposer visite du stock ou échantillon avant offre volume. Relais assistant tiers du 26/10 (dédupliqué Gmail/Contacts) — e-mail « vérifié » par le relais, à re-confirmer sur site officiel avant envoi. NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi</t>
+        </is>
+      </c>
       <c r="P68" s="15" t="inlineStr">
         <is>
           <t>2e liste (12/10)</t>
+        </is>
+      </c>
+      <c r="Q68" t="inlineStr">
+        <is>
+          <t>christophe.devaux@granits-materiaux.fr</t>
         </is>
       </c>
     </row>
@@ -6810,11 +6823,24 @@
         </is>
       </c>
       <c r="M78" s="21" t="n"/>
-      <c r="N78" s="21" t="n"/>
-      <c r="O78" s="21" t="n"/>
+      <c r="N78" s="21" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi</t>
+        </is>
+      </c>
+      <c r="O78" s="21" t="inlineStr">
+        <is>
+          <t>[26/10] E-mail apporté par le relais tiers : marbrestendances@orange.fr. Eslettes (76) — chantiers sur mesure et petites palettes. Relais assistant tiers du 26/10 (dédupliqué Gmail/Contacts) — e-mail « vérifié » par le relais, à re-confirmer sur site officiel avant envoi. NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi</t>
+        </is>
+      </c>
       <c r="P78" s="15" t="inlineStr">
         <is>
           <t>2e liste (12/10)</t>
+        </is>
+      </c>
+      <c r="Q78" t="inlineStr">
+        <is>
+          <t>marbrestendances@orange.fr</t>
         </is>
       </c>
     </row>
@@ -18798,7 +18824,7 @@
           <t>Rénovation générale / plomberie / chauffage en Île-de-France — chantiers salle de bains et sols visibles sur son Instagram (236 K abonnés, compte vérifié) : acheteur potentiel de dallage pour ses chantiers, et relais d'audience possible.</t>
         </is>
       </c>
-      <c r="J266" t="inlineStr">
+      <c r="J266" s="12" t="inlineStr">
         <is>
           <t>06 12 38 05 34</t>
         </is>
@@ -18830,46 +18856,1036 @@
       </c>
     </row>
     <row r="267" ht="15" customHeight="1" s="13">
-      <c r="L267" s="12" t="n"/>
+      <c r="A267" t="n">
+        <v>267</v>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C267" t="n">
+        <v>1</v>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>Fournisseur dallage/pavage pro+particuli</t>
+        </is>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>Adi Roc</t>
+        </is>
+      </c>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>Evran (22)</t>
+        </is>
+      </c>
+      <c r="G267" t="inlineStr">
+        <is>
+          <t>Bretagne</t>
+        </is>
+      </c>
+      <c r="H267" t="inlineStr">
+        <is>
+          <t>Très forte adéquation : vend déjà de la pierre d'Égypte. Approche : échantillon + lot test puis palettes.</t>
+        </is>
+      </c>
+      <c r="I267" t="inlineStr">
+        <is>
+          <t>https://www.adi-roc.fr</t>
+        </is>
+      </c>
+      <c r="J267" t="inlineStr">
+        <is>
+          <t>06 28 04 92 93</t>
+        </is>
+      </c>
+      <c r="K267" t="inlineStr">
+        <is>
+          <t>Relais assistant (26/10)</t>
+        </is>
+      </c>
+      <c r="L267" s="12" t="inlineStr">
+        <is>
+          <t>À contacter (formulaire/tél) — EN ATTENTE</t>
+        </is>
+      </c>
+      <c r="N267" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi</t>
+        </is>
+      </c>
+      <c r="O267" t="inlineStr">
+        <is>
+          <t>[26/10] Relais assistant tiers du 26/10 (dédupliqué Gmail/Contacts) — e-mail « vérifié » par le relais, à re-confirmer sur site officiel avant envoi. Pas d'e-mail publié : formulaire du site ou téléphone. NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi</t>
+        </is>
+      </c>
+      <c r="P267" t="inlineStr">
+        <is>
+          <t>5e liste — relais (26/10)</t>
+        </is>
+      </c>
     </row>
     <row r="268" ht="15" customHeight="1" s="13">
-      <c r="L268" s="12" t="n"/>
+      <c r="A268" t="n">
+        <v>268</v>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C268" t="n">
+        <v>1</v>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Négoce pavage/dallage, stockage annoncé </t>
+        </is>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>Espace TP Distribution</t>
+        </is>
+      </c>
+      <c r="F268" t="inlineStr">
+        <is>
+          <t>Vaux-le-Pénil (77)</t>
+        </is>
+      </c>
+      <c r="G268" t="inlineStr">
+        <is>
+          <t>Île-de-France</t>
+        </is>
+      </c>
+      <c r="H268" t="inlineStr">
+        <is>
+          <t>Cible majeure pour 25–500 m² ou revente par palettes.</t>
+        </is>
+      </c>
+      <c r="I268" t="inlineStr">
+        <is>
+          <t>https://www.espacetp.fr</t>
+        </is>
+      </c>
+      <c r="J268" t="inlineStr">
+        <is>
+          <t>01 64 19 19 16</t>
+        </is>
+      </c>
+      <c r="K268" t="inlineStr">
+        <is>
+          <t>Relais assistant (26/10)</t>
+        </is>
+      </c>
+      <c r="L268" s="12" t="inlineStr">
+        <is>
+          <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
+        </is>
+      </c>
+      <c r="N268" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi</t>
+        </is>
+      </c>
+      <c r="O268" t="inlineStr">
+        <is>
+          <t>[26/10] Relais assistant tiers du 26/10 (dédupliqué Gmail/Contacts) — e-mail « vérifié » par le relais, à re-confirmer sur site officiel avant envoi.  NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi</t>
+        </is>
+      </c>
+      <c r="P268" t="inlineStr">
+        <is>
+          <t>5e liste — relais (26/10)</t>
+        </is>
+      </c>
+      <c r="Q268" t="inlineStr">
+        <is>
+          <t>contact@espacetp.fr</t>
+        </is>
+      </c>
     </row>
     <row r="269" ht="15" customHeight="1" s="13">
-      <c r="L269" s="12" t="n"/>
+      <c r="A269" t="n">
+        <v>269</v>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C269" t="n">
+        <v>1</v>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>Revendeur pierre naturelle, &gt;1 000 m² d'</t>
+        </is>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>Kei-Stone Les Alluets-le-Roi</t>
+        </is>
+      </c>
+      <c r="F269" t="inlineStr">
+        <is>
+          <t>Les Alluets-le-Roi (78)</t>
+        </is>
+      </c>
+      <c r="G269" t="inlineStr">
+        <is>
+          <t>Île-de-France</t>
+        </is>
+      </c>
+      <c r="H269" t="inlineStr">
+        <is>
+          <t>Présenter MINYALA comme gamme calcaire beige disponible rapidement depuis Gennevilliers.</t>
+        </is>
+      </c>
+      <c r="I269" t="inlineStr">
+        <is>
+          <t>https://www.kei-stone.fr</t>
+        </is>
+      </c>
+      <c r="J269" t="inlineStr">
+        <is>
+          <t>01 39 75 55 60</t>
+        </is>
+      </c>
+      <c r="K269" t="inlineStr">
+        <is>
+          <t>Relais assistant (26/10)</t>
+        </is>
+      </c>
+      <c r="L269" s="12" t="inlineStr">
+        <is>
+          <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
+        </is>
+      </c>
+      <c r="N269" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi</t>
+        </is>
+      </c>
+      <c r="O269" t="inlineStr">
+        <is>
+          <t>[26/10] Relais assistant tiers du 26/10 (dédupliqué Gmail/Contacts) — e-mail « vérifié » par le relais, à re-confirmer sur site officiel avant envoi.  NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi</t>
+        </is>
+      </c>
+      <c r="P269" t="inlineStr">
+        <is>
+          <t>5e liste — relais (26/10)</t>
+        </is>
+      </c>
+      <c r="Q269" t="inlineStr">
+        <is>
+          <t>contact78@kei-stone.fr</t>
+        </is>
+      </c>
     </row>
     <row r="270" ht="15" customHeight="1" s="13">
-      <c r="L270" s="12" t="n"/>
+      <c r="A270" t="n">
+        <v>270</v>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C270" t="n">
+        <v>1</v>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>Négoce avec showroom 350 m² : dalles, pa</t>
+        </is>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>Hestia Pierre &amp; Jardin</t>
+        </is>
+      </c>
+      <c r="F270" t="inlineStr">
+        <is>
+          <t>Hillion (22)</t>
+        </is>
+      </c>
+      <c r="G270" t="inlineStr">
+        <is>
+          <t>Bretagne</t>
+        </is>
+      </c>
+      <c r="H270" t="inlineStr">
+        <is>
+          <t>Partenariat revendeur : échantillon + conditions par palette.</t>
+        </is>
+      </c>
+      <c r="I270" t="inlineStr">
+        <is>
+          <t>https://www.hestia.bzh</t>
+        </is>
+      </c>
+      <c r="J270" t="inlineStr">
+        <is>
+          <t>02 96 52 33 04</t>
+        </is>
+      </c>
+      <c r="K270" t="inlineStr">
+        <is>
+          <t>Relais assistant (26/10)</t>
+        </is>
+      </c>
+      <c r="L270" s="12" t="inlineStr">
+        <is>
+          <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
+        </is>
+      </c>
+      <c r="N270" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi</t>
+        </is>
+      </c>
+      <c r="O270" t="inlineStr">
+        <is>
+          <t>[26/10] Relais assistant tiers du 26/10 (dédupliqué Gmail/Contacts) — e-mail « vérifié » par le relais, à re-confirmer sur site officiel avant envoi.  NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi</t>
+        </is>
+      </c>
+      <c r="P270" t="inlineStr">
+        <is>
+          <t>5e liste — relais (26/10)</t>
+        </is>
+      </c>
+      <c r="Q270" t="inlineStr">
+        <is>
+          <t>bonjour@hestia.bzh</t>
+        </is>
+      </c>
     </row>
     <row r="271" ht="15" customHeight="1" s="13">
-      <c r="L271" s="12" t="n"/>
+      <c r="A271" t="n">
+        <v>271</v>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C271" t="n">
+        <v>1</v>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>Importateur direct de calcaires et pierr</t>
+        </is>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>Dalle Décor</t>
+        </is>
+      </c>
+      <c r="F271" t="inlineStr">
+        <is>
+          <t>Galluis (78)</t>
+        </is>
+      </c>
+      <c r="G271" t="inlineStr">
+        <is>
+          <t>Île-de-France</t>
+        </is>
+      </c>
+      <c r="H271" t="inlineStr">
+        <is>
+          <t>Demander s'ils reprennent des lots déjà importés et disponibles localement.</t>
+        </is>
+      </c>
+      <c r="J271" t="inlineStr">
+        <is>
+          <t>09 74 56 22 36</t>
+        </is>
+      </c>
+      <c r="K271" t="inlineStr">
+        <is>
+          <t>Relais assistant (26/10)</t>
+        </is>
+      </c>
+      <c r="L271" s="12" t="inlineStr">
+        <is>
+          <t>À contacter (formulaire/tél) — EN ATTENTE</t>
+        </is>
+      </c>
+      <c r="N271" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi</t>
+        </is>
+      </c>
+      <c r="O271" t="inlineStr">
+        <is>
+          <t>[26/10] Relais assistant tiers du 26/10 (dédupliqué Gmail/Contacts) — e-mail « vérifié » par le relais, à re-confirmer sur site officiel avant envoi. Pas d'e-mail publié : téléphone. NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi</t>
+        </is>
+      </c>
+      <c r="P271" t="inlineStr">
+        <is>
+          <t>5e liste — relais (26/10)</t>
+        </is>
+      </c>
     </row>
     <row r="272" ht="15" customHeight="1" s="13">
-      <c r="L272" s="12" t="n"/>
+      <c r="A272" t="n">
+        <v>272</v>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C272" t="n">
+        <v>1</v>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>Vente et pose de dallages, pavés, bordur</t>
+        </is>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>Les Paveurs d'Eure-et-Loir</t>
+        </is>
+      </c>
+      <c r="F272" t="inlineStr">
+        <is>
+          <t>Cherisy (28)</t>
+        </is>
+      </c>
+      <c r="G272" t="inlineStr">
+        <is>
+          <t>IdF/Eure/Normandie</t>
+        </is>
+      </c>
+      <c r="H272" t="inlineStr">
+        <is>
+          <t>Très bon profil pour fourniture de lots de 25 à plusieurs centaines de m² (la pose reste la leur).</t>
+        </is>
+      </c>
+      <c r="J272" t="inlineStr">
+        <is>
+          <t>06 87 53 33 76</t>
+        </is>
+      </c>
+      <c r="K272" t="inlineStr">
+        <is>
+          <t>Relais assistant (26/10)</t>
+        </is>
+      </c>
+      <c r="L272" s="12" t="inlineStr">
+        <is>
+          <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
+        </is>
+      </c>
+      <c r="N272" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi</t>
+        </is>
+      </c>
+      <c r="O272" t="inlineStr">
+        <is>
+          <t>[26/10] Relais assistant tiers du 26/10 (dédupliqué Gmail/Contacts) — e-mail « vérifié » par le relais, à re-confirmer sur site officiel avant envoi.  NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi</t>
+        </is>
+      </c>
+      <c r="P272" t="inlineStr">
+        <is>
+          <t>5e liste — relais (26/10)</t>
+        </is>
+      </c>
+      <c r="Q272" t="inlineStr">
+        <is>
+          <t>lespaveurs.eureetloir@orange.fr</t>
+        </is>
+      </c>
     </row>
     <row r="273" ht="15" customHeight="1" s="13">
-      <c r="L273" s="12" t="n"/>
+      <c r="A273" t="n">
+        <v>273</v>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C273" t="n">
+        <v>1</v>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>Fournisseur pierre naturelle constructio</t>
+        </is>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>MC Pierre</t>
+        </is>
+      </c>
+      <c r="F273" t="inlineStr">
+        <is>
+          <t>Courtry (77)</t>
+        </is>
+      </c>
+      <c r="G273" t="inlineStr">
+        <is>
+          <t>Île-de-France</t>
+        </is>
+      </c>
+      <c r="H273" t="inlineStr">
+        <is>
+          <t>Tester l'intérêt pour une gamme complémentaire calcaire égyptien 30×60×2.</t>
+        </is>
+      </c>
+      <c r="J273" t="inlineStr">
+        <is>
+          <t>06 25 28 12 12</t>
+        </is>
+      </c>
+      <c r="K273" t="inlineStr">
+        <is>
+          <t>Relais assistant (26/10)</t>
+        </is>
+      </c>
+      <c r="L273" s="12" t="inlineStr">
+        <is>
+          <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
+        </is>
+      </c>
+      <c r="N273" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi</t>
+        </is>
+      </c>
+      <c r="O273" t="inlineStr">
+        <is>
+          <t>[26/10] Relais assistant tiers du 26/10 (dédupliqué Gmail/Contacts) — e-mail « vérifié » par le relais, à re-confirmer sur site officiel avant envoi.  NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi</t>
+        </is>
+      </c>
+      <c r="P273" t="inlineStr">
+        <is>
+          <t>5e liste — relais (26/10)</t>
+        </is>
+      </c>
+      <c r="Q273" t="inlineStr">
+        <is>
+          <t>contact@mc-pierre.com</t>
+        </is>
+      </c>
     </row>
     <row r="274" ht="15" customHeight="1" s="13">
-      <c r="L274" s="12" t="n"/>
+      <c r="A274" t="n">
+        <v>274</v>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C274" t="n">
+        <v>2</v>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>Bureau d'études paysager + showroom, ven</t>
+        </is>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>Esprit Vert Design</t>
+        </is>
+      </c>
+      <c r="F274" t="inlineStr">
+        <is>
+          <t>Ploërmel (56)</t>
+        </is>
+      </c>
+      <c r="G274" t="inlineStr">
+        <is>
+          <t>Bretagne</t>
+        </is>
+      </c>
+      <c r="H274" t="inlineStr">
+        <is>
+          <t>Fiche architecte (photos, texture, dimensions, prix) adaptée.</t>
+        </is>
+      </c>
+      <c r="J274" t="inlineStr">
+        <is>
+          <t>02 97 72 97 51</t>
+        </is>
+      </c>
+      <c r="K274" t="inlineStr">
+        <is>
+          <t>Relais assistant (26/10)</t>
+        </is>
+      </c>
+      <c r="L274" s="12" t="inlineStr">
+        <is>
+          <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
+        </is>
+      </c>
+      <c r="N274" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi</t>
+        </is>
+      </c>
+      <c r="O274" t="inlineStr">
+        <is>
+          <t>[26/10] Relais assistant tiers du 26/10 (dédupliqué Gmail/Contacts) — e-mail « vérifié » par le relais, à re-confirmer sur site officiel avant envoi.  NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi</t>
+        </is>
+      </c>
+      <c r="P274" t="inlineStr">
+        <is>
+          <t>5e liste — relais (26/10)</t>
+        </is>
+      </c>
+      <c r="Q274" t="inlineStr">
+        <is>
+          <t>contact@esprit-vert-design.fr</t>
+        </is>
+      </c>
     </row>
     <row r="275" ht="15" customHeight="1" s="13">
-      <c r="L275" s="12" t="n"/>
+      <c r="A275" t="n">
+        <v>275</v>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C275" t="n">
+        <v>2</v>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Terrassement et aménagements : dallage, </t>
+        </is>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>Guevel TP</t>
+        </is>
+      </c>
+      <c r="F275" t="inlineStr">
+        <is>
+          <t>Betton (35)</t>
+        </is>
+      </c>
+      <c r="G275" t="inlineStr">
+        <is>
+          <t>Bretagne</t>
+        </is>
+      </c>
+      <c r="H275" t="inlineStr">
+        <is>
+          <t>Pierre pour terrasses/aménagements privés — ne pas lier l'offre à un marché public précis.</t>
+        </is>
+      </c>
+      <c r="I275" t="inlineStr">
+        <is>
+          <t>https://www.guevel-tp.fr</t>
+        </is>
+      </c>
+      <c r="J275" t="inlineStr">
+        <is>
+          <t>06 08 40 35 42</t>
+        </is>
+      </c>
+      <c r="K275" t="inlineStr">
+        <is>
+          <t>Relais assistant (26/10)</t>
+        </is>
+      </c>
+      <c r="L275" s="12" t="inlineStr">
+        <is>
+          <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
+        </is>
+      </c>
+      <c r="N275" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi</t>
+        </is>
+      </c>
+      <c r="O275" t="inlineStr">
+        <is>
+          <t>[26/10] Relais assistant tiers du 26/10 (dédupliqué Gmail/Contacts) — e-mail « vérifié » par le relais, à re-confirmer sur site officiel avant envoi.  NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi</t>
+        </is>
+      </c>
+      <c r="P275" t="inlineStr">
+        <is>
+          <t>5e liste — relais (26/10)</t>
+        </is>
+      </c>
+      <c r="Q275" t="inlineStr">
+        <is>
+          <t>contact@guevel-tp.fr</t>
+        </is>
+      </c>
     </row>
     <row r="276" ht="15" customHeight="1" s="13">
-      <c r="L276" s="12" t="n"/>
+      <c r="A276" t="n">
+        <v>276</v>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C276" t="n">
+        <v>2</v>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pavage/dallage bassin rennais, surfaces </t>
+        </is>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>Peron Aménagement Minéral</t>
+        </is>
+      </c>
+      <c r="F276" t="inlineStr">
+        <is>
+          <t>Vieux-Vy-sur-Couesnon (35)</t>
+        </is>
+      </c>
+      <c r="G276" t="inlineStr">
+        <is>
+          <t>Bretagne</t>
+        </is>
+      </c>
+      <c r="H276" t="inlineStr">
+        <is>
+          <t>Correspond au minimum 25 m² : tarif pierre seule + transport séparé.</t>
+        </is>
+      </c>
+      <c r="J276" t="inlineStr">
+        <is>
+          <t>02 99 39 51 02</t>
+        </is>
+      </c>
+      <c r="K276" t="inlineStr">
+        <is>
+          <t>Relais assistant (26/10)</t>
+        </is>
+      </c>
+      <c r="L276" s="12" t="inlineStr">
+        <is>
+          <t>À contacter (formulaire/tél) — EN ATTENTE</t>
+        </is>
+      </c>
+      <c r="N276" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi</t>
+        </is>
+      </c>
+      <c r="O276" t="inlineStr">
+        <is>
+          <t>[26/10] Relais assistant tiers du 26/10 (dédupliqué Gmail/Contacts) — e-mail « vérifié » par le relais, à re-confirmer sur site officiel avant envoi. Pas d'e-mail publié : téléphone. NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi</t>
+        </is>
+      </c>
+      <c r="P276" t="inlineStr">
+        <is>
+          <t>5e liste — relais (26/10)</t>
+        </is>
+      </c>
     </row>
     <row r="277" ht="15" customHeight="1" s="13">
-      <c r="L277" s="12" t="n"/>
+      <c r="A277" t="n">
+        <v>277</v>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C277" t="n">
+        <v>3</v>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>TP/voirie — lauréat d'un lot voirie Renn</t>
+        </is>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>Eurovia Ille-et-Vilaine</t>
+        </is>
+      </c>
+      <c r="F277" t="inlineStr">
+        <is>
+          <t>Rennes (35)</t>
+        </is>
+      </c>
+      <c r="G277" t="inlineStr">
+        <is>
+          <t>Bretagne</t>
+        </is>
+      </c>
+      <c r="H277" t="inlineStr">
+        <is>
+          <t>Voirie marchés rennais — voir minyala/marches-publics.md : rien ne prouve que MINYALA (2 cm) convient ni qu'ils soumissionneront.</t>
+        </is>
+      </c>
+      <c r="J277" t="inlineStr">
+        <is>
+          <t>02 99 05 03 00</t>
+        </is>
+      </c>
+      <c r="K277" t="inlineStr">
+        <is>
+          <t>Relais assistant (26/10)</t>
+        </is>
+      </c>
+      <c r="L277" s="12" t="inlineStr">
+        <is>
+          <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
+        </is>
+      </c>
+      <c r="N277" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi</t>
+        </is>
+      </c>
+      <c r="O277" t="inlineStr">
+        <is>
+          <t>[26/10] Relais assistant tiers du 26/10 (dédupliqué Gmail/Contacts) — e-mail « vérifié » par le relais, à re-confirmer sur site officiel avant envoi.  NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi</t>
+        </is>
+      </c>
+      <c r="P277" t="inlineStr">
+        <is>
+          <t>5e liste — relais (26/10)</t>
+        </is>
+      </c>
+      <c r="Q277" t="inlineStr">
+        <is>
+          <t>ille-et-vilaine@eurovia.com</t>
+        </is>
+      </c>
     </row>
     <row r="278" ht="15" customHeight="1" s="13">
-      <c r="L278" s="12" t="n"/>
+      <c r="A278" t="n">
+        <v>278</v>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C278" t="n">
+        <v>3</v>
+      </c>
+      <c r="D278" t="inlineStr">
+        <is>
+          <t>TP/voirie — lauréat de plusieurs lots du</t>
+        </is>
+      </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>Colas Rennes</t>
+        </is>
+      </c>
+      <c r="F278" t="inlineStr">
+        <is>
+          <t>Rennes (35)</t>
+        </is>
+      </c>
+      <c r="G278" t="inlineStr">
+        <is>
+          <t>Bretagne</t>
+        </is>
+      </c>
+      <c r="H278" t="inlineStr">
+        <is>
+          <t>Idem Eurovia — prérequis techniques (FNTP 3451, DoP, essais) non réunis à ce jour.</t>
+        </is>
+      </c>
+      <c r="J278" t="inlineStr">
+        <is>
+          <t>02 99 59 25 91</t>
+        </is>
+      </c>
+      <c r="K278" t="inlineStr">
+        <is>
+          <t>Relais assistant (26/10)</t>
+        </is>
+      </c>
+      <c r="L278" s="12" t="inlineStr">
+        <is>
+          <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
+        </is>
+      </c>
+      <c r="N278" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi</t>
+        </is>
+      </c>
+      <c r="O278" t="inlineStr">
+        <is>
+          <t>[26/10] Relais assistant tiers du 26/10 (dédupliqué Gmail/Contacts) — e-mail « vérifié » par le relais, à re-confirmer sur site officiel avant envoi.  NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi</t>
+        </is>
+      </c>
+      <c r="P278" t="inlineStr">
+        <is>
+          <t>5e liste — relais (26/10)</t>
+        </is>
+      </c>
+      <c r="Q278" t="inlineStr">
+        <is>
+          <t>contact.rennes@colas.com</t>
+        </is>
+      </c>
     </row>
     <row r="279" ht="15" customHeight="1" s="13">
-      <c r="L279" s="12" t="n"/>
+      <c r="A279" t="n">
+        <v>279</v>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C279" t="n">
+        <v>3</v>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>TP/voirie — lauréat d'un lot</t>
+        </is>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>Keravis (Groupe Lessard)</t>
+        </is>
+      </c>
+      <c r="F279" t="inlineStr">
+        <is>
+          <t>L'Hermitage (35)</t>
+        </is>
+      </c>
+      <c r="G279" t="inlineStr">
+        <is>
+          <t>Bretagne</t>
+        </is>
+      </c>
+      <c r="H279" t="inlineStr">
+        <is>
+          <t>Idem — voir mémo marchés publics.</t>
+        </is>
+      </c>
+      <c r="J279" t="inlineStr">
+        <is>
+          <t>02 99 64 07 64</t>
+        </is>
+      </c>
+      <c r="K279" t="inlineStr">
+        <is>
+          <t>Relais assistant (26/10)</t>
+        </is>
+      </c>
+      <c r="L279" s="12" t="inlineStr">
+        <is>
+          <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
+        </is>
+      </c>
+      <c r="N279" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi</t>
+        </is>
+      </c>
+      <c r="O279" t="inlineStr">
+        <is>
+          <t>[26/10] Relais assistant tiers du 26/10 (dédupliqué Gmail/Contacts) — e-mail « vérifié » par le relais, à re-confirmer sur site officiel avant envoi.  NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi</t>
+        </is>
+      </c>
+      <c r="P279" t="inlineStr">
+        <is>
+          <t>5e liste — relais (26/10)</t>
+        </is>
+      </c>
+      <c r="Q279" t="inlineStr">
+        <is>
+          <t>secretariat.keravis@lessard.fr</t>
+        </is>
+      </c>
     </row>
     <row r="280" ht="15" customHeight="1" s="13">
-      <c r="L280" s="12" t="n"/>
+      <c r="A280" t="n">
+        <v>280</v>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C280" t="n">
+        <v>3</v>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>TP rennais : routes et aménagements</t>
+        </is>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>SRTP (Groupe Pigeon)</t>
+        </is>
+      </c>
+      <c r="F280" t="inlineStr">
+        <is>
+          <t>Domloup (35)</t>
+        </is>
+      </c>
+      <c r="G280" t="inlineStr">
+        <is>
+          <t>Bretagne</t>
+        </is>
+      </c>
+      <c r="H280" t="inlineStr">
+        <is>
+          <t>Idem — voir mémo marchés publics.</t>
+        </is>
+      </c>
+      <c r="J280" t="inlineStr">
+        <is>
+          <t>02 99 41 65 70</t>
+        </is>
+      </c>
+      <c r="K280" t="inlineStr">
+        <is>
+          <t>Relais assistant (26/10)</t>
+        </is>
+      </c>
+      <c r="L280" s="12" t="inlineStr">
+        <is>
+          <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
+        </is>
+      </c>
+      <c r="N280" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi</t>
+        </is>
+      </c>
+      <c r="O280" t="inlineStr">
+        <is>
+          <t>[26/10] Relais assistant tiers du 26/10 (dédupliqué Gmail/Contacts) — e-mail « vérifié » par le relais, à re-confirmer sur site officiel avant envoi.  NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi</t>
+        </is>
+      </c>
+      <c r="P280" t="inlineStr">
+        <is>
+          <t>5e liste — relais (26/10)</t>
+        </is>
+      </c>
+      <c r="Q280" t="inlineStr">
+        <is>
+          <t>srtp@groupe-pigeon.com</t>
+        </is>
+      </c>
     </row>
     <row r="281" ht="15" customHeight="1" s="13">
       <c r="L281" s="12" t="n"/>

</xml_diff>

<commit_message>
5e liste — recherche (26/10) : 31 prospects vérifiés ajoutés (12 P1), 1 doublon écarté (Dalle Décor), 3 concurrents marqués prudence — AUCUN ENVOI
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xqm9tFtdvLdJdkiWw2VVp6
</commit_message>
<xml_diff>
--- a/minyala/clients-potentiels.xlsx
+++ b/minyala/clients-potentiels.xlsx
@@ -6177,7 +6177,7 @@
           <t>2e liste (12/10)</t>
         </is>
       </c>
-      <c r="Q68" t="inlineStr">
+      <c r="Q68" s="12" t="inlineStr">
         <is>
           <t>christophe.devaux@granits-materiaux.fr</t>
         </is>
@@ -6838,7 +6838,7 @@
           <t>2e liste (12/10)</t>
         </is>
       </c>
-      <c r="Q78" t="inlineStr">
+      <c r="Q78" s="12" t="inlineStr">
         <is>
           <t>marbrestendances@orange.fr</t>
         </is>
@@ -18856,53 +18856,53 @@
       </c>
     </row>
     <row r="267" ht="15" customHeight="1" s="13">
-      <c r="A267" t="n">
+      <c r="A267" s="12" t="n">
         <v>267</v>
       </c>
-      <c r="B267" t="inlineStr">
+      <c r="B267" s="12" t="inlineStr">
         <is>
           <t>Pro France</t>
         </is>
       </c>
-      <c r="C267" t="n">
+      <c r="C267" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="D267" t="inlineStr">
+      <c r="D267" s="12" t="inlineStr">
         <is>
           <t>Fournisseur dallage/pavage pro+particuli</t>
         </is>
       </c>
-      <c r="E267" t="inlineStr">
+      <c r="E267" s="12" t="inlineStr">
         <is>
           <t>Adi Roc</t>
         </is>
       </c>
-      <c r="F267" t="inlineStr">
+      <c r="F267" s="12" t="inlineStr">
         <is>
           <t>Evran (22)</t>
         </is>
       </c>
-      <c r="G267" t="inlineStr">
+      <c r="G267" s="12" t="inlineStr">
         <is>
           <t>Bretagne</t>
         </is>
       </c>
-      <c r="H267" t="inlineStr">
+      <c r="H267" s="12" t="inlineStr">
         <is>
           <t>Très forte adéquation : vend déjà de la pierre d'Égypte. Approche : échantillon + lot test puis palettes.</t>
         </is>
       </c>
-      <c r="I267" t="inlineStr">
+      <c r="I267" s="12" t="inlineStr">
         <is>
           <t>https://www.adi-roc.fr</t>
         </is>
       </c>
-      <c r="J267" t="inlineStr">
+      <c r="J267" s="12" t="inlineStr">
         <is>
           <t>06 28 04 92 93</t>
         </is>
       </c>
-      <c r="K267" t="inlineStr">
+      <c r="K267" s="12" t="inlineStr">
         <is>
           <t>Relais assistant (26/10)</t>
         </is>
@@ -18912,70 +18912,70 @@
           <t>À contacter (formulaire/tél) — EN ATTENTE</t>
         </is>
       </c>
-      <c r="N267" t="inlineStr">
+      <c r="N267" s="12" t="inlineStr">
         <is>
           <t>NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi</t>
         </is>
       </c>
-      <c r="O267" t="inlineStr">
+      <c r="O267" s="12" t="inlineStr">
         <is>
           <t>[26/10] Relais assistant tiers du 26/10 (dédupliqué Gmail/Contacts) — e-mail « vérifié » par le relais, à re-confirmer sur site officiel avant envoi. Pas d'e-mail publié : formulaire du site ou téléphone. NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi</t>
         </is>
       </c>
-      <c r="P267" t="inlineStr">
+      <c r="P267" s="12" t="inlineStr">
         <is>
           <t>5e liste — relais (26/10)</t>
         </is>
       </c>
     </row>
     <row r="268" ht="15" customHeight="1" s="13">
-      <c r="A268" t="n">
+      <c r="A268" s="12" t="n">
         <v>268</v>
       </c>
-      <c r="B268" t="inlineStr">
+      <c r="B268" s="12" t="inlineStr">
         <is>
           <t>Pro France</t>
         </is>
       </c>
-      <c r="C268" t="n">
+      <c r="C268" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="D268" t="inlineStr">
+      <c r="D268" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Négoce pavage/dallage, stockage annoncé </t>
         </is>
       </c>
-      <c r="E268" t="inlineStr">
+      <c r="E268" s="12" t="inlineStr">
         <is>
           <t>Espace TP Distribution</t>
         </is>
       </c>
-      <c r="F268" t="inlineStr">
+      <c r="F268" s="12" t="inlineStr">
         <is>
           <t>Vaux-le-Pénil (77)</t>
         </is>
       </c>
-      <c r="G268" t="inlineStr">
+      <c r="G268" s="12" t="inlineStr">
         <is>
           <t>Île-de-France</t>
         </is>
       </c>
-      <c r="H268" t="inlineStr">
+      <c r="H268" s="12" t="inlineStr">
         <is>
           <t>Cible majeure pour 25–500 m² ou revente par palettes.</t>
         </is>
       </c>
-      <c r="I268" t="inlineStr">
+      <c r="I268" s="12" t="inlineStr">
         <is>
           <t>https://www.espacetp.fr</t>
         </is>
       </c>
-      <c r="J268" t="inlineStr">
+      <c r="J268" s="12" t="inlineStr">
         <is>
           <t>01 64 19 19 16</t>
         </is>
       </c>
-      <c r="K268" t="inlineStr">
+      <c r="K268" s="12" t="inlineStr">
         <is>
           <t>Relais assistant (26/10)</t>
         </is>
@@ -18985,75 +18985,75 @@
           <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
         </is>
       </c>
-      <c r="N268" t="inlineStr">
+      <c r="N268" s="12" t="inlineStr">
         <is>
           <t>NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi</t>
         </is>
       </c>
-      <c r="O268" t="inlineStr">
+      <c r="O268" s="12" t="inlineStr">
         <is>
           <t>[26/10] Relais assistant tiers du 26/10 (dédupliqué Gmail/Contacts) — e-mail « vérifié » par le relais, à re-confirmer sur site officiel avant envoi.  NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi</t>
         </is>
       </c>
-      <c r="P268" t="inlineStr">
+      <c r="P268" s="12" t="inlineStr">
         <is>
           <t>5e liste — relais (26/10)</t>
         </is>
       </c>
-      <c r="Q268" t="inlineStr">
+      <c r="Q268" s="12" t="inlineStr">
         <is>
           <t>contact@espacetp.fr</t>
         </is>
       </c>
     </row>
     <row r="269" ht="15" customHeight="1" s="13">
-      <c r="A269" t="n">
+      <c r="A269" s="12" t="n">
         <v>269</v>
       </c>
-      <c r="B269" t="inlineStr">
+      <c r="B269" s="12" t="inlineStr">
         <is>
           <t>Pro France</t>
         </is>
       </c>
-      <c r="C269" t="n">
+      <c r="C269" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="D269" t="inlineStr">
+      <c r="D269" s="12" t="inlineStr">
         <is>
           <t>Revendeur pierre naturelle, &gt;1 000 m² d'</t>
         </is>
       </c>
-      <c r="E269" t="inlineStr">
+      <c r="E269" s="12" t="inlineStr">
         <is>
           <t>Kei-Stone Les Alluets-le-Roi</t>
         </is>
       </c>
-      <c r="F269" t="inlineStr">
+      <c r="F269" s="12" t="inlineStr">
         <is>
           <t>Les Alluets-le-Roi (78)</t>
         </is>
       </c>
-      <c r="G269" t="inlineStr">
+      <c r="G269" s="12" t="inlineStr">
         <is>
           <t>Île-de-France</t>
         </is>
       </c>
-      <c r="H269" t="inlineStr">
+      <c r="H269" s="12" t="inlineStr">
         <is>
           <t>Présenter MINYALA comme gamme calcaire beige disponible rapidement depuis Gennevilliers.</t>
         </is>
       </c>
-      <c r="I269" t="inlineStr">
+      <c r="I269" s="12" t="inlineStr">
         <is>
           <t>https://www.kei-stone.fr</t>
         </is>
       </c>
-      <c r="J269" t="inlineStr">
+      <c r="J269" s="12" t="inlineStr">
         <is>
           <t>01 39 75 55 60</t>
         </is>
       </c>
-      <c r="K269" t="inlineStr">
+      <c r="K269" s="12" t="inlineStr">
         <is>
           <t>Relais assistant (26/10)</t>
         </is>
@@ -19063,75 +19063,75 @@
           <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
         </is>
       </c>
-      <c r="N269" t="inlineStr">
+      <c r="N269" s="12" t="inlineStr">
         <is>
           <t>NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi</t>
         </is>
       </c>
-      <c r="O269" t="inlineStr">
+      <c r="O269" s="12" t="inlineStr">
         <is>
           <t>[26/10] Relais assistant tiers du 26/10 (dédupliqué Gmail/Contacts) — e-mail « vérifié » par le relais, à re-confirmer sur site officiel avant envoi.  NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi</t>
         </is>
       </c>
-      <c r="P269" t="inlineStr">
+      <c r="P269" s="12" t="inlineStr">
         <is>
           <t>5e liste — relais (26/10)</t>
         </is>
       </c>
-      <c r="Q269" t="inlineStr">
+      <c r="Q269" s="12" t="inlineStr">
         <is>
           <t>contact78@kei-stone.fr</t>
         </is>
       </c>
     </row>
     <row r="270" ht="15" customHeight="1" s="13">
-      <c r="A270" t="n">
+      <c r="A270" s="12" t="n">
         <v>270</v>
       </c>
-      <c r="B270" t="inlineStr">
+      <c r="B270" s="12" t="inlineStr">
         <is>
           <t>Pro France</t>
         </is>
       </c>
-      <c r="C270" t="n">
+      <c r="C270" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="D270" t="inlineStr">
+      <c r="D270" s="12" t="inlineStr">
         <is>
           <t>Négoce avec showroom 350 m² : dalles, pa</t>
         </is>
       </c>
-      <c r="E270" t="inlineStr">
+      <c r="E270" s="12" t="inlineStr">
         <is>
           <t>Hestia Pierre &amp; Jardin</t>
         </is>
       </c>
-      <c r="F270" t="inlineStr">
+      <c r="F270" s="12" t="inlineStr">
         <is>
           <t>Hillion (22)</t>
         </is>
       </c>
-      <c r="G270" t="inlineStr">
+      <c r="G270" s="12" t="inlineStr">
         <is>
           <t>Bretagne</t>
         </is>
       </c>
-      <c r="H270" t="inlineStr">
+      <c r="H270" s="12" t="inlineStr">
         <is>
           <t>Partenariat revendeur : échantillon + conditions par palette.</t>
         </is>
       </c>
-      <c r="I270" t="inlineStr">
+      <c r="I270" s="12" t="inlineStr">
         <is>
           <t>https://www.hestia.bzh</t>
         </is>
       </c>
-      <c r="J270" t="inlineStr">
+      <c r="J270" s="12" t="inlineStr">
         <is>
           <t>02 96 52 33 04</t>
         </is>
       </c>
-      <c r="K270" t="inlineStr">
+      <c r="K270" s="12" t="inlineStr">
         <is>
           <t>Relais assistant (26/10)</t>
         </is>
@@ -19141,70 +19141,70 @@
           <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
         </is>
       </c>
-      <c r="N270" t="inlineStr">
+      <c r="N270" s="12" t="inlineStr">
         <is>
           <t>NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi</t>
         </is>
       </c>
-      <c r="O270" t="inlineStr">
+      <c r="O270" s="12" t="inlineStr">
         <is>
           <t>[26/10] Relais assistant tiers du 26/10 (dédupliqué Gmail/Contacts) — e-mail « vérifié » par le relais, à re-confirmer sur site officiel avant envoi.  NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi</t>
         </is>
       </c>
-      <c r="P270" t="inlineStr">
+      <c r="P270" s="12" t="inlineStr">
         <is>
           <t>5e liste — relais (26/10)</t>
         </is>
       </c>
-      <c r="Q270" t="inlineStr">
+      <c r="Q270" s="12" t="inlineStr">
         <is>
           <t>bonjour@hestia.bzh</t>
         </is>
       </c>
     </row>
     <row r="271" ht="15" customHeight="1" s="13">
-      <c r="A271" t="n">
+      <c r="A271" s="12" t="n">
         <v>271</v>
       </c>
-      <c r="B271" t="inlineStr">
+      <c r="B271" s="12" t="inlineStr">
         <is>
           <t>Pro France</t>
         </is>
       </c>
-      <c r="C271" t="n">
+      <c r="C271" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="D271" t="inlineStr">
+      <c r="D271" s="12" t="inlineStr">
         <is>
           <t>Importateur direct de calcaires et pierr</t>
         </is>
       </c>
-      <c r="E271" t="inlineStr">
+      <c r="E271" s="12" t="inlineStr">
         <is>
           <t>Dalle Décor</t>
         </is>
       </c>
-      <c r="F271" t="inlineStr">
+      <c r="F271" s="12" t="inlineStr">
         <is>
           <t>Galluis (78)</t>
         </is>
       </c>
-      <c r="G271" t="inlineStr">
+      <c r="G271" s="12" t="inlineStr">
         <is>
           <t>Île-de-France</t>
         </is>
       </c>
-      <c r="H271" t="inlineStr">
+      <c r="H271" s="12" t="inlineStr">
         <is>
           <t>Demander s'ils reprennent des lots déjà importés et disponibles localement.</t>
         </is>
       </c>
-      <c r="J271" t="inlineStr">
+      <c r="J271" s="12" t="inlineStr">
         <is>
           <t>09 74 56 22 36</t>
         </is>
       </c>
-      <c r="K271" t="inlineStr">
+      <c r="K271" s="12" t="inlineStr">
         <is>
           <t>Relais assistant (26/10)</t>
         </is>
@@ -19214,65 +19214,65 @@
           <t>À contacter (formulaire/tél) — EN ATTENTE</t>
         </is>
       </c>
-      <c r="N271" t="inlineStr">
+      <c r="N271" s="12" t="inlineStr">
         <is>
           <t>NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi</t>
         </is>
       </c>
-      <c r="O271" t="inlineStr">
+      <c r="O271" s="12" t="inlineStr">
         <is>
           <t>[26/10] Relais assistant tiers du 26/10 (dédupliqué Gmail/Contacts) — e-mail « vérifié » par le relais, à re-confirmer sur site officiel avant envoi. Pas d'e-mail publié : téléphone. NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi</t>
         </is>
       </c>
-      <c r="P271" t="inlineStr">
+      <c r="P271" s="12" t="inlineStr">
         <is>
           <t>5e liste — relais (26/10)</t>
         </is>
       </c>
     </row>
     <row r="272" ht="15" customHeight="1" s="13">
-      <c r="A272" t="n">
+      <c r="A272" s="12" t="n">
         <v>272</v>
       </c>
-      <c r="B272" t="inlineStr">
+      <c r="B272" s="12" t="inlineStr">
         <is>
           <t>Pro France</t>
         </is>
       </c>
-      <c r="C272" t="n">
+      <c r="C272" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="D272" t="inlineStr">
+      <c r="D272" s="12" t="inlineStr">
         <is>
           <t>Vente et pose de dallages, pavés, bordur</t>
         </is>
       </c>
-      <c r="E272" t="inlineStr">
+      <c r="E272" s="12" t="inlineStr">
         <is>
           <t>Les Paveurs d'Eure-et-Loir</t>
         </is>
       </c>
-      <c r="F272" t="inlineStr">
+      <c r="F272" s="12" t="inlineStr">
         <is>
           <t>Cherisy (28)</t>
         </is>
       </c>
-      <c r="G272" t="inlineStr">
+      <c r="G272" s="12" t="inlineStr">
         <is>
           <t>IdF/Eure/Normandie</t>
         </is>
       </c>
-      <c r="H272" t="inlineStr">
+      <c r="H272" s="12" t="inlineStr">
         <is>
           <t>Très bon profil pour fourniture de lots de 25 à plusieurs centaines de m² (la pose reste la leur).</t>
         </is>
       </c>
-      <c r="J272" t="inlineStr">
+      <c r="J272" s="12" t="inlineStr">
         <is>
           <t>06 87 53 33 76</t>
         </is>
       </c>
-      <c r="K272" t="inlineStr">
+      <c r="K272" s="12" t="inlineStr">
         <is>
           <t>Relais assistant (26/10)</t>
         </is>
@@ -19282,70 +19282,70 @@
           <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
         </is>
       </c>
-      <c r="N272" t="inlineStr">
+      <c r="N272" s="12" t="inlineStr">
         <is>
           <t>NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi</t>
         </is>
       </c>
-      <c r="O272" t="inlineStr">
+      <c r="O272" s="12" t="inlineStr">
         <is>
           <t>[26/10] Relais assistant tiers du 26/10 (dédupliqué Gmail/Contacts) — e-mail « vérifié » par le relais, à re-confirmer sur site officiel avant envoi.  NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi</t>
         </is>
       </c>
-      <c r="P272" t="inlineStr">
+      <c r="P272" s="12" t="inlineStr">
         <is>
           <t>5e liste — relais (26/10)</t>
         </is>
       </c>
-      <c r="Q272" t="inlineStr">
+      <c r="Q272" s="12" t="inlineStr">
         <is>
           <t>lespaveurs.eureetloir@orange.fr</t>
         </is>
       </c>
     </row>
     <row r="273" ht="15" customHeight="1" s="13">
-      <c r="A273" t="n">
+      <c r="A273" s="12" t="n">
         <v>273</v>
       </c>
-      <c r="B273" t="inlineStr">
+      <c r="B273" s="12" t="inlineStr">
         <is>
           <t>Pro France</t>
         </is>
       </c>
-      <c r="C273" t="n">
+      <c r="C273" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="D273" t="inlineStr">
+      <c r="D273" s="12" t="inlineStr">
         <is>
           <t>Fournisseur pierre naturelle constructio</t>
         </is>
       </c>
-      <c r="E273" t="inlineStr">
+      <c r="E273" s="12" t="inlineStr">
         <is>
           <t>MC Pierre</t>
         </is>
       </c>
-      <c r="F273" t="inlineStr">
+      <c r="F273" s="12" t="inlineStr">
         <is>
           <t>Courtry (77)</t>
         </is>
       </c>
-      <c r="G273" t="inlineStr">
+      <c r="G273" s="12" t="inlineStr">
         <is>
           <t>Île-de-France</t>
         </is>
       </c>
-      <c r="H273" t="inlineStr">
+      <c r="H273" s="12" t="inlineStr">
         <is>
           <t>Tester l'intérêt pour une gamme complémentaire calcaire égyptien 30×60×2.</t>
         </is>
       </c>
-      <c r="J273" t="inlineStr">
+      <c r="J273" s="12" t="inlineStr">
         <is>
           <t>06 25 28 12 12</t>
         </is>
       </c>
-      <c r="K273" t="inlineStr">
+      <c r="K273" s="12" t="inlineStr">
         <is>
           <t>Relais assistant (26/10)</t>
         </is>
@@ -19355,70 +19355,70 @@
           <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
         </is>
       </c>
-      <c r="N273" t="inlineStr">
+      <c r="N273" s="12" t="inlineStr">
         <is>
           <t>NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi</t>
         </is>
       </c>
-      <c r="O273" t="inlineStr">
+      <c r="O273" s="12" t="inlineStr">
         <is>
           <t>[26/10] Relais assistant tiers du 26/10 (dédupliqué Gmail/Contacts) — e-mail « vérifié » par le relais, à re-confirmer sur site officiel avant envoi.  NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi</t>
         </is>
       </c>
-      <c r="P273" t="inlineStr">
+      <c r="P273" s="12" t="inlineStr">
         <is>
           <t>5e liste — relais (26/10)</t>
         </is>
       </c>
-      <c r="Q273" t="inlineStr">
+      <c r="Q273" s="12" t="inlineStr">
         <is>
           <t>contact@mc-pierre.com</t>
         </is>
       </c>
     </row>
     <row r="274" ht="15" customHeight="1" s="13">
-      <c r="A274" t="n">
+      <c r="A274" s="12" t="n">
         <v>274</v>
       </c>
-      <c r="B274" t="inlineStr">
+      <c r="B274" s="12" t="inlineStr">
         <is>
           <t>Pro France</t>
         </is>
       </c>
-      <c r="C274" t="n">
+      <c r="C274" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="D274" t="inlineStr">
+      <c r="D274" s="12" t="inlineStr">
         <is>
           <t>Bureau d'études paysager + showroom, ven</t>
         </is>
       </c>
-      <c r="E274" t="inlineStr">
+      <c r="E274" s="12" t="inlineStr">
         <is>
           <t>Esprit Vert Design</t>
         </is>
       </c>
-      <c r="F274" t="inlineStr">
+      <c r="F274" s="12" t="inlineStr">
         <is>
           <t>Ploërmel (56)</t>
         </is>
       </c>
-      <c r="G274" t="inlineStr">
+      <c r="G274" s="12" t="inlineStr">
         <is>
           <t>Bretagne</t>
         </is>
       </c>
-      <c r="H274" t="inlineStr">
+      <c r="H274" s="12" t="inlineStr">
         <is>
           <t>Fiche architecte (photos, texture, dimensions, prix) adaptée.</t>
         </is>
       </c>
-      <c r="J274" t="inlineStr">
+      <c r="J274" s="12" t="inlineStr">
         <is>
           <t>02 97 72 97 51</t>
         </is>
       </c>
-      <c r="K274" t="inlineStr">
+      <c r="K274" s="12" t="inlineStr">
         <is>
           <t>Relais assistant (26/10)</t>
         </is>
@@ -19428,75 +19428,75 @@
           <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
         </is>
       </c>
-      <c r="N274" t="inlineStr">
+      <c r="N274" s="12" t="inlineStr">
         <is>
           <t>NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi</t>
         </is>
       </c>
-      <c r="O274" t="inlineStr">
+      <c r="O274" s="12" t="inlineStr">
         <is>
           <t>[26/10] Relais assistant tiers du 26/10 (dédupliqué Gmail/Contacts) — e-mail « vérifié » par le relais, à re-confirmer sur site officiel avant envoi.  NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi</t>
         </is>
       </c>
-      <c r="P274" t="inlineStr">
+      <c r="P274" s="12" t="inlineStr">
         <is>
           <t>5e liste — relais (26/10)</t>
         </is>
       </c>
-      <c r="Q274" t="inlineStr">
+      <c r="Q274" s="12" t="inlineStr">
         <is>
           <t>contact@esprit-vert-design.fr</t>
         </is>
       </c>
     </row>
     <row r="275" ht="15" customHeight="1" s="13">
-      <c r="A275" t="n">
+      <c r="A275" s="12" t="n">
         <v>275</v>
       </c>
-      <c r="B275" t="inlineStr">
+      <c r="B275" s="12" t="inlineStr">
         <is>
           <t>Pro France</t>
         </is>
       </c>
-      <c r="C275" t="n">
+      <c r="C275" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="D275" t="inlineStr">
+      <c r="D275" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Terrassement et aménagements : dallage, </t>
         </is>
       </c>
-      <c r="E275" t="inlineStr">
+      <c r="E275" s="12" t="inlineStr">
         <is>
           <t>Guevel TP</t>
         </is>
       </c>
-      <c r="F275" t="inlineStr">
+      <c r="F275" s="12" t="inlineStr">
         <is>
           <t>Betton (35)</t>
         </is>
       </c>
-      <c r="G275" t="inlineStr">
+      <c r="G275" s="12" t="inlineStr">
         <is>
           <t>Bretagne</t>
         </is>
       </c>
-      <c r="H275" t="inlineStr">
+      <c r="H275" s="12" t="inlineStr">
         <is>
           <t>Pierre pour terrasses/aménagements privés — ne pas lier l'offre à un marché public précis.</t>
         </is>
       </c>
-      <c r="I275" t="inlineStr">
+      <c r="I275" s="12" t="inlineStr">
         <is>
           <t>https://www.guevel-tp.fr</t>
         </is>
       </c>
-      <c r="J275" t="inlineStr">
+      <c r="J275" s="12" t="inlineStr">
         <is>
           <t>06 08 40 35 42</t>
         </is>
       </c>
-      <c r="K275" t="inlineStr">
+      <c r="K275" s="12" t="inlineStr">
         <is>
           <t>Relais assistant (26/10)</t>
         </is>
@@ -19506,70 +19506,70 @@
           <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
         </is>
       </c>
-      <c r="N275" t="inlineStr">
+      <c r="N275" s="12" t="inlineStr">
         <is>
           <t>NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi</t>
         </is>
       </c>
-      <c r="O275" t="inlineStr">
+      <c r="O275" s="12" t="inlineStr">
         <is>
           <t>[26/10] Relais assistant tiers du 26/10 (dédupliqué Gmail/Contacts) — e-mail « vérifié » par le relais, à re-confirmer sur site officiel avant envoi.  NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi</t>
         </is>
       </c>
-      <c r="P275" t="inlineStr">
+      <c r="P275" s="12" t="inlineStr">
         <is>
           <t>5e liste — relais (26/10)</t>
         </is>
       </c>
-      <c r="Q275" t="inlineStr">
+      <c r="Q275" s="12" t="inlineStr">
         <is>
           <t>contact@guevel-tp.fr</t>
         </is>
       </c>
     </row>
     <row r="276" ht="15" customHeight="1" s="13">
-      <c r="A276" t="n">
+      <c r="A276" s="12" t="n">
         <v>276</v>
       </c>
-      <c r="B276" t="inlineStr">
+      <c r="B276" s="12" t="inlineStr">
         <is>
           <t>Pro France</t>
         </is>
       </c>
-      <c r="C276" t="n">
+      <c r="C276" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="D276" t="inlineStr">
+      <c r="D276" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Pavage/dallage bassin rennais, surfaces </t>
         </is>
       </c>
-      <c r="E276" t="inlineStr">
+      <c r="E276" s="12" t="inlineStr">
         <is>
           <t>Peron Aménagement Minéral</t>
         </is>
       </c>
-      <c r="F276" t="inlineStr">
+      <c r="F276" s="12" t="inlineStr">
         <is>
           <t>Vieux-Vy-sur-Couesnon (35)</t>
         </is>
       </c>
-      <c r="G276" t="inlineStr">
+      <c r="G276" s="12" t="inlineStr">
         <is>
           <t>Bretagne</t>
         </is>
       </c>
-      <c r="H276" t="inlineStr">
+      <c r="H276" s="12" t="inlineStr">
         <is>
           <t>Correspond au minimum 25 m² : tarif pierre seule + transport séparé.</t>
         </is>
       </c>
-      <c r="J276" t="inlineStr">
+      <c r="J276" s="12" t="inlineStr">
         <is>
           <t>02 99 39 51 02</t>
         </is>
       </c>
-      <c r="K276" t="inlineStr">
+      <c r="K276" s="12" t="inlineStr">
         <is>
           <t>Relais assistant (26/10)</t>
         </is>
@@ -19579,65 +19579,65 @@
           <t>À contacter (formulaire/tél) — EN ATTENTE</t>
         </is>
       </c>
-      <c r="N276" t="inlineStr">
+      <c r="N276" s="12" t="inlineStr">
         <is>
           <t>NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi</t>
         </is>
       </c>
-      <c r="O276" t="inlineStr">
+      <c r="O276" s="12" t="inlineStr">
         <is>
           <t>[26/10] Relais assistant tiers du 26/10 (dédupliqué Gmail/Contacts) — e-mail « vérifié » par le relais, à re-confirmer sur site officiel avant envoi. Pas d'e-mail publié : téléphone. NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi</t>
         </is>
       </c>
-      <c r="P276" t="inlineStr">
+      <c r="P276" s="12" t="inlineStr">
         <is>
           <t>5e liste — relais (26/10)</t>
         </is>
       </c>
     </row>
     <row r="277" ht="15" customHeight="1" s="13">
-      <c r="A277" t="n">
+      <c r="A277" s="12" t="n">
         <v>277</v>
       </c>
-      <c r="B277" t="inlineStr">
+      <c r="B277" s="12" t="inlineStr">
         <is>
           <t>Pro France</t>
         </is>
       </c>
-      <c r="C277" t="n">
+      <c r="C277" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="D277" t="inlineStr">
+      <c r="D277" s="12" t="inlineStr">
         <is>
           <t>TP/voirie — lauréat d'un lot voirie Renn</t>
         </is>
       </c>
-      <c r="E277" t="inlineStr">
+      <c r="E277" s="12" t="inlineStr">
         <is>
           <t>Eurovia Ille-et-Vilaine</t>
         </is>
       </c>
-      <c r="F277" t="inlineStr">
+      <c r="F277" s="12" t="inlineStr">
         <is>
           <t>Rennes (35)</t>
         </is>
       </c>
-      <c r="G277" t="inlineStr">
+      <c r="G277" s="12" t="inlineStr">
         <is>
           <t>Bretagne</t>
         </is>
       </c>
-      <c r="H277" t="inlineStr">
+      <c r="H277" s="12" t="inlineStr">
         <is>
           <t>Voirie marchés rennais — voir minyala/marches-publics.md : rien ne prouve que MINYALA (2 cm) convient ni qu'ils soumissionneront.</t>
         </is>
       </c>
-      <c r="J277" t="inlineStr">
+      <c r="J277" s="12" t="inlineStr">
         <is>
           <t>02 99 05 03 00</t>
         </is>
       </c>
-      <c r="K277" t="inlineStr">
+      <c r="K277" s="12" t="inlineStr">
         <is>
           <t>Relais assistant (26/10)</t>
         </is>
@@ -19647,70 +19647,70 @@
           <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
         </is>
       </c>
-      <c r="N277" t="inlineStr">
+      <c r="N277" s="12" t="inlineStr">
         <is>
           <t>NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi</t>
         </is>
       </c>
-      <c r="O277" t="inlineStr">
+      <c r="O277" s="12" t="inlineStr">
         <is>
           <t>[26/10] Relais assistant tiers du 26/10 (dédupliqué Gmail/Contacts) — e-mail « vérifié » par le relais, à re-confirmer sur site officiel avant envoi.  NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi</t>
         </is>
       </c>
-      <c r="P277" t="inlineStr">
+      <c r="P277" s="12" t="inlineStr">
         <is>
           <t>5e liste — relais (26/10)</t>
         </is>
       </c>
-      <c r="Q277" t="inlineStr">
+      <c r="Q277" s="12" t="inlineStr">
         <is>
           <t>ille-et-vilaine@eurovia.com</t>
         </is>
       </c>
     </row>
     <row r="278" ht="15" customHeight="1" s="13">
-      <c r="A278" t="n">
+      <c r="A278" s="12" t="n">
         <v>278</v>
       </c>
-      <c r="B278" t="inlineStr">
+      <c r="B278" s="12" t="inlineStr">
         <is>
           <t>Pro France</t>
         </is>
       </c>
-      <c r="C278" t="n">
+      <c r="C278" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="D278" t="inlineStr">
+      <c r="D278" s="12" t="inlineStr">
         <is>
           <t>TP/voirie — lauréat de plusieurs lots du</t>
         </is>
       </c>
-      <c r="E278" t="inlineStr">
+      <c r="E278" s="12" t="inlineStr">
         <is>
           <t>Colas Rennes</t>
         </is>
       </c>
-      <c r="F278" t="inlineStr">
+      <c r="F278" s="12" t="inlineStr">
         <is>
           <t>Rennes (35)</t>
         </is>
       </c>
-      <c r="G278" t="inlineStr">
+      <c r="G278" s="12" t="inlineStr">
         <is>
           <t>Bretagne</t>
         </is>
       </c>
-      <c r="H278" t="inlineStr">
+      <c r="H278" s="12" t="inlineStr">
         <is>
           <t>Idem Eurovia — prérequis techniques (FNTP 3451, DoP, essais) non réunis à ce jour.</t>
         </is>
       </c>
-      <c r="J278" t="inlineStr">
+      <c r="J278" s="12" t="inlineStr">
         <is>
           <t>02 99 59 25 91</t>
         </is>
       </c>
-      <c r="K278" t="inlineStr">
+      <c r="K278" s="12" t="inlineStr">
         <is>
           <t>Relais assistant (26/10)</t>
         </is>
@@ -19720,70 +19720,70 @@
           <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
         </is>
       </c>
-      <c r="N278" t="inlineStr">
+      <c r="N278" s="12" t="inlineStr">
         <is>
           <t>NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi</t>
         </is>
       </c>
-      <c r="O278" t="inlineStr">
+      <c r="O278" s="12" t="inlineStr">
         <is>
           <t>[26/10] Relais assistant tiers du 26/10 (dédupliqué Gmail/Contacts) — e-mail « vérifié » par le relais, à re-confirmer sur site officiel avant envoi.  NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi</t>
         </is>
       </c>
-      <c r="P278" t="inlineStr">
+      <c r="P278" s="12" t="inlineStr">
         <is>
           <t>5e liste — relais (26/10)</t>
         </is>
       </c>
-      <c r="Q278" t="inlineStr">
+      <c r="Q278" s="12" t="inlineStr">
         <is>
           <t>contact.rennes@colas.com</t>
         </is>
       </c>
     </row>
     <row r="279" ht="15" customHeight="1" s="13">
-      <c r="A279" t="n">
+      <c r="A279" s="12" t="n">
         <v>279</v>
       </c>
-      <c r="B279" t="inlineStr">
+      <c r="B279" s="12" t="inlineStr">
         <is>
           <t>Pro France</t>
         </is>
       </c>
-      <c r="C279" t="n">
+      <c r="C279" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="D279" t="inlineStr">
+      <c r="D279" s="12" t="inlineStr">
         <is>
           <t>TP/voirie — lauréat d'un lot</t>
         </is>
       </c>
-      <c r="E279" t="inlineStr">
+      <c r="E279" s="12" t="inlineStr">
         <is>
           <t>Keravis (Groupe Lessard)</t>
         </is>
       </c>
-      <c r="F279" t="inlineStr">
+      <c r="F279" s="12" t="inlineStr">
         <is>
           <t>L'Hermitage (35)</t>
         </is>
       </c>
-      <c r="G279" t="inlineStr">
+      <c r="G279" s="12" t="inlineStr">
         <is>
           <t>Bretagne</t>
         </is>
       </c>
-      <c r="H279" t="inlineStr">
+      <c r="H279" s="12" t="inlineStr">
         <is>
           <t>Idem — voir mémo marchés publics.</t>
         </is>
       </c>
-      <c r="J279" t="inlineStr">
+      <c r="J279" s="12" t="inlineStr">
         <is>
           <t>02 99 64 07 64</t>
         </is>
       </c>
-      <c r="K279" t="inlineStr">
+      <c r="K279" s="12" t="inlineStr">
         <is>
           <t>Relais assistant (26/10)</t>
         </is>
@@ -19793,70 +19793,70 @@
           <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
         </is>
       </c>
-      <c r="N279" t="inlineStr">
+      <c r="N279" s="12" t="inlineStr">
         <is>
           <t>NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi</t>
         </is>
       </c>
-      <c r="O279" t="inlineStr">
+      <c r="O279" s="12" t="inlineStr">
         <is>
           <t>[26/10] Relais assistant tiers du 26/10 (dédupliqué Gmail/Contacts) — e-mail « vérifié » par le relais, à re-confirmer sur site officiel avant envoi.  NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi</t>
         </is>
       </c>
-      <c r="P279" t="inlineStr">
+      <c r="P279" s="12" t="inlineStr">
         <is>
           <t>5e liste — relais (26/10)</t>
         </is>
       </c>
-      <c r="Q279" t="inlineStr">
+      <c r="Q279" s="12" t="inlineStr">
         <is>
           <t>secretariat.keravis@lessard.fr</t>
         </is>
       </c>
     </row>
     <row r="280" ht="15" customHeight="1" s="13">
-      <c r="A280" t="n">
+      <c r="A280" s="12" t="n">
         <v>280</v>
       </c>
-      <c r="B280" t="inlineStr">
+      <c r="B280" s="12" t="inlineStr">
         <is>
           <t>Pro France</t>
         </is>
       </c>
-      <c r="C280" t="n">
+      <c r="C280" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="D280" t="inlineStr">
+      <c r="D280" s="12" t="inlineStr">
         <is>
           <t>TP rennais : routes et aménagements</t>
         </is>
       </c>
-      <c r="E280" t="inlineStr">
+      <c r="E280" s="12" t="inlineStr">
         <is>
           <t>SRTP (Groupe Pigeon)</t>
         </is>
       </c>
-      <c r="F280" t="inlineStr">
+      <c r="F280" s="12" t="inlineStr">
         <is>
           <t>Domloup (35)</t>
         </is>
       </c>
-      <c r="G280" t="inlineStr">
+      <c r="G280" s="12" t="inlineStr">
         <is>
           <t>Bretagne</t>
         </is>
       </c>
-      <c r="H280" t="inlineStr">
+      <c r="H280" s="12" t="inlineStr">
         <is>
           <t>Idem — voir mémo marchés publics.</t>
         </is>
       </c>
-      <c r="J280" t="inlineStr">
+      <c r="J280" s="12" t="inlineStr">
         <is>
           <t>02 99 41 65 70</t>
         </is>
       </c>
-      <c r="K280" t="inlineStr">
+      <c r="K280" s="12" t="inlineStr">
         <is>
           <t>Relais assistant (26/10)</t>
         </is>
@@ -19866,119 +19866,2384 @@
           <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
         </is>
       </c>
-      <c r="N280" t="inlineStr">
+      <c r="N280" s="12" t="inlineStr">
         <is>
           <t>NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi</t>
         </is>
       </c>
-      <c r="O280" t="inlineStr">
+      <c r="O280" s="12" t="inlineStr">
         <is>
           <t>[26/10] Relais assistant tiers du 26/10 (dédupliqué Gmail/Contacts) — e-mail « vérifié » par le relais, à re-confirmer sur site officiel avant envoi.  NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi</t>
         </is>
       </c>
-      <c r="P280" t="inlineStr">
+      <c r="P280" s="12" t="inlineStr">
         <is>
           <t>5e liste — relais (26/10)</t>
         </is>
       </c>
-      <c r="Q280" t="inlineStr">
+      <c r="Q280" s="12" t="inlineStr">
         <is>
           <t>srtp@groupe-pigeon.com</t>
         </is>
       </c>
     </row>
     <row r="281" ht="15" customHeight="1" s="13">
-      <c r="L281" s="12" t="n"/>
+      <c r="A281" t="n">
+        <v>281</v>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C281" t="n">
+        <v>1</v>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>importateurs</t>
+        </is>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>Marbrerie Arnaud (SUD PIERRE)</t>
+        </is>
+      </c>
+      <c r="F281" t="inlineStr">
+        <is>
+          <t>Colombiers / Béziers</t>
+        </is>
+      </c>
+      <c r="G281" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="H281" t="inlineStr">
+        <is>
+          <t>Confirmée : « Importateur et distributeur de pierre naturelle depuis 2012 », import direct Turquie, Égypte, Chine (page d'accueil) ; showroom 700 m² à Béziers, adresse Route de Nar…</t>
+        </is>
+      </c>
+      <c r="I281" t="inlineStr">
+        <is>
+          <t>https://www.marbreriearnaud34.com/</t>
+        </is>
+      </c>
+      <c r="J281" t="inlineStr">
+        <is>
+          <t>04 67 35 82 22</t>
+        </is>
+      </c>
+      <c r="K281" t="inlineStr">
+        <is>
+          <t>Recherche Claude (26/10)</t>
+        </is>
+      </c>
+      <c r="L281" s="12" t="inlineStr">
+        <is>
+          <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
+        </is>
+      </c>
+      <c r="N281" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="O281" t="inlineStr">
+        <is>
+          <t>[26/10] Recherche vérifiée (segment importateurs). Confirmée : « Importateur et distributeur de pierre naturelle depuis 2012 », import direct Turquie, Égypte, Chine (page d'accueil) ; showroom 700 m² à Béziers, adresse Route de Narbonne à Colombiers. Villes conformes. E-mail lu textuellement dans les mentions légales (« e-mail : j.andreo@marbrerie-arnaud.com », propriétaire SUD PIERRE). Le domaine de l'e-mail (marbrerie-arnaud.com) diffère du domaine du site, mais c'est bien l'adresse publiée officiellement. Téléphone confirmé sur mentions légales et accueil. Domaine hors liste d'exclusion. Source e-mail : https://www.marbreriearnaud34.com/mentions-legales/.  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="P281" t="inlineStr">
+        <is>
+          <t>5e liste — recherche (26/10)</t>
+        </is>
+      </c>
+      <c r="Q281" t="inlineStr">
+        <is>
+          <t>j.andreo@marbrerie-arnaud.com</t>
+        </is>
+      </c>
     </row>
     <row r="282" ht="15" customHeight="1" s="13">
-      <c r="L282" s="12" t="n"/>
+      <c r="A282" t="n">
+        <v>282</v>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C282" t="n">
+        <v>1</v>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>importateurs</t>
+        </is>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>Artemis (Artemis Prestige)</t>
+        </is>
+      </c>
+      <c r="F282" t="inlineStr">
+        <is>
+          <t>Cabriès (Plan de Campagne) ; entrepôt à Simiane-Collongue</t>
+        </is>
+      </c>
+      <c r="G282" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="H282" t="inlineStr">
+        <is>
+          <t>Confirmée : importateur-vendeur de pierre naturelle (travertin, marbre, pierre d'Égypte, grès cérame), livraison France entière. Showroom Expobat Plan de Campagne 13480 Cabriès + e…</t>
+        </is>
+      </c>
+      <c r="I282" t="inlineStr">
+        <is>
+          <t>https://www.artemis-prestige.com/</t>
+        </is>
+      </c>
+      <c r="J282" t="inlineStr">
+        <is>
+          <t>04 42 31 41 40</t>
+        </is>
+      </c>
+      <c r="K282" t="inlineStr">
+        <is>
+          <t>Recherche Claude (26/10)</t>
+        </is>
+      </c>
+      <c r="L282" s="12" t="inlineStr">
+        <is>
+          <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
+        </is>
+      </c>
+      <c r="N282" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="O282" t="inlineStr">
+        <is>
+          <t>[26/10] Recherche vérifiée (segment importateurs). Confirmée : importateur-vendeur de pierre naturelle (travertin, marbre, pierre d'Égypte, grès cérame), livraison France entière. Showroom Expobat Plan de Campagne 13480 Cabriès + entrepôt logistique 13109 Simiane-Collongue confirmés sur la page contact. E-mail présent textuellement sur la page contact (texte du lien et mailto). Téléphone confirmé. Pierre d'Égypte explicitement au catalogue. Domaine hors liste d'exclusion. Source e-mail : https://www.artemis-prestige.com/contact.html.  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="P282" t="inlineStr">
+        <is>
+          <t>5e liste — recherche (26/10)</t>
+        </is>
+      </c>
+      <c r="Q282" t="inlineStr">
+        <is>
+          <t>artemis-prestige@orange.fr</t>
+        </is>
+      </c>
     </row>
     <row r="283" ht="15" customHeight="1" s="13">
-      <c r="L283" s="12" t="n"/>
+      <c r="A283" t="n">
+        <v>283</v>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C283" t="n">
+        <v>1</v>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>importateurs</t>
+        </is>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>Minéral Pierre Naturelle (Pierre de l'Est SAS)</t>
+        </is>
+      </c>
+      <c r="F283" t="inlineStr">
+        <is>
+          <t>Woustviller (magasins Lyon, Strasbourg, Nancy, Beaune, Thion</t>
+        </is>
+      </c>
+      <c r="G283" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="H283" t="inlineStr">
+        <is>
+          <t>Confirmée : spécialiste pierre naturelle (travertin, calcaire, marbre, granit...), 7 magasins France/Allemagne dont Lyon, Strasbourg, Nancy, Beaune, Thionville. Mentions légales : …</t>
+        </is>
+      </c>
+      <c r="I283" t="inlineStr">
+        <is>
+          <t>https://www.mineral-pierre-naturelle.fr/</t>
+        </is>
+      </c>
+      <c r="J283" t="inlineStr">
+        <is>
+          <t>03 60 12 33 53</t>
+        </is>
+      </c>
+      <c r="K283" t="inlineStr">
+        <is>
+          <t>Recherche Claude (26/10)</t>
+        </is>
+      </c>
+      <c r="L283" s="12" t="inlineStr">
+        <is>
+          <t>À contacter (formulaire/tél) — EN ATTENTE</t>
+        </is>
+      </c>
+      <c r="N283" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="O283" t="inlineStr">
+        <is>
+          <t>[26/10] Recherche vérifiée (segment importateurs). Confirmée : spécialiste pierre naturelle (travertin, calcaire, marbre, granit...), 7 magasins France/Allemagne dont Lyon, Strasbourg, Nancy, Beaune, Thionville. Mentions légales : Pierre de l'Est SAS, 44 Rue de Nancy, 57915 Woustviller — raison sociale et ville confirmées. AUCUN e-mail publié : vérifié sur l'accueil et les mentions légales (contact par téléphone ou formulaire uniquement). Repli téléphone VÉRIFIÉ : 03 60 12 33 53 affiché sur l'accueil (« Conseil d'expert ») et dans les mentions légales. Le produit Sinai Pearl n'était pas visible sur la portion d'accueil lue, mais l'activité calcaire/travertin est confirmée. Domaine hors liste d'exclusion. Source e-mail : aucune (pas d e-mail publié).  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="P283" t="inlineStr">
+        <is>
+          <t>5e liste — recherche (26/10)</t>
+        </is>
+      </c>
     </row>
     <row r="284" ht="15" customHeight="1" s="13">
-      <c r="L284" s="12" t="n"/>
+      <c r="A284" t="n">
+        <v>284</v>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C284" t="n">
+        <v>1</v>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>importateurs</t>
+        </is>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>Nimex International</t>
+        </is>
+      </c>
+      <c r="F284" t="inlineStr">
+        <is>
+          <t>Caissargues (dépôt à Nîmes)</t>
+        </is>
+      </c>
+      <c r="G284" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="H284" t="inlineStr">
+        <is>
+          <t>Confirmée : importateur-distributeur de pierre naturelle, marbre, granit, travertin ; approvisionnement direct carrières (Espagne, Italie, Portugal, Grèce, Turquie, ÉGYPTE, Inde) ;…</t>
+        </is>
+      </c>
+      <c r="I284" t="inlineStr">
+        <is>
+          <t>https://www.nimexinternational.fr/</t>
+        </is>
+      </c>
+      <c r="J284" t="inlineStr">
+        <is>
+          <t>04 30 22 01 75</t>
+        </is>
+      </c>
+      <c r="K284" t="inlineStr">
+        <is>
+          <t>Recherche Claude (26/10)</t>
+        </is>
+      </c>
+      <c r="L284" s="12" t="inlineStr">
+        <is>
+          <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
+        </is>
+      </c>
+      <c r="N284" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="O284" t="inlineStr">
+        <is>
+          <t>[26/10] Recherche vérifiée (segment importateurs). Confirmée : importateur-distributeur de pierre naturelle, marbre, granit, travertin ; approvisionnement direct carrières (Espagne, Italie, Portugal, Grèce, Turquie, ÉGYPTE, Inde) ; dépôt à Nîmes, vente et livraison France entière. Adresse : 14 avenue de la Vistrenque, 30132 Caissargues — ville confirmée. E-mail présent textuellement dans le pied de page du site officiel. Téléphone confirmé. L'Égypte figure parmi les pays d'approvisionnement cités. Domaine hors liste d'exclusion. Source e-mail : https://www.nimexinternational.fr/.  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="P284" t="inlineStr">
+        <is>
+          <t>5e liste — recherche (26/10)</t>
+        </is>
+      </c>
+      <c r="Q284" t="inlineStr">
+        <is>
+          <t>nimex.international@wanadoo.fr</t>
+        </is>
+      </c>
     </row>
     <row r="285" ht="15" customHeight="1" s="13">
-      <c r="L285" s="12" t="n"/>
+      <c r="A285" t="n">
+        <v>285</v>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C285" t="n">
+        <v>1</v>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>importateurs</t>
+        </is>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>Travertin.fr</t>
+        </is>
+      </c>
+      <c r="F285" t="inlineStr">
+        <is>
+          <t>Fos-sur-Mer (centre logistique)</t>
+        </is>
+      </c>
+      <c r="G285" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="H285" t="inlineStr">
+        <is>
+          <t>Confirmée : le site se décrit comme « un importateur et un grossiste spécialisé en travertin » (carrières Turquie/Italie), dalles, carrelages, margelles, livraison France entière. …</t>
+        </is>
+      </c>
+      <c r="I285" t="inlineStr">
+        <is>
+          <t>https://www.travertin.fr/</t>
+        </is>
+      </c>
+      <c r="J285" t="inlineStr">
+        <is>
+          <t>09 70 70 73 75</t>
+        </is>
+      </c>
+      <c r="K285" t="inlineStr">
+        <is>
+          <t>Recherche Claude (26/10)</t>
+        </is>
+      </c>
+      <c r="L285" s="12" t="inlineStr">
+        <is>
+          <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
+        </is>
+      </c>
+      <c r="N285" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="O285" t="inlineStr">
+        <is>
+          <t>[26/10] Recherche vérifiée (segment importateurs). Confirmée : le site se décrit comme « un importateur et un grossiste spécialisé en travertin » (carrières Turquie/Italie), dalles, carrelages, margelles, livraison France entière. Adresse : Centre Logistique, 13270 Fos-sur-Mer — ville confirmée. E-mail présent textuellement dans le bloc contact du pied de page, sous l'adresse de Fos-sur-Mer. Téléphone confirmé (en-tête et pied de page). Domaine hors liste d'exclusion. Source e-mail : https://www.travertin.fr/.  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="P285" t="inlineStr">
+        <is>
+          <t>5e liste — recherche (26/10)</t>
+        </is>
+      </c>
+      <c r="Q285" t="inlineStr">
+        <is>
+          <t>info@travertin.fr</t>
+        </is>
+      </c>
     </row>
     <row r="286" ht="15" customHeight="1" s="13">
-      <c r="L286" s="12" t="n"/>
+      <c r="A286" t="n">
+        <v>286</v>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C286" t="n">
+        <v>2</v>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>importateurs</t>
+        </is>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>Espace Travertin (EURL GNPS Espace Carrelage)</t>
+        </is>
+      </c>
+      <c r="F286" t="inlineStr">
+        <is>
+          <t>Bollène</t>
+        </is>
+      </c>
+      <c r="G286" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="H286" t="inlineStr">
+        <is>
+          <t>Confirmée partiellement : vente de travertin (dallage, margelles, plinthes, vasques, 200+ références) avec page « Devenir Revendeur » et prix de gros revendiqués ; adresse Impasse …</t>
+        </is>
+      </c>
+      <c r="I286" t="inlineStr">
+        <is>
+          <t>https://www.espace-travertin.fr/</t>
+        </is>
+      </c>
+      <c r="J286" t="inlineStr">
+        <is>
+          <t>07 68 18 70 32</t>
+        </is>
+      </c>
+      <c r="K286" t="inlineStr">
+        <is>
+          <t>Recherche Claude (26/10)</t>
+        </is>
+      </c>
+      <c r="L286" s="12" t="inlineStr">
+        <is>
+          <t>À contacter (formulaire/tél) — EN ATTENTE</t>
+        </is>
+      </c>
+      <c r="N286" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="O286" t="inlineStr">
+        <is>
+          <t>[26/10] Recherche vérifiée (segment importateurs). Confirmée partiellement : vente de travertin (dallage, margelles, plinthes, vasques, 200+ références) avec page « Devenir Revendeur » et prix de gros revendiqués ; adresse Impasse de la Rode, 84500 Bollène confirmée. Le site vend aussi aux particuliers (pas uniquement B2B). Le siège à Étoile-sur-Rhône et la raison sociale GNPS n'apparaissent pas sur la page d'accueil (le PDF CGV mentionne « stone-diffusion-centre »). AUCUN e-mail publié sur la page d'accueil (vérifié). Repli téléphone VÉRIFIÉ : 07 68 18 70 32 affiché deux fois en haut de page en lien cliquable. Domaine hors liste d'exclusion. Profil un peu plus B2C que revendiqué, mais canal revendeur réel. Source e-mail : aucune (pas d e-mail publié). ⚠️ CONCURRENT suivi dans la veille prix (ambiguïtés marbre/calcaire) — approche uniquement « reprise de lot revendeur ». NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="P286" t="inlineStr">
+        <is>
+          <t>5e liste — recherche (26/10)</t>
+        </is>
+      </c>
     </row>
     <row r="287" ht="15" customHeight="1" s="13">
-      <c r="L287" s="12" t="n"/>
+      <c r="A287" t="n">
+        <v>287</v>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C287" t="n">
+        <v>1</v>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>importateurs</t>
+        </is>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>DMC Miller</t>
+        </is>
+      </c>
+      <c r="F287" t="inlineStr">
+        <is>
+          <t>Pertuis (dépôt également à Gujan-Mestras, 33)</t>
+        </is>
+      </c>
+      <c r="G287" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="H287" t="inlineStr">
+        <is>
+          <t>Confirmée : distributeur spécialiste du travertin (dalles 1er/2e choix, margelles, plinthes, mosaïques, pavés granit), vente au m², livraison France entière. Adresse 315 Rue Benjam…</t>
+        </is>
+      </c>
+      <c r="I287" t="inlineStr">
+        <is>
+          <t>https://www.dmcmiller.com/</t>
+        </is>
+      </c>
+      <c r="J287" t="inlineStr">
+        <is>
+          <t>06 66 55 44 42</t>
+        </is>
+      </c>
+      <c r="K287" t="inlineStr">
+        <is>
+          <t>Recherche Claude (26/10)</t>
+        </is>
+      </c>
+      <c r="L287" s="12" t="inlineStr">
+        <is>
+          <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
+        </is>
+      </c>
+      <c r="N287" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="O287" t="inlineStr">
+        <is>
+          <t>[26/10] Recherche vérifiée (segment importateurs). Confirmée : distributeur spécialiste du travertin (dalles 1er/2e choix, margelles, plinthes, mosaïques, pavés granit), vente au m², livraison France entière. Adresse 315 Rue Benjamin Franklin, 84120 Pertuis + dépôts Pertuis et Gujan-Mestras — villes confirmées. E-mail présent textuellement dans le pied de page (lien mailto). Téléphone confirmé (affiché 0666554442 en en-tête, pied de page et lien WhatsApp). Domaine hors liste d'exclusion. Source e-mail : https://www.dmcmiller.com/.  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="P287" t="inlineStr">
+        <is>
+          <t>5e liste — recherche (26/10)</t>
+        </is>
+      </c>
+      <c r="Q287" t="inlineStr">
+        <is>
+          <t>contact@dmcmiller.com</t>
+        </is>
+      </c>
     </row>
     <row r="288" ht="15" customHeight="1" s="13">
-      <c r="L288" s="12" t="n"/>
+      <c r="A288" t="n">
+        <v>288</v>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C288" t="n">
+        <v>1</v>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>importateurs</t>
+        </is>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>Cupa Stone France (Cupa Pierres Distribution)</t>
+        </is>
+      </c>
+      <c r="F288" t="inlineStr">
+        <is>
+          <t>Changé (Le Mans) — réseau national d'agences</t>
+        </is>
+      </c>
+      <c r="G288" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="H288" t="inlineStr">
+        <is>
+          <t>Confirmée : distributeur national de pierre naturelle avec agences au Mans (Changé), Tours, Rennes, Nantes, Lyon, Aix-en-Provence, Quimper, Pau, Limoges, Cholet, Muzillac, La Roche…</t>
+        </is>
+      </c>
+      <c r="I288" t="inlineStr">
+        <is>
+          <t>https://www.cupastone.fr/</t>
+        </is>
+      </c>
+      <c r="J288" t="inlineStr">
+        <is>
+          <t>+33 2 43 85 06 84</t>
+        </is>
+      </c>
+      <c r="K288" t="inlineStr">
+        <is>
+          <t>Recherche Claude (26/10)</t>
+        </is>
+      </c>
+      <c r="L288" s="12" t="inlineStr">
+        <is>
+          <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
+        </is>
+      </c>
+      <c r="N288" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="O288" t="inlineStr">
+        <is>
+          <t>[26/10] Recherche vérifiée (segment importateurs). Confirmée : distributeur national de pierre naturelle avec agences au Mans (Changé), Tours, Rennes, Nantes, Lyon, Aix-en-Provence, Quimper, Pau, Limoges, Cholet, Muzillac, La Roche-sur-Yon, etc. (groupe présent aussi en Espagne/Portugal). Le téléphone +33 2 43 85 06 84 est bien celui de l'agence Le Mans (Changé), contact Amandine Renard. E-mail contact@cupastone.fr présent textuellement sur la page points de vente, répété pour la plupart des agences françaises (dont Le Mans). D'autres e-mails nominatifs existent (cleger@cupastone.fr Bordeaux, lgasse@cupastone.com Paris-IdF, sbatmale@cupastone.com Toulouse, fmadehors@cupastone.com Nord-Est) si un ciblage régional est préféré. Domaine hors liste d'exclusion. Source e-mail : https://www.cupastone.fr/points-de-vente/.  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="P288" t="inlineStr">
+        <is>
+          <t>5e liste — recherche (26/10)</t>
+        </is>
+      </c>
+      <c r="Q288" t="inlineStr">
+        <is>
+          <t>contact@cupastone.fr</t>
+        </is>
+      </c>
     </row>
     <row r="289" ht="15" customHeight="1" s="13">
-      <c r="L289" s="12" t="n"/>
+      <c r="A289" t="n">
+        <v>289</v>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C289" t="n">
+        <v>2</v>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>importateurs</t>
+        </is>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>Ti'ma Stone</t>
+        </is>
+      </c>
+      <c r="F289" t="inlineStr">
+        <is>
+          <t>Lunel (non confirmée sur le site)</t>
+        </is>
+      </c>
+      <c r="G289" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="H289" t="inlineStr">
+        <is>
+          <t>Confirmée pour l'activité : vente en ligne de pierre naturelle France entière (dallage, parement, margelles, zellige, vasques), travertin très présent, liens « Grossiste dallage » …</t>
+        </is>
+      </c>
+      <c r="I289" t="inlineStr">
+        <is>
+          <t>https://timastone.com/</t>
+        </is>
+      </c>
+      <c r="J289" t="inlineStr">
+        <is>
+          <t>04 15 54 01 25</t>
+        </is>
+      </c>
+      <c r="K289" t="inlineStr">
+        <is>
+          <t>Recherche Claude (26/10)</t>
+        </is>
+      </c>
+      <c r="L289" s="12" t="inlineStr">
+        <is>
+          <t>À contacter (formulaire/tél) — EN ATTENTE</t>
+        </is>
+      </c>
+      <c r="N289" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="O289" t="inlineStr">
+        <is>
+          <t>[26/10] Recherche vérifiée (segment importateurs). Confirmée pour l'activité : vente en ligne de pierre naturelle France entière (dallage, parement, margelles, zellige, vasques), travertin très présent, liens « Grossiste dallage » et « Fournisseur carrelage » + espace pro. La VILLE n'est PAS confirmée : aucune adresse ni ville sur la page d'accueil, et les pages /mentions-legales/ et /contact/ renvoient un 404 aux URL standards. AUCUN e-mail publié sur la page d'accueil (vérifié). Repli téléphone VÉRIFIÉ : 04 15 54 01 25 affiché en en-tête et pied de page (horaires lun-ven 9h-12h / 14h-18h). Domaine hors liste d'exclusion. Site vivant et actif, mais profil plutôt vente en ligne avec volet grossiste ; localisation Lunel à reconfirmer par téléphone avant tout engagement logistique. Source e-mail : aucune (pas d e-mail publié). ⚠️ CONCURRENT suivi dans la veille prix (42,46–59,96 €/m²) — approche uniquement « reprise de lot revendeur », aucune info sensible. NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="P289" t="inlineStr">
+        <is>
+          <t>5e liste — recherche (26/10)</t>
+        </is>
+      </c>
     </row>
     <row r="290" ht="15" customHeight="1" s="13">
-      <c r="L290" s="12" t="n"/>
+      <c r="A290" t="n">
+        <v>290</v>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C290" t="n">
+        <v>2</v>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>importateurs</t>
+        </is>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>BH Matériaux (groupe Holding Laffont)</t>
+        </is>
+      </c>
+      <c r="F290" t="inlineStr">
+        <is>
+          <t>Lauzerte</t>
+        </is>
+      </c>
+      <c r="G290" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="H290" t="inlineStr">
+        <is>
+          <t>Confirmée : grossiste revendiqué (« Votre grossiste ») en matériaux de construction/rénovation/décoration avec le travertin et le dallage pierre naturelle en gamme majeure (dallage…</t>
+        </is>
+      </c>
+      <c r="I290" t="inlineStr">
+        <is>
+          <t>https://bh-materiaux.com/</t>
+        </is>
+      </c>
+      <c r="J290" t="inlineStr">
+        <is>
+          <t>05 63 95 39 08</t>
+        </is>
+      </c>
+      <c r="K290" t="inlineStr">
+        <is>
+          <t>Recherche Claude (26/10)</t>
+        </is>
+      </c>
+      <c r="L290" s="12" t="inlineStr">
+        <is>
+          <t>À contacter (formulaire/tél) — EN ATTENTE</t>
+        </is>
+      </c>
+      <c r="N290" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="O290" t="inlineStr">
+        <is>
+          <t>[26/10] Recherche vérifiée (segment importateurs). Confirmée : grossiste revendiqué (« Votre grossiste ») en matériaux de construction/rénovation/décoration avec le travertin et le dallage pierre naturelle en gamme majeure (dallages du monde, parement, graviers, pas japonais) ; particuliers et professionnels ; retrait au dépôt de Lauzerte. Adresse 138 route de Montbarla, 82110 Lauzerte confirmée. Groupe Holding Laffont confirmé (Osagra, Laffont TP, Laffont Granulats...). AUCUN e-mail publié (vérifié sur la page d'accueil : téléphone et formulaire de rappel uniquement). Repli téléphone VÉRIFIÉ : 05 63 95 39 08 répété en en-tête et sections contact. ATTENTION : le site confirme « membre du réseau FRANCE MATERIAUX » dont le domaine france-materiaux.fr figure dans la liste d'exclusion ; le domaine propre bh-materiaux.com n'y figure pas — retenu, mais à arbitrer côté donneur d'ordre avant contact. Source e-mail : aucune (pas d e-mail publié).  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="P290" t="inlineStr">
+        <is>
+          <t>5e liste — recherche (26/10)</t>
+        </is>
+      </c>
     </row>
     <row r="291" ht="15" customHeight="1" s="13">
-      <c r="L291" s="12" t="n"/>
+      <c r="A291" t="n">
+        <v>291</v>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C291" t="n">
+        <v>2</v>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>marbreries-idf</t>
+        </is>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>Les Marbreries de la Seine (LMS Paris)</t>
+        </is>
+      </c>
+      <c r="F291" t="inlineStr">
+        <is>
+          <t>Les Pavillons-sous-Bois (ateliers) / Paris 7e (showroom)</t>
+        </is>
+      </c>
+      <c r="G291" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="H291" t="inlineStr">
+        <is>
+          <t>Confirmée : marbrerie haute décoration (architecture, mobilier, objets d'art) ; showroom 33 rue de Verneuil 75007 Paris, ateliers et logistique 2/8 allée de Londres 93320 Les Pavil…</t>
+        </is>
+      </c>
+      <c r="I291" t="inlineStr">
+        <is>
+          <t>https://www.lesmarbreriesdelaseine.com</t>
+        </is>
+      </c>
+      <c r="J291" t="inlineStr">
+        <is>
+          <t>+33 1 48 48 10 00 (showroom) / +33 1 48 48 59 76 (ateliers)</t>
+        </is>
+      </c>
+      <c r="K291" t="inlineStr">
+        <is>
+          <t>Recherche Claude (26/10)</t>
+        </is>
+      </c>
+      <c r="L291" s="12" t="inlineStr">
+        <is>
+          <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
+        </is>
+      </c>
+      <c r="N291" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="O291" t="inlineStr">
+        <is>
+          <t>[26/10] Recherche vérifiée (segment marbreries-idf). Confirmée : marbrerie haute décoration (architecture, mobilier, objets d'art) ; showroom 33 rue de Verneuil 75007 Paris, ateliers et logistique 2/8 allée de Londres 93320 Les Pavillons-sous-Bois. E-mail info@lmsparis.com lu textuellement sur la page contact du site officiel (un second e-mail info@lmsmiami.com concerne l'antenne de Miami, à ignorer). Téléphones confirmés. Domaine hors liste d'exclusion. Site officiel, pas un annuaire. Source e-mail : https://www.lesmarbreriesdelaseine.com/contact.  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="P291" t="inlineStr">
+        <is>
+          <t>5e liste — recherche (26/10)</t>
+        </is>
+      </c>
+      <c r="Q291" t="inlineStr">
+        <is>
+          <t>info@lmsparis.com</t>
+        </is>
+      </c>
     </row>
     <row r="292" ht="15" customHeight="1" s="13">
-      <c r="L292" s="12" t="n"/>
+      <c r="A292" t="n">
+        <v>292</v>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C292" t="n">
+        <v>2</v>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>marbreries-idf</t>
+        </is>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>Marbre Import</t>
+        </is>
+      </c>
+      <c r="F292" t="inlineStr">
+        <is>
+          <t>Paris 19e (118 av. Jean Jaurès) ; autre adresse affichée : B</t>
+        </is>
+      </c>
+      <c r="G292" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="H292" t="inlineStr">
+        <is>
+          <t>Confirmée : spécialiste de la pierre naturelle (marbre, granit, dalles, blocs), vente aux particuliers et professionnels (marbriers, architectes, constructeurs).</t>
+        </is>
+      </c>
+      <c r="I292" t="inlineStr">
+        <is>
+          <t>https://www.marbre-import.fr</t>
+        </is>
+      </c>
+      <c r="J292" t="inlineStr">
+        <is>
+          <t>09 72 15 80 01</t>
+        </is>
+      </c>
+      <c r="K292" t="inlineStr">
+        <is>
+          <t>Recherche Claude (26/10)</t>
+        </is>
+      </c>
+      <c r="L292" s="12" t="inlineStr">
+        <is>
+          <t>À contacter (formulaire/tél) — EN ATTENTE</t>
+        </is>
+      </c>
+      <c r="N292" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="O292" t="inlineStr">
+        <is>
+          <t>[26/10] Recherche vérifiée (segment marbreries-idf). Confirmée : spécialiste de la pierre naturelle (marbre, granit, dalles, blocs), vente aux particuliers et professionnels (marbriers, architectes, constructeurs). AUCUN e-mail publié sur la page contact du site officiel : formulaire de devis uniquement. Retenu sur la base du téléphone vérifié 09 72 15 80 01 (affiché textuellement et en lien tel: sur la page contact). Attention : la page contact affiche Paris 19e et Bordeaux ; le showroom de Villejuif annoncé dans le candidat n'y apparaît pas — à confirmer par téléphone. Domaine hors liste d'exclusion. Source e-mail : aucune (pas d e-mail publié). ⚠️ CONCURRENT suivi dans la veille prix (Crema Marfil Espagne, lot promo 20 € HT) — prudence, approche reprise de lot uniquement. NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="P292" t="inlineStr">
+        <is>
+          <t>5e liste — recherche (26/10)</t>
+        </is>
+      </c>
     </row>
     <row r="293" ht="15" customHeight="1" s="13">
-      <c r="L293" s="12" t="n"/>
+      <c r="A293" t="n">
+        <v>293</v>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C293" t="n">
+        <v>2</v>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>marbreries-idf</t>
+        </is>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>Arthema Marbre (marbrerie SPIMA)</t>
+        </is>
+      </c>
+      <c r="F293" t="inlineStr">
+        <is>
+          <t>Paris 3e (showroom 34 rue de Poitou, Le Marais)</t>
+        </is>
+      </c>
+      <c r="G293" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="H293" t="inlineStr">
+        <is>
+          <t>Confirmée : marbrerie de décoration sur mesure (marbre, pierre calcaire, travertin, onyx, granit, quartzite), fabrication en atelier partenaire SPIMA et pose ; clientèle d'architec…</t>
+        </is>
+      </c>
+      <c r="I293" t="inlineStr">
+        <is>
+          <t>https://arthema-marbre.com</t>
+        </is>
+      </c>
+      <c r="J293" t="inlineStr">
+        <is>
+          <t>01 42 71 79 09 / 06 19 26 42 68</t>
+        </is>
+      </c>
+      <c r="K293" t="inlineStr">
+        <is>
+          <t>Recherche Claude (26/10)</t>
+        </is>
+      </c>
+      <c r="L293" s="12" t="inlineStr">
+        <is>
+          <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
+        </is>
+      </c>
+      <c r="N293" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="O293" t="inlineStr">
+        <is>
+          <t>[26/10] Recherche vérifiée (segment marbreries-idf). Confirmée : marbrerie de décoration sur mesure (marbre, pierre calcaire, travertin, onyx, granit, quartzite), fabrication en atelier partenaire SPIMA et pose ; clientèle d'architectes et décorateurs. E-mail lu textuellement sur la page d'accueil du site officiel. Un mobile supplémentaire (06 19 26 42 68) y figure aussi. Travail explicite des pierres calcaires et travertins confirmé. Domaine hors liste d'exclusion. Source e-mail : https://arthema-marbre.com/.  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="P293" t="inlineStr">
+        <is>
+          <t>5e liste — recherche (26/10)</t>
+        </is>
+      </c>
+      <c r="Q293" t="inlineStr">
+        <is>
+          <t>contact@arthema-marbre.com</t>
+        </is>
+      </c>
     </row>
     <row r="294" ht="15" customHeight="1" s="13">
-      <c r="L294" s="12" t="n"/>
+      <c r="A294" t="n">
+        <v>294</v>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C294" t="n">
+        <v>2</v>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>marbreries-idf</t>
+        </is>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>Atelier Matière</t>
+        </is>
+      </c>
+      <c r="F294" t="inlineStr">
+        <is>
+          <t>Paris 16e (19 rue Vital) et Paris 17e (36 rue Brunel)</t>
+        </is>
+      </c>
+      <c r="G294" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="H294" t="inlineStr">
+        <is>
+          <t>Confirmée : studio/showroom de pierre naturelle, marbre et terrazzo haut de gamme depuis 2012, distribution et pose sur rendez-vous ; deux showrooms parisiens confirmés.</t>
+        </is>
+      </c>
+      <c r="I294" t="inlineStr">
+        <is>
+          <t>https://www.ateliermatiere.fr</t>
+        </is>
+      </c>
+      <c r="J294" t="inlineStr">
+        <is>
+          <t>01 45 04 57 65</t>
+        </is>
+      </c>
+      <c r="K294" t="inlineStr">
+        <is>
+          <t>Recherche Claude (26/10)</t>
+        </is>
+      </c>
+      <c r="L294" s="12" t="inlineStr">
+        <is>
+          <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
+        </is>
+      </c>
+      <c r="N294" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="O294" t="inlineStr">
+        <is>
+          <t>[26/10] Recherche vérifiée (segment marbreries-idf). Confirmée : studio/showroom de pierre naturelle, marbre et terrazzo haut de gamme depuis 2012, distribution et pose sur rendez-vous ; deux showrooms parisiens confirmés. E-mail lu textuellement sur la page Pierre du site officiel ; téléphone confirmé. Domaine hors liste d'exclusion. Site officiel, pas un annuaire. Source e-mail : https://www.ateliermatiere.fr/pierre.  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="P294" t="inlineStr">
+        <is>
+          <t>5e liste — recherche (26/10)</t>
+        </is>
+      </c>
+      <c r="Q294" t="inlineStr">
+        <is>
+          <t>info@ateliermatiere.fr</t>
+        </is>
+      </c>
     </row>
     <row r="295" ht="15" customHeight="1" s="13">
-      <c r="L295" s="12" t="n"/>
+      <c r="A295" t="n">
+        <v>295</v>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C295" t="n">
+        <v>2</v>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>marbreries-idf</t>
+        </is>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>Artefacts Paris</t>
+        </is>
+      </c>
+      <c r="F295" t="inlineStr">
+        <is>
+          <t>Paris 7e (showroom 17 bis passage Jean Nicot) ; atelier à Né</t>
+        </is>
+      </c>
+      <c r="G295" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="H295" t="inlineStr">
+        <is>
+          <t>Confirmée : marbrerie fine et pierre de taille, revêtements durs en pierre naturelle pour la construction et l'agencement de luxe ; showroom Paris 7e et atelier/bureau d'études à N…</t>
+        </is>
+      </c>
+      <c r="I295" t="inlineStr">
+        <is>
+          <t>https://www.artefacts-paris.com</t>
+        </is>
+      </c>
+      <c r="K295" t="inlineStr">
+        <is>
+          <t>Recherche Claude (26/10)</t>
+        </is>
+      </c>
+      <c r="L295" s="12" t="inlineStr">
+        <is>
+          <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
+        </is>
+      </c>
+      <c r="N295" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="O295" t="inlineStr">
+        <is>
+          <t>[26/10] Recherche vérifiée (segment marbreries-idf). Confirmée : marbrerie fine et pierre de taille, revêtements durs en pierre naturelle pour la construction et l'agencement de luxe ; showroom Paris 7e et atelier/bureau d'études à Nérac (47600) confirmés. E-mail lu textuellement sur le site officiel. Aucun téléphone affiché sur la page. L'atelier de façonnage est bien hors IdF (Nérac, 47) comme signalé, mais la vitrine commerciale et les chantiers sont parisiens. Domaine hors liste d'exclusion. Source e-mail : https://www.artefacts-paris.com.  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="P295" t="inlineStr">
+        <is>
+          <t>5e liste — recherche (26/10)</t>
+        </is>
+      </c>
+      <c r="Q295" t="inlineStr">
+        <is>
+          <t>info@artefacts-paris.com</t>
+        </is>
+      </c>
     </row>
     <row r="296" ht="15" customHeight="1" s="13">
-      <c r="L296" s="12" t="n"/>
+      <c r="A296" t="n">
+        <v>296</v>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C296" t="n">
+        <v>2</v>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>marbreries-idf</t>
+        </is>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>H. Chevalier</t>
+        </is>
+      </c>
+      <c r="F296" t="inlineStr">
+        <is>
+          <t>Suresnes (26 rue Henri Regnault, 92150)</t>
+        </is>
+      </c>
+      <c r="G296" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="H296" t="inlineStr">
+        <is>
+          <t>Confirmée : restauration du patrimoine bâti depuis 1946 (maçonnerie-pierre, restauration de sculpture, hôtels particuliers et châteaux), 250 salariés, 80 M€ de CA ; adresse à Sures…</t>
+        </is>
+      </c>
+      <c r="I296" t="inlineStr">
+        <is>
+          <t>https://www.hchevalier.com</t>
+        </is>
+      </c>
+      <c r="J296" t="inlineStr">
+        <is>
+          <t>01 45 06 83 33</t>
+        </is>
+      </c>
+      <c r="K296" t="inlineStr">
+        <is>
+          <t>Recherche Claude (26/10)</t>
+        </is>
+      </c>
+      <c r="L296" s="12" t="inlineStr">
+        <is>
+          <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
+        </is>
+      </c>
+      <c r="N296" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="O296" t="inlineStr">
+        <is>
+          <t>[26/10] Recherche vérifiée (segment marbreries-idf). Confirmée : restauration du patrimoine bâti depuis 1946 (maçonnerie-pierre, restauration de sculpture, hôtels particuliers et châteaux), 250 salariés, 80 M€ de CA ; adresse à Suresnes confirmée. E-mail et téléphone lus textuellement sur la page d'accueil du site officiel. Domaine hors liste d'exclusion. Profil patrimoine/monuments : pertinence moyenne pour un calcaire égyptien standard, comme indiqué dans le candidat. Source e-mail : https://www.hchevalier.com.  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="P296" t="inlineStr">
+        <is>
+          <t>5e liste — recherche (26/10)</t>
+        </is>
+      </c>
+      <c r="Q296" t="inlineStr">
+        <is>
+          <t>contact@hchevalier.com</t>
+        </is>
+      </c>
     </row>
     <row r="297" ht="15" customHeight="1" s="13">
-      <c r="L297" s="12" t="n"/>
+      <c r="A297" t="n">
+        <v>297</v>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C297" t="n">
+        <v>2</v>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>marbreries-idf</t>
+        </is>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>Vexin Patrimoine</t>
+        </is>
+      </c>
+      <c r="F297" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Secteur Vexin / Île-de-France (95) — aucune adresse précise </t>
+        </is>
+      </c>
+      <c r="G297" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="H297" t="inlineStr">
+        <is>
+          <t>Confirmée : tailleur de pierre (taille sur mesure intérieur/extérieur, restauration historique, création, sols en pierre), plus de 15 ans d'expérience, clients pro et particuliers,…</t>
+        </is>
+      </c>
+      <c r="I297" t="inlineStr">
+        <is>
+          <t>https://vexinpatrimoine.fr</t>
+        </is>
+      </c>
+      <c r="J297" t="inlineStr">
+        <is>
+          <t>01 30 73 86 50</t>
+        </is>
+      </c>
+      <c r="K297" t="inlineStr">
+        <is>
+          <t>Recherche Claude (26/10)</t>
+        </is>
+      </c>
+      <c r="L297" s="12" t="inlineStr">
+        <is>
+          <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
+        </is>
+      </c>
+      <c r="N297" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="O297" t="inlineStr">
+        <is>
+          <t>[26/10] Recherche vérifiée (segment marbreries-idf). Confirmée : tailleur de pierre (taille sur mesure intérieur/extérieur, restauration historique, création, sols en pierre), plus de 15 ans d'expérience, clients pro et particuliers, zone Vexin/Île-de-France. Deux graphies sur le site : le pied de page affiche textuellement contact@vexinpatrimoine.fr (correct) ; la barre latérale affiche la coquille « contat@vexinpatrimoine.fr ». Utiliser contact@vexinpatrimoine.fr. Téléphone confirmé (affiché deux fois). Aucune ville précise publiée, cohérent avec le candidat. Domaine hors liste d'exclusion. Source e-mail : https://vexinpatrimoine.fr/.  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="P297" t="inlineStr">
+        <is>
+          <t>5e liste — recherche (26/10)</t>
+        </is>
+      </c>
+      <c r="Q297" t="inlineStr">
+        <is>
+          <t>contact@vexinpatrimoine.fr</t>
+        </is>
+      </c>
     </row>
     <row r="298" ht="15" customHeight="1" s="13">
-      <c r="L298" s="12" t="n"/>
+      <c r="A298" t="n">
+        <v>298</v>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C298" t="n">
+        <v>2</v>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>marbreries-idf</t>
+        </is>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>Accolade Artisans</t>
+        </is>
+      </c>
+      <c r="F298" t="inlineStr">
+        <is>
+          <t>Viarmes (14 rue Kleinpeter, 95270)</t>
+        </is>
+      </c>
+      <c r="G298" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="H298" t="inlineStr">
+        <is>
+          <t>Confirmée : taille de pierre et maçonnerie de restauration du bâti ancien (certification Qualibat restauration pierre de taille et maçonnerie du patrimoine) ; adresse à Viarmes (95…</t>
+        </is>
+      </c>
+      <c r="I298" t="inlineStr">
+        <is>
+          <t>https://www.accoladeartisans.fr</t>
+        </is>
+      </c>
+      <c r="J298" t="inlineStr">
+        <is>
+          <t>06 27 85 91 92</t>
+        </is>
+      </c>
+      <c r="K298" t="inlineStr">
+        <is>
+          <t>Recherche Claude (26/10)</t>
+        </is>
+      </c>
+      <c r="L298" s="12" t="inlineStr">
+        <is>
+          <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
+        </is>
+      </c>
+      <c r="N298" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="O298" t="inlineStr">
+        <is>
+          <t>[26/10] Recherche vérifiée (segment marbreries-idf). Confirmée : taille de pierre et maçonnerie de restauration du bâti ancien (certification Qualibat restauration pierre de taille et maçonnerie du patrimoine) ; adresse à Viarmes (95270) confirmée. E-mail lu textuellement dans la section Coordonnées du pied de page ; téléphone confirmé (en-tête et pied de page). Domaine hors liste d'exclusion. Site officiel, pas un annuaire. Source e-mail : https://www.accoladeartisans.fr/taille-de-pierre.htm.  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="P298" t="inlineStr">
+        <is>
+          <t>5e liste — recherche (26/10)</t>
+        </is>
+      </c>
+      <c r="Q298" t="inlineStr">
+        <is>
+          <t>contact@accoladeartisans.fr</t>
+        </is>
+      </c>
     </row>
     <row r="299" ht="15" customHeight="1" s="13">
-      <c r="L299" s="12" t="n"/>
+      <c r="A299" t="n">
+        <v>299</v>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C299" t="n">
+        <v>2</v>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>marbreries-idf</t>
+        </is>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>Techno Pierre</t>
+        </is>
+      </c>
+      <c r="F299" t="inlineStr">
+        <is>
+          <t>Vanves (35 rue Aristide Briand, 92170)</t>
+        </is>
+      </c>
+      <c r="G299" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="H299" t="inlineStr">
+        <is>
+          <t>Confirmée : tailleur de pierres et marbrier du bâtiment (taille de pierre, marbrerie, rénovation et revêtement de façades en pierre, marbre et granit) ; adresse à Vanves confirmée.</t>
+        </is>
+      </c>
+      <c r="I299" t="inlineStr">
+        <is>
+          <t>https://www.technopierre.fr</t>
+        </is>
+      </c>
+      <c r="J299" t="inlineStr">
+        <is>
+          <t>09 74 56 39 83</t>
+        </is>
+      </c>
+      <c r="K299" t="inlineStr">
+        <is>
+          <t>Recherche Claude (26/10)</t>
+        </is>
+      </c>
+      <c r="L299" s="12" t="inlineStr">
+        <is>
+          <t>À contacter (formulaire/tél) — EN ATTENTE</t>
+        </is>
+      </c>
+      <c r="N299" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="O299" t="inlineStr">
+        <is>
+          <t>[26/10] Recherche vérifiée (segment marbreries-idf). Confirmée : tailleur de pierres et marbrier du bâtiment (taille de pierre, marbrerie, rénovation et revêtement de façades en pierre, marbre et granit) ; adresse à Vanves confirmée. AUCUN e-mail publié sur le site officiel : la page contactez-nous.php ne propose qu'un formulaire (le lien « E-mail » pointe vers ce formulaire, pas vers une adresse). Retenu sur la base du téléphone vérifié 09 74 56 39 83, affiché plusieurs fois sur la page. Domaine hors liste d'exclusion. Source e-mail : aucune (pas d e-mail publié).  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="P299" t="inlineStr">
+        <is>
+          <t>5e liste — recherche (26/10)</t>
+        </is>
+      </c>
     </row>
     <row r="300" ht="15" customHeight="1" s="13">
-      <c r="L300" s="12" t="n"/>
+      <c r="A300" t="n">
+        <v>300</v>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C300" t="n">
+        <v>1</v>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>normandie</t>
+        </is>
+      </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>Guilloux Matériaux</t>
+        </is>
+      </c>
+      <c r="F300" t="inlineStr">
+        <is>
+          <t>Cormeilles (27) et Rouen (76) — siège Saint-Pair-sur-Mer (50</t>
+        </is>
+      </c>
+      <c r="G300" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="H300" t="inlineStr">
+        <is>
+          <t>Confirmé : négoce indépendant de matériaux de construction, 10 agences en Normandie (dont Cormeilles 27 et Rouen 76), scierie/atelier à Vire, siège à Saint-Pair-sur-Mer (50380).</t>
+        </is>
+      </c>
+      <c r="I300" t="inlineStr">
+        <is>
+          <t>https://www.guillouxmateriaux.com</t>
+        </is>
+      </c>
+      <c r="J300" t="inlineStr">
+        <is>
+          <t>02 33 48 14 44 (siège) ; agence Cormeilles 02 32 57 15 98 ; agence Rouen 02 32 12 11 80</t>
+        </is>
+      </c>
+      <c r="K300" t="inlineStr">
+        <is>
+          <t>Recherche Claude (26/10)</t>
+        </is>
+      </c>
+      <c r="L300" s="12" t="inlineStr">
+        <is>
+          <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
+        </is>
+      </c>
+      <c r="N300" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="O300" t="inlineStr">
+        <is>
+          <t>[26/10] Recherche vérifiée (segment normandie). Confirmé : négoce indépendant de matériaux de construction, 10 agences en Normandie (dont Cormeilles 27 et Rouen 76), scierie/atelier à Vire, siège à Saint-Pair-sur-Mer (50380). E-mail lu TEXTUELLEMENT sur les mentions légales (responsable de la publication). Attention : le domaine de l'e-mail (guilloux-materiaux.com, avec tiret) diffère du domaine du site (guillouxmateriaux.com) — c'est bien ce qu'affiche le site officiel. Téléphones siège/Cormeilles/Rouen tous confirmés sur la même page. Hors liste d'exclusion. Source e-mail : https://www.guillouxmateriaux.com/mentions-legales-guilloux-materiaux-le-specialiste-des-materiaux-de-construction/.  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="P300" t="inlineStr">
+        <is>
+          <t>5e liste — recherche (26/10)</t>
+        </is>
+      </c>
+      <c r="Q300" t="inlineStr">
+        <is>
+          <t>bonjour@guilloux-materiaux.com</t>
+        </is>
+      </c>
     </row>
     <row r="301" ht="15" customHeight="1" s="13">
-      <c r="L301" s="12" t="n"/>
+      <c r="A301" t="n">
+        <v>301</v>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C301" t="n">
+        <v>1</v>
+      </c>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>normandie</t>
+        </is>
+      </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>Sani 27 (« Le Géant du carrelage »)</t>
+        </is>
+      </c>
+      <c r="F301" t="inlineStr">
+        <is>
+          <t>Angerville-la-Campagne (27930), ZAC de Villeneuve — près d'É</t>
+        </is>
+      </c>
+      <c r="G301" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="H301" t="inlineStr">
+        <is>
+          <t>Confirmé : magasin spécialiste du carrelage (« le plus grand magasin de carrelage ») avec sanitaire, robinetterie et meubles de salle de bain ; adresse ZAC de Villeneuve, 27930 Ang…</t>
+        </is>
+      </c>
+      <c r="I301" t="inlineStr">
+        <is>
+          <t>https://sani27.com</t>
+        </is>
+      </c>
+      <c r="J301" t="inlineStr">
+        <is>
+          <t>02 32 28 00 12</t>
+        </is>
+      </c>
+      <c r="K301" t="inlineStr">
+        <is>
+          <t>Recherche Claude (26/10)</t>
+        </is>
+      </c>
+      <c r="L301" s="12" t="inlineStr">
+        <is>
+          <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
+        </is>
+      </c>
+      <c r="N301" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="O301" t="inlineStr">
+        <is>
+          <t>[26/10] Recherche vérifiée (segment normandie). Confirmé : magasin spécialiste du carrelage (« le plus grand magasin de carrelage ») avec sanitaire, robinetterie et meubles de salle de bain ; adresse ZAC de Villeneuve, 27930 Angerville-la-Campagne, zone d'Évreux. contact@sani27.fr est écrit TEXTUELLEMENT dans le pied de page du site officiel. Divergence confirmée : le lien mailto associé pointe vers sani27@wanadoo.fr — en cas de non-réponse sur contact@sani27.fr, utiliser sani27@wanadoo.fr en seconde adresse. Téléphone 02 32 28 00 12 confirmé. Hors liste d'exclusion. Source e-mail : https://sani27.com/.  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="P301" t="inlineStr">
+        <is>
+          <t>5e liste — recherche (26/10)</t>
+        </is>
+      </c>
+      <c r="Q301" t="inlineStr">
+        <is>
+          <t>contact@sani27.fr</t>
+        </is>
+      </c>
     </row>
     <row r="302" ht="15" customHeight="1" s="13">
-      <c r="L302" s="12" t="n"/>
+      <c r="A302" t="n">
+        <v>302</v>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C302" t="n">
+        <v>1</v>
+      </c>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>normandie</t>
+        </is>
+      </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>BCA Matériaux Anciens</t>
+        </is>
+      </c>
+      <c r="F302" t="inlineStr">
+        <is>
+          <t>Méry-Corbon (14370) et Pont-l'Évêque (14130) — siège Segré-e</t>
+        </is>
+      </c>
+      <c r="G302" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="H302" t="inlineStr">
+        <is>
+          <t>Confirmé : « Spécialiste des matériaux anciens » — dallages et carrelages anciens en pierre, parquets anciens, tomettes, pavés, parements pierre, cheminées ; deux agences normandes…</t>
+        </is>
+      </c>
+      <c r="I302" t="inlineStr">
+        <is>
+          <t>https://www.bca-materiauxanciens.com</t>
+        </is>
+      </c>
+      <c r="J302" t="inlineStr">
+        <is>
+          <t>02 31 23 95 87 (Méry-Corbon) ; 02 61 67 23 40 (Pont-l'Évêque) ; +33 (0)2 41 61 62 40 (siège)</t>
+        </is>
+      </c>
+      <c r="K302" t="inlineStr">
+        <is>
+          <t>Recherche Claude (26/10)</t>
+        </is>
+      </c>
+      <c r="L302" s="12" t="inlineStr">
+        <is>
+          <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
+        </is>
+      </c>
+      <c r="N302" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="O302" t="inlineStr">
+        <is>
+          <t>[26/10] Recherche vérifiée (segment normandie). Confirmé : « Spécialiste des matériaux anciens » — dallages et carrelages anciens en pierre, parquets anciens, tomettes, pavés, parements pierre, cheminées ; deux agences normandes (Méry-Corbon et Pont-l'Évêque), siège en Pays de la Loire. normandie@bcamateriaux.com (agence Méry-Corbon) lu TEXTUELLEMENT sur le site officiel, ainsi que pontleveque@bcamateriaux.com, info@bcamateriaux.com et david@bcamateriaux.com (anglais). Tous les téléphones confirmés. Cœur de métier aligné (dallages pierre par lots). Hors liste d'exclusion. Source e-mail : https://www.bca-materiauxanciens.com.  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="P302" t="inlineStr">
+        <is>
+          <t>5e liste — recherche (26/10)</t>
+        </is>
+      </c>
+      <c r="Q302" t="inlineStr">
+        <is>
+          <t>normandie@bcamateriaux.com</t>
+        </is>
+      </c>
     </row>
     <row r="303" ht="15" customHeight="1" s="13">
-      <c r="L303" s="12" t="n"/>
+      <c r="A303" t="n">
+        <v>303</v>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C303" t="n">
+        <v>2</v>
+      </c>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>normandie</t>
+        </is>
+      </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>Adéquate - Marbrerie Décorative</t>
+        </is>
+      </c>
+      <c r="F303" t="inlineStr">
+        <is>
+          <t>Seulline (14310), ZA Eco 5 — près de Caen</t>
+        </is>
+      </c>
+      <c r="G303" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="H303" t="inlineStr">
+        <is>
+          <t>Confirmé : marbrerie décorative avec showroom (visites sur rendez-vous), ZA Eco 5 n° 7 et 9, 14310 Seulline, « près de Caen en Normandie ».</t>
+        </is>
+      </c>
+      <c r="I303" t="inlineStr">
+        <is>
+          <t>https://www.adequatemarbrerie.fr</t>
+        </is>
+      </c>
+      <c r="J303" t="inlineStr">
+        <is>
+          <t>02 31 24 11 22</t>
+        </is>
+      </c>
+      <c r="K303" t="inlineStr">
+        <is>
+          <t>Recherche Claude (26/10)</t>
+        </is>
+      </c>
+      <c r="L303" s="12" t="inlineStr">
+        <is>
+          <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
+        </is>
+      </c>
+      <c r="N303" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="O303" t="inlineStr">
+        <is>
+          <t>[26/10] Recherche vérifiée (segment normandie). Confirmé : marbrerie décorative avec showroom (visites sur rendez-vous), ZA Eco 5 n° 7 et 9, 14310 Seulline, « près de Caen en Normandie ». contact@adequatemarbrerie.fr lu TEXTUELLEMENT sur la page contact du site officiel (en texte et en lien mailto, concordants). Téléphone confirmé. Hors liste d'exclusion. Source e-mail : https://www.adequatemarbrerie.fr/contact.  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="P303" t="inlineStr">
+        <is>
+          <t>5e liste — recherche (26/10)</t>
+        </is>
+      </c>
+      <c r="Q303" t="inlineStr">
+        <is>
+          <t>contact@adequatemarbrerie.fr</t>
+        </is>
+      </c>
     </row>
     <row r="304" ht="15" customHeight="1" s="13">
-      <c r="L304" s="12" t="n"/>
+      <c r="A304" t="n">
+        <v>304</v>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C304" t="n">
+        <v>2</v>
+      </c>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>normandie</t>
+        </is>
+      </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>Motte Décoration</t>
+        </is>
+      </c>
+      <c r="F304" t="inlineStr">
+        <is>
+          <t>Le Pré-d'Auge (14340), 10 Chemin des Vatines — entre Cambrem</t>
+        </is>
+      </c>
+      <c r="G304" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="H304" t="inlineStr">
+        <is>
+          <t>Confirmé via sources tierces : société MOTTE DECORATION immatriculée (SIREN 844835728, taille/façonnage/finissage de pierres) au Pré-d'Auge (14340) ; marbrerie décorative familiale…</t>
+        </is>
+      </c>
+      <c r="I304" t="inlineStr">
+        <is>
+          <t>https://www.mottedecoration.com</t>
+        </is>
+      </c>
+      <c r="J304" t="inlineStr">
+        <is>
+          <t>02 31 32 22 00</t>
+        </is>
+      </c>
+      <c r="K304" t="inlineStr">
+        <is>
+          <t>Recherche Claude (26/10)</t>
+        </is>
+      </c>
+      <c r="L304" s="12" t="inlineStr">
+        <is>
+          <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
+        </is>
+      </c>
+      <c r="N304" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="O304" t="inlineStr">
+        <is>
+          <t>[26/10] Recherche vérifiée (segment normandie). Confirmé via sources tierces : société MOTTE DECORATION immatriculée (SIREN 844835728, taille/façonnage/finissage de pierres) au Pré-d'Auge (14340) ; marbrerie décorative familiale (marbre, granit, quartz, pierre naturelle) intervenant sur toute la Normandie — societe.com, Initiative Calvados, Pages Jaunes et index du site officiel concordants. E-mail NON confirmé textuellement : le site officiel refuse toute lecture automatisée (HTTP 401 sur l'accueil et la page contact), vérification visuelle impossible ici. L'index du moteur de recherche attribue bien contact@mottedecoration.com et le 02 31 32 22 00 au site officiel, et le téléphone est corroboré par plusieurs sources indépendantes. Retenu sur REPLI TÉLÉPHONE vérifié (02 31 32 22 00) ; ne pas utiliser l'e-mail avant confirmation visuelle sur le site. Hors liste d'exclusion. Entreprise réelle, en France, site vivant (blocage anti-robot, pas site mort). Source e-mail : aucune (pas d e-mail publié).  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="P304" t="inlineStr">
+        <is>
+          <t>5e liste — recherche (26/10)</t>
+        </is>
+      </c>
+      <c r="Q304" t="inlineStr">
+        <is>
+          <t>contact@mottedecoration.com</t>
+        </is>
+      </c>
     </row>
     <row r="305" ht="15" customHeight="1" s="13">
-      <c r="L305" s="12" t="n"/>
+      <c r="A305" t="n">
+        <v>305</v>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C305" t="n">
+        <v>2</v>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>normandie</t>
+        </is>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>Carreau Déco (SARL)</t>
+        </is>
+      </c>
+      <c r="F305" t="inlineStr">
+        <is>
+          <t>Évreux (27) ; autres magasins : Barentin, Tourville-la-Riviè</t>
+        </is>
+      </c>
+      <c r="G305" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="H305" t="inlineStr">
+        <is>
+          <t>Confirmé : enseigne de carrelage (« Carrelage haut de gamme, sol et mur ») — grès cérame, dalles, faïence, intérieur/extérieur ; 6 points de vente confirmés dont Évreux, Barentin, …</t>
+        </is>
+      </c>
+      <c r="I305" t="inlineStr">
+        <is>
+          <t>https://www.carreaudeco.com</t>
+        </is>
+      </c>
+      <c r="J305" t="inlineStr">
+        <is>
+          <t>02 32 30 62 04 (Évreux) ; 02 37 21 27 80 (Lèves/standard) ; 02 78 77 51 00 (Barentin) ; 02 78 77 09 77 (Tourville) ; 02 78 93 05 05 (Montivilliers) ; 02 37 46 23 27 (Vernouillet)</t>
+        </is>
+      </c>
+      <c r="K305" t="inlineStr">
+        <is>
+          <t>Recherche Claude (26/10)</t>
+        </is>
+      </c>
+      <c r="L305" s="12" t="inlineStr">
+        <is>
+          <t>À contacter (formulaire/tél) — EN ATTENTE</t>
+        </is>
+      </c>
+      <c r="N305" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="O305" t="inlineStr">
+        <is>
+          <t>[26/10] Recherche vérifiée (segment normandie). Confirmé : enseigne de carrelage (« Carrelage haut de gamme, sol et mur ») — grès cérame, dalles, faïence, intérieur/extérieur ; 6 points de vente confirmés dont Évreux, Barentin, Tourville-la-Rivière et Montivilliers. AUCUN e-mail publié textuellement sur le site officiel (formulaire de contact uniquement) — vérifié. Retenu sur REPLI TÉLÉPHONE : les 6 numéros de magasins sont confirmés sur le site officiel, dont Évreux 02 32 30 62 04 et le standard de Lèves 02 37 21 27 80. Hors liste d'exclusion. Source e-mail : aucune (pas d e-mail publié).  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="P305" t="inlineStr">
+        <is>
+          <t>5e liste — recherche (26/10)</t>
+        </is>
+      </c>
     </row>
     <row r="306" ht="15" customHeight="1" s="13">
-      <c r="L306" s="12" t="n"/>
+      <c r="A306" t="n">
+        <v>306</v>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C306" t="n">
+        <v>2</v>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>normandie</t>
+        </is>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>Carré &amp; Déco (SAS Fortin Design)</t>
+        </is>
+      </c>
+      <c r="F306" t="inlineStr">
+        <is>
+          <t>Colombelles (14460), 6 rue de la Métallurgie — agglomération</t>
+        </is>
+      </c>
+      <c r="G306" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="H306" t="inlineStr">
+        <is>
+          <t>Confirmé : magasin de carrelage et céramique avec showroom (« votre expert en carrelage et céramique à proximité de Caen »), pierre naturelle présente en gamme extérieure (activité…</t>
+        </is>
+      </c>
+      <c r="I306" t="inlineStr">
+        <is>
+          <t>https://carre-deco.fr</t>
+        </is>
+      </c>
+      <c r="J306" t="inlineStr">
+        <is>
+          <t>02 31 34 40 50</t>
+        </is>
+      </c>
+      <c r="K306" t="inlineStr">
+        <is>
+          <t>Recherche Claude (26/10)</t>
+        </is>
+      </c>
+      <c r="L306" s="12" t="inlineStr">
+        <is>
+          <t>À contacter (formulaire/tél) — EN ATTENTE</t>
+        </is>
+      </c>
+      <c r="N306" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="O306" t="inlineStr">
+        <is>
+          <t>[26/10] Recherche vérifiée (segment normandie). Confirmé : magasin de carrelage et céramique avec showroom (« votre expert en carrelage et céramique à proximité de Caen »), pierre naturelle présente en gamme extérieure (activité secondaire). AUCUN e-mail publié textuellement sur le site officiel (formulaire uniquement) — vérifié. Retenu sur REPLI TÉLÉPHONE : 02 31 34 40 50 confirmé sur le site officiel, adresse Colombelles confirmée. Nuance : la pierre naturelle n'est pas son cœur de métier (carrelage/céramique d'abord). Hors liste d'exclusion. Source e-mail : aucune (pas d e-mail publié).  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="P306" t="inlineStr">
+        <is>
+          <t>5e liste — recherche (26/10)</t>
+        </is>
+      </c>
     </row>
     <row r="307" ht="15" customHeight="1" s="13">
-      <c r="L307" s="12" t="n"/>
+      <c r="A307" t="n">
+        <v>307</v>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C307" t="n">
+        <v>2</v>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>destockage-exterieur</t>
+        </is>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>Vallois (groupe Spie batignolles paysage) — agence Val de Seine</t>
+        </is>
+      </c>
+      <c r="F307" t="inlineStr">
+        <is>
+          <t>Val-de-Reuil (27100, Z.A la Comminière) — agence IDF à Trapp</t>
+        </is>
+      </c>
+      <c r="G307" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="H307" t="inlineStr">
+        <is>
+          <t>Confirmée : « aménagements paysagers » dans le Grand Ouest, société de Spie batignolles paysage (vérifié sur la page d'accueil) ; la page contact confirme l'agence Val de Seine à V…</t>
+        </is>
+      </c>
+      <c r="I307" t="inlineStr">
+        <is>
+          <t>https://www.vallois.eu/</t>
+        </is>
+      </c>
+      <c r="J307" t="inlineStr">
+        <is>
+          <t>02 32 40 32 30 (Val de Seine) ; 01 30 16 07 00 (IDF Trappes)</t>
+        </is>
+      </c>
+      <c r="K307" t="inlineStr">
+        <is>
+          <t>Recherche Claude (26/10)</t>
+        </is>
+      </c>
+      <c r="L307" s="12" t="inlineStr">
+        <is>
+          <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
+        </is>
+      </c>
+      <c r="N307" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="O307" t="inlineStr">
+        <is>
+          <t>[26/10] Recherche vérifiée (segment destockage-exterieur). Confirmée : « aménagements paysagers » dans le Grand Ouest, société de Spie batignolles paysage (vérifié sur la page d'accueil) ; la page contact confirme l'agence Val de Seine à Val-de-Reuil 27100 et l'agence IDF à Trappes 78190. E-mail lu textuellement dans la fiche « Agence Val de Seine » de la page contact ; les deux téléphones y figurent aussi textuellement. Précision : la page contact donne comme siège social de Spie batignolles paysage Nanterre (92) et comme siège administratif St Hymer (14) ; Mirville (76210) est l'adresse de l'agence de l'Estuaire, pas du siège. Hors liste d'exclusion. Candidat solide. Source e-mail : https://www.vallois.eu/contact.  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="P307" t="inlineStr">
+        <is>
+          <t>5e liste — recherche (26/10)</t>
+        </is>
+      </c>
+      <c r="Q307" t="inlineStr">
+        <is>
+          <t>agence-valdeseine@vallois.eu</t>
+        </is>
+      </c>
     </row>
     <row r="308" ht="15" customHeight="1" s="13">
-      <c r="L308" s="12" t="n"/>
+      <c r="A308" t="n">
+        <v>308</v>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C308" t="n">
+        <v>1</v>
+      </c>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>destockage-exterieur</t>
+        </is>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>Tricycle Environnement / Bâticycle</t>
+        </is>
+      </c>
+      <c r="F308" t="inlineStr">
+        <is>
+          <t>Gennevilliers (120 rue du Moulin de Cage, 92230)</t>
+        </is>
+      </c>
+      <c r="G308" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="H308" t="inlineStr">
+        <is>
+          <t>Confirmée : « Matériaux BTP d'occasion », « Réemploi de matériaux de second œuvre », « Curage de bâtiment » — réemploi/revente de matériaux de construction, vérifié sur le site off…</t>
+        </is>
+      </c>
+      <c r="I308" t="inlineStr">
+        <is>
+          <t>https://www.tricycle-environnement.fr/</t>
+        </is>
+      </c>
+      <c r="J308" t="inlineStr">
+        <is>
+          <t>07 60 62 41 36</t>
+        </is>
+      </c>
+      <c r="K308" t="inlineStr">
+        <is>
+          <t>Recherche Claude (26/10)</t>
+        </is>
+      </c>
+      <c r="L308" s="12" t="inlineStr">
+        <is>
+          <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
+        </is>
+      </c>
+      <c r="N308" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="O308" t="inlineStr">
+        <is>
+          <t>[26/10] Recherche vérifiée (segment destockage-exterieur). Confirmée : « Matériaux BTP d'occasion », « Réemploi de matériaux de second œuvre », « Curage de bâtiment » — réemploi/revente de matériaux de construction, vérifié sur le site officiel. E-mail lu textuellement en en-tête ET en pied de page ; téléphone confirmé sous deux formats (+33 7 60 62 41 36 / 07 60 62 41 36) ; adresse 120 rue du Moulin de Cage, 92230 Gennevilliers confirmée en pied de page — la ville même du stock. Hors liste d'exclusion. Candidat solide. Source e-mail : https://www.tricycle-environnement.fr/.  📍 Même ville que le dépôt (Gennevilliers) — réemploi : bon candidat reprise de lot. NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="P308" t="inlineStr">
+        <is>
+          <t>5e liste — recherche (26/10)</t>
+        </is>
+      </c>
+      <c r="Q308" t="inlineStr">
+        <is>
+          <t>contact@tri-cycle.fr</t>
+        </is>
+      </c>
     </row>
     <row r="309" ht="15" customHeight="1" s="13">
-      <c r="L309" s="12" t="n"/>
+      <c r="A309" t="n">
+        <v>309</v>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C309" t="n">
+        <v>2</v>
+      </c>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>destockage-exterieur</t>
+        </is>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>Minéka</t>
+        </is>
+      </c>
+      <c r="F309" t="inlineStr">
+        <is>
+          <t>Villeurbanne (182 rue de la Poudrette, 69100)</t>
+        </is>
+      </c>
+      <c r="G309" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="H309" t="inlineStr">
+        <is>
+          <t>Confirmée : adresse « 182 rue de la Poudrette 69100 VILLEURBANNE » vérifiée dans les mentions légales, qui mentionnent aussi le magasin « Minéstock » (« Venez nous voir au Minéstoc…</t>
+        </is>
+      </c>
+      <c r="I309" t="inlineStr">
+        <is>
+          <t>https://mineka.fr/</t>
+        </is>
+      </c>
+      <c r="K309" t="inlineStr">
+        <is>
+          <t>Recherche Claude (26/10)</t>
+        </is>
+      </c>
+      <c r="L309" s="12" t="inlineStr">
+        <is>
+          <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
+        </is>
+      </c>
+      <c r="N309" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="O309" t="inlineStr">
+        <is>
+          <t>[26/10] Recherche vérifiée (segment destockage-exterieur). Confirmée : adresse « 182 rue de la Poudrette 69100 VILLEURBANNE » vérifiée dans les mentions légales, qui mentionnent aussi le magasin « Minéstock » (« Venez nous voir au Minéstock ») — structure de collecte/revente avec point de vente physique, pas une pure marketplace. E-mail lu textuellement dans les mentions légales (« Adresse électronique : contact@mineka.fr »), seule adresse de la page. AUCUN téléphone publié : le contact ne pourra se faire que par e-mail (vérifié). En France (Lyon/Villeurbanne) ; limite logistique : loin des stocks de Vernon/Gennevilliers, retrait à organiser. Hors liste d'exclusion. Source e-mail : https://mineka.fr/mentions-legales/.  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="P309" t="inlineStr">
+        <is>
+          <t>5e liste — recherche (26/10)</t>
+        </is>
+      </c>
+      <c r="Q309" t="inlineStr">
+        <is>
+          <t>contact@mineka.fr</t>
+        </is>
+      </c>
     </row>
     <row r="310" ht="15" customHeight="1" s="13">
-      <c r="L310" s="12" t="n"/>
+      <c r="A310" t="n">
+        <v>310</v>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C310" t="n">
+        <v>2</v>
+      </c>
+      <c r="D310" t="inlineStr">
+        <is>
+          <t>destockage-exterieur</t>
+        </is>
+      </c>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>Pinson Paysage (groupe Osmaïa)</t>
+        </is>
+      </c>
+      <c r="F310" t="inlineStr">
+        <is>
+          <t>Andilly (13 avenue des Cures, 95580)</t>
+        </is>
+      </c>
+      <c r="G310" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="H310" t="inlineStr">
+        <is>
+          <t>Confirmée : page « Nous contacter » vérifiée — siège « 13 Avenue des Cures, 95580 Andilly » ; activités « Création », « Entretien » (espaces verts) et « Génie écologique » affichée…</t>
+        </is>
+      </c>
+      <c r="I310" t="inlineStr">
+        <is>
+          <t>https://www.pinson-paysage.com/</t>
+        </is>
+      </c>
+      <c r="K310" t="inlineStr">
+        <is>
+          <t>Recherche Claude (26/10)</t>
+        </is>
+      </c>
+      <c r="L310" s="12" t="inlineStr">
+        <is>
+          <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
+        </is>
+      </c>
+      <c r="N310" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="O310" t="inlineStr">
+        <is>
+          <t>[26/10] Recherche vérifiée (segment destockage-exterieur). Confirmée : page « Nous contacter » vérifiée — siège « 13 Avenue des Cures, 95580 Andilly » ; activités « Création », « Entretien » (espaces verts) et « Génie écologique » affichées, cohérentes avec une entreprise paysagère IDF. E-mail lu textuellement (seule adresse de la page). AUCUN téléphone sur la page contact (formulaire uniquement) : contact par e-mail vérifié. Réserve maintenue : le site met en avant le végétal/génie écologique plus que la maçonnerie minérale — pertinence segment (b) à pondérer. Hors liste d'exclusion. Source e-mail : https://www.pinson-paysage.com/nous-contacter/.  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="P310" t="inlineStr">
+        <is>
+          <t>5e liste — recherche (26/10)</t>
+        </is>
+      </c>
+      <c r="Q310" t="inlineStr">
+        <is>
+          <t>pinson@pinson-paysage.com</t>
+        </is>
+      </c>
     </row>
     <row r="311" ht="15" customHeight="1" s="13">
-      <c r="L311" s="12" t="n"/>
+      <c r="A311" t="n">
+        <v>311</v>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C311" t="n">
+        <v>1</v>
+      </c>
+      <c r="D311" t="inlineStr">
+        <is>
+          <t>destockage-exterieur</t>
+        </is>
+      </c>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>NOZ (centrale d'achat S.F.N.)</t>
+        </is>
+      </c>
+      <c r="F311" t="inlineStr">
+        <is>
+          <t>Saint-Berthevin (53940)</t>
+        </is>
+      </c>
+      <c r="G311" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="H311" t="inlineStr">
+        <is>
+          <t>Confirmée : page contact vérifiée — adresse « 53940 Saint-Berthevin – France », formulaire avec champ « Vous êtes ? » incluant « Je suis un fournisseur » et objet « Besoin de désto…</t>
+        </is>
+      </c>
+      <c r="I311" t="inlineStr">
+        <is>
+          <t>https://www.noz.fr/</t>
+        </is>
+      </c>
+      <c r="J311" t="inlineStr">
+        <is>
+          <t>02 43 01 53 54</t>
+        </is>
+      </c>
+      <c r="K311" t="inlineStr">
+        <is>
+          <t>Recherche Claude (26/10)</t>
+        </is>
+      </c>
+      <c r="L311" s="12" t="inlineStr">
+        <is>
+          <t>À contacter (formulaire/tél) — EN ATTENTE</t>
+        </is>
+      </c>
+      <c r="N311" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="O311" t="inlineStr">
+        <is>
+          <t>[26/10] Recherche vérifiée (segment destockage-exterieur). Confirmée : page contact vérifiée — adresse « 53940 Saint-Berthevin – France », formulaire avec champ « Vous êtes ? » incluant « Je suis un fournisseur » et objet « Besoin de déstockage », cohérent avec l'activité de rachat de surstocks/lots. RETENU SANS E-MAIL : aucun e-mail publié sur https://www.noz.fr/contactez-nous/ (revérifié le 26/10/2026 — le seul mot « Email » est un champ de formulaire), mais le téléphone 02 43 01 53 54 y est écrit textuellement et vérifié ; contact via ce numéro ou le formulaire fournisseur « Besoin de déstockage ». Hors liste d'exclusion. Réserve : lot minéral lourd atypique dans leur mix. Source e-mail : aucune (pas d e-mail publié).  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="P311" t="inlineStr">
+        <is>
+          <t>5e liste — recherche (26/10)</t>
+        </is>
+      </c>
     </row>
     <row r="312" ht="15" customHeight="1" s="13">
       <c r="L312" s="12" t="n"/>

</xml_diff>

<commit_message>
Croisement fichier prospects 26/10 : 7 ajouts, 3 corrections, plan d'attaque
- Corrections : Le Monde de la Pierre = déjà contacté 12/10 (faux « nouveau »
  du fichier, non ré-ajouté) ; Marbre Import = contacté le 20/10, ne pas
  réexpédier ; La Roche Taillée enrichie (e-mail + tél).
- 17 fiches enrichies (téléphones, e-mails alternatifs, divergences notées :
  Tricycle, Eurovia, Keravis, Guilloux, Cupa IdF, NOZ, Espace Travertin…).
- 7 nouvelles sociétés « 5e liste — croisement (26/10) » : ILDEI, La Marbrerie
  Contemporaine, Paris Roches, Alpha Marbre, Caudron, Facomat, MasterPierre.
- Nouveau plan d'attaque 27/10 : vagues 1-3, Top 8, verrou global zéro envoi,
  règles d'identité (From réel info@pierredegypte.online via Network Solutions,
  interdiction customerservice@/Hotmail).
- CSV ré-exporté (garde-fou prix OK, 317 lignes).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xqm9tFtdvLdJdkiWw2VVp6
</commit_message>
<xml_diff>
--- a/minyala/clients-potentiels.xlsx
+++ b/minyala/clients-potentiels.xlsx
@@ -6357,7 +6357,11 @@
           <t>www.la-roche-taillee.fr</t>
         </is>
       </c>
-      <c r="J71" s="15" t="n"/>
+      <c r="J71" s="15" t="inlineStr">
+        <is>
+          <t>02 35 72 01 62</t>
+        </is>
+      </c>
       <c r="K71" s="20" t="inlineStr">
         <is>
           <t>Voir</t>
@@ -6370,10 +6374,19 @@
       </c>
       <c r="M71" s="21" t="n"/>
       <c r="N71" s="21" t="n"/>
-      <c r="O71" s="21" t="n"/>
+      <c r="O71" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> [26/10 croisement fichier propriétaire] E-mail et tél apportés par le fichier (Sotteville-lès-Rouen). NE RIEN ENVOYER — vrai From info@pierredegypte.online via Network Solutions à vérifier avant tout contact</t>
+        </is>
+      </c>
       <c r="P71" s="15" t="inlineStr">
         <is>
           <t>2e liste (12/10)</t>
+        </is>
+      </c>
+      <c r="Q71" t="inlineStr">
+        <is>
+          <t>contact@la-roche-taillee.fr</t>
         </is>
       </c>
     </row>
@@ -18894,7 +18907,7 @@
       </c>
       <c r="I267" s="12" t="inlineStr">
         <is>
-          <t>https://www.adi-roc.fr</t>
+          <t>https://www.adiroc.fr/produit/pierre-egypte/</t>
         </is>
       </c>
       <c r="J267" s="12" t="inlineStr">
@@ -18919,7 +18932,7 @@
       </c>
       <c r="O267" s="12" t="inlineStr">
         <is>
-          <t>[26/10] Relais assistant tiers du 26/10 (dédupliqué Gmail/Contacts) — e-mail « vérifié » par le relais, à re-confirmer sur site officiel avant envoi. Pas d'e-mail publié : formulaire du site ou téléphone. NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi</t>
+          <t>[26/10] Relais assistant tiers du 26/10 (dédupliqué Gmail/Contacts) — e-mail « vérifié » par le relais, à re-confirmer sur site officiel avant envoi. Pas d'e-mail publié : formulaire du site ou téléphone. NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi [26/10 croisement fichier propriétaire] Site/preuve (fichier) : adiroc.fr — page « pierre d'Égypte 20 mm » confirmée. Limite : peut déjà avoir un fournisseur égyptien.</t>
         </is>
       </c>
       <c r="P267" s="12" t="inlineStr">
@@ -19148,7 +19161,7 @@
       </c>
       <c r="O270" s="12" t="inlineStr">
         <is>
-          <t>[26/10] Relais assistant tiers du 26/10 (dédupliqué Gmail/Contacts) — e-mail « vérifié » par le relais, à re-confirmer sur site officiel avant envoi.  NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi</t>
+          <t>[26/10] Relais assistant tiers du 26/10 (dédupliqué Gmail/Contacts) — e-mail « vérifié » par le relais, à re-confirmer sur site officiel avant envoi.  NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi [26/10 croisement fichier propriétaire] Le fichier précise : vend déjà une gamme « Egypta » → angle « second fournisseur différencié ».</t>
         </is>
       </c>
       <c r="P270" s="12" t="inlineStr">
@@ -19269,7 +19282,7 @@
       </c>
       <c r="J272" s="12" t="inlineStr">
         <is>
-          <t>06 87 53 33 76</t>
+          <t>06 87 53 33 76 / 02 37 48 79 91</t>
         </is>
       </c>
       <c r="K272" s="12" t="inlineStr">
@@ -19342,7 +19355,7 @@
       </c>
       <c r="J273" s="12" t="inlineStr">
         <is>
-          <t>06 25 28 12 12</t>
+          <t>06 25 28 12 12 / 07 73 60 46 37</t>
         </is>
       </c>
       <c r="K273" s="12" t="inlineStr">
@@ -19654,7 +19667,7 @@
       </c>
       <c r="O277" s="12" t="inlineStr">
         <is>
-          <t>[26/10] Relais assistant tiers du 26/10 (dédupliqué Gmail/Contacts) — e-mail « vérifié » par le relais, à re-confirmer sur site officiel avant envoi.  NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi</t>
+          <t>[26/10] Relais assistant tiers du 26/10 (dédupliqué Gmail/Contacts) — e-mail « vérifié » par le relais, à re-confirmer sur site officiel avant envoi.  NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi [26/10 croisement fichier propriétaire] ⚠️ Coordonnées divergentes : relais du 26/10 matin = ille-de-vilaine@eurovia.com / 02 99 05 03 00 ; fichier du soir = « agence locale à confirmer ». À CONFIRMER avant tout contact.</t>
         </is>
       </c>
       <c r="P277" s="12" t="inlineStr">
@@ -19800,7 +19813,7 @@
       </c>
       <c r="O279" s="12" t="inlineStr">
         <is>
-          <t>[26/10] Relais assistant tiers du 26/10 (dédupliqué Gmail/Contacts) — e-mail « vérifié » par le relais, à re-confirmer sur site officiel avant envoi.  NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi</t>
+          <t>[26/10] Relais assistant tiers du 26/10 (dédupliqué Gmail/Contacts) — e-mail « vérifié » par le relais, à re-confirmer sur site officiel avant envoi.  NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi [26/10 croisement fichier propriétaire] Deux e-mails relevés : secretariat.keravis@lessard.fr (relais) et keravis@lessard.fr (fichier) — confirmer le bon.</t>
         </is>
       </c>
       <c r="P279" s="12" t="inlineStr">
@@ -19888,53 +19901,53 @@
       </c>
     </row>
     <row r="281" ht="15" customHeight="1" s="13">
-      <c r="A281" t="n">
+      <c r="A281" s="12" t="n">
         <v>281</v>
       </c>
-      <c r="B281" t="inlineStr">
+      <c r="B281" s="12" t="inlineStr">
         <is>
           <t>Pro France</t>
         </is>
       </c>
-      <c r="C281" t="n">
+      <c r="C281" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="D281" t="inlineStr">
+      <c r="D281" s="12" t="inlineStr">
         <is>
           <t>importateurs</t>
         </is>
       </c>
-      <c r="E281" t="inlineStr">
+      <c r="E281" s="12" t="inlineStr">
         <is>
           <t>Marbrerie Arnaud (SUD PIERRE)</t>
         </is>
       </c>
-      <c r="F281" t="inlineStr">
+      <c r="F281" s="12" t="inlineStr">
         <is>
           <t>Colombiers / Béziers</t>
         </is>
       </c>
-      <c r="G281" t="inlineStr">
+      <c r="G281" s="12" t="inlineStr">
         <is>
           <t>France</t>
         </is>
       </c>
-      <c r="H281" t="inlineStr">
+      <c r="H281" s="12" t="inlineStr">
         <is>
           <t>Confirmée : « Importateur et distributeur de pierre naturelle depuis 2012 », import direct Turquie, Égypte, Chine (page d'accueil) ; showroom 700 m² à Béziers, adresse Route de Nar…</t>
         </is>
       </c>
-      <c r="I281" t="inlineStr">
+      <c r="I281" s="12" t="inlineStr">
         <is>
           <t>https://www.marbreriearnaud34.com/</t>
         </is>
       </c>
-      <c r="J281" t="inlineStr">
+      <c r="J281" s="12" t="inlineStr">
         <is>
           <t>04 67 35 82 22</t>
         </is>
       </c>
-      <c r="K281" t="inlineStr">
+      <c r="K281" s="12" t="inlineStr">
         <is>
           <t>Recherche Claude (26/10)</t>
         </is>
@@ -19944,75 +19957,75 @@
           <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
         </is>
       </c>
-      <c r="N281" t="inlineStr">
+      <c r="N281" s="12" t="inlineStr">
         <is>
           <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
         </is>
       </c>
-      <c r="O281" t="inlineStr">
+      <c r="O281" s="12" t="inlineStr">
         <is>
           <t>[26/10] Recherche vérifiée (segment importateurs). Confirmée : « Importateur et distributeur de pierre naturelle depuis 2012 », import direct Turquie, Égypte, Chine (page d'accueil) ; showroom 700 m² à Béziers, adresse Route de Narbonne à Colombiers. Villes conformes. E-mail lu textuellement dans les mentions légales (« e-mail : j.andreo@marbrerie-arnaud.com », propriétaire SUD PIERRE). Le domaine de l'e-mail (marbrerie-arnaud.com) diffère du domaine du site, mais c'est bien l'adresse publiée officiellement. Téléphone confirmé sur mentions légales et accueil. Domaine hors liste d'exclusion. Source e-mail : https://www.marbreriearnaud34.com/mentions-legales/.  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
         </is>
       </c>
-      <c r="P281" t="inlineStr">
+      <c r="P281" s="12" t="inlineStr">
         <is>
           <t>5e liste — recherche (26/10)</t>
         </is>
       </c>
-      <c r="Q281" t="inlineStr">
+      <c r="Q281" s="12" t="inlineStr">
         <is>
           <t>j.andreo@marbrerie-arnaud.com</t>
         </is>
       </c>
     </row>
     <row r="282" ht="15" customHeight="1" s="13">
-      <c r="A282" t="n">
+      <c r="A282" s="12" t="n">
         <v>282</v>
       </c>
-      <c r="B282" t="inlineStr">
+      <c r="B282" s="12" t="inlineStr">
         <is>
           <t>Pro France</t>
         </is>
       </c>
-      <c r="C282" t="n">
+      <c r="C282" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="D282" t="inlineStr">
+      <c r="D282" s="12" t="inlineStr">
         <is>
           <t>importateurs</t>
         </is>
       </c>
-      <c r="E282" t="inlineStr">
+      <c r="E282" s="12" t="inlineStr">
         <is>
           <t>Artemis (Artemis Prestige)</t>
         </is>
       </c>
-      <c r="F282" t="inlineStr">
+      <c r="F282" s="12" t="inlineStr">
         <is>
           <t>Cabriès (Plan de Campagne) ; entrepôt à Simiane-Collongue</t>
         </is>
       </c>
-      <c r="G282" t="inlineStr">
+      <c r="G282" s="12" t="inlineStr">
         <is>
           <t>France</t>
         </is>
       </c>
-      <c r="H282" t="inlineStr">
+      <c r="H282" s="12" t="inlineStr">
         <is>
           <t>Confirmée : importateur-vendeur de pierre naturelle (travertin, marbre, pierre d'Égypte, grès cérame), livraison France entière. Showroom Expobat Plan de Campagne 13480 Cabriès + e…</t>
         </is>
       </c>
-      <c r="I282" t="inlineStr">
+      <c r="I282" s="12" t="inlineStr">
         <is>
           <t>https://www.artemis-prestige.com/</t>
         </is>
       </c>
-      <c r="J282" t="inlineStr">
+      <c r="J282" s="12" t="inlineStr">
         <is>
           <t>04 42 31 41 40</t>
         </is>
       </c>
-      <c r="K282" t="inlineStr">
+      <c r="K282" s="12" t="inlineStr">
         <is>
           <t>Recherche Claude (26/10)</t>
         </is>
@@ -20022,75 +20035,75 @@
           <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
         </is>
       </c>
-      <c r="N282" t="inlineStr">
+      <c r="N282" s="12" t="inlineStr">
         <is>
           <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
         </is>
       </c>
-      <c r="O282" t="inlineStr">
+      <c r="O282" s="12" t="inlineStr">
         <is>
           <t>[26/10] Recherche vérifiée (segment importateurs). Confirmée : importateur-vendeur de pierre naturelle (travertin, marbre, pierre d'Égypte, grès cérame), livraison France entière. Showroom Expobat Plan de Campagne 13480 Cabriès + entrepôt logistique 13109 Simiane-Collongue confirmés sur la page contact. E-mail présent textuellement sur la page contact (texte du lien et mailto). Téléphone confirmé. Pierre d'Égypte explicitement au catalogue. Domaine hors liste d'exclusion. Source e-mail : https://www.artemis-prestige.com/contact.html.  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
         </is>
       </c>
-      <c r="P282" t="inlineStr">
+      <c r="P282" s="12" t="inlineStr">
         <is>
           <t>5e liste — recherche (26/10)</t>
         </is>
       </c>
-      <c r="Q282" t="inlineStr">
+      <c r="Q282" s="12" t="inlineStr">
         <is>
           <t>artemis-prestige@orange.fr</t>
         </is>
       </c>
     </row>
     <row r="283" ht="15" customHeight="1" s="13">
-      <c r="A283" t="n">
+      <c r="A283" s="12" t="n">
         <v>283</v>
       </c>
-      <c r="B283" t="inlineStr">
+      <c r="B283" s="12" t="inlineStr">
         <is>
           <t>Pro France</t>
         </is>
       </c>
-      <c r="C283" t="n">
+      <c r="C283" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="D283" t="inlineStr">
+      <c r="D283" s="12" t="inlineStr">
         <is>
           <t>importateurs</t>
         </is>
       </c>
-      <c r="E283" t="inlineStr">
+      <c r="E283" s="12" t="inlineStr">
         <is>
           <t>Minéral Pierre Naturelle (Pierre de l'Est SAS)</t>
         </is>
       </c>
-      <c r="F283" t="inlineStr">
+      <c r="F283" s="12" t="inlineStr">
         <is>
           <t>Woustviller (magasins Lyon, Strasbourg, Nancy, Beaune, Thion</t>
         </is>
       </c>
-      <c r="G283" t="inlineStr">
+      <c r="G283" s="12" t="inlineStr">
         <is>
           <t>France</t>
         </is>
       </c>
-      <c r="H283" t="inlineStr">
+      <c r="H283" s="12" t="inlineStr">
         <is>
           <t>Confirmée : spécialiste pierre naturelle (travertin, calcaire, marbre, granit...), 7 magasins France/Allemagne dont Lyon, Strasbourg, Nancy, Beaune, Thionville. Mentions légales : …</t>
         </is>
       </c>
-      <c r="I283" t="inlineStr">
+      <c r="I283" s="12" t="inlineStr">
         <is>
           <t>https://www.mineral-pierre-naturelle.fr/</t>
         </is>
       </c>
-      <c r="J283" t="inlineStr">
-        <is>
-          <t>03 60 12 33 53</t>
-        </is>
-      </c>
-      <c r="K283" t="inlineStr">
+      <c r="J283" s="12" t="inlineStr">
+        <is>
+          <t>03 60 12 33 53 / 03 87 98 67 37</t>
+        </is>
+      </c>
+      <c r="K283" s="12" t="inlineStr">
         <is>
           <t>Recherche Claude (26/10)</t>
         </is>
@@ -20100,70 +20113,70 @@
           <t>À contacter (formulaire/tél) — EN ATTENTE</t>
         </is>
       </c>
-      <c r="N283" t="inlineStr">
+      <c r="N283" s="12" t="inlineStr">
         <is>
           <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
         </is>
       </c>
-      <c r="O283" t="inlineStr">
-        <is>
-          <t>[26/10] Recherche vérifiée (segment importateurs). Confirmée : spécialiste pierre naturelle (travertin, calcaire, marbre, granit...), 7 magasins France/Allemagne dont Lyon, Strasbourg, Nancy, Beaune, Thionville. Mentions légales : Pierre de l'Est SAS, 44 Rue de Nancy, 57915 Woustviller — raison sociale et ville confirmées. AUCUN e-mail publié : vérifié sur l'accueil et les mentions légales (contact par téléphone ou formulaire uniquement). Repli téléphone VÉRIFIÉ : 03 60 12 33 53 affiché sur l'accueil (« Conseil d'expert ») et dans les mentions légales. Le produit Sinai Pearl n'était pas visible sur la portion d'accueil lue, mais l'activité calcaire/travertin est confirmée. Domaine hors liste d'exclusion. Source e-mail : aucune (pas d e-mail publié).  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
-        </is>
-      </c>
-      <c r="P283" t="inlineStr">
+      <c r="O283" s="12" t="inlineStr">
+        <is>
+          <t>[26/10] Recherche vérifiée (segment importateurs). Confirmée : spécialiste pierre naturelle (travertin, calcaire, marbre, granit...), 7 magasins France/Allemagne dont Lyon, Strasbourg, Nancy, Beaune, Thionville. Mentions légales : Pierre de l'Est SAS, 44 Rue de Nancy, 57915 Woustviller — raison sociale et ville confirmées. AUCUN e-mail publié : vérifié sur l'accueil et les mentions légales (contact par téléphone ou formulaire uniquement). Repli téléphone VÉRIFIÉ : 03 60 12 33 53 affiché sur l'accueil (« Conseil d'expert ») et dans les mentions légales. Le produit Sinai Pearl n'était pas visible sur la portion d'accueil lue, mais l'activité calcaire/travertin est confirmée. Domaine hors liste d'exclusion. Source e-mail : aucune (pas d e-mail publié).  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi [26/10 croisement fichier propriétaire] 2e téléphone (fichier) : 03 87 98 67 37.</t>
+        </is>
+      </c>
+      <c r="P283" s="12" t="inlineStr">
         <is>
           <t>5e liste — recherche (26/10)</t>
         </is>
       </c>
     </row>
     <row r="284" ht="15" customHeight="1" s="13">
-      <c r="A284" t="n">
+      <c r="A284" s="12" t="n">
         <v>284</v>
       </c>
-      <c r="B284" t="inlineStr">
+      <c r="B284" s="12" t="inlineStr">
         <is>
           <t>Pro France</t>
         </is>
       </c>
-      <c r="C284" t="n">
+      <c r="C284" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="D284" t="inlineStr">
+      <c r="D284" s="12" t="inlineStr">
         <is>
           <t>importateurs</t>
         </is>
       </c>
-      <c r="E284" t="inlineStr">
+      <c r="E284" s="12" t="inlineStr">
         <is>
           <t>Nimex International</t>
         </is>
       </c>
-      <c r="F284" t="inlineStr">
+      <c r="F284" s="12" t="inlineStr">
         <is>
           <t>Caissargues (dépôt à Nîmes)</t>
         </is>
       </c>
-      <c r="G284" t="inlineStr">
+      <c r="G284" s="12" t="inlineStr">
         <is>
           <t>France</t>
         </is>
       </c>
-      <c r="H284" t="inlineStr">
+      <c r="H284" s="12" t="inlineStr">
         <is>
           <t>Confirmée : importateur-distributeur de pierre naturelle, marbre, granit, travertin ; approvisionnement direct carrières (Espagne, Italie, Portugal, Grèce, Turquie, ÉGYPTE, Inde) ;…</t>
         </is>
       </c>
-      <c r="I284" t="inlineStr">
+      <c r="I284" s="12" t="inlineStr">
         <is>
           <t>https://www.nimexinternational.fr/</t>
         </is>
       </c>
-      <c r="J284" t="inlineStr">
+      <c r="J284" s="12" t="inlineStr">
         <is>
           <t>04 30 22 01 75</t>
         </is>
       </c>
-      <c r="K284" t="inlineStr">
+      <c r="K284" s="12" t="inlineStr">
         <is>
           <t>Recherche Claude (26/10)</t>
         </is>
@@ -20173,75 +20186,75 @@
           <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
         </is>
       </c>
-      <c r="N284" t="inlineStr">
+      <c r="N284" s="12" t="inlineStr">
         <is>
           <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
         </is>
       </c>
-      <c r="O284" t="inlineStr">
+      <c r="O284" s="12" t="inlineStr">
         <is>
           <t>[26/10] Recherche vérifiée (segment importateurs). Confirmée : importateur-distributeur de pierre naturelle, marbre, granit, travertin ; approvisionnement direct carrières (Espagne, Italie, Portugal, Grèce, Turquie, ÉGYPTE, Inde) ; dépôt à Nîmes, vente et livraison France entière. Adresse : 14 avenue de la Vistrenque, 30132 Caissargues — ville confirmée. E-mail présent textuellement dans le pied de page du site officiel. Téléphone confirmé. L'Égypte figure parmi les pays d'approvisionnement cités. Domaine hors liste d'exclusion. Source e-mail : https://www.nimexinternational.fr/.  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
         </is>
       </c>
-      <c r="P284" t="inlineStr">
+      <c r="P284" s="12" t="inlineStr">
         <is>
           <t>5e liste — recherche (26/10)</t>
         </is>
       </c>
-      <c r="Q284" t="inlineStr">
+      <c r="Q284" s="12" t="inlineStr">
         <is>
           <t>nimex.international@wanadoo.fr</t>
         </is>
       </c>
     </row>
     <row r="285" ht="15" customHeight="1" s="13">
-      <c r="A285" t="n">
+      <c r="A285" s="12" t="n">
         <v>285</v>
       </c>
-      <c r="B285" t="inlineStr">
+      <c r="B285" s="12" t="inlineStr">
         <is>
           <t>Pro France</t>
         </is>
       </c>
-      <c r="C285" t="n">
+      <c r="C285" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="D285" t="inlineStr">
+      <c r="D285" s="12" t="inlineStr">
         <is>
           <t>importateurs</t>
         </is>
       </c>
-      <c r="E285" t="inlineStr">
+      <c r="E285" s="12" t="inlineStr">
         <is>
           <t>Travertin.fr</t>
         </is>
       </c>
-      <c r="F285" t="inlineStr">
+      <c r="F285" s="12" t="inlineStr">
         <is>
           <t>Fos-sur-Mer (centre logistique)</t>
         </is>
       </c>
-      <c r="G285" t="inlineStr">
+      <c r="G285" s="12" t="inlineStr">
         <is>
           <t>France</t>
         </is>
       </c>
-      <c r="H285" t="inlineStr">
+      <c r="H285" s="12" t="inlineStr">
         <is>
           <t>Confirmée : le site se décrit comme « un importateur et un grossiste spécialisé en travertin » (carrières Turquie/Italie), dalles, carrelages, margelles, livraison France entière. …</t>
         </is>
       </c>
-      <c r="I285" t="inlineStr">
+      <c r="I285" s="12" t="inlineStr">
         <is>
           <t>https://www.travertin.fr/</t>
         </is>
       </c>
-      <c r="J285" t="inlineStr">
+      <c r="J285" s="12" t="inlineStr">
         <is>
           <t>09 70 70 73 75</t>
         </is>
       </c>
-      <c r="K285" t="inlineStr">
+      <c r="K285" s="12" t="inlineStr">
         <is>
           <t>Recherche Claude (26/10)</t>
         </is>
@@ -20251,75 +20264,75 @@
           <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
         </is>
       </c>
-      <c r="N285" t="inlineStr">
+      <c r="N285" s="12" t="inlineStr">
         <is>
           <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
         </is>
       </c>
-      <c r="O285" t="inlineStr">
+      <c r="O285" s="12" t="inlineStr">
         <is>
           <t>[26/10] Recherche vérifiée (segment importateurs). Confirmée : le site se décrit comme « un importateur et un grossiste spécialisé en travertin » (carrières Turquie/Italie), dalles, carrelages, margelles, livraison France entière. Adresse : Centre Logistique, 13270 Fos-sur-Mer — ville confirmée. E-mail présent textuellement dans le bloc contact du pied de page, sous l'adresse de Fos-sur-Mer. Téléphone confirmé (en-tête et pied de page). Domaine hors liste d'exclusion. Source e-mail : https://www.travertin.fr/.  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
         </is>
       </c>
-      <c r="P285" t="inlineStr">
+      <c r="P285" s="12" t="inlineStr">
         <is>
           <t>5e liste — recherche (26/10)</t>
         </is>
       </c>
-      <c r="Q285" t="inlineStr">
+      <c r="Q285" s="12" t="inlineStr">
         <is>
           <t>info@travertin.fr</t>
         </is>
       </c>
     </row>
     <row r="286" ht="15" customHeight="1" s="13">
-      <c r="A286" t="n">
+      <c r="A286" s="12" t="n">
         <v>286</v>
       </c>
-      <c r="B286" t="inlineStr">
+      <c r="B286" s="12" t="inlineStr">
         <is>
           <t>Pro France</t>
         </is>
       </c>
-      <c r="C286" t="n">
+      <c r="C286" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="D286" t="inlineStr">
+      <c r="D286" s="12" t="inlineStr">
         <is>
           <t>importateurs</t>
         </is>
       </c>
-      <c r="E286" t="inlineStr">
+      <c r="E286" s="12" t="inlineStr">
         <is>
           <t>Espace Travertin (EURL GNPS Espace Carrelage)</t>
         </is>
       </c>
-      <c r="F286" t="inlineStr">
+      <c r="F286" s="12" t="inlineStr">
         <is>
           <t>Bollène</t>
         </is>
       </c>
-      <c r="G286" t="inlineStr">
+      <c r="G286" s="12" t="inlineStr">
         <is>
           <t>France</t>
         </is>
       </c>
-      <c r="H286" t="inlineStr">
+      <c r="H286" s="12" t="inlineStr">
         <is>
           <t>Confirmée partiellement : vente de travertin (dallage, margelles, plinthes, vasques, 200+ références) avec page « Devenir Revendeur » et prix de gros revendiqués ; adresse Impasse …</t>
         </is>
       </c>
-      <c r="I286" t="inlineStr">
+      <c r="I286" s="12" t="inlineStr">
         <is>
           <t>https://www.espace-travertin.fr/</t>
         </is>
       </c>
-      <c r="J286" t="inlineStr">
+      <c r="J286" s="12" t="inlineStr">
         <is>
           <t>07 68 18 70 32</t>
         </is>
       </c>
-      <c r="K286" t="inlineStr">
+      <c r="K286" s="12" t="inlineStr">
         <is>
           <t>Recherche Claude (26/10)</t>
         </is>
@@ -20329,70 +20342,75 @@
           <t>À contacter (formulaire/tél) — EN ATTENTE</t>
         </is>
       </c>
-      <c r="N286" t="inlineStr">
+      <c r="N286" s="12" t="inlineStr">
         <is>
           <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
         </is>
       </c>
-      <c r="O286" t="inlineStr">
-        <is>
-          <t>[26/10] Recherche vérifiée (segment importateurs). Confirmée partiellement : vente de travertin (dallage, margelles, plinthes, vasques, 200+ références) avec page « Devenir Revendeur » et prix de gros revendiqués ; adresse Impasse de la Rode, 84500 Bollène confirmée. Le site vend aussi aux particuliers (pas uniquement B2B). Le siège à Étoile-sur-Rhône et la raison sociale GNPS n'apparaissent pas sur la page d'accueil (le PDF CGV mentionne « stone-diffusion-centre »). AUCUN e-mail publié sur la page d'accueil (vérifié). Repli téléphone VÉRIFIÉ : 07 68 18 70 32 affiché deux fois en haut de page en lien cliquable. Domaine hors liste d'exclusion. Profil un peu plus B2C que revendiqué, mais canal revendeur réel. Source e-mail : aucune (pas d e-mail publié). ⚠️ CONCURRENT suivi dans la veille prix (ambiguïtés marbre/calcaire) — approche uniquement « reprise de lot revendeur ». NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
-        </is>
-      </c>
-      <c r="P286" t="inlineStr">
+      <c r="O286" s="12" t="inlineStr">
+        <is>
+          <t>[26/10] Recherche vérifiée (segment importateurs). Confirmée partiellement : vente de travertin (dallage, margelles, plinthes, vasques, 200+ références) avec page « Devenir Revendeur » et prix de gros revendiqués ; adresse Impasse de la Rode, 84500 Bollène confirmée. Le site vend aussi aux particuliers (pas uniquement B2B). Le siège à Étoile-sur-Rhône et la raison sociale GNPS n'apparaissent pas sur la page d'accueil (le PDF CGV mentionne « stone-diffusion-centre »). AUCUN e-mail publié sur la page d'accueil (vérifié). Repli téléphone VÉRIFIÉ : 07 68 18 70 32 affiché deux fois en haut de page en lien cliquable. Domaine hors liste d'exclusion. Profil un peu plus B2C que revendiqué, mais canal revendeur réel. Source e-mail : aucune (pas d e-mail publié). ⚠️ CONCURRENT suivi dans la veille prix (ambiguïtés marbre/calcaire) — approche uniquement « reprise de lot revendeur ». NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi [26/10 croisement fichier propriétaire] E-mail apporté par le fichier : contactgnps26@gmail.com (Étoile-sur-Rhône). ⚠️ Identité exploitant contradictoire — VALIDER LA SOCIÉTÉ avant contact (consigne fichier).</t>
+        </is>
+      </c>
+      <c r="P286" s="12" t="inlineStr">
         <is>
           <t>5e liste — recherche (26/10)</t>
         </is>
       </c>
+      <c r="Q286" t="inlineStr">
+        <is>
+          <t>contactgnps26@gmail.com</t>
+        </is>
+      </c>
     </row>
     <row r="287" ht="15" customHeight="1" s="13">
-      <c r="A287" t="n">
+      <c r="A287" s="12" t="n">
         <v>287</v>
       </c>
-      <c r="B287" t="inlineStr">
+      <c r="B287" s="12" t="inlineStr">
         <is>
           <t>Pro France</t>
         </is>
       </c>
-      <c r="C287" t="n">
+      <c r="C287" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="D287" t="inlineStr">
+      <c r="D287" s="12" t="inlineStr">
         <is>
           <t>importateurs</t>
         </is>
       </c>
-      <c r="E287" t="inlineStr">
+      <c r="E287" s="12" t="inlineStr">
         <is>
           <t>DMC Miller</t>
         </is>
       </c>
-      <c r="F287" t="inlineStr">
+      <c r="F287" s="12" t="inlineStr">
         <is>
           <t>Pertuis (dépôt également à Gujan-Mestras, 33)</t>
         </is>
       </c>
-      <c r="G287" t="inlineStr">
+      <c r="G287" s="12" t="inlineStr">
         <is>
           <t>France</t>
         </is>
       </c>
-      <c r="H287" t="inlineStr">
+      <c r="H287" s="12" t="inlineStr">
         <is>
           <t>Confirmée : distributeur spécialiste du travertin (dalles 1er/2e choix, margelles, plinthes, mosaïques, pavés granit), vente au m², livraison France entière. Adresse 315 Rue Benjam…</t>
         </is>
       </c>
-      <c r="I287" t="inlineStr">
+      <c r="I287" s="12" t="inlineStr">
         <is>
           <t>https://www.dmcmiller.com/</t>
         </is>
       </c>
-      <c r="J287" t="inlineStr">
+      <c r="J287" s="12" t="inlineStr">
         <is>
           <t>06 66 55 44 42</t>
         </is>
       </c>
-      <c r="K287" t="inlineStr">
+      <c r="K287" s="12" t="inlineStr">
         <is>
           <t>Recherche Claude (26/10)</t>
         </is>
@@ -20402,75 +20420,75 @@
           <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
         </is>
       </c>
-      <c r="N287" t="inlineStr">
+      <c r="N287" s="12" t="inlineStr">
         <is>
           <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
         </is>
       </c>
-      <c r="O287" t="inlineStr">
+      <c r="O287" s="12" t="inlineStr">
         <is>
           <t>[26/10] Recherche vérifiée (segment importateurs). Confirmée : distributeur spécialiste du travertin (dalles 1er/2e choix, margelles, plinthes, mosaïques, pavés granit), vente au m², livraison France entière. Adresse 315 Rue Benjamin Franklin, 84120 Pertuis + dépôts Pertuis et Gujan-Mestras — villes confirmées. E-mail présent textuellement dans le pied de page (lien mailto). Téléphone confirmé (affiché 0666554442 en en-tête, pied de page et lien WhatsApp). Domaine hors liste d'exclusion. Source e-mail : https://www.dmcmiller.com/.  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
         </is>
       </c>
-      <c r="P287" t="inlineStr">
+      <c r="P287" s="12" t="inlineStr">
         <is>
           <t>5e liste — recherche (26/10)</t>
         </is>
       </c>
-      <c r="Q287" t="inlineStr">
+      <c r="Q287" s="12" t="inlineStr">
         <is>
           <t>contact@dmcmiller.com</t>
         </is>
       </c>
     </row>
     <row r="288" ht="15" customHeight="1" s="13">
-      <c r="A288" t="n">
+      <c r="A288" s="12" t="n">
         <v>288</v>
       </c>
-      <c r="B288" t="inlineStr">
+      <c r="B288" s="12" t="inlineStr">
         <is>
           <t>Pro France</t>
         </is>
       </c>
-      <c r="C288" t="n">
+      <c r="C288" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="D288" t="inlineStr">
+      <c r="D288" s="12" t="inlineStr">
         <is>
           <t>importateurs</t>
         </is>
       </c>
-      <c r="E288" t="inlineStr">
+      <c r="E288" s="12" t="inlineStr">
         <is>
           <t>Cupa Stone France (Cupa Pierres Distribution)</t>
         </is>
       </c>
-      <c r="F288" t="inlineStr">
+      <c r="F288" s="12" t="inlineStr">
         <is>
           <t>Changé (Le Mans) — réseau national d'agences</t>
         </is>
       </c>
-      <c r="G288" t="inlineStr">
+      <c r="G288" s="12" t="inlineStr">
         <is>
           <t>France</t>
         </is>
       </c>
-      <c r="H288" t="inlineStr">
+      <c r="H288" s="12" t="inlineStr">
         <is>
           <t>Confirmée : distributeur national de pierre naturelle avec agences au Mans (Changé), Tours, Rennes, Nantes, Lyon, Aix-en-Provence, Quimper, Pau, Limoges, Cholet, Muzillac, La Roche…</t>
         </is>
       </c>
-      <c r="I288" t="inlineStr">
+      <c r="I288" s="12" t="inlineStr">
         <is>
           <t>https://www.cupastone.fr/</t>
         </is>
       </c>
-      <c r="J288" t="inlineStr">
+      <c r="J288" s="12" t="inlineStr">
         <is>
           <t>+33 2 43 85 06 84</t>
         </is>
       </c>
-      <c r="K288" t="inlineStr">
+      <c r="K288" s="12" t="inlineStr">
         <is>
           <t>Recherche Claude (26/10)</t>
         </is>
@@ -20480,75 +20498,75 @@
           <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
         </is>
       </c>
-      <c r="N288" t="inlineStr">
+      <c r="N288" s="12" t="inlineStr">
         <is>
           <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
         </is>
       </c>
-      <c r="O288" t="inlineStr">
-        <is>
-          <t>[26/10] Recherche vérifiée (segment importateurs). Confirmée : distributeur national de pierre naturelle avec agences au Mans (Changé), Tours, Rennes, Nantes, Lyon, Aix-en-Provence, Quimper, Pau, Limoges, Cholet, Muzillac, La Roche-sur-Yon, etc. (groupe présent aussi en Espagne/Portugal). Le téléphone +33 2 43 85 06 84 est bien celui de l'agence Le Mans (Changé), contact Amandine Renard. E-mail contact@cupastone.fr présent textuellement sur la page points de vente, répété pour la plupart des agences françaises (dont Le Mans). D'autres e-mails nominatifs existent (cleger@cupastone.fr Bordeaux, lgasse@cupastone.com Paris-IdF, sbatmale@cupastone.com Toulouse, fmadehors@cupastone.com Nord-Est) si un ciblage régional est préféré. Domaine hors liste d'exclusion. Source e-mail : https://www.cupastone.fr/points-de-vente/.  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
-        </is>
-      </c>
-      <c r="P288" t="inlineStr">
+      <c r="O288" s="12" t="inlineStr">
+        <is>
+          <t>[26/10] Recherche vérifiée (segment importateurs). Confirmée : distributeur national de pierre naturelle avec agences au Mans (Changé), Tours, Rennes, Nantes, Lyon, Aix-en-Provence, Quimper, Pau, Limoges, Cholet, Muzillac, La Roche-sur-Yon, etc. (groupe présent aussi en Espagne/Portugal). Le téléphone +33 2 43 85 06 84 est bien celui de l'agence Le Mans (Changé), contact Amandine Renard. E-mail contact@cupastone.fr présent textuellement sur la page points de vente, répété pour la plupart des agences françaises (dont Le Mans). D'autres e-mails nominatifs existent (cleger@cupastone.fr Bordeaux, lgasse@cupastone.com Paris-IdF, sbatmale@cupastone.com Toulouse, fmadehors@cupastone.com Nord-Est) si un ciblage régional est préféré. Domaine hors liste d'exclusion. Source e-mail : https://www.cupastone.fr/points-de-vente/.  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi [26/10 croisement fichier propriétaire] Ciblage régional préféré (fichier) : agence Paris/IdF à Coignières — lgasse@cupastone.com, 01 30 49 69 91. Sinon contact@cupastone.fr (Le Mans, vérifié).</t>
+        </is>
+      </c>
+      <c r="P288" s="12" t="inlineStr">
         <is>
           <t>5e liste — recherche (26/10)</t>
         </is>
       </c>
-      <c r="Q288" t="inlineStr">
+      <c r="Q288" s="12" t="inlineStr">
         <is>
           <t>contact@cupastone.fr</t>
         </is>
       </c>
     </row>
     <row r="289" ht="15" customHeight="1" s="13">
-      <c r="A289" t="n">
+      <c r="A289" s="12" t="n">
         <v>289</v>
       </c>
-      <c r="B289" t="inlineStr">
+      <c r="B289" s="12" t="inlineStr">
         <is>
           <t>Pro France</t>
         </is>
       </c>
-      <c r="C289" t="n">
+      <c r="C289" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="D289" t="inlineStr">
+      <c r="D289" s="12" t="inlineStr">
         <is>
           <t>importateurs</t>
         </is>
       </c>
-      <c r="E289" t="inlineStr">
+      <c r="E289" s="12" t="inlineStr">
         <is>
           <t>Ti'ma Stone</t>
         </is>
       </c>
-      <c r="F289" t="inlineStr">
+      <c r="F289" s="12" t="inlineStr">
         <is>
           <t>Lunel (non confirmée sur le site)</t>
         </is>
       </c>
-      <c r="G289" t="inlineStr">
+      <c r="G289" s="12" t="inlineStr">
         <is>
           <t>France</t>
         </is>
       </c>
-      <c r="H289" t="inlineStr">
+      <c r="H289" s="12" t="inlineStr">
         <is>
           <t>Confirmée pour l'activité : vente en ligne de pierre naturelle France entière (dallage, parement, margelles, zellige, vasques), travertin très présent, liens « Grossiste dallage » …</t>
         </is>
       </c>
-      <c r="I289" t="inlineStr">
+      <c r="I289" s="12" t="inlineStr">
         <is>
           <t>https://timastone.com/</t>
         </is>
       </c>
-      <c r="J289" t="inlineStr">
+      <c r="J289" s="12" t="inlineStr">
         <is>
           <t>04 15 54 01 25</t>
         </is>
       </c>
-      <c r="K289" t="inlineStr">
+      <c r="K289" s="12" t="inlineStr">
         <is>
           <t>Recherche Claude (26/10)</t>
         </is>
@@ -20558,70 +20576,70 @@
           <t>À contacter (formulaire/tél) — EN ATTENTE</t>
         </is>
       </c>
-      <c r="N289" t="inlineStr">
+      <c r="N289" s="12" t="inlineStr">
         <is>
           <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
         </is>
       </c>
-      <c r="O289" t="inlineStr">
+      <c r="O289" s="12" t="inlineStr">
         <is>
           <t>[26/10] Recherche vérifiée (segment importateurs). Confirmée pour l'activité : vente en ligne de pierre naturelle France entière (dallage, parement, margelles, zellige, vasques), travertin très présent, liens « Grossiste dallage » et « Fournisseur carrelage » + espace pro. La VILLE n'est PAS confirmée : aucune adresse ni ville sur la page d'accueil, et les pages /mentions-legales/ et /contact/ renvoient un 404 aux URL standards. AUCUN e-mail publié sur la page d'accueil (vérifié). Repli téléphone VÉRIFIÉ : 04 15 54 01 25 affiché en en-tête et pied de page (horaires lun-ven 9h-12h / 14h-18h). Domaine hors liste d'exclusion. Site vivant et actif, mais profil plutôt vente en ligne avec volet grossiste ; localisation Lunel à reconfirmer par téléphone avant tout engagement logistique. Source e-mail : aucune (pas d e-mail publié). ⚠️ CONCURRENT suivi dans la veille prix (42,46–59,96 €/m²) — approche uniquement « reprise de lot revendeur », aucune info sensible. NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
         </is>
       </c>
-      <c r="P289" t="inlineStr">
+      <c r="P289" s="12" t="inlineStr">
         <is>
           <t>5e liste — recherche (26/10)</t>
         </is>
       </c>
     </row>
     <row r="290" ht="15" customHeight="1" s="13">
-      <c r="A290" t="n">
+      <c r="A290" s="12" t="n">
         <v>290</v>
       </c>
-      <c r="B290" t="inlineStr">
+      <c r="B290" s="12" t="inlineStr">
         <is>
           <t>Pro France</t>
         </is>
       </c>
-      <c r="C290" t="n">
+      <c r="C290" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="D290" t="inlineStr">
+      <c r="D290" s="12" t="inlineStr">
         <is>
           <t>importateurs</t>
         </is>
       </c>
-      <c r="E290" t="inlineStr">
+      <c r="E290" s="12" t="inlineStr">
         <is>
           <t>BH Matériaux (groupe Holding Laffont)</t>
         </is>
       </c>
-      <c r="F290" t="inlineStr">
+      <c r="F290" s="12" t="inlineStr">
         <is>
           <t>Lauzerte</t>
         </is>
       </c>
-      <c r="G290" t="inlineStr">
+      <c r="G290" s="12" t="inlineStr">
         <is>
           <t>France</t>
         </is>
       </c>
-      <c r="H290" t="inlineStr">
+      <c r="H290" s="12" t="inlineStr">
         <is>
           <t>Confirmée : grossiste revendiqué (« Votre grossiste ») en matériaux de construction/rénovation/décoration avec le travertin et le dallage pierre naturelle en gamme majeure (dallage…</t>
         </is>
       </c>
-      <c r="I290" t="inlineStr">
+      <c r="I290" s="12" t="inlineStr">
         <is>
           <t>https://bh-materiaux.com/</t>
         </is>
       </c>
-      <c r="J290" t="inlineStr">
+      <c r="J290" s="12" t="inlineStr">
         <is>
           <t>05 63 95 39 08</t>
         </is>
       </c>
-      <c r="K290" t="inlineStr">
+      <c r="K290" s="12" t="inlineStr">
         <is>
           <t>Recherche Claude (26/10)</t>
         </is>
@@ -20631,70 +20649,70 @@
           <t>À contacter (formulaire/tél) — EN ATTENTE</t>
         </is>
       </c>
-      <c r="N290" t="inlineStr">
+      <c r="N290" s="12" t="inlineStr">
         <is>
           <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
         </is>
       </c>
-      <c r="O290" t="inlineStr">
+      <c r="O290" s="12" t="inlineStr">
         <is>
           <t>[26/10] Recherche vérifiée (segment importateurs). Confirmée : grossiste revendiqué (« Votre grossiste ») en matériaux de construction/rénovation/décoration avec le travertin et le dallage pierre naturelle en gamme majeure (dallages du monde, parement, graviers, pas japonais) ; particuliers et professionnels ; retrait au dépôt de Lauzerte. Adresse 138 route de Montbarla, 82110 Lauzerte confirmée. Groupe Holding Laffont confirmé (Osagra, Laffont TP, Laffont Granulats...). AUCUN e-mail publié (vérifié sur la page d'accueil : téléphone et formulaire de rappel uniquement). Repli téléphone VÉRIFIÉ : 05 63 95 39 08 répété en en-tête et sections contact. ATTENTION : le site confirme « membre du réseau FRANCE MATERIAUX » dont le domaine france-materiaux.fr figure dans la liste d'exclusion ; le domaine propre bh-materiaux.com n'y figure pas — retenu, mais à arbitrer côté donneur d'ordre avant contact. Source e-mail : aucune (pas d e-mail publié).  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
         </is>
       </c>
-      <c r="P290" t="inlineStr">
+      <c r="P290" s="12" t="inlineStr">
         <is>
           <t>5e liste — recherche (26/10)</t>
         </is>
       </c>
     </row>
     <row r="291" ht="15" customHeight="1" s="13">
-      <c r="A291" t="n">
+      <c r="A291" s="12" t="n">
         <v>291</v>
       </c>
-      <c r="B291" t="inlineStr">
+      <c r="B291" s="12" t="inlineStr">
         <is>
           <t>Pro France</t>
         </is>
       </c>
-      <c r="C291" t="n">
+      <c r="C291" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="D291" t="inlineStr">
+      <c r="D291" s="12" t="inlineStr">
         <is>
           <t>marbreries-idf</t>
         </is>
       </c>
-      <c r="E291" t="inlineStr">
+      <c r="E291" s="12" t="inlineStr">
         <is>
           <t>Les Marbreries de la Seine (LMS Paris)</t>
         </is>
       </c>
-      <c r="F291" t="inlineStr">
+      <c r="F291" s="12" t="inlineStr">
         <is>
           <t>Les Pavillons-sous-Bois (ateliers) / Paris 7e (showroom)</t>
         </is>
       </c>
-      <c r="G291" t="inlineStr">
+      <c r="G291" s="12" t="inlineStr">
         <is>
           <t>France</t>
         </is>
       </c>
-      <c r="H291" t="inlineStr">
+      <c r="H291" s="12" t="inlineStr">
         <is>
           <t>Confirmée : marbrerie haute décoration (architecture, mobilier, objets d'art) ; showroom 33 rue de Verneuil 75007 Paris, ateliers et logistique 2/8 allée de Londres 93320 Les Pavil…</t>
         </is>
       </c>
-      <c r="I291" t="inlineStr">
+      <c r="I291" s="12" t="inlineStr">
         <is>
           <t>https://www.lesmarbreriesdelaseine.com</t>
         </is>
       </c>
-      <c r="J291" t="inlineStr">
+      <c r="J291" s="12" t="inlineStr">
         <is>
           <t>+33 1 48 48 10 00 (showroom) / +33 1 48 48 59 76 (ateliers)</t>
         </is>
       </c>
-      <c r="K291" t="inlineStr">
+      <c r="K291" s="12" t="inlineStr">
         <is>
           <t>Recherche Claude (26/10)</t>
         </is>
@@ -20704,1567 +20722,2072 @@
           <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
         </is>
       </c>
-      <c r="N291" t="inlineStr">
+      <c r="N291" s="12" t="inlineStr">
         <is>
           <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
         </is>
       </c>
-      <c r="O291" t="inlineStr">
+      <c r="O291" s="12" t="inlineStr">
         <is>
           <t>[26/10] Recherche vérifiée (segment marbreries-idf). Confirmée : marbrerie haute décoration (architecture, mobilier, objets d'art) ; showroom 33 rue de Verneuil 75007 Paris, ateliers et logistique 2/8 allée de Londres 93320 Les Pavillons-sous-Bois. E-mail info@lmsparis.com lu textuellement sur la page contact du site officiel (un second e-mail info@lmsmiami.com concerne l'antenne de Miami, à ignorer). Téléphones confirmés. Domaine hors liste d'exclusion. Site officiel, pas un annuaire. Source e-mail : https://www.lesmarbreriesdelaseine.com/contact.  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
         </is>
       </c>
-      <c r="P291" t="inlineStr">
+      <c r="P291" s="12" t="inlineStr">
         <is>
           <t>5e liste — recherche (26/10)</t>
         </is>
       </c>
-      <c r="Q291" t="inlineStr">
+      <c r="Q291" s="12" t="inlineStr">
         <is>
           <t>info@lmsparis.com</t>
         </is>
       </c>
     </row>
     <row r="292" ht="15" customHeight="1" s="13">
-      <c r="A292" t="n">
+      <c r="A292" s="12" t="n">
         <v>292</v>
       </c>
-      <c r="B292" t="inlineStr">
+      <c r="B292" s="12" t="inlineStr">
         <is>
           <t>Pro France</t>
         </is>
       </c>
-      <c r="C292" t="n">
+      <c r="C292" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="D292" t="inlineStr">
+      <c r="D292" s="12" t="inlineStr">
         <is>
           <t>marbreries-idf</t>
         </is>
       </c>
-      <c r="E292" t="inlineStr">
+      <c r="E292" s="12" t="inlineStr">
         <is>
           <t>Marbre Import</t>
         </is>
       </c>
-      <c r="F292" t="inlineStr">
+      <c r="F292" s="12" t="inlineStr">
         <is>
           <t>Paris 19e (118 av. Jean Jaurès) ; autre adresse affichée : B</t>
         </is>
       </c>
-      <c r="G292" t="inlineStr">
+      <c r="G292" s="12" t="inlineStr">
         <is>
           <t>France</t>
         </is>
       </c>
-      <c r="H292" t="inlineStr">
+      <c r="H292" s="12" t="inlineStr">
         <is>
           <t>Confirmée : spécialiste de la pierre naturelle (marbre, granit, dalles, blocs), vente aux particuliers et professionnels (marbriers, architectes, constructeurs).</t>
         </is>
       </c>
-      <c r="I292" t="inlineStr">
+      <c r="I292" s="12" t="inlineStr">
         <is>
           <t>https://www.marbre-import.fr</t>
         </is>
       </c>
-      <c r="J292" t="inlineStr">
+      <c r="J292" s="12" t="inlineStr">
         <is>
           <t>09 72 15 80 01</t>
         </is>
       </c>
-      <c r="K292" t="inlineStr">
+      <c r="K292" s="12" t="inlineStr">
         <is>
           <t>Recherche Claude (26/10)</t>
         </is>
       </c>
       <c r="L292" s="12" t="inlineStr">
         <is>
+          <t>Contacté le 20/10 (Gmail) — ne pas réexpédier</t>
+        </is>
+      </c>
+      <c r="N292" s="12" t="inlineStr">
+        <is>
+          <t>Vérifier s'il y a eu réponse au message du 20/10 ; AUCUN nouvel envoi</t>
+        </is>
+      </c>
+      <c r="O292" s="12" t="inlineStr">
+        <is>
+          <t>[26/10] Recherche vérifiée (segment marbreries-idf). Confirmée : spécialiste de la pierre naturelle (marbre, granit, dalles, blocs), vente aux particuliers et professionnels (marbriers, architectes, constructeurs). AUCUN e-mail publié sur la page contact du site officiel : formulaire de devis uniquement. Retenu sur la base du téléphone vérifié 09 72 15 80 01 (affiché textuellement et en lien tel: sur la page contact). Attention : la page contact affiche Paris 19e et Bordeaux ; le showroom de Villejuif annoncé dans le candidat n'y apparaît pas — à confirmer par téléphone. Domaine hors liste d'exclusion. Source e-mail : aucune (pas d e-mail publié). ⚠️ CONCURRENT suivi dans la veille prix (Crema Marfil Espagne, lot promo 20 € HT) — prudence, approche reprise de lot uniquement. NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi [26/10 croisement fichier propriétaire] Le fichier indique « Déjà contacté — Gmail 20/10/2026 » (canal propriétaire/tiers). Correction du statut : plus un prospect vierge.</t>
+        </is>
+      </c>
+      <c r="P292" s="12" t="inlineStr">
+        <is>
+          <t>5e liste — recherche (26/10)</t>
+        </is>
+      </c>
+      <c r="Q292" t="inlineStr">
+        <is>
+          <t>contact@marbre-import.fr</t>
+        </is>
+      </c>
+    </row>
+    <row r="293" ht="15" customHeight="1" s="13">
+      <c r="A293" s="12" t="n">
+        <v>293</v>
+      </c>
+      <c r="B293" s="12" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C293" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="D293" s="12" t="inlineStr">
+        <is>
+          <t>marbreries-idf</t>
+        </is>
+      </c>
+      <c r="E293" s="12" t="inlineStr">
+        <is>
+          <t>Arthema Marbre (marbrerie SPIMA)</t>
+        </is>
+      </c>
+      <c r="F293" s="12" t="inlineStr">
+        <is>
+          <t>Paris 3e (showroom 34 rue de Poitou, Le Marais)</t>
+        </is>
+      </c>
+      <c r="G293" s="12" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="H293" s="12" t="inlineStr">
+        <is>
+          <t>Confirmée : marbrerie de décoration sur mesure (marbre, pierre calcaire, travertin, onyx, granit, quartzite), fabrication en atelier partenaire SPIMA et pose ; clientèle d'architec…</t>
+        </is>
+      </c>
+      <c r="I293" s="12" t="inlineStr">
+        <is>
+          <t>https://arthema-marbre.com</t>
+        </is>
+      </c>
+      <c r="J293" s="12" t="inlineStr">
+        <is>
+          <t>01 42 71 79 09 / 06 19 26 42 68</t>
+        </is>
+      </c>
+      <c r="K293" s="12" t="inlineStr">
+        <is>
+          <t>Recherche Claude (26/10)</t>
+        </is>
+      </c>
+      <c r="L293" s="12" t="inlineStr">
+        <is>
+          <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
+        </is>
+      </c>
+      <c r="N293" s="12" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="O293" s="12" t="inlineStr">
+        <is>
+          <t>[26/10] Recherche vérifiée (segment marbreries-idf). Confirmée : marbrerie de décoration sur mesure (marbre, pierre calcaire, travertin, onyx, granit, quartzite), fabrication en atelier partenaire SPIMA et pose ; clientèle d'architectes et décorateurs. E-mail lu textuellement sur la page d'accueil du site officiel. Un mobile supplémentaire (06 19 26 42 68) y figure aussi. Travail explicite des pierres calcaires et travertins confirmé. Domaine hors liste d'exclusion. Source e-mail : https://arthema-marbre.com/.  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="P293" s="12" t="inlineStr">
+        <is>
+          <t>5e liste — recherche (26/10)</t>
+        </is>
+      </c>
+      <c r="Q293" s="12" t="inlineStr">
+        <is>
+          <t>contact@arthema-marbre.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="294" ht="15" customHeight="1" s="13">
+      <c r="A294" s="12" t="n">
+        <v>294</v>
+      </c>
+      <c r="B294" s="12" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C294" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="D294" s="12" t="inlineStr">
+        <is>
+          <t>marbreries-idf</t>
+        </is>
+      </c>
+      <c r="E294" s="12" t="inlineStr">
+        <is>
+          <t>Atelier Matière</t>
+        </is>
+      </c>
+      <c r="F294" s="12" t="inlineStr">
+        <is>
+          <t>Paris 16e (19 rue Vital) et Paris 17e (36 rue Brunel)</t>
+        </is>
+      </c>
+      <c r="G294" s="12" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="H294" s="12" t="inlineStr">
+        <is>
+          <t>Confirmée : studio/showroom de pierre naturelle, marbre et terrazzo haut de gamme depuis 2012, distribution et pose sur rendez-vous ; deux showrooms parisiens confirmés.</t>
+        </is>
+      </c>
+      <c r="I294" s="12" t="inlineStr">
+        <is>
+          <t>https://www.ateliermatiere.fr</t>
+        </is>
+      </c>
+      <c r="J294" s="12" t="inlineStr">
+        <is>
+          <t>01 45 04 57 65</t>
+        </is>
+      </c>
+      <c r="K294" s="12" t="inlineStr">
+        <is>
+          <t>Recherche Claude (26/10)</t>
+        </is>
+      </c>
+      <c r="L294" s="12" t="inlineStr">
+        <is>
+          <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
+        </is>
+      </c>
+      <c r="N294" s="12" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="O294" s="12" t="inlineStr">
+        <is>
+          <t>[26/10] Recherche vérifiée (segment marbreries-idf). Confirmée : studio/showroom de pierre naturelle, marbre et terrazzo haut de gamme depuis 2012, distribution et pose sur rendez-vous ; deux showrooms parisiens confirmés. E-mail lu textuellement sur la page Pierre du site officiel ; téléphone confirmé. Domaine hors liste d'exclusion. Site officiel, pas un annuaire. Source e-mail : https://www.ateliermatiere.fr/pierre.  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="P294" s="12" t="inlineStr">
+        <is>
+          <t>5e liste — recherche (26/10)</t>
+        </is>
+      </c>
+      <c r="Q294" s="12" t="inlineStr">
+        <is>
+          <t>info@ateliermatiere.fr</t>
+        </is>
+      </c>
+    </row>
+    <row r="295" ht="15" customHeight="1" s="13">
+      <c r="A295" s="12" t="n">
+        <v>295</v>
+      </c>
+      <c r="B295" s="12" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C295" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="D295" s="12" t="inlineStr">
+        <is>
+          <t>marbreries-idf</t>
+        </is>
+      </c>
+      <c r="E295" s="12" t="inlineStr">
+        <is>
+          <t>Artefacts Paris</t>
+        </is>
+      </c>
+      <c r="F295" s="12" t="inlineStr">
+        <is>
+          <t>Paris 7e (showroom 17 bis passage Jean Nicot) ; atelier à Né</t>
+        </is>
+      </c>
+      <c r="G295" s="12" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="H295" s="12" t="inlineStr">
+        <is>
+          <t>Confirmée : marbrerie fine et pierre de taille, revêtements durs en pierre naturelle pour la construction et l'agencement de luxe ; showroom Paris 7e et atelier/bureau d'études à N…</t>
+        </is>
+      </c>
+      <c r="I295" s="12" t="inlineStr">
+        <is>
+          <t>https://www.artefacts-paris.com</t>
+        </is>
+      </c>
+      <c r="K295" s="12" t="inlineStr">
+        <is>
+          <t>Recherche Claude (26/10)</t>
+        </is>
+      </c>
+      <c r="L295" s="12" t="inlineStr">
+        <is>
+          <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
+        </is>
+      </c>
+      <c r="N295" s="12" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="O295" s="12" t="inlineStr">
+        <is>
+          <t>[26/10] Recherche vérifiée (segment marbreries-idf). Confirmée : marbrerie fine et pierre de taille, revêtements durs en pierre naturelle pour la construction et l'agencement de luxe ; showroom Paris 7e et atelier/bureau d'études à Nérac (47600) confirmés. E-mail lu textuellement sur le site officiel. Aucun téléphone affiché sur la page. L'atelier de façonnage est bien hors IdF (Nérac, 47) comme signalé, mais la vitrine commerciale et les chantiers sont parisiens. Domaine hors liste d'exclusion. Source e-mail : https://www.artefacts-paris.com.  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="P295" s="12" t="inlineStr">
+        <is>
+          <t>5e liste — recherche (26/10)</t>
+        </is>
+      </c>
+      <c r="Q295" s="12" t="inlineStr">
+        <is>
+          <t>info@artefacts-paris.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="296" ht="15" customHeight="1" s="13">
+      <c r="A296" s="12" t="n">
+        <v>296</v>
+      </c>
+      <c r="B296" s="12" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C296" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="D296" s="12" t="inlineStr">
+        <is>
+          <t>marbreries-idf</t>
+        </is>
+      </c>
+      <c r="E296" s="12" t="inlineStr">
+        <is>
+          <t>H. Chevalier</t>
+        </is>
+      </c>
+      <c r="F296" s="12" t="inlineStr">
+        <is>
+          <t>Suresnes (26 rue Henri Regnault, 92150)</t>
+        </is>
+      </c>
+      <c r="G296" s="12" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="H296" s="12" t="inlineStr">
+        <is>
+          <t>Confirmée : restauration du patrimoine bâti depuis 1946 (maçonnerie-pierre, restauration de sculpture, hôtels particuliers et châteaux), 250 salariés, 80 M€ de CA ; adresse à Sures…</t>
+        </is>
+      </c>
+      <c r="I296" s="12" t="inlineStr">
+        <is>
+          <t>https://www.hchevalier.com</t>
+        </is>
+      </c>
+      <c r="J296" s="12" t="inlineStr">
+        <is>
+          <t>01 45 06 83 33</t>
+        </is>
+      </c>
+      <c r="K296" s="12" t="inlineStr">
+        <is>
+          <t>Recherche Claude (26/10)</t>
+        </is>
+      </c>
+      <c r="L296" s="12" t="inlineStr">
+        <is>
+          <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
+        </is>
+      </c>
+      <c r="N296" s="12" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="O296" s="12" t="inlineStr">
+        <is>
+          <t>[26/10] Recherche vérifiée (segment marbreries-idf). Confirmée : restauration du patrimoine bâti depuis 1946 (maçonnerie-pierre, restauration de sculpture, hôtels particuliers et châteaux), 250 salariés, 80 M€ de CA ; adresse à Suresnes confirmée. E-mail et téléphone lus textuellement sur la page d'accueil du site officiel. Domaine hors liste d'exclusion. Profil patrimoine/monuments : pertinence moyenne pour un calcaire égyptien standard, comme indiqué dans le candidat. Source e-mail : https://www.hchevalier.com.  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="P296" s="12" t="inlineStr">
+        <is>
+          <t>5e liste — recherche (26/10)</t>
+        </is>
+      </c>
+      <c r="Q296" s="12" t="inlineStr">
+        <is>
+          <t>contact@hchevalier.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="297" ht="15" customHeight="1" s="13">
+      <c r="A297" s="12" t="n">
+        <v>297</v>
+      </c>
+      <c r="B297" s="12" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C297" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="D297" s="12" t="inlineStr">
+        <is>
+          <t>marbreries-idf</t>
+        </is>
+      </c>
+      <c r="E297" s="12" t="inlineStr">
+        <is>
+          <t>Vexin Patrimoine</t>
+        </is>
+      </c>
+      <c r="F297" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Secteur Vexin / Île-de-France (95) — aucune adresse précise </t>
+        </is>
+      </c>
+      <c r="G297" s="12" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="H297" s="12" t="inlineStr">
+        <is>
+          <t>Confirmée : tailleur de pierre (taille sur mesure intérieur/extérieur, restauration historique, création, sols en pierre), plus de 15 ans d'expérience, clients pro et particuliers,…</t>
+        </is>
+      </c>
+      <c r="I297" s="12" t="inlineStr">
+        <is>
+          <t>https://vexinpatrimoine.fr</t>
+        </is>
+      </c>
+      <c r="J297" s="12" t="inlineStr">
+        <is>
+          <t>01 30 73 86 50</t>
+        </is>
+      </c>
+      <c r="K297" s="12" t="inlineStr">
+        <is>
+          <t>Recherche Claude (26/10)</t>
+        </is>
+      </c>
+      <c r="L297" s="12" t="inlineStr">
+        <is>
+          <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
+        </is>
+      </c>
+      <c r="N297" s="12" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="O297" s="12" t="inlineStr">
+        <is>
+          <t>[26/10] Recherche vérifiée (segment marbreries-idf). Confirmée : tailleur de pierre (taille sur mesure intérieur/extérieur, restauration historique, création, sols en pierre), plus de 15 ans d'expérience, clients pro et particuliers, zone Vexin/Île-de-France. Deux graphies sur le site : le pied de page affiche textuellement contact@vexinpatrimoine.fr (correct) ; la barre latérale affiche la coquille « contat@vexinpatrimoine.fr ». Utiliser contact@vexinpatrimoine.fr. Téléphone confirmé (affiché deux fois). Aucune ville précise publiée, cohérent avec le candidat. Domaine hors liste d'exclusion. Source e-mail : https://vexinpatrimoine.fr/.  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="P297" s="12" t="inlineStr">
+        <is>
+          <t>5e liste — recherche (26/10)</t>
+        </is>
+      </c>
+      <c r="Q297" s="12" t="inlineStr">
+        <is>
+          <t>contact@vexinpatrimoine.fr</t>
+        </is>
+      </c>
+    </row>
+    <row r="298" ht="15" customHeight="1" s="13">
+      <c r="A298" s="12" t="n">
+        <v>298</v>
+      </c>
+      <c r="B298" s="12" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C298" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="D298" s="12" t="inlineStr">
+        <is>
+          <t>marbreries-idf</t>
+        </is>
+      </c>
+      <c r="E298" s="12" t="inlineStr">
+        <is>
+          <t>Accolade Artisans</t>
+        </is>
+      </c>
+      <c r="F298" s="12" t="inlineStr">
+        <is>
+          <t>Viarmes (14 rue Kleinpeter, 95270)</t>
+        </is>
+      </c>
+      <c r="G298" s="12" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="H298" s="12" t="inlineStr">
+        <is>
+          <t>Confirmée : taille de pierre et maçonnerie de restauration du bâti ancien (certification Qualibat restauration pierre de taille et maçonnerie du patrimoine) ; adresse à Viarmes (95…</t>
+        </is>
+      </c>
+      <c r="I298" s="12" t="inlineStr">
+        <is>
+          <t>https://www.accoladeartisans.fr</t>
+        </is>
+      </c>
+      <c r="J298" s="12" t="inlineStr">
+        <is>
+          <t>06 27 85 91 92</t>
+        </is>
+      </c>
+      <c r="K298" s="12" t="inlineStr">
+        <is>
+          <t>Recherche Claude (26/10)</t>
+        </is>
+      </c>
+      <c r="L298" s="12" t="inlineStr">
+        <is>
+          <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
+        </is>
+      </c>
+      <c r="N298" s="12" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="O298" s="12" t="inlineStr">
+        <is>
+          <t>[26/10] Recherche vérifiée (segment marbreries-idf). Confirmée : taille de pierre et maçonnerie de restauration du bâti ancien (certification Qualibat restauration pierre de taille et maçonnerie du patrimoine) ; adresse à Viarmes (95270) confirmée. E-mail lu textuellement dans la section Coordonnées du pied de page ; téléphone confirmé (en-tête et pied de page). Domaine hors liste d'exclusion. Site officiel, pas un annuaire. Source e-mail : https://www.accoladeartisans.fr/taille-de-pierre.htm.  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="P298" s="12" t="inlineStr">
+        <is>
+          <t>5e liste — recherche (26/10)</t>
+        </is>
+      </c>
+      <c r="Q298" s="12" t="inlineStr">
+        <is>
+          <t>contact@accoladeartisans.fr</t>
+        </is>
+      </c>
+    </row>
+    <row r="299" ht="15" customHeight="1" s="13">
+      <c r="A299" s="12" t="n">
+        <v>299</v>
+      </c>
+      <c r="B299" s="12" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C299" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="D299" s="12" t="inlineStr">
+        <is>
+          <t>marbreries-idf</t>
+        </is>
+      </c>
+      <c r="E299" s="12" t="inlineStr">
+        <is>
+          <t>Techno Pierre</t>
+        </is>
+      </c>
+      <c r="F299" s="12" t="inlineStr">
+        <is>
+          <t>Vanves (35 rue Aristide Briand, 92170)</t>
+        </is>
+      </c>
+      <c r="G299" s="12" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="H299" s="12" t="inlineStr">
+        <is>
+          <t>Confirmée : tailleur de pierres et marbrier du bâtiment (taille de pierre, marbrerie, rénovation et revêtement de façades en pierre, marbre et granit) ; adresse à Vanves confirmée.</t>
+        </is>
+      </c>
+      <c r="I299" s="12" t="inlineStr">
+        <is>
+          <t>https://www.technopierre.fr</t>
+        </is>
+      </c>
+      <c r="J299" s="12" t="inlineStr">
+        <is>
+          <t>09 74 56 39 83</t>
+        </is>
+      </c>
+      <c r="K299" s="12" t="inlineStr">
+        <is>
+          <t>Recherche Claude (26/10)</t>
+        </is>
+      </c>
+      <c r="L299" s="12" t="inlineStr">
+        <is>
           <t>À contacter (formulaire/tél) — EN ATTENTE</t>
         </is>
       </c>
-      <c r="N292" t="inlineStr">
+      <c r="N299" s="12" t="inlineStr">
         <is>
           <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
         </is>
       </c>
-      <c r="O292" t="inlineStr">
-        <is>
-          <t>[26/10] Recherche vérifiée (segment marbreries-idf). Confirmée : spécialiste de la pierre naturelle (marbre, granit, dalles, blocs), vente aux particuliers et professionnels (marbriers, architectes, constructeurs). AUCUN e-mail publié sur la page contact du site officiel : formulaire de devis uniquement. Retenu sur la base du téléphone vérifié 09 72 15 80 01 (affiché textuellement et en lien tel: sur la page contact). Attention : la page contact affiche Paris 19e et Bordeaux ; le showroom de Villejuif annoncé dans le candidat n'y apparaît pas — à confirmer par téléphone. Domaine hors liste d'exclusion. Source e-mail : aucune (pas d e-mail publié). ⚠️ CONCURRENT suivi dans la veille prix (Crema Marfil Espagne, lot promo 20 € HT) — prudence, approche reprise de lot uniquement. NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
-        </is>
-      </c>
-      <c r="P292" t="inlineStr">
+      <c r="O299" s="12" t="inlineStr">
+        <is>
+          <t>[26/10] Recherche vérifiée (segment marbreries-idf). Confirmée : tailleur de pierres et marbrier du bâtiment (taille de pierre, marbrerie, rénovation et revêtement de façades en pierre, marbre et granit) ; adresse à Vanves confirmée. AUCUN e-mail publié sur le site officiel : la page contactez-nous.php ne propose qu'un formulaire (le lien « E-mail » pointe vers ce formulaire, pas vers une adresse). Retenu sur la base du téléphone vérifié 09 74 56 39 83, affiché plusieurs fois sur la page. Domaine hors liste d'exclusion. Source e-mail : aucune (pas d e-mail publié).  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="P299" s="12" t="inlineStr">
         <is>
           <t>5e liste — recherche (26/10)</t>
         </is>
       </c>
     </row>
-    <row r="293" ht="15" customHeight="1" s="13">
-      <c r="A293" t="n">
-        <v>293</v>
-      </c>
-      <c r="B293" t="inlineStr">
+    <row r="300" ht="15" customHeight="1" s="13">
+      <c r="A300" s="12" t="n">
+        <v>300</v>
+      </c>
+      <c r="B300" s="12" t="inlineStr">
         <is>
           <t>Pro France</t>
         </is>
       </c>
-      <c r="C293" t="n">
+      <c r="C300" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D300" s="12" t="inlineStr">
+        <is>
+          <t>normandie</t>
+        </is>
+      </c>
+      <c r="E300" s="12" t="inlineStr">
+        <is>
+          <t>Guilloux Matériaux</t>
+        </is>
+      </c>
+      <c r="F300" s="12" t="inlineStr">
+        <is>
+          <t>Cormeilles (27) et Rouen (76) — siège Saint-Pair-sur-Mer (50</t>
+        </is>
+      </c>
+      <c r="G300" s="12" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="H300" s="12" t="inlineStr">
+        <is>
+          <t>Confirmé : négoce indépendant de matériaux de construction, 10 agences en Normandie (dont Cormeilles 27 et Rouen 76), scierie/atelier à Vire, siège à Saint-Pair-sur-Mer (50380).</t>
+        </is>
+      </c>
+      <c r="I300" s="12" t="inlineStr">
+        <is>
+          <t>https://www.guillouxmateriaux.com</t>
+        </is>
+      </c>
+      <c r="J300" s="12" t="inlineStr">
+        <is>
+          <t>02 33 48 14 44 (siège) ; agence Cormeilles 02 32 57 15 98 ; agence Rouen 02 32 12 11 80</t>
+        </is>
+      </c>
+      <c r="K300" s="12" t="inlineStr">
+        <is>
+          <t>Recherche Claude (26/10)</t>
+        </is>
+      </c>
+      <c r="L300" s="12" t="inlineStr">
+        <is>
+          <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
+        </is>
+      </c>
+      <c r="N300" s="12" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="O300" s="12" t="inlineStr">
+        <is>
+          <t>[26/10] Recherche vérifiée (segment normandie). Confirmé : négoce indépendant de matériaux de construction, 10 agences en Normandie (dont Cormeilles 27 et Rouen 76), scierie/atelier à Vire, siège à Saint-Pair-sur-Mer (50380). E-mail lu TEXTUELLEMENT sur les mentions légales (responsable de la publication). Attention : le domaine de l'e-mail (guilloux-materiaux.com, avec tiret) diffère du domaine du site (guillouxmateriaux.com) — c'est bien ce qu'affiche le site officiel. Téléphones siège/Cormeilles/Rouen tous confirmés sur la même page. Hors liste d'exclusion. Source e-mail : https://www.guillouxmateriaux.com/mentions-legales-guilloux-materiaux-le-specialiste-des-materiaux-de-construction/.  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi [26/10 croisement fichier propriétaire] Divergence e-mail : fichier donne contact@guilloux-materiaux.com « à revalider » ; notre vérification site officielle a lu bonjour@guilloux-materiaux.com → conserver bonjour@.</t>
+        </is>
+      </c>
+      <c r="P300" s="12" t="inlineStr">
+        <is>
+          <t>5e liste — recherche (26/10)</t>
+        </is>
+      </c>
+      <c r="Q300" s="12" t="inlineStr">
+        <is>
+          <t>bonjour@guilloux-materiaux.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="301" ht="15" customHeight="1" s="13">
+      <c r="A301" s="12" t="n">
+        <v>301</v>
+      </c>
+      <c r="B301" s="12" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C301" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D301" s="12" t="inlineStr">
+        <is>
+          <t>normandie</t>
+        </is>
+      </c>
+      <c r="E301" s="12" t="inlineStr">
+        <is>
+          <t>Sani 27 (« Le Géant du carrelage »)</t>
+        </is>
+      </c>
+      <c r="F301" s="12" t="inlineStr">
+        <is>
+          <t>Angerville-la-Campagne (27930), ZAC de Villeneuve — près d'É</t>
+        </is>
+      </c>
+      <c r="G301" s="12" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="H301" s="12" t="inlineStr">
+        <is>
+          <t>Confirmé : magasin spécialiste du carrelage (« le plus grand magasin de carrelage ») avec sanitaire, robinetterie et meubles de salle de bain ; adresse ZAC de Villeneuve, 27930 Ang…</t>
+        </is>
+      </c>
+      <c r="I301" s="12" t="inlineStr">
+        <is>
+          <t>https://sani27.com</t>
+        </is>
+      </c>
+      <c r="J301" s="12" t="inlineStr">
+        <is>
+          <t>02 32 28 00 12</t>
+        </is>
+      </c>
+      <c r="K301" s="12" t="inlineStr">
+        <is>
+          <t>Recherche Claude (26/10)</t>
+        </is>
+      </c>
+      <c r="L301" s="12" t="inlineStr">
+        <is>
+          <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
+        </is>
+      </c>
+      <c r="N301" s="12" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="O301" s="12" t="inlineStr">
+        <is>
+          <t>[26/10] Recherche vérifiée (segment normandie). Confirmé : magasin spécialiste du carrelage (« le plus grand magasin de carrelage ») avec sanitaire, robinetterie et meubles de salle de bain ; adresse ZAC de Villeneuve, 27930 Angerville-la-Campagne, zone d'Évreux. contact@sani27.fr est écrit TEXTUELLEMENT dans le pied de page du site officiel. Divergence confirmée : le lien mailto associé pointe vers sani27@wanadoo.fr — en cas de non-réponse sur contact@sani27.fr, utiliser sani27@wanadoo.fr en seconde adresse. Téléphone 02 32 28 00 12 confirmé. Hors liste d'exclusion. Source e-mail : https://sani27.com/.  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="P301" s="12" t="inlineStr">
+        <is>
+          <t>5e liste — recherche (26/10)</t>
+        </is>
+      </c>
+      <c r="Q301" s="12" t="inlineStr">
+        <is>
+          <t>contact@sani27.fr</t>
+        </is>
+      </c>
+    </row>
+    <row r="302" ht="15" customHeight="1" s="13">
+      <c r="A302" s="12" t="n">
+        <v>302</v>
+      </c>
+      <c r="B302" s="12" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C302" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D302" s="12" t="inlineStr">
+        <is>
+          <t>normandie</t>
+        </is>
+      </c>
+      <c r="E302" s="12" t="inlineStr">
+        <is>
+          <t>BCA Matériaux Anciens</t>
+        </is>
+      </c>
+      <c r="F302" s="12" t="inlineStr">
+        <is>
+          <t>Méry-Corbon (14370) et Pont-l'Évêque (14130) — siège Segré-e</t>
+        </is>
+      </c>
+      <c r="G302" s="12" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="H302" s="12" t="inlineStr">
+        <is>
+          <t>Confirmé : « Spécialiste des matériaux anciens » — dallages et carrelages anciens en pierre, parquets anciens, tomettes, pavés, parements pierre, cheminées ; deux agences normandes…</t>
+        </is>
+      </c>
+      <c r="I302" s="12" t="inlineStr">
+        <is>
+          <t>https://www.bca-materiauxanciens.com</t>
+        </is>
+      </c>
+      <c r="J302" s="12" t="inlineStr">
+        <is>
+          <t>02 31 23 95 87 (Méry-Corbon) ; 02 61 67 23 40 (Pont-l'Évêque) ; +33 (0)2 41 61 62 40 (siège)</t>
+        </is>
+      </c>
+      <c r="K302" s="12" t="inlineStr">
+        <is>
+          <t>Recherche Claude (26/10)</t>
+        </is>
+      </c>
+      <c r="L302" s="12" t="inlineStr">
+        <is>
+          <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
+        </is>
+      </c>
+      <c r="N302" s="12" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="O302" s="12" t="inlineStr">
+        <is>
+          <t>[26/10] Recherche vérifiée (segment normandie). Confirmé : « Spécialiste des matériaux anciens » — dallages et carrelages anciens en pierre, parquets anciens, tomettes, pavés, parements pierre, cheminées ; deux agences normandes (Méry-Corbon et Pont-l'Évêque), siège en Pays de la Loire. normandie@bcamateriaux.com (agence Méry-Corbon) lu TEXTUELLEMENT sur le site officiel, ainsi que pontleveque@bcamateriaux.com, info@bcamateriaux.com et david@bcamateriaux.com (anglais). Tous les téléphones confirmés. Cœur de métier aligné (dallages pierre par lots). Hors liste d'exclusion. Source e-mail : https://www.bca-materiauxanciens.com.  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="P302" s="12" t="inlineStr">
+        <is>
+          <t>5e liste — recherche (26/10)</t>
+        </is>
+      </c>
+      <c r="Q302" s="12" t="inlineStr">
+        <is>
+          <t>normandie@bcamateriaux.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="303" ht="15" customHeight="1" s="13">
+      <c r="A303" s="12" t="n">
+        <v>303</v>
+      </c>
+      <c r="B303" s="12" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C303" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="D293" t="inlineStr">
-        <is>
-          <t>marbreries-idf</t>
-        </is>
-      </c>
-      <c r="E293" t="inlineStr">
-        <is>
-          <t>Arthema Marbre (marbrerie SPIMA)</t>
-        </is>
-      </c>
-      <c r="F293" t="inlineStr">
-        <is>
-          <t>Paris 3e (showroom 34 rue de Poitou, Le Marais)</t>
-        </is>
-      </c>
-      <c r="G293" t="inlineStr">
+      <c r="D303" s="12" t="inlineStr">
+        <is>
+          <t>normandie</t>
+        </is>
+      </c>
+      <c r="E303" s="12" t="inlineStr">
+        <is>
+          <t>Adéquate - Marbrerie Décorative</t>
+        </is>
+      </c>
+      <c r="F303" s="12" t="inlineStr">
+        <is>
+          <t>Seulline (14310), ZA Eco 5 — près de Caen</t>
+        </is>
+      </c>
+      <c r="G303" s="12" t="inlineStr">
         <is>
           <t>France</t>
         </is>
       </c>
-      <c r="H293" t="inlineStr">
-        <is>
-          <t>Confirmée : marbrerie de décoration sur mesure (marbre, pierre calcaire, travertin, onyx, granit, quartzite), fabrication en atelier partenaire SPIMA et pose ; clientèle d'architec…</t>
-        </is>
-      </c>
-      <c r="I293" t="inlineStr">
-        <is>
-          <t>https://arthema-marbre.com</t>
-        </is>
-      </c>
-      <c r="J293" t="inlineStr">
-        <is>
-          <t>01 42 71 79 09 / 06 19 26 42 68</t>
-        </is>
-      </c>
-      <c r="K293" t="inlineStr">
+      <c r="H303" s="12" t="inlineStr">
+        <is>
+          <t>Confirmé : marbrerie décorative avec showroom (visites sur rendez-vous), ZA Eco 5 n° 7 et 9, 14310 Seulline, « près de Caen en Normandie ».</t>
+        </is>
+      </c>
+      <c r="I303" s="12" t="inlineStr">
+        <is>
+          <t>https://www.adequatemarbrerie.fr</t>
+        </is>
+      </c>
+      <c r="J303" s="12" t="inlineStr">
+        <is>
+          <t>02 31 24 11 22</t>
+        </is>
+      </c>
+      <c r="K303" s="12" t="inlineStr">
         <is>
           <t>Recherche Claude (26/10)</t>
         </is>
       </c>
-      <c r="L293" s="12" t="inlineStr">
+      <c r="L303" s="12" t="inlineStr">
         <is>
           <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
         </is>
       </c>
-      <c r="N293" t="inlineStr">
+      <c r="N303" s="12" t="inlineStr">
         <is>
           <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
         </is>
       </c>
-      <c r="O293" t="inlineStr">
-        <is>
-          <t>[26/10] Recherche vérifiée (segment marbreries-idf). Confirmée : marbrerie de décoration sur mesure (marbre, pierre calcaire, travertin, onyx, granit, quartzite), fabrication en atelier partenaire SPIMA et pose ; clientèle d'architectes et décorateurs. E-mail lu textuellement sur la page d'accueil du site officiel. Un mobile supplémentaire (06 19 26 42 68) y figure aussi. Travail explicite des pierres calcaires et travertins confirmé. Domaine hors liste d'exclusion. Source e-mail : https://arthema-marbre.com/.  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
-        </is>
-      </c>
-      <c r="P293" t="inlineStr">
+      <c r="O303" s="12" t="inlineStr">
+        <is>
+          <t>[26/10] Recherche vérifiée (segment normandie). Confirmé : marbrerie décorative avec showroom (visites sur rendez-vous), ZA Eco 5 n° 7 et 9, 14310 Seulline, « près de Caen en Normandie ». contact@adequatemarbrerie.fr lu TEXTUELLEMENT sur la page contact du site officiel (en texte et en lien mailto, concordants). Téléphone confirmé. Hors liste d'exclusion. Source e-mail : https://www.adequatemarbrerie.fr/contact.  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="P303" s="12" t="inlineStr">
         <is>
           <t>5e liste — recherche (26/10)</t>
         </is>
       </c>
-      <c r="Q293" t="inlineStr">
-        <is>
-          <t>contact@arthema-marbre.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="294" ht="15" customHeight="1" s="13">
-      <c r="A294" t="n">
-        <v>294</v>
-      </c>
-      <c r="B294" t="inlineStr">
+      <c r="Q303" s="12" t="inlineStr">
+        <is>
+          <t>contact@adequatemarbrerie.fr</t>
+        </is>
+      </c>
+    </row>
+    <row r="304" ht="15" customHeight="1" s="13">
+      <c r="A304" s="12" t="n">
+        <v>304</v>
+      </c>
+      <c r="B304" s="12" t="inlineStr">
         <is>
           <t>Pro France</t>
         </is>
       </c>
-      <c r="C294" t="n">
+      <c r="C304" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="D294" t="inlineStr">
-        <is>
-          <t>marbreries-idf</t>
-        </is>
-      </c>
-      <c r="E294" t="inlineStr">
-        <is>
-          <t>Atelier Matière</t>
-        </is>
-      </c>
-      <c r="F294" t="inlineStr">
-        <is>
-          <t>Paris 16e (19 rue Vital) et Paris 17e (36 rue Brunel)</t>
-        </is>
-      </c>
-      <c r="G294" t="inlineStr">
+      <c r="D304" s="12" t="inlineStr">
+        <is>
+          <t>normandie</t>
+        </is>
+      </c>
+      <c r="E304" s="12" t="inlineStr">
+        <is>
+          <t>Motte Décoration</t>
+        </is>
+      </c>
+      <c r="F304" s="12" t="inlineStr">
+        <is>
+          <t>Le Pré-d'Auge (14340), 10 Chemin des Vatines — entre Cambrem</t>
+        </is>
+      </c>
+      <c r="G304" s="12" t="inlineStr">
         <is>
           <t>France</t>
         </is>
       </c>
-      <c r="H294" t="inlineStr">
-        <is>
-          <t>Confirmée : studio/showroom de pierre naturelle, marbre et terrazzo haut de gamme depuis 2012, distribution et pose sur rendez-vous ; deux showrooms parisiens confirmés.</t>
-        </is>
-      </c>
-      <c r="I294" t="inlineStr">
-        <is>
-          <t>https://www.ateliermatiere.fr</t>
-        </is>
-      </c>
-      <c r="J294" t="inlineStr">
-        <is>
-          <t>01 45 04 57 65</t>
-        </is>
-      </c>
-      <c r="K294" t="inlineStr">
+      <c r="H304" s="12" t="inlineStr">
+        <is>
+          <t>Confirmé via sources tierces : société MOTTE DECORATION immatriculée (SIREN 844835728, taille/façonnage/finissage de pierres) au Pré-d'Auge (14340) ; marbrerie décorative familiale…</t>
+        </is>
+      </c>
+      <c r="I304" s="12" t="inlineStr">
+        <is>
+          <t>https://www.mottedecoration.com</t>
+        </is>
+      </c>
+      <c r="J304" s="12" t="inlineStr">
+        <is>
+          <t>02 31 32 22 00</t>
+        </is>
+      </c>
+      <c r="K304" s="12" t="inlineStr">
         <is>
           <t>Recherche Claude (26/10)</t>
         </is>
       </c>
-      <c r="L294" s="12" t="inlineStr">
+      <c r="L304" s="12" t="inlineStr">
         <is>
           <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
         </is>
       </c>
-      <c r="N294" t="inlineStr">
+      <c r="N304" s="12" t="inlineStr">
         <is>
           <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
         </is>
       </c>
-      <c r="O294" t="inlineStr">
-        <is>
-          <t>[26/10] Recherche vérifiée (segment marbreries-idf). Confirmée : studio/showroom de pierre naturelle, marbre et terrazzo haut de gamme depuis 2012, distribution et pose sur rendez-vous ; deux showrooms parisiens confirmés. E-mail lu textuellement sur la page Pierre du site officiel ; téléphone confirmé. Domaine hors liste d'exclusion. Site officiel, pas un annuaire. Source e-mail : https://www.ateliermatiere.fr/pierre.  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
-        </is>
-      </c>
-      <c r="P294" t="inlineStr">
+      <c r="O304" s="12" t="inlineStr">
+        <is>
+          <t>[26/10] Recherche vérifiée (segment normandie). Confirmé via sources tierces : société MOTTE DECORATION immatriculée (SIREN 844835728, taille/façonnage/finissage de pierres) au Pré-d'Auge (14340) ; marbrerie décorative familiale (marbre, granit, quartz, pierre naturelle) intervenant sur toute la Normandie — societe.com, Initiative Calvados, Pages Jaunes et index du site officiel concordants. E-mail NON confirmé textuellement : le site officiel refuse toute lecture automatisée (HTTP 401 sur l'accueil et la page contact), vérification visuelle impossible ici. L'index du moteur de recherche attribue bien contact@mottedecoration.com et le 02 31 32 22 00 au site officiel, et le téléphone est corroboré par plusieurs sources indépendantes. Retenu sur REPLI TÉLÉPHONE vérifié (02 31 32 22 00) ; ne pas utiliser l'e-mail avant confirmation visuelle sur le site. Hors liste d'exclusion. Entreprise réelle, en France, site vivant (blocage anti-robot, pas site mort). Source e-mail : aucune (pas d e-mail publié).  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="P304" s="12" t="inlineStr">
         <is>
           <t>5e liste — recherche (26/10)</t>
         </is>
       </c>
-      <c r="Q294" t="inlineStr">
-        <is>
-          <t>info@ateliermatiere.fr</t>
-        </is>
-      </c>
-    </row>
-    <row r="295" ht="15" customHeight="1" s="13">
-      <c r="A295" t="n">
-        <v>295</v>
-      </c>
-      <c r="B295" t="inlineStr">
+      <c r="Q304" s="12" t="inlineStr">
+        <is>
+          <t>contact@mottedecoration.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="305" ht="15" customHeight="1" s="13">
+      <c r="A305" s="12" t="n">
+        <v>305</v>
+      </c>
+      <c r="B305" s="12" t="inlineStr">
         <is>
           <t>Pro France</t>
         </is>
       </c>
-      <c r="C295" t="n">
+      <c r="C305" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="D295" t="inlineStr">
-        <is>
-          <t>marbreries-idf</t>
-        </is>
-      </c>
-      <c r="E295" t="inlineStr">
-        <is>
-          <t>Artefacts Paris</t>
-        </is>
-      </c>
-      <c r="F295" t="inlineStr">
-        <is>
-          <t>Paris 7e (showroom 17 bis passage Jean Nicot) ; atelier à Né</t>
-        </is>
-      </c>
-      <c r="G295" t="inlineStr">
+      <c r="D305" s="12" t="inlineStr">
+        <is>
+          <t>normandie</t>
+        </is>
+      </c>
+      <c r="E305" s="12" t="inlineStr">
+        <is>
+          <t>Carreau Déco (SARL)</t>
+        </is>
+      </c>
+      <c r="F305" s="12" t="inlineStr">
+        <is>
+          <t>Évreux (27) ; autres magasins : Barentin, Tourville-la-Riviè</t>
+        </is>
+      </c>
+      <c r="G305" s="12" t="inlineStr">
         <is>
           <t>France</t>
         </is>
       </c>
-      <c r="H295" t="inlineStr">
-        <is>
-          <t>Confirmée : marbrerie fine et pierre de taille, revêtements durs en pierre naturelle pour la construction et l'agencement de luxe ; showroom Paris 7e et atelier/bureau d'études à N…</t>
-        </is>
-      </c>
-      <c r="I295" t="inlineStr">
-        <is>
-          <t>https://www.artefacts-paris.com</t>
-        </is>
-      </c>
-      <c r="K295" t="inlineStr">
+      <c r="H305" s="12" t="inlineStr">
+        <is>
+          <t>Confirmé : enseigne de carrelage (« Carrelage haut de gamme, sol et mur ») — grès cérame, dalles, faïence, intérieur/extérieur ; 6 points de vente confirmés dont Évreux, Barentin, …</t>
+        </is>
+      </c>
+      <c r="I305" s="12" t="inlineStr">
+        <is>
+          <t>https://www.carreaudeco.com</t>
+        </is>
+      </c>
+      <c r="J305" s="12" t="inlineStr">
+        <is>
+          <t>02 32 30 62 04 (Évreux) ; 02 37 21 27 80 (Lèves/standard) ; 02 78 77 51 00 (Barentin) ; 02 78 77 09 77 (Tourville) ; 02 78 93 05 05 (Montivilliers) ; 02 37 46 23 27 (Vernouillet)</t>
+        </is>
+      </c>
+      <c r="K305" s="12" t="inlineStr">
         <is>
           <t>Recherche Claude (26/10)</t>
         </is>
       </c>
-      <c r="L295" s="12" t="inlineStr">
+      <c r="L305" s="12" t="inlineStr">
+        <is>
+          <t>À contacter (formulaire/tél) — EN ATTENTE</t>
+        </is>
+      </c>
+      <c r="N305" s="12" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="O305" s="12" t="inlineStr">
+        <is>
+          <t>[26/10] Recherche vérifiée (segment normandie). Confirmé : enseigne de carrelage (« Carrelage haut de gamme, sol et mur ») — grès cérame, dalles, faïence, intérieur/extérieur ; 6 points de vente confirmés dont Évreux, Barentin, Tourville-la-Rivière et Montivilliers. AUCUN e-mail publié textuellement sur le site officiel (formulaire de contact uniquement) — vérifié. Retenu sur REPLI TÉLÉPHONE : les 6 numéros de magasins sont confirmés sur le site officiel, dont Évreux 02 32 30 62 04 et le standard de Lèves 02 37 21 27 80. Hors liste d'exclusion. Source e-mail : aucune (pas d e-mail publié).  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="P305" s="12" t="inlineStr">
+        <is>
+          <t>5e liste — recherche (26/10)</t>
+        </is>
+      </c>
+    </row>
+    <row r="306" ht="15" customHeight="1" s="13">
+      <c r="A306" s="12" t="n">
+        <v>306</v>
+      </c>
+      <c r="B306" s="12" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C306" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="D306" s="12" t="inlineStr">
+        <is>
+          <t>normandie</t>
+        </is>
+      </c>
+      <c r="E306" s="12" t="inlineStr">
+        <is>
+          <t>Carré &amp; Déco (SAS Fortin Design)</t>
+        </is>
+      </c>
+      <c r="F306" s="12" t="inlineStr">
+        <is>
+          <t>Colombelles (14460), 6 rue de la Métallurgie — agglomération</t>
+        </is>
+      </c>
+      <c r="G306" s="12" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="H306" s="12" t="inlineStr">
+        <is>
+          <t>Confirmé : magasin de carrelage et céramique avec showroom (« votre expert en carrelage et céramique à proximité de Caen »), pierre naturelle présente en gamme extérieure (activité…</t>
+        </is>
+      </c>
+      <c r="I306" s="12" t="inlineStr">
+        <is>
+          <t>https://carre-deco.fr</t>
+        </is>
+      </c>
+      <c r="J306" s="12" t="inlineStr">
+        <is>
+          <t>02 31 34 40 50</t>
+        </is>
+      </c>
+      <c r="K306" s="12" t="inlineStr">
+        <is>
+          <t>Recherche Claude (26/10)</t>
+        </is>
+      </c>
+      <c r="L306" s="12" t="inlineStr">
+        <is>
+          <t>À contacter (formulaire/tél) — EN ATTENTE</t>
+        </is>
+      </c>
+      <c r="N306" s="12" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="O306" s="12" t="inlineStr">
+        <is>
+          <t>[26/10] Recherche vérifiée (segment normandie). Confirmé : magasin de carrelage et céramique avec showroom (« votre expert en carrelage et céramique à proximité de Caen »), pierre naturelle présente en gamme extérieure (activité secondaire). AUCUN e-mail publié textuellement sur le site officiel (formulaire uniquement) — vérifié. Retenu sur REPLI TÉLÉPHONE : 02 31 34 40 50 confirmé sur le site officiel, adresse Colombelles confirmée. Nuance : la pierre naturelle n'est pas son cœur de métier (carrelage/céramique d'abord). Hors liste d'exclusion. Source e-mail : aucune (pas d e-mail publié).  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="P306" s="12" t="inlineStr">
+        <is>
+          <t>5e liste — recherche (26/10)</t>
+        </is>
+      </c>
+    </row>
+    <row r="307" ht="15" customHeight="1" s="13">
+      <c r="A307" s="12" t="n">
+        <v>307</v>
+      </c>
+      <c r="B307" s="12" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C307" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="D307" s="12" t="inlineStr">
+        <is>
+          <t>destockage-exterieur</t>
+        </is>
+      </c>
+      <c r="E307" s="12" t="inlineStr">
+        <is>
+          <t>Vallois (groupe Spie batignolles paysage) — agence Val de Seine</t>
+        </is>
+      </c>
+      <c r="F307" s="12" t="inlineStr">
+        <is>
+          <t>Val-de-Reuil (27100, Z.A la Comminière) — agence IDF à Trapp</t>
+        </is>
+      </c>
+      <c r="G307" s="12" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="H307" s="12" t="inlineStr">
+        <is>
+          <t>Confirmée : « aménagements paysagers » dans le Grand Ouest, société de Spie batignolles paysage (vérifié sur la page d'accueil) ; la page contact confirme l'agence Val de Seine à V…</t>
+        </is>
+      </c>
+      <c r="I307" s="12" t="inlineStr">
+        <is>
+          <t>https://www.vallois.eu/</t>
+        </is>
+      </c>
+      <c r="J307" s="12" t="inlineStr">
+        <is>
+          <t>02 32 40 32 30 (Val de Seine) ; 01 30 16 07 00 (IDF Trappes)</t>
+        </is>
+      </c>
+      <c r="K307" s="12" t="inlineStr">
+        <is>
+          <t>Recherche Claude (26/10)</t>
+        </is>
+      </c>
+      <c r="L307" s="12" t="inlineStr">
         <is>
           <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
         </is>
       </c>
-      <c r="N295" t="inlineStr">
+      <c r="N307" s="12" t="inlineStr">
         <is>
           <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
         </is>
       </c>
-      <c r="O295" t="inlineStr">
-        <is>
-          <t>[26/10] Recherche vérifiée (segment marbreries-idf). Confirmée : marbrerie fine et pierre de taille, revêtements durs en pierre naturelle pour la construction et l'agencement de luxe ; showroom Paris 7e et atelier/bureau d'études à Nérac (47600) confirmés. E-mail lu textuellement sur le site officiel. Aucun téléphone affiché sur la page. L'atelier de façonnage est bien hors IdF (Nérac, 47) comme signalé, mais la vitrine commerciale et les chantiers sont parisiens. Domaine hors liste d'exclusion. Source e-mail : https://www.artefacts-paris.com.  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
-        </is>
-      </c>
-      <c r="P295" t="inlineStr">
+      <c r="O307" s="12" t="inlineStr">
+        <is>
+          <t>[26/10] Recherche vérifiée (segment destockage-exterieur). Confirmée : « aménagements paysagers » dans le Grand Ouest, société de Spie batignolles paysage (vérifié sur la page d'accueil) ; la page contact confirme l'agence Val de Seine à Val-de-Reuil 27100 et l'agence IDF à Trappes 78190. E-mail lu textuellement dans la fiche « Agence Val de Seine » de la page contact ; les deux téléphones y figurent aussi textuellement. Précision : la page contact donne comme siège social de Spie batignolles paysage Nanterre (92) et comme siège administratif St Hymer (14) ; Mirville (76210) est l'adresse de l'agence de l'Estuaire, pas du siège. Hors liste d'exclusion. Candidat solide. Source e-mail : https://www.vallois.eu/contact.  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi [26/10 croisement fichier propriétaire] Variante IdF (fichier) : agence-idf@vallois.eu / 01 30 16 07 00 — choisir l'agence selon le chantier.</t>
+        </is>
+      </c>
+      <c r="P307" s="12" t="inlineStr">
         <is>
           <t>5e liste — recherche (26/10)</t>
         </is>
       </c>
-      <c r="Q295" t="inlineStr">
-        <is>
-          <t>info@artefacts-paris.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="296" ht="15" customHeight="1" s="13">
-      <c r="A296" t="n">
-        <v>296</v>
-      </c>
-      <c r="B296" t="inlineStr">
+      <c r="Q307" s="12" t="inlineStr">
+        <is>
+          <t>agence-valdeseine@vallois.eu</t>
+        </is>
+      </c>
+    </row>
+    <row r="308" ht="15" customHeight="1" s="13">
+      <c r="A308" s="12" t="n">
+        <v>308</v>
+      </c>
+      <c r="B308" s="12" t="inlineStr">
         <is>
           <t>Pro France</t>
         </is>
       </c>
-      <c r="C296" t="n">
+      <c r="C308" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D308" s="12" t="inlineStr">
+        <is>
+          <t>destockage-exterieur</t>
+        </is>
+      </c>
+      <c r="E308" s="12" t="inlineStr">
+        <is>
+          <t>Tricycle Environnement / Bâticycle</t>
+        </is>
+      </c>
+      <c r="F308" s="12" t="inlineStr">
+        <is>
+          <t>Gennevilliers (120 rue du Moulin de Cage, 92230)</t>
+        </is>
+      </c>
+      <c r="G308" s="12" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="H308" s="12" t="inlineStr">
+        <is>
+          <t>Confirmée : « Matériaux BTP d'occasion », « Réemploi de matériaux de second œuvre », « Curage de bâtiment » — réemploi/revente de matériaux de construction, vérifié sur le site off…</t>
+        </is>
+      </c>
+      <c r="I308" s="12" t="inlineStr">
+        <is>
+          <t>https://www.tricycle-environnement.fr/</t>
+        </is>
+      </c>
+      <c r="J308" s="12" t="inlineStr">
+        <is>
+          <t>07 60 62 41 36 / 06 99 57 37 28</t>
+        </is>
+      </c>
+      <c r="K308" s="12" t="inlineStr">
+        <is>
+          <t>Recherche Claude (26/10)</t>
+        </is>
+      </c>
+      <c r="L308" s="12" t="inlineStr">
+        <is>
+          <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
+        </is>
+      </c>
+      <c r="N308" s="12" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="O308" s="12" t="inlineStr">
+        <is>
+          <t>[26/10] Recherche vérifiée (segment destockage-exterieur). Confirmée : « Matériaux BTP d'occasion », « Réemploi de matériaux de second œuvre », « Curage de bâtiment » — réemploi/revente de matériaux de construction, vérifié sur le site officiel. E-mail lu textuellement en en-tête ET en pied de page ; téléphone confirmé sous deux formats (+33 7 60 62 41 36 / 07 60 62 41 36) ; adresse 120 rue du Moulin de Cage, 92230 Gennevilliers confirmée en pied de page — la ville même du stock. Hors liste d'exclusion. Candidat solide. Source e-mail : https://www.tricycle-environnement.fr/.  📍 Même ville que le dépôt (Gennevilliers) — réemploi : bon candidat reprise de lot. NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi [26/10 croisement fichier propriétaire] 2e canal relevé par le fichier : contact@bati-cycle.fr / 06 99 57 37 28 (marque Bâticycle). Choisir UNE voie à l'envoi.</t>
+        </is>
+      </c>
+      <c r="P308" s="12" t="inlineStr">
+        <is>
+          <t>5e liste — recherche (26/10)</t>
+        </is>
+      </c>
+      <c r="Q308" s="12" t="inlineStr">
+        <is>
+          <t>contact@tri-cycle.fr</t>
+        </is>
+      </c>
+    </row>
+    <row r="309" ht="15" customHeight="1" s="13">
+      <c r="A309" s="12" t="n">
+        <v>309</v>
+      </c>
+      <c r="B309" s="12" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C309" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="D296" t="inlineStr">
-        <is>
-          <t>marbreries-idf</t>
-        </is>
-      </c>
-      <c r="E296" t="inlineStr">
-        <is>
-          <t>H. Chevalier</t>
-        </is>
-      </c>
-      <c r="F296" t="inlineStr">
-        <is>
-          <t>Suresnes (26 rue Henri Regnault, 92150)</t>
-        </is>
-      </c>
-      <c r="G296" t="inlineStr">
+      <c r="D309" s="12" t="inlineStr">
+        <is>
+          <t>destockage-exterieur</t>
+        </is>
+      </c>
+      <c r="E309" s="12" t="inlineStr">
+        <is>
+          <t>Minéka</t>
+        </is>
+      </c>
+      <c r="F309" s="12" t="inlineStr">
+        <is>
+          <t>Villeurbanne (182 rue de la Poudrette, 69100)</t>
+        </is>
+      </c>
+      <c r="G309" s="12" t="inlineStr">
         <is>
           <t>France</t>
         </is>
       </c>
-      <c r="H296" t="inlineStr">
-        <is>
-          <t>Confirmée : restauration du patrimoine bâti depuis 1946 (maçonnerie-pierre, restauration de sculpture, hôtels particuliers et châteaux), 250 salariés, 80 M€ de CA ; adresse à Sures…</t>
-        </is>
-      </c>
-      <c r="I296" t="inlineStr">
-        <is>
-          <t>https://www.hchevalier.com</t>
-        </is>
-      </c>
-      <c r="J296" t="inlineStr">
-        <is>
-          <t>01 45 06 83 33</t>
-        </is>
-      </c>
-      <c r="K296" t="inlineStr">
+      <c r="H309" s="12" t="inlineStr">
+        <is>
+          <t>Confirmée : adresse « 182 rue de la Poudrette 69100 VILLEURBANNE » vérifiée dans les mentions légales, qui mentionnent aussi le magasin « Minéstock » (« Venez nous voir au Minéstoc…</t>
+        </is>
+      </c>
+      <c r="I309" s="12" t="inlineStr">
+        <is>
+          <t>https://mineka.fr/</t>
+        </is>
+      </c>
+      <c r="J309" t="inlineStr">
+        <is>
+          <t>04 78 52 86 28</t>
+        </is>
+      </c>
+      <c r="K309" s="12" t="inlineStr">
         <is>
           <t>Recherche Claude (26/10)</t>
         </is>
       </c>
-      <c r="L296" s="12" t="inlineStr">
+      <c r="L309" s="12" t="inlineStr">
         <is>
           <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
         </is>
       </c>
-      <c r="N296" t="inlineStr">
+      <c r="N309" s="12" t="inlineStr">
         <is>
           <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
         </is>
       </c>
-      <c r="O296" t="inlineStr">
-        <is>
-          <t>[26/10] Recherche vérifiée (segment marbreries-idf). Confirmée : restauration du patrimoine bâti depuis 1946 (maçonnerie-pierre, restauration de sculpture, hôtels particuliers et châteaux), 250 salariés, 80 M€ de CA ; adresse à Suresnes confirmée. E-mail et téléphone lus textuellement sur la page d'accueil du site officiel. Domaine hors liste d'exclusion. Profil patrimoine/monuments : pertinence moyenne pour un calcaire égyptien standard, comme indiqué dans le candidat. Source e-mail : https://www.hchevalier.com.  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
-        </is>
-      </c>
-      <c r="P296" t="inlineStr">
+      <c r="O309" s="12" t="inlineStr">
+        <is>
+          <t>[26/10] Recherche vérifiée (segment destockage-exterieur). Confirmée : adresse « 182 rue de la Poudrette 69100 VILLEURBANNE » vérifiée dans les mentions légales, qui mentionnent aussi le magasin « Minéstock » (« Venez nous voir au Minéstock ») — structure de collecte/revente avec point de vente physique, pas une pure marketplace. E-mail lu textuellement dans les mentions légales (« Adresse électronique : contact@mineka.fr »), seule adresse de la page. AUCUN téléphone publié : le contact ne pourra se faire que par e-mail (vérifié). En France (Lyon/Villeurbanne) ; limite logistique : loin des stocks de Vernon/Gennevilliers, retrait à organiser. Hors liste d'exclusion. Source e-mail : https://mineka.fr/mentions-legales/.  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi [26/10 croisement fichier propriétaire] Canal collecte préféré (fichier) : collecte@mineka.fr.</t>
+        </is>
+      </c>
+      <c r="P309" s="12" t="inlineStr">
         <is>
           <t>5e liste — recherche (26/10)</t>
         </is>
       </c>
-      <c r="Q296" t="inlineStr">
-        <is>
-          <t>contact@hchevalier.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="297" ht="15" customHeight="1" s="13">
-      <c r="A297" t="n">
-        <v>297</v>
-      </c>
-      <c r="B297" t="inlineStr">
+      <c r="Q309" s="12" t="inlineStr">
+        <is>
+          <t>collecte@mineka.fr</t>
+        </is>
+      </c>
+    </row>
+    <row r="310" ht="15" customHeight="1" s="13">
+      <c r="A310" s="12" t="n">
+        <v>310</v>
+      </c>
+      <c r="B310" s="12" t="inlineStr">
         <is>
           <t>Pro France</t>
         </is>
       </c>
-      <c r="C297" t="n">
+      <c r="C310" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="D297" t="inlineStr">
-        <is>
-          <t>marbreries-idf</t>
-        </is>
-      </c>
-      <c r="E297" t="inlineStr">
-        <is>
-          <t>Vexin Patrimoine</t>
-        </is>
-      </c>
-      <c r="F297" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Secteur Vexin / Île-de-France (95) — aucune adresse précise </t>
-        </is>
-      </c>
-      <c r="G297" t="inlineStr">
+      <c r="D310" s="12" t="inlineStr">
+        <is>
+          <t>destockage-exterieur</t>
+        </is>
+      </c>
+      <c r="E310" s="12" t="inlineStr">
+        <is>
+          <t>Pinson Paysage (groupe Osmaïa)</t>
+        </is>
+      </c>
+      <c r="F310" s="12" t="inlineStr">
+        <is>
+          <t>Andilly (13 avenue des Cures, 95580)</t>
+        </is>
+      </c>
+      <c r="G310" s="12" t="inlineStr">
         <is>
           <t>France</t>
         </is>
       </c>
-      <c r="H297" t="inlineStr">
-        <is>
-          <t>Confirmée : tailleur de pierre (taille sur mesure intérieur/extérieur, restauration historique, création, sols en pierre), plus de 15 ans d'expérience, clients pro et particuliers,…</t>
-        </is>
-      </c>
-      <c r="I297" t="inlineStr">
-        <is>
-          <t>https://vexinpatrimoine.fr</t>
-        </is>
-      </c>
-      <c r="J297" t="inlineStr">
-        <is>
-          <t>01 30 73 86 50</t>
-        </is>
-      </c>
-      <c r="K297" t="inlineStr">
+      <c r="H310" s="12" t="inlineStr">
+        <is>
+          <t>Confirmée : page « Nous contacter » vérifiée — siège « 13 Avenue des Cures, 95580 Andilly » ; activités « Création », « Entretien » (espaces verts) et « Génie écologique » affichée…</t>
+        </is>
+      </c>
+      <c r="I310" s="12" t="inlineStr">
+        <is>
+          <t>https://www.pinson-paysage.com/</t>
+        </is>
+      </c>
+      <c r="J310" t="inlineStr">
+        <is>
+          <t>01 34 16 61 01</t>
+        </is>
+      </c>
+      <c r="K310" s="12" t="inlineStr">
         <is>
           <t>Recherche Claude (26/10)</t>
         </is>
       </c>
-      <c r="L297" s="12" t="inlineStr">
+      <c r="L310" s="12" t="inlineStr">
         <is>
           <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
         </is>
       </c>
-      <c r="N297" t="inlineStr">
+      <c r="N310" s="12" t="inlineStr">
         <is>
           <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
         </is>
       </c>
-      <c r="O297" t="inlineStr">
-        <is>
-          <t>[26/10] Recherche vérifiée (segment marbreries-idf). Confirmée : tailleur de pierre (taille sur mesure intérieur/extérieur, restauration historique, création, sols en pierre), plus de 15 ans d'expérience, clients pro et particuliers, zone Vexin/Île-de-France. Deux graphies sur le site : le pied de page affiche textuellement contact@vexinpatrimoine.fr (correct) ; la barre latérale affiche la coquille « contat@vexinpatrimoine.fr ». Utiliser contact@vexinpatrimoine.fr. Téléphone confirmé (affiché deux fois). Aucune ville précise publiée, cohérent avec le candidat. Domaine hors liste d'exclusion. Source e-mail : https://vexinpatrimoine.fr/.  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
-        </is>
-      </c>
-      <c r="P297" t="inlineStr">
+      <c r="O310" s="12" t="inlineStr">
+        <is>
+          <t>[26/10] Recherche vérifiée (segment destockage-exterieur). Confirmée : page « Nous contacter » vérifiée — siège « 13 Avenue des Cures, 95580 Andilly » ; activités « Création », « Entretien » (espaces verts) et « Génie écologique » affichées, cohérentes avec une entreprise paysagère IDF. E-mail lu textuellement (seule adresse de la page). AUCUN téléphone sur la page contact (formulaire uniquement) : contact par e-mail vérifié. Réserve maintenue : le site met en avant le végétal/génie écologique plus que la maçonnerie minérale — pertinence segment (b) à pondérer. Hors liste d'exclusion. Source e-mail : https://www.pinson-paysage.com/nous-contacter/.  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="P310" s="12" t="inlineStr">
         <is>
           <t>5e liste — recherche (26/10)</t>
         </is>
       </c>
-      <c r="Q297" t="inlineStr">
-        <is>
-          <t>contact@vexinpatrimoine.fr</t>
-        </is>
-      </c>
-    </row>
-    <row r="298" ht="15" customHeight="1" s="13">
-      <c r="A298" t="n">
-        <v>298</v>
-      </c>
-      <c r="B298" t="inlineStr">
+      <c r="Q310" s="12" t="inlineStr">
+        <is>
+          <t>pinson@pinson-paysage.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="311" ht="15" customHeight="1" s="13">
+      <c r="A311" s="12" t="n">
+        <v>311</v>
+      </c>
+      <c r="B311" s="12" t="inlineStr">
         <is>
           <t>Pro France</t>
         </is>
       </c>
-      <c r="C298" t="n">
+      <c r="C311" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D311" s="12" t="inlineStr">
+        <is>
+          <t>destockage-exterieur</t>
+        </is>
+      </c>
+      <c r="E311" s="12" t="inlineStr">
+        <is>
+          <t>NOZ (centrale d'achat S.F.N.)</t>
+        </is>
+      </c>
+      <c r="F311" s="12" t="inlineStr">
+        <is>
+          <t>Saint-Berthevin (53940)</t>
+        </is>
+      </c>
+      <c r="G311" s="12" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="H311" s="12" t="inlineStr">
+        <is>
+          <t>Confirmée : page contact vérifiée — adresse « 53940 Saint-Berthevin – France », formulaire avec champ « Vous êtes ? » incluant « Je suis un fournisseur » et objet « Besoin de désto…</t>
+        </is>
+      </c>
+      <c r="I311" s="12" t="inlineStr">
+        <is>
+          <t>https://www.noz.fr/</t>
+        </is>
+      </c>
+      <c r="J311" s="12" t="inlineStr">
+        <is>
+          <t>02 43 01 53 54</t>
+        </is>
+      </c>
+      <c r="K311" s="12" t="inlineStr">
+        <is>
+          <t>Recherche Claude (26/10)</t>
+        </is>
+      </c>
+      <c r="L311" s="12" t="inlineStr">
+        <is>
+          <t>À contacter (formulaire/tél) — EN ATTENTE</t>
+        </is>
+      </c>
+      <c r="N311" s="12" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
+        </is>
+      </c>
+      <c r="O311" s="12" t="inlineStr">
+        <is>
+          <t>[26/10] Recherche vérifiée (segment destockage-exterieur). Confirmée : page contact vérifiée — adresse « 53940 Saint-Berthevin – France », formulaire avec champ « Vous êtes ? » incluant « Je suis un fournisseur » et objet « Besoin de déstockage », cohérent avec l'activité de rachat de surstocks/lots. RETENU SANS E-MAIL : aucun e-mail publié sur https://www.noz.fr/contactez-nous/ (revérifié le 26/10/2026 — le seul mot « Email » est un champ de formulaire), mais le téléphone 02 43 01 53 54 y est écrit textuellement et vérifié ; contact via ce numéro ou le formulaire fournisseur « Besoin de déstockage ». Hors liste d'exclusion. Réserve : lot minéral lourd atypique dans leur mix. Source e-mail : aucune (pas d e-mail publié).  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi [26/10 croisement fichier propriétaire] E-mail noz@noz.fr apporté par le fichier — NON vérifié sur site officiel, à confirmer avant envoi.</t>
+        </is>
+      </c>
+      <c r="P311" s="12" t="inlineStr">
+        <is>
+          <t>5e liste — recherche (26/10)</t>
+        </is>
+      </c>
+      <c r="Q311" t="inlineStr">
+        <is>
+          <t>noz@noz.fr</t>
+        </is>
+      </c>
+    </row>
+    <row r="312" ht="15" customHeight="1" s="13">
+      <c r="A312" t="n">
+        <v>312</v>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C312" t="n">
         <v>2</v>
       </c>
-      <c r="D298" t="inlineStr">
-        <is>
-          <t>marbreries-idf</t>
-        </is>
-      </c>
-      <c r="E298" t="inlineStr">
-        <is>
-          <t>Accolade Artisans</t>
-        </is>
-      </c>
-      <c r="F298" t="inlineStr">
-        <is>
-          <t>Viarmes (14 rue Kleinpeter, 95270)</t>
-        </is>
-      </c>
-      <c r="G298" t="inlineStr">
-        <is>
-          <t>France</t>
-        </is>
-      </c>
-      <c r="H298" t="inlineStr">
-        <is>
-          <t>Confirmée : taille de pierre et maçonnerie de restauration du bâti ancien (certification Qualibat restauration pierre de taille et maçonnerie du patrimoine) ; adresse à Viarmes (95…</t>
-        </is>
-      </c>
-      <c r="I298" t="inlineStr">
-        <is>
-          <t>https://www.accoladeartisans.fr</t>
-        </is>
-      </c>
-      <c r="J298" t="inlineStr">
-        <is>
-          <t>06 27 85 91 92</t>
-        </is>
-      </c>
-      <c r="K298" t="inlineStr">
-        <is>
-          <t>Recherche Claude (26/10)</t>
-        </is>
-      </c>
-      <c r="L298" s="12" t="inlineStr">
+      <c r="D312" t="inlineStr">
+        <is>
+          <t>Marbrerie / pierre</t>
+        </is>
+      </c>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>ILDEI</t>
+        </is>
+      </c>
+      <c r="F312" t="inlineStr">
+        <is>
+          <t>Le Plessis-Pâté (91)</t>
+        </is>
+      </c>
+      <c r="G312" t="inlineStr">
+        <is>
+          <t>Île-de-France</t>
+        </is>
+      </c>
+      <c r="H312" t="inlineStr">
+        <is>
+          <t>Marbrerie / pierre</t>
+        </is>
+      </c>
+      <c r="J312" t="inlineStr">
+        <is>
+          <t>01 60 84 11 00</t>
+        </is>
+      </c>
+      <c r="K312" t="inlineStr">
+        <is>
+          <t>Croisement fichier (26/10)</t>
+        </is>
+      </c>
+      <c r="L312" s="12" t="inlineStr">
         <is>
           <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
         </is>
       </c>
-      <c r="N298" t="inlineStr">
-        <is>
-          <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
-        </is>
-      </c>
-      <c r="O298" t="inlineStr">
-        <is>
-          <t>[26/10] Recherche vérifiée (segment marbreries-idf). Confirmée : taille de pierre et maçonnerie de restauration du bâti ancien (certification Qualibat restauration pierre de taille et maçonnerie du patrimoine) ; adresse à Viarmes (95270) confirmée. E-mail lu textuellement dans la section Coordonnées du pied de page ; téléphone confirmé (en-tête et pied de page). Domaine hors liste d'exclusion. Site officiel, pas un annuaire. Source e-mail : https://www.accoladeartisans.fr/taille-de-pierre.htm.  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
-        </is>
-      </c>
-      <c r="P298" t="inlineStr">
-        <is>
-          <t>5e liste — recherche (26/10)</t>
-        </is>
-      </c>
-      <c r="Q298" t="inlineStr">
-        <is>
-          <t>contact@accoladeartisans.fr</t>
-        </is>
-      </c>
-    </row>
-    <row r="299" ht="15" customHeight="1" s="13">
-      <c r="A299" t="n">
-        <v>299</v>
-      </c>
-      <c r="B299" t="inlineStr">
+      <c r="N312" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER — vrai From info@pierredegypte.online via Network Solutions à vérifier avant tout contact</t>
+        </is>
+      </c>
+      <c r="O312" t="inlineStr">
+        <is>
+          <t>[26/10 croisement fichier propriétaire] Apporté par le fichier propriétaire du 26/10 (origine « Recherche 31 » de son côté). E-mail à re-vérifier sur site officiel avant envoi. NE RIEN ENVOYER — vrai From info@pierredegypte.online via Network Solutions à vérifier avant tout contact</t>
+        </is>
+      </c>
+      <c r="P312" t="inlineStr">
+        <is>
+          <t>5e liste — croisement (26/10)</t>
+        </is>
+      </c>
+      <c r="Q312" t="inlineStr">
+        <is>
+          <t>contact@ildei.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="313" ht="15" customHeight="1" s="13">
+      <c r="A313" t="n">
+        <v>313</v>
+      </c>
+      <c r="B313" t="inlineStr">
         <is>
           <t>Pro France</t>
         </is>
       </c>
-      <c r="C299" t="n">
+      <c r="C313" t="n">
         <v>2</v>
       </c>
-      <c r="D299" t="inlineStr">
-        <is>
-          <t>marbreries-idf</t>
-        </is>
-      </c>
-      <c r="E299" t="inlineStr">
-        <is>
-          <t>Techno Pierre</t>
-        </is>
-      </c>
-      <c r="F299" t="inlineStr">
-        <is>
-          <t>Vanves (35 rue Aristide Briand, 92170)</t>
-        </is>
-      </c>
-      <c r="G299" t="inlineStr">
-        <is>
-          <t>France</t>
-        </is>
-      </c>
-      <c r="H299" t="inlineStr">
-        <is>
-          <t>Confirmée : tailleur de pierres et marbrier du bâtiment (taille de pierre, marbrerie, rénovation et revêtement de façades en pierre, marbre et granit) ; adresse à Vanves confirmée.</t>
-        </is>
-      </c>
-      <c r="I299" t="inlineStr">
-        <is>
-          <t>https://www.technopierre.fr</t>
-        </is>
-      </c>
-      <c r="J299" t="inlineStr">
-        <is>
-          <t>09 74 56 39 83</t>
-        </is>
-      </c>
-      <c r="K299" t="inlineStr">
-        <is>
-          <t>Recherche Claude (26/10)</t>
-        </is>
-      </c>
-      <c r="L299" s="12" t="inlineStr">
-        <is>
-          <t>À contacter (formulaire/tél) — EN ATTENTE</t>
-        </is>
-      </c>
-      <c r="N299" t="inlineStr">
-        <is>
-          <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
-        </is>
-      </c>
-      <c r="O299" t="inlineStr">
-        <is>
-          <t>[26/10] Recherche vérifiée (segment marbreries-idf). Confirmée : tailleur de pierres et marbrier du bâtiment (taille de pierre, marbrerie, rénovation et revêtement de façades en pierre, marbre et granit) ; adresse à Vanves confirmée. AUCUN e-mail publié sur le site officiel : la page contactez-nous.php ne propose qu'un formulaire (le lien « E-mail » pointe vers ce formulaire, pas vers une adresse). Retenu sur la base du téléphone vérifié 09 74 56 39 83, affiché plusieurs fois sur la page. Domaine hors liste d'exclusion. Source e-mail : aucune (pas d e-mail publié).  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
-        </is>
-      </c>
-      <c r="P299" t="inlineStr">
-        <is>
-          <t>5e liste — recherche (26/10)</t>
-        </is>
-      </c>
-    </row>
-    <row r="300" ht="15" customHeight="1" s="13">
-      <c r="A300" t="n">
-        <v>300</v>
-      </c>
-      <c r="B300" t="inlineStr">
+      <c r="D313" t="inlineStr">
+        <is>
+          <t>Marbrerie</t>
+        </is>
+      </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>La Marbrerie Contemporaine</t>
+        </is>
+      </c>
+      <c r="F313" t="inlineStr">
+        <is>
+          <t>Bagnolet (93)</t>
+        </is>
+      </c>
+      <c r="G313" t="inlineStr">
+        <is>
+          <t>Île-de-France</t>
+        </is>
+      </c>
+      <c r="H313" t="inlineStr">
+        <is>
+          <t>Marbrerie</t>
+        </is>
+      </c>
+      <c r="J313" t="inlineStr">
+        <is>
+          <t>01 48 97 00 13</t>
+        </is>
+      </c>
+      <c r="K313" t="inlineStr">
+        <is>
+          <t>Croisement fichier (26/10)</t>
+        </is>
+      </c>
+      <c r="L313" s="12" t="inlineStr">
+        <is>
+          <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
+        </is>
+      </c>
+      <c r="N313" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER — vrai From info@pierredegypte.online via Network Solutions à vérifier avant tout contact</t>
+        </is>
+      </c>
+      <c r="O313" t="inlineStr">
+        <is>
+          <t>[26/10 croisement fichier propriétaire] Apporté par le fichier propriétaire du 26/10 (origine « Recherche 31 » de son côté). E-mail à re-vérifier sur site officiel avant envoi. NE RIEN ENVOYER — vrai From info@pierredegypte.online via Network Solutions à vérifier avant tout contact</t>
+        </is>
+      </c>
+      <c r="P313" t="inlineStr">
+        <is>
+          <t>5e liste — croisement (26/10)</t>
+        </is>
+      </c>
+      <c r="Q313" t="inlineStr">
+        <is>
+          <t>contact@la-marbrerie-contemporaine.fr</t>
+        </is>
+      </c>
+    </row>
+    <row r="314" ht="15" customHeight="1" s="13">
+      <c r="A314" t="n">
+        <v>314</v>
+      </c>
+      <c r="B314" t="inlineStr">
         <is>
           <t>Pro France</t>
         </is>
       </c>
-      <c r="C300" t="n">
-        <v>1</v>
-      </c>
-      <c r="D300" t="inlineStr">
-        <is>
-          <t>normandie</t>
-        </is>
-      </c>
-      <c r="E300" t="inlineStr">
-        <is>
-          <t>Guilloux Matériaux</t>
-        </is>
-      </c>
-      <c r="F300" t="inlineStr">
-        <is>
-          <t>Cormeilles (27) et Rouen (76) — siège Saint-Pair-sur-Mer (50</t>
-        </is>
-      </c>
-      <c r="G300" t="inlineStr">
-        <is>
-          <t>France</t>
-        </is>
-      </c>
-      <c r="H300" t="inlineStr">
-        <is>
-          <t>Confirmé : négoce indépendant de matériaux de construction, 10 agences en Normandie (dont Cormeilles 27 et Rouen 76), scierie/atelier à Vire, siège à Saint-Pair-sur-Mer (50380).</t>
-        </is>
-      </c>
-      <c r="I300" t="inlineStr">
-        <is>
-          <t>https://www.guillouxmateriaux.com</t>
-        </is>
-      </c>
-      <c r="J300" t="inlineStr">
-        <is>
-          <t>02 33 48 14 44 (siège) ; agence Cormeilles 02 32 57 15 98 ; agence Rouen 02 32 12 11 80</t>
-        </is>
-      </c>
-      <c r="K300" t="inlineStr">
-        <is>
-          <t>Recherche Claude (26/10)</t>
-        </is>
-      </c>
-      <c r="L300" s="12" t="inlineStr">
+      <c r="C314" t="n">
+        <v>2</v>
+      </c>
+      <c r="D314" t="inlineStr">
+        <is>
+          <t>Marbrerie / négoce pierre</t>
+        </is>
+      </c>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>Paris Roches</t>
+        </is>
+      </c>
+      <c r="F314" t="inlineStr">
+        <is>
+          <t>Vitry-sur-Seine (94)</t>
+        </is>
+      </c>
+      <c r="G314" t="inlineStr">
+        <is>
+          <t>Île-de-France</t>
+        </is>
+      </c>
+      <c r="H314" t="inlineStr">
+        <is>
+          <t>Marbrerie / négoce pierre</t>
+        </is>
+      </c>
+      <c r="J314" t="inlineStr">
+        <is>
+          <t>01 47 26 00 99</t>
+        </is>
+      </c>
+      <c r="K314" t="inlineStr">
+        <is>
+          <t>Croisement fichier (26/10)</t>
+        </is>
+      </c>
+      <c r="L314" s="12" t="inlineStr">
         <is>
           <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
         </is>
       </c>
-      <c r="N300" t="inlineStr">
-        <is>
-          <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
-        </is>
-      </c>
-      <c r="O300" t="inlineStr">
-        <is>
-          <t>[26/10] Recherche vérifiée (segment normandie). Confirmé : négoce indépendant de matériaux de construction, 10 agences en Normandie (dont Cormeilles 27 et Rouen 76), scierie/atelier à Vire, siège à Saint-Pair-sur-Mer (50380). E-mail lu TEXTUELLEMENT sur les mentions légales (responsable de la publication). Attention : le domaine de l'e-mail (guilloux-materiaux.com, avec tiret) diffère du domaine du site (guillouxmateriaux.com) — c'est bien ce qu'affiche le site officiel. Téléphones siège/Cormeilles/Rouen tous confirmés sur la même page. Hors liste d'exclusion. Source e-mail : https://www.guillouxmateriaux.com/mentions-legales-guilloux-materiaux-le-specialiste-des-materiaux-de-construction/.  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
-        </is>
-      </c>
-      <c r="P300" t="inlineStr">
-        <is>
-          <t>5e liste — recherche (26/10)</t>
-        </is>
-      </c>
-      <c r="Q300" t="inlineStr">
-        <is>
-          <t>bonjour@guilloux-materiaux.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="301" ht="15" customHeight="1" s="13">
-      <c r="A301" t="n">
-        <v>301</v>
-      </c>
-      <c r="B301" t="inlineStr">
+      <c r="N314" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER — vrai From info@pierredegypte.online via Network Solutions à vérifier avant tout contact</t>
+        </is>
+      </c>
+      <c r="O314" t="inlineStr">
+        <is>
+          <t>[26/10 croisement fichier propriétaire] Apporté par le fichier propriétaire du 26/10 (origine « Recherche 31 » de son côté). E-mail à re-vérifier sur site officiel avant envoi. NE RIEN ENVOYER — vrai From info@pierredegypte.online via Network Solutions à vérifier avant tout contact</t>
+        </is>
+      </c>
+      <c r="P314" t="inlineStr">
+        <is>
+          <t>5e liste — croisement (26/10)</t>
+        </is>
+      </c>
+      <c r="Q314" t="inlineStr">
+        <is>
+          <t>paris-roches@orange.fr</t>
+        </is>
+      </c>
+    </row>
+    <row r="315" ht="15" customHeight="1" s="13">
+      <c r="A315" t="n">
+        <v>315</v>
+      </c>
+      <c r="B315" t="inlineStr">
         <is>
           <t>Pro France</t>
         </is>
       </c>
-      <c r="C301" t="n">
-        <v>1</v>
-      </c>
-      <c r="D301" t="inlineStr">
-        <is>
-          <t>normandie</t>
-        </is>
-      </c>
-      <c r="E301" t="inlineStr">
-        <is>
-          <t>Sani 27 (« Le Géant du carrelage »)</t>
-        </is>
-      </c>
-      <c r="F301" t="inlineStr">
-        <is>
-          <t>Angerville-la-Campagne (27930), ZAC de Villeneuve — près d'É</t>
-        </is>
-      </c>
-      <c r="G301" t="inlineStr">
-        <is>
-          <t>France</t>
-        </is>
-      </c>
-      <c r="H301" t="inlineStr">
-        <is>
-          <t>Confirmé : magasin spécialiste du carrelage (« le plus grand magasin de carrelage ») avec sanitaire, robinetterie et meubles de salle de bain ; adresse ZAC de Villeneuve, 27930 Ang…</t>
-        </is>
-      </c>
-      <c r="I301" t="inlineStr">
-        <is>
-          <t>https://sani27.com</t>
-        </is>
-      </c>
-      <c r="J301" t="inlineStr">
-        <is>
-          <t>02 32 28 00 12</t>
-        </is>
-      </c>
-      <c r="K301" t="inlineStr">
-        <is>
-          <t>Recherche Claude (26/10)</t>
-        </is>
-      </c>
-      <c r="L301" s="12" t="inlineStr">
+      <c r="C315" t="n">
+        <v>2</v>
+      </c>
+      <c r="D315" t="inlineStr">
+        <is>
+          <t>Marbrerie</t>
+        </is>
+      </c>
+      <c r="E315" t="inlineStr">
+        <is>
+          <t>Alpha Marbre</t>
+        </is>
+      </c>
+      <c r="F315" t="inlineStr">
+        <is>
+          <t>Coubert (77)</t>
+        </is>
+      </c>
+      <c r="G315" t="inlineStr">
+        <is>
+          <t>Île-de-France</t>
+        </is>
+      </c>
+      <c r="H315" t="inlineStr">
+        <is>
+          <t>Marbrerie</t>
+        </is>
+      </c>
+      <c r="J315" t="inlineStr">
+        <is>
+          <t>01 64 16 03 69</t>
+        </is>
+      </c>
+      <c r="K315" t="inlineStr">
+        <is>
+          <t>Croisement fichier (26/10)</t>
+        </is>
+      </c>
+      <c r="L315" s="12" t="inlineStr">
         <is>
           <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
         </is>
       </c>
-      <c r="N301" t="inlineStr">
-        <is>
-          <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
-        </is>
-      </c>
-      <c r="O301" t="inlineStr">
-        <is>
-          <t>[26/10] Recherche vérifiée (segment normandie). Confirmé : magasin spécialiste du carrelage (« le plus grand magasin de carrelage ») avec sanitaire, robinetterie et meubles de salle de bain ; adresse ZAC de Villeneuve, 27930 Angerville-la-Campagne, zone d'Évreux. contact@sani27.fr est écrit TEXTUELLEMENT dans le pied de page du site officiel. Divergence confirmée : le lien mailto associé pointe vers sani27@wanadoo.fr — en cas de non-réponse sur contact@sani27.fr, utiliser sani27@wanadoo.fr en seconde adresse. Téléphone 02 32 28 00 12 confirmé. Hors liste d'exclusion. Source e-mail : https://sani27.com/.  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
-        </is>
-      </c>
-      <c r="P301" t="inlineStr">
-        <is>
-          <t>5e liste — recherche (26/10)</t>
-        </is>
-      </c>
-      <c r="Q301" t="inlineStr">
-        <is>
-          <t>contact@sani27.fr</t>
-        </is>
-      </c>
-    </row>
-    <row r="302" ht="15" customHeight="1" s="13">
-      <c r="A302" t="n">
-        <v>302</v>
-      </c>
-      <c r="B302" t="inlineStr">
+      <c r="N315" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER — vrai From info@pierredegypte.online via Network Solutions à vérifier avant tout contact</t>
+        </is>
+      </c>
+      <c r="O315" t="inlineStr">
+        <is>
+          <t>[26/10 croisement fichier propriétaire] Apporté par le fichier propriétaire du 26/10 (origine « Recherche 31 » de son côté). E-mail à re-vérifier sur site officiel avant envoi. NE RIEN ENVOYER — vrai From info@pierredegypte.online via Network Solutions à vérifier avant tout contact</t>
+        </is>
+      </c>
+      <c r="P315" t="inlineStr">
+        <is>
+          <t>5e liste — croisement (26/10)</t>
+        </is>
+      </c>
+      <c r="Q315" t="inlineStr">
+        <is>
+          <t>alpha.marbre@laposte.net</t>
+        </is>
+      </c>
+    </row>
+    <row r="316" ht="15" customHeight="1" s="13">
+      <c r="A316" t="n">
+        <v>316</v>
+      </c>
+      <c r="B316" t="inlineStr">
         <is>
           <t>Pro France</t>
         </is>
       </c>
-      <c r="C302" t="n">
-        <v>1</v>
-      </c>
-      <c r="D302" t="inlineStr">
-        <is>
-          <t>normandie</t>
-        </is>
-      </c>
-      <c r="E302" t="inlineStr">
-        <is>
-          <t>BCA Matériaux Anciens</t>
-        </is>
-      </c>
-      <c r="F302" t="inlineStr">
-        <is>
-          <t>Méry-Corbon (14370) et Pont-l'Évêque (14130) — siège Segré-e</t>
-        </is>
-      </c>
-      <c r="G302" t="inlineStr">
-        <is>
-          <t>France</t>
-        </is>
-      </c>
-      <c r="H302" t="inlineStr">
-        <is>
-          <t>Confirmé : « Spécialiste des matériaux anciens » — dallages et carrelages anciens en pierre, parquets anciens, tomettes, pavés, parements pierre, cheminées ; deux agences normandes…</t>
-        </is>
-      </c>
-      <c r="I302" t="inlineStr">
-        <is>
-          <t>https://www.bca-materiauxanciens.com</t>
-        </is>
-      </c>
-      <c r="J302" t="inlineStr">
-        <is>
-          <t>02 31 23 95 87 (Méry-Corbon) ; 02 61 67 23 40 (Pont-l'Évêque) ; +33 (0)2 41 61 62 40 (siège)</t>
-        </is>
-      </c>
-      <c r="K302" t="inlineStr">
-        <is>
-          <t>Recherche Claude (26/10)</t>
-        </is>
-      </c>
-      <c r="L302" s="12" t="inlineStr">
+      <c r="C316" t="n">
+        <v>2</v>
+      </c>
+      <c r="D316" t="inlineStr">
+        <is>
+          <t>Marbrerie</t>
+        </is>
+      </c>
+      <c r="E316" t="inlineStr">
+        <is>
+          <t>Marbrerie Christian Caudron</t>
+        </is>
+      </c>
+      <c r="F316" t="inlineStr">
+        <is>
+          <t>Noisy-le-Sec (93)</t>
+        </is>
+      </c>
+      <c r="G316" t="inlineStr">
+        <is>
+          <t>Île-de-France</t>
+        </is>
+      </c>
+      <c r="H316" t="inlineStr">
+        <is>
+          <t>Marbrerie</t>
+        </is>
+      </c>
+      <c r="J316" t="inlineStr">
+        <is>
+          <t>06 30 60 75 01</t>
+        </is>
+      </c>
+      <c r="K316" t="inlineStr">
+        <is>
+          <t>Croisement fichier (26/10)</t>
+        </is>
+      </c>
+      <c r="L316" s="12" t="inlineStr">
         <is>
           <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
         </is>
       </c>
-      <c r="N302" t="inlineStr">
-        <is>
-          <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
-        </is>
-      </c>
-      <c r="O302" t="inlineStr">
-        <is>
-          <t>[26/10] Recherche vérifiée (segment normandie). Confirmé : « Spécialiste des matériaux anciens » — dallages et carrelages anciens en pierre, parquets anciens, tomettes, pavés, parements pierre, cheminées ; deux agences normandes (Méry-Corbon et Pont-l'Évêque), siège en Pays de la Loire. normandie@bcamateriaux.com (agence Méry-Corbon) lu TEXTUELLEMENT sur le site officiel, ainsi que pontleveque@bcamateriaux.com, info@bcamateriaux.com et david@bcamateriaux.com (anglais). Tous les téléphones confirmés. Cœur de métier aligné (dallages pierre par lots). Hors liste d'exclusion. Source e-mail : https://www.bca-materiauxanciens.com.  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
-        </is>
-      </c>
-      <c r="P302" t="inlineStr">
-        <is>
-          <t>5e liste — recherche (26/10)</t>
-        </is>
-      </c>
-      <c r="Q302" t="inlineStr">
-        <is>
-          <t>normandie@bcamateriaux.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="303" ht="15" customHeight="1" s="13">
-      <c r="A303" t="n">
-        <v>303</v>
-      </c>
-      <c r="B303" t="inlineStr">
+      <c r="N316" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER — vrai From info@pierredegypte.online via Network Solutions à vérifier avant tout contact</t>
+        </is>
+      </c>
+      <c r="O316" t="inlineStr">
+        <is>
+          <t>[26/10 croisement fichier propriétaire] Apporté par le fichier propriétaire du 26/10 (origine « Recherche 31 » de son côté). E-mail à re-vérifier sur site officiel avant envoi. NE RIEN ENVOYER — vrai From info@pierredegypte.online via Network Solutions à vérifier avant tout contact</t>
+        </is>
+      </c>
+      <c r="P316" t="inlineStr">
+        <is>
+          <t>5e liste — croisement (26/10)</t>
+        </is>
+      </c>
+      <c r="Q316" t="inlineStr">
+        <is>
+          <t>atelier-marbre@orange.fr</t>
+        </is>
+      </c>
+    </row>
+    <row r="317" ht="15" customHeight="1" s="13">
+      <c r="A317" t="n">
+        <v>317</v>
+      </c>
+      <c r="B317" t="inlineStr">
         <is>
           <t>Pro France</t>
         </is>
       </c>
-      <c r="C303" t="n">
+      <c r="C317" t="n">
         <v>2</v>
       </c>
-      <c r="D303" t="inlineStr">
-        <is>
-          <t>normandie</t>
-        </is>
-      </c>
-      <c r="E303" t="inlineStr">
-        <is>
-          <t>Adéquate - Marbrerie Décorative</t>
-        </is>
-      </c>
-      <c r="F303" t="inlineStr">
-        <is>
-          <t>Seulline (14310), ZA Eco 5 — près de Caen</t>
-        </is>
-      </c>
-      <c r="G303" t="inlineStr">
-        <is>
-          <t>France</t>
-        </is>
-      </c>
-      <c r="H303" t="inlineStr">
-        <is>
-          <t>Confirmé : marbrerie décorative avec showroom (visites sur rendez-vous), ZA Eco 5 n° 7 et 9, 14310 Seulline, « près de Caen en Normandie ».</t>
-        </is>
-      </c>
-      <c r="I303" t="inlineStr">
-        <is>
-          <t>https://www.adequatemarbrerie.fr</t>
-        </is>
-      </c>
-      <c r="J303" t="inlineStr">
-        <is>
-          <t>02 31 24 11 22</t>
-        </is>
-      </c>
-      <c r="K303" t="inlineStr">
-        <is>
-          <t>Recherche Claude (26/10)</t>
-        </is>
-      </c>
-      <c r="L303" s="12" t="inlineStr">
+      <c r="D317" t="inlineStr">
+        <is>
+          <t>Négoce matériaux</t>
+        </is>
+      </c>
+      <c r="E317" t="inlineStr">
+        <is>
+          <t>Facomat</t>
+        </is>
+      </c>
+      <c r="F317" t="inlineStr">
+        <is>
+          <t>Buchy (76)</t>
+        </is>
+      </c>
+      <c r="G317" t="inlineStr">
+        <is>
+          <t>Normandie</t>
+        </is>
+      </c>
+      <c r="H317" t="inlineStr">
+        <is>
+          <t>Négoce matériaux</t>
+        </is>
+      </c>
+      <c r="K317" t="inlineStr">
+        <is>
+          <t>Croisement fichier (26/10)</t>
+        </is>
+      </c>
+      <c r="L317" s="12" t="inlineStr">
         <is>
           <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
         </is>
       </c>
-      <c r="N303" t="inlineStr">
-        <is>
-          <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
-        </is>
-      </c>
-      <c r="O303" t="inlineStr">
-        <is>
-          <t>[26/10] Recherche vérifiée (segment normandie). Confirmé : marbrerie décorative avec showroom (visites sur rendez-vous), ZA Eco 5 n° 7 et 9, 14310 Seulline, « près de Caen en Normandie ». contact@adequatemarbrerie.fr lu TEXTUELLEMENT sur la page contact du site officiel (en texte et en lien mailto, concordants). Téléphone confirmé. Hors liste d'exclusion. Source e-mail : https://www.adequatemarbrerie.fr/contact.  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
-        </is>
-      </c>
-      <c r="P303" t="inlineStr">
-        <is>
-          <t>5e liste — recherche (26/10)</t>
-        </is>
-      </c>
-      <c r="Q303" t="inlineStr">
-        <is>
-          <t>contact@adequatemarbrerie.fr</t>
-        </is>
-      </c>
-    </row>
-    <row r="304" ht="15" customHeight="1" s="13">
-      <c r="A304" t="n">
-        <v>304</v>
-      </c>
-      <c r="B304" t="inlineStr">
+      <c r="N317" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER — vrai From info@pierredegypte.online via Network Solutions à vérifier avant tout contact</t>
+        </is>
+      </c>
+      <c r="O317" t="inlineStr">
+        <is>
+          <t>[26/10 croisement fichier propriétaire] Apporté par le fichier propriétaire du 26/10 (origine « Recherche 31 » de son côté). E-mail à re-vérifier sur site officiel avant envoi. NE RIEN ENVOYER — vrai From info@pierredegypte.online via Network Solutions à vérifier avant tout contact</t>
+        </is>
+      </c>
+      <c r="P317" t="inlineStr">
+        <is>
+          <t>5e liste — croisement (26/10)</t>
+        </is>
+      </c>
+      <c r="Q317" t="inlineStr">
+        <is>
+          <t>facomat76@wanadoo.fr</t>
+        </is>
+      </c>
+    </row>
+    <row r="318" ht="15" customHeight="1" s="13">
+      <c r="A318" t="n">
+        <v>318</v>
+      </c>
+      <c r="B318" t="inlineStr">
         <is>
           <t>Pro France</t>
         </is>
       </c>
-      <c r="C304" t="n">
+      <c r="C318" t="n">
         <v>2</v>
       </c>
-      <c r="D304" t="inlineStr">
-        <is>
-          <t>normandie</t>
-        </is>
-      </c>
-      <c r="E304" t="inlineStr">
-        <is>
-          <t>Motte Décoration</t>
-        </is>
-      </c>
-      <c r="F304" t="inlineStr">
-        <is>
-          <t>Le Pré-d'Auge (14340), 10 Chemin des Vatines — entre Cambrem</t>
-        </is>
-      </c>
-      <c r="G304" t="inlineStr">
-        <is>
-          <t>France</t>
-        </is>
-      </c>
-      <c r="H304" t="inlineStr">
-        <is>
-          <t>Confirmé via sources tierces : société MOTTE DECORATION immatriculée (SIREN 844835728, taille/façonnage/finissage de pierres) au Pré-d'Auge (14340) ; marbrerie décorative familiale…</t>
-        </is>
-      </c>
-      <c r="I304" t="inlineStr">
-        <is>
-          <t>https://www.mottedecoration.com</t>
-        </is>
-      </c>
-      <c r="J304" t="inlineStr">
-        <is>
-          <t>02 31 32 22 00</t>
-        </is>
-      </c>
-      <c r="K304" t="inlineStr">
-        <is>
-          <t>Recherche Claude (26/10)</t>
-        </is>
-      </c>
-      <c r="L304" s="12" t="inlineStr">
+      <c r="D318" t="inlineStr">
+        <is>
+          <t>Négoce pierre</t>
+        </is>
+      </c>
+      <c r="E318" t="inlineStr">
+        <is>
+          <t>MasterPierre Caen</t>
+        </is>
+      </c>
+      <c r="F318" t="inlineStr">
+        <is>
+          <t>Mondeville (14)</t>
+        </is>
+      </c>
+      <c r="G318" t="inlineStr">
+        <is>
+          <t>Normandie</t>
+        </is>
+      </c>
+      <c r="H318" t="inlineStr">
+        <is>
+          <t>Négoce pierre</t>
+        </is>
+      </c>
+      <c r="J318" t="inlineStr">
+        <is>
+          <t>02 31 52 42 77</t>
+        </is>
+      </c>
+      <c r="K318" t="inlineStr">
+        <is>
+          <t>Croisement fichier (26/10)</t>
+        </is>
+      </c>
+      <c r="L318" s="12" t="inlineStr">
         <is>
           <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
         </is>
       </c>
-      <c r="N304" t="inlineStr">
-        <is>
-          <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
-        </is>
-      </c>
-      <c r="O304" t="inlineStr">
-        <is>
-          <t>[26/10] Recherche vérifiée (segment normandie). Confirmé via sources tierces : société MOTTE DECORATION immatriculée (SIREN 844835728, taille/façonnage/finissage de pierres) au Pré-d'Auge (14340) ; marbrerie décorative familiale (marbre, granit, quartz, pierre naturelle) intervenant sur toute la Normandie — societe.com, Initiative Calvados, Pages Jaunes et index du site officiel concordants. E-mail NON confirmé textuellement : le site officiel refuse toute lecture automatisée (HTTP 401 sur l'accueil et la page contact), vérification visuelle impossible ici. L'index du moteur de recherche attribue bien contact@mottedecoration.com et le 02 31 32 22 00 au site officiel, et le téléphone est corroboré par plusieurs sources indépendantes. Retenu sur REPLI TÉLÉPHONE vérifié (02 31 32 22 00) ; ne pas utiliser l'e-mail avant confirmation visuelle sur le site. Hors liste d'exclusion. Entreprise réelle, en France, site vivant (blocage anti-robot, pas site mort). Source e-mail : aucune (pas d e-mail publié).  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
-        </is>
-      </c>
-      <c r="P304" t="inlineStr">
-        <is>
-          <t>5e liste — recherche (26/10)</t>
-        </is>
-      </c>
-      <c r="Q304" t="inlineStr">
-        <is>
-          <t>contact@mottedecoration.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="305" ht="15" customHeight="1" s="13">
-      <c r="A305" t="n">
-        <v>305</v>
-      </c>
-      <c r="B305" t="inlineStr">
-        <is>
-          <t>Pro France</t>
-        </is>
-      </c>
-      <c r="C305" t="n">
-        <v>2</v>
-      </c>
-      <c r="D305" t="inlineStr">
-        <is>
-          <t>normandie</t>
-        </is>
-      </c>
-      <c r="E305" t="inlineStr">
-        <is>
-          <t>Carreau Déco (SARL)</t>
-        </is>
-      </c>
-      <c r="F305" t="inlineStr">
-        <is>
-          <t>Évreux (27) ; autres magasins : Barentin, Tourville-la-Riviè</t>
-        </is>
-      </c>
-      <c r="G305" t="inlineStr">
-        <is>
-          <t>France</t>
-        </is>
-      </c>
-      <c r="H305" t="inlineStr">
-        <is>
-          <t>Confirmé : enseigne de carrelage (« Carrelage haut de gamme, sol et mur ») — grès cérame, dalles, faïence, intérieur/extérieur ; 6 points de vente confirmés dont Évreux, Barentin, …</t>
-        </is>
-      </c>
-      <c r="I305" t="inlineStr">
-        <is>
-          <t>https://www.carreaudeco.com</t>
-        </is>
-      </c>
-      <c r="J305" t="inlineStr">
-        <is>
-          <t>02 32 30 62 04 (Évreux) ; 02 37 21 27 80 (Lèves/standard) ; 02 78 77 51 00 (Barentin) ; 02 78 77 09 77 (Tourville) ; 02 78 93 05 05 (Montivilliers) ; 02 37 46 23 27 (Vernouillet)</t>
-        </is>
-      </c>
-      <c r="K305" t="inlineStr">
-        <is>
-          <t>Recherche Claude (26/10)</t>
-        </is>
-      </c>
-      <c r="L305" s="12" t="inlineStr">
-        <is>
-          <t>À contacter (formulaire/tél) — EN ATTENTE</t>
-        </is>
-      </c>
-      <c r="N305" t="inlineStr">
-        <is>
-          <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
-        </is>
-      </c>
-      <c r="O305" t="inlineStr">
-        <is>
-          <t>[26/10] Recherche vérifiée (segment normandie). Confirmé : enseigne de carrelage (« Carrelage haut de gamme, sol et mur ») — grès cérame, dalles, faïence, intérieur/extérieur ; 6 points de vente confirmés dont Évreux, Barentin, Tourville-la-Rivière et Montivilliers. AUCUN e-mail publié textuellement sur le site officiel (formulaire de contact uniquement) — vérifié. Retenu sur REPLI TÉLÉPHONE : les 6 numéros de magasins sont confirmés sur le site officiel, dont Évreux 02 32 30 62 04 et le standard de Lèves 02 37 21 27 80. Hors liste d'exclusion. Source e-mail : aucune (pas d e-mail publié).  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
-        </is>
-      </c>
-      <c r="P305" t="inlineStr">
-        <is>
-          <t>5e liste — recherche (26/10)</t>
-        </is>
-      </c>
-    </row>
-    <row r="306" ht="15" customHeight="1" s="13">
-      <c r="A306" t="n">
-        <v>306</v>
-      </c>
-      <c r="B306" t="inlineStr">
-        <is>
-          <t>Pro France</t>
-        </is>
-      </c>
-      <c r="C306" t="n">
-        <v>2</v>
-      </c>
-      <c r="D306" t="inlineStr">
-        <is>
-          <t>normandie</t>
-        </is>
-      </c>
-      <c r="E306" t="inlineStr">
-        <is>
-          <t>Carré &amp; Déco (SAS Fortin Design)</t>
-        </is>
-      </c>
-      <c r="F306" t="inlineStr">
-        <is>
-          <t>Colombelles (14460), 6 rue de la Métallurgie — agglomération</t>
-        </is>
-      </c>
-      <c r="G306" t="inlineStr">
-        <is>
-          <t>France</t>
-        </is>
-      </c>
-      <c r="H306" t="inlineStr">
-        <is>
-          <t>Confirmé : magasin de carrelage et céramique avec showroom (« votre expert en carrelage et céramique à proximité de Caen »), pierre naturelle présente en gamme extérieure (activité…</t>
-        </is>
-      </c>
-      <c r="I306" t="inlineStr">
-        <is>
-          <t>https://carre-deco.fr</t>
-        </is>
-      </c>
-      <c r="J306" t="inlineStr">
-        <is>
-          <t>02 31 34 40 50</t>
-        </is>
-      </c>
-      <c r="K306" t="inlineStr">
-        <is>
-          <t>Recherche Claude (26/10)</t>
-        </is>
-      </c>
-      <c r="L306" s="12" t="inlineStr">
-        <is>
-          <t>À contacter (formulaire/tél) — EN ATTENTE</t>
-        </is>
-      </c>
-      <c r="N306" t="inlineStr">
-        <is>
-          <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
-        </is>
-      </c>
-      <c r="O306" t="inlineStr">
-        <is>
-          <t>[26/10] Recherche vérifiée (segment normandie). Confirmé : magasin de carrelage et céramique avec showroom (« votre expert en carrelage et céramique à proximité de Caen »), pierre naturelle présente en gamme extérieure (activité secondaire). AUCUN e-mail publié textuellement sur le site officiel (formulaire uniquement) — vérifié. Retenu sur REPLI TÉLÉPHONE : 02 31 34 40 50 confirmé sur le site officiel, adresse Colombelles confirmée. Nuance : la pierre naturelle n'est pas son cœur de métier (carrelage/céramique d'abord). Hors liste d'exclusion. Source e-mail : aucune (pas d e-mail publié).  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
-        </is>
-      </c>
-      <c r="P306" t="inlineStr">
-        <is>
-          <t>5e liste — recherche (26/10)</t>
-        </is>
-      </c>
-    </row>
-    <row r="307" ht="15" customHeight="1" s="13">
-      <c r="A307" t="n">
-        <v>307</v>
-      </c>
-      <c r="B307" t="inlineStr">
-        <is>
-          <t>Pro France</t>
-        </is>
-      </c>
-      <c r="C307" t="n">
-        <v>2</v>
-      </c>
-      <c r="D307" t="inlineStr">
-        <is>
-          <t>destockage-exterieur</t>
-        </is>
-      </c>
-      <c r="E307" t="inlineStr">
-        <is>
-          <t>Vallois (groupe Spie batignolles paysage) — agence Val de Seine</t>
-        </is>
-      </c>
-      <c r="F307" t="inlineStr">
-        <is>
-          <t>Val-de-Reuil (27100, Z.A la Comminière) — agence IDF à Trapp</t>
-        </is>
-      </c>
-      <c r="G307" t="inlineStr">
-        <is>
-          <t>France</t>
-        </is>
-      </c>
-      <c r="H307" t="inlineStr">
-        <is>
-          <t>Confirmée : « aménagements paysagers » dans le Grand Ouest, société de Spie batignolles paysage (vérifié sur la page d'accueil) ; la page contact confirme l'agence Val de Seine à V…</t>
-        </is>
-      </c>
-      <c r="I307" t="inlineStr">
-        <is>
-          <t>https://www.vallois.eu/</t>
-        </is>
-      </c>
-      <c r="J307" t="inlineStr">
-        <is>
-          <t>02 32 40 32 30 (Val de Seine) ; 01 30 16 07 00 (IDF Trappes)</t>
-        </is>
-      </c>
-      <c r="K307" t="inlineStr">
-        <is>
-          <t>Recherche Claude (26/10)</t>
-        </is>
-      </c>
-      <c r="L307" s="12" t="inlineStr">
-        <is>
-          <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
-        </is>
-      </c>
-      <c r="N307" t="inlineStr">
-        <is>
-          <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
-        </is>
-      </c>
-      <c r="O307" t="inlineStr">
-        <is>
-          <t>[26/10] Recherche vérifiée (segment destockage-exterieur). Confirmée : « aménagements paysagers » dans le Grand Ouest, société de Spie batignolles paysage (vérifié sur la page d'accueil) ; la page contact confirme l'agence Val de Seine à Val-de-Reuil 27100 et l'agence IDF à Trappes 78190. E-mail lu textuellement dans la fiche « Agence Val de Seine » de la page contact ; les deux téléphones y figurent aussi textuellement. Précision : la page contact donne comme siège social de Spie batignolles paysage Nanterre (92) et comme siège administratif St Hymer (14) ; Mirville (76210) est l'adresse de l'agence de l'Estuaire, pas du siège. Hors liste d'exclusion. Candidat solide. Source e-mail : https://www.vallois.eu/contact.  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
-        </is>
-      </c>
-      <c r="P307" t="inlineStr">
-        <is>
-          <t>5e liste — recherche (26/10)</t>
-        </is>
-      </c>
-      <c r="Q307" t="inlineStr">
-        <is>
-          <t>agence-valdeseine@vallois.eu</t>
-        </is>
-      </c>
-    </row>
-    <row r="308" ht="15" customHeight="1" s="13">
-      <c r="A308" t="n">
-        <v>308</v>
-      </c>
-      <c r="B308" t="inlineStr">
-        <is>
-          <t>Pro France</t>
-        </is>
-      </c>
-      <c r="C308" t="n">
-        <v>1</v>
-      </c>
-      <c r="D308" t="inlineStr">
-        <is>
-          <t>destockage-exterieur</t>
-        </is>
-      </c>
-      <c r="E308" t="inlineStr">
-        <is>
-          <t>Tricycle Environnement / Bâticycle</t>
-        </is>
-      </c>
-      <c r="F308" t="inlineStr">
-        <is>
-          <t>Gennevilliers (120 rue du Moulin de Cage, 92230)</t>
-        </is>
-      </c>
-      <c r="G308" t="inlineStr">
-        <is>
-          <t>France</t>
-        </is>
-      </c>
-      <c r="H308" t="inlineStr">
-        <is>
-          <t>Confirmée : « Matériaux BTP d'occasion », « Réemploi de matériaux de second œuvre », « Curage de bâtiment » — réemploi/revente de matériaux de construction, vérifié sur le site off…</t>
-        </is>
-      </c>
-      <c r="I308" t="inlineStr">
-        <is>
-          <t>https://www.tricycle-environnement.fr/</t>
-        </is>
-      </c>
-      <c r="J308" t="inlineStr">
-        <is>
-          <t>07 60 62 41 36</t>
-        </is>
-      </c>
-      <c r="K308" t="inlineStr">
-        <is>
-          <t>Recherche Claude (26/10)</t>
-        </is>
-      </c>
-      <c r="L308" s="12" t="inlineStr">
-        <is>
-          <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
-        </is>
-      </c>
-      <c r="N308" t="inlineStr">
-        <is>
-          <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
-        </is>
-      </c>
-      <c r="O308" t="inlineStr">
-        <is>
-          <t>[26/10] Recherche vérifiée (segment destockage-exterieur). Confirmée : « Matériaux BTP d'occasion », « Réemploi de matériaux de second œuvre », « Curage de bâtiment » — réemploi/revente de matériaux de construction, vérifié sur le site officiel. E-mail lu textuellement en en-tête ET en pied de page ; téléphone confirmé sous deux formats (+33 7 60 62 41 36 / 07 60 62 41 36) ; adresse 120 rue du Moulin de Cage, 92230 Gennevilliers confirmée en pied de page — la ville même du stock. Hors liste d'exclusion. Candidat solide. Source e-mail : https://www.tricycle-environnement.fr/.  📍 Même ville que le dépôt (Gennevilliers) — réemploi : bon candidat reprise de lot. NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
-        </is>
-      </c>
-      <c r="P308" t="inlineStr">
-        <is>
-          <t>5e liste — recherche (26/10)</t>
-        </is>
-      </c>
-      <c r="Q308" t="inlineStr">
-        <is>
-          <t>contact@tri-cycle.fr</t>
-        </is>
-      </c>
-    </row>
-    <row r="309" ht="15" customHeight="1" s="13">
-      <c r="A309" t="n">
-        <v>309</v>
-      </c>
-      <c r="B309" t="inlineStr">
-        <is>
-          <t>Pro France</t>
-        </is>
-      </c>
-      <c r="C309" t="n">
-        <v>2</v>
-      </c>
-      <c r="D309" t="inlineStr">
-        <is>
-          <t>destockage-exterieur</t>
-        </is>
-      </c>
-      <c r="E309" t="inlineStr">
-        <is>
-          <t>Minéka</t>
-        </is>
-      </c>
-      <c r="F309" t="inlineStr">
-        <is>
-          <t>Villeurbanne (182 rue de la Poudrette, 69100)</t>
-        </is>
-      </c>
-      <c r="G309" t="inlineStr">
-        <is>
-          <t>France</t>
-        </is>
-      </c>
-      <c r="H309" t="inlineStr">
-        <is>
-          <t>Confirmée : adresse « 182 rue de la Poudrette 69100 VILLEURBANNE » vérifiée dans les mentions légales, qui mentionnent aussi le magasin « Minéstock » (« Venez nous voir au Minéstoc…</t>
-        </is>
-      </c>
-      <c r="I309" t="inlineStr">
-        <is>
-          <t>https://mineka.fr/</t>
-        </is>
-      </c>
-      <c r="K309" t="inlineStr">
-        <is>
-          <t>Recherche Claude (26/10)</t>
-        </is>
-      </c>
-      <c r="L309" s="12" t="inlineStr">
-        <is>
-          <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
-        </is>
-      </c>
-      <c r="N309" t="inlineStr">
-        <is>
-          <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
-        </is>
-      </c>
-      <c r="O309" t="inlineStr">
-        <is>
-          <t>[26/10] Recherche vérifiée (segment destockage-exterieur). Confirmée : adresse « 182 rue de la Poudrette 69100 VILLEURBANNE » vérifiée dans les mentions légales, qui mentionnent aussi le magasin « Minéstock » (« Venez nous voir au Minéstock ») — structure de collecte/revente avec point de vente physique, pas une pure marketplace. E-mail lu textuellement dans les mentions légales (« Adresse électronique : contact@mineka.fr »), seule adresse de la page. AUCUN téléphone publié : le contact ne pourra se faire que par e-mail (vérifié). En France (Lyon/Villeurbanne) ; limite logistique : loin des stocks de Vernon/Gennevilliers, retrait à organiser. Hors liste d'exclusion. Source e-mail : https://mineka.fr/mentions-legales/.  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
-        </is>
-      </c>
-      <c r="P309" t="inlineStr">
-        <is>
-          <t>5e liste — recherche (26/10)</t>
-        </is>
-      </c>
-      <c r="Q309" t="inlineStr">
-        <is>
-          <t>contact@mineka.fr</t>
-        </is>
-      </c>
-    </row>
-    <row r="310" ht="15" customHeight="1" s="13">
-      <c r="A310" t="n">
-        <v>310</v>
-      </c>
-      <c r="B310" t="inlineStr">
-        <is>
-          <t>Pro France</t>
-        </is>
-      </c>
-      <c r="C310" t="n">
-        <v>2</v>
-      </c>
-      <c r="D310" t="inlineStr">
-        <is>
-          <t>destockage-exterieur</t>
-        </is>
-      </c>
-      <c r="E310" t="inlineStr">
-        <is>
-          <t>Pinson Paysage (groupe Osmaïa)</t>
-        </is>
-      </c>
-      <c r="F310" t="inlineStr">
-        <is>
-          <t>Andilly (13 avenue des Cures, 95580)</t>
-        </is>
-      </c>
-      <c r="G310" t="inlineStr">
-        <is>
-          <t>France</t>
-        </is>
-      </c>
-      <c r="H310" t="inlineStr">
-        <is>
-          <t>Confirmée : page « Nous contacter » vérifiée — siège « 13 Avenue des Cures, 95580 Andilly » ; activités « Création », « Entretien » (espaces verts) et « Génie écologique » affichée…</t>
-        </is>
-      </c>
-      <c r="I310" t="inlineStr">
-        <is>
-          <t>https://www.pinson-paysage.com/</t>
-        </is>
-      </c>
-      <c r="K310" t="inlineStr">
-        <is>
-          <t>Recherche Claude (26/10)</t>
-        </is>
-      </c>
-      <c r="L310" s="12" t="inlineStr">
-        <is>
-          <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
-        </is>
-      </c>
-      <c r="N310" t="inlineStr">
-        <is>
-          <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
-        </is>
-      </c>
-      <c r="O310" t="inlineStr">
-        <is>
-          <t>[26/10] Recherche vérifiée (segment destockage-exterieur). Confirmée : page « Nous contacter » vérifiée — siège « 13 Avenue des Cures, 95580 Andilly » ; activités « Création », « Entretien » (espaces verts) et « Génie écologique » affichées, cohérentes avec une entreprise paysagère IDF. E-mail lu textuellement (seule adresse de la page). AUCUN téléphone sur la page contact (formulaire uniquement) : contact par e-mail vérifié. Réserve maintenue : le site met en avant le végétal/génie écologique plus que la maçonnerie minérale — pertinence segment (b) à pondérer. Hors liste d'exclusion. Source e-mail : https://www.pinson-paysage.com/nous-contacter/.  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
-        </is>
-      </c>
-      <c r="P310" t="inlineStr">
-        <is>
-          <t>5e liste — recherche (26/10)</t>
-        </is>
-      </c>
-      <c r="Q310" t="inlineStr">
-        <is>
-          <t>pinson@pinson-paysage.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="311" ht="15" customHeight="1" s="13">
-      <c r="A311" t="n">
-        <v>311</v>
-      </c>
-      <c r="B311" t="inlineStr">
-        <is>
-          <t>Pro France</t>
-        </is>
-      </c>
-      <c r="C311" t="n">
-        <v>1</v>
-      </c>
-      <c r="D311" t="inlineStr">
-        <is>
-          <t>destockage-exterieur</t>
-        </is>
-      </c>
-      <c r="E311" t="inlineStr">
-        <is>
-          <t>NOZ (centrale d'achat S.F.N.)</t>
-        </is>
-      </c>
-      <c r="F311" t="inlineStr">
-        <is>
-          <t>Saint-Berthevin (53940)</t>
-        </is>
-      </c>
-      <c r="G311" t="inlineStr">
-        <is>
-          <t>France</t>
-        </is>
-      </c>
-      <c r="H311" t="inlineStr">
-        <is>
-          <t>Confirmée : page contact vérifiée — adresse « 53940 Saint-Berthevin – France », formulaire avec champ « Vous êtes ? » incluant « Je suis un fournisseur » et objet « Besoin de désto…</t>
-        </is>
-      </c>
-      <c r="I311" t="inlineStr">
-        <is>
-          <t>https://www.noz.fr/</t>
-        </is>
-      </c>
-      <c r="J311" t="inlineStr">
-        <is>
-          <t>02 43 01 53 54</t>
-        </is>
-      </c>
-      <c r="K311" t="inlineStr">
-        <is>
-          <t>Recherche Claude (26/10)</t>
-        </is>
-      </c>
-      <c r="L311" s="12" t="inlineStr">
-        <is>
-          <t>À contacter (formulaire/tél) — EN ATTENTE</t>
-        </is>
-      </c>
-      <c r="N311" t="inlineStr">
-        <is>
-          <t>NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
-        </is>
-      </c>
-      <c r="O311" t="inlineStr">
-        <is>
-          <t>[26/10] Recherche vérifiée (segment destockage-exterieur). Confirmée : page contact vérifiée — adresse « 53940 Saint-Berthevin – France », formulaire avec champ « Vous êtes ? » incluant « Je suis un fournisseur » et objet « Besoin de déstockage », cohérent avec l'activité de rachat de surstocks/lots. RETENU SANS E-MAIL : aucun e-mail publié sur https://www.noz.fr/contactez-nous/ (revérifié le 26/10/2026 — le seul mot « Email » est un champ de formulaire), mais le téléphone 02 43 01 53 54 y est écrit textuellement et vérifié ; contact via ce numéro ou le formulaire fournisseur « Besoin de déstockage ». Hors liste d'exclusion. Réserve : lot minéral lourd atypique dans leur mix. Source e-mail : aucune (pas d e-mail publié).  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi</t>
-        </is>
-      </c>
-      <c r="P311" t="inlineStr">
-        <is>
-          <t>5e liste — recherche (26/10)</t>
-        </is>
-      </c>
-    </row>
-    <row r="312" ht="15" customHeight="1" s="13">
-      <c r="L312" s="12" t="n"/>
-    </row>
-    <row r="313" ht="15" customHeight="1" s="13">
-      <c r="L313" s="12" t="n"/>
-    </row>
-    <row r="314" ht="15" customHeight="1" s="13">
-      <c r="L314" s="12" t="n"/>
-    </row>
-    <row r="315" ht="15" customHeight="1" s="13">
-      <c r="L315" s="12" t="n"/>
-    </row>
-    <row r="316" ht="15" customHeight="1" s="13">
-      <c r="L316" s="12" t="n"/>
-    </row>
-    <row r="317" ht="15" customHeight="1" s="13">
-      <c r="L317" s="12" t="n"/>
-    </row>
-    <row r="318" ht="15" customHeight="1" s="13">
-      <c r="L318" s="12" t="n"/>
+      <c r="N318" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER — vrai From info@pierredegypte.online via Network Solutions à vérifier avant tout contact</t>
+        </is>
+      </c>
+      <c r="O318" t="inlineStr">
+        <is>
+          <t>[26/10 croisement fichier propriétaire] Apporté par le fichier propriétaire du 26/10 (origine « Recherche 31 » de son côté). E-mail à re-vérifier sur site officiel avant envoi. ⚠️ Domaine masterpierre.com déjà croisé dans nos sources : vérifier l'historique avant envoi. NE RIEN ENVOYER — vrai From info@pierredegypte.online via Network Solutions à vérifier avant tout contact</t>
+        </is>
+      </c>
+      <c r="P318" t="inlineStr">
+        <is>
+          <t>5e liste — croisement (26/10)</t>
+        </is>
+      </c>
+      <c r="Q318" t="inlineStr">
+        <is>
+          <t>caen@masterpierre.com</t>
+        </is>
+      </c>
     </row>
     <row r="319" ht="15" customHeight="1" s="13">
       <c r="L319" s="12" t="n"/>

</xml_diff>

<commit_message>
Dalle Décor : angle « Revendeurs à 35 € » (relevé 26/10 soir)
Importateur depuis 1972, ~30 min de Gennevilliers, achète en lot.
Jamais contacté — verrou d'envoi inchangé.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xqm9tFtdvLdJdkiWw2VVp6
</commit_message>
<xml_diff>
--- a/minyala/clients-potentiels.xlsx
+++ b/minyala/clients-potentiels.xlsx
@@ -6384,7 +6384,7 @@
           <t>2e liste (12/10)</t>
         </is>
       </c>
-      <c r="Q71" t="inlineStr">
+      <c r="Q71" s="12" t="inlineStr">
         <is>
           <t>contact@la-roche-taillee.fr</t>
         </is>
@@ -19234,7 +19234,7 @@
       </c>
       <c r="O271" s="12" t="inlineStr">
         <is>
-          <t>[26/10] Relais assistant tiers du 26/10 (dédupliqué Gmail/Contacts) — e-mail « vérifié » par le relais, à re-confirmer sur site officiel avant envoi. Pas d'e-mail publié : téléphone. NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi</t>
+          <t>[26/10] Relais assistant tiers du 26/10 (dédupliqué Gmail/Contacts) — e-mail « vérifié » par le relais, à re-confirmer sur site officiel avant envoi. Pas d'e-mail publié : téléphone. NE RIEN ENVOYER (ordre du 26/10) — vérifier d'abord l'expéditeur réel info@pierredegypte.online (Network Solutions), puis re-vérifier l'e-mail sur le site officiel avant tout envoi [26/10 relevé revendeurs] Angle revendeur confirmé : importateur de pierre depuis 1972, à ~30 min du stock de Gennevilliers, achète en lot — cible « Revendeurs à 35 € » (revente au détail plus chère). Jamais contacté.</t>
         </is>
       </c>
       <c r="P271" s="12" t="inlineStr">
@@ -20357,7 +20357,7 @@
           <t>5e liste — recherche (26/10)</t>
         </is>
       </c>
-      <c r="Q286" t="inlineStr">
+      <c r="Q286" s="12" t="inlineStr">
         <is>
           <t>contactgnps26@gmail.com</t>
         </is>
@@ -20815,7 +20815,7 @@
           <t>5e liste — recherche (26/10)</t>
         </is>
       </c>
-      <c r="Q292" t="inlineStr">
+      <c r="Q292" s="12" t="inlineStr">
         <is>
           <t>contact@marbre-import.fr</t>
         </is>
@@ -22091,7 +22091,7 @@
           <t>https://mineka.fr/</t>
         </is>
       </c>
-      <c r="J309" t="inlineStr">
+      <c r="J309" s="12" t="inlineStr">
         <is>
           <t>04 78 52 86 28</t>
         </is>
@@ -22169,7 +22169,7 @@
           <t>https://www.pinson-paysage.com/</t>
         </is>
       </c>
-      <c r="J310" t="inlineStr">
+      <c r="J310" s="12" t="inlineStr">
         <is>
           <t>01 34 16 61 01</t>
         </is>
@@ -22277,55 +22277,55 @@
           <t>5e liste — recherche (26/10)</t>
         </is>
       </c>
-      <c r="Q311" t="inlineStr">
+      <c r="Q311" s="12" t="inlineStr">
         <is>
           <t>noz@noz.fr</t>
         </is>
       </c>
     </row>
     <row r="312" ht="15" customHeight="1" s="13">
-      <c r="A312" t="n">
+      <c r="A312" s="12" t="n">
         <v>312</v>
       </c>
-      <c r="B312" t="inlineStr">
+      <c r="B312" s="12" t="inlineStr">
         <is>
           <t>Pro France</t>
         </is>
       </c>
-      <c r="C312" t="n">
+      <c r="C312" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="D312" t="inlineStr">
+      <c r="D312" s="12" t="inlineStr">
         <is>
           <t>Marbrerie / pierre</t>
         </is>
       </c>
-      <c r="E312" t="inlineStr">
+      <c r="E312" s="12" t="inlineStr">
         <is>
           <t>ILDEI</t>
         </is>
       </c>
-      <c r="F312" t="inlineStr">
+      <c r="F312" s="12" t="inlineStr">
         <is>
           <t>Le Plessis-Pâté (91)</t>
         </is>
       </c>
-      <c r="G312" t="inlineStr">
+      <c r="G312" s="12" t="inlineStr">
         <is>
           <t>Île-de-France</t>
         </is>
       </c>
-      <c r="H312" t="inlineStr">
+      <c r="H312" s="12" t="inlineStr">
         <is>
           <t>Marbrerie / pierre</t>
         </is>
       </c>
-      <c r="J312" t="inlineStr">
+      <c r="J312" s="12" t="inlineStr">
         <is>
           <t>01 60 84 11 00</t>
         </is>
       </c>
-      <c r="K312" t="inlineStr">
+      <c r="K312" s="12" t="inlineStr">
         <is>
           <t>Croisement fichier (26/10)</t>
         </is>
@@ -22335,70 +22335,70 @@
           <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
         </is>
       </c>
-      <c r="N312" t="inlineStr">
+      <c r="N312" s="12" t="inlineStr">
         <is>
           <t>NE RIEN ENVOYER — vrai From info@pierredegypte.online via Network Solutions à vérifier avant tout contact</t>
         </is>
       </c>
-      <c r="O312" t="inlineStr">
+      <c r="O312" s="12" t="inlineStr">
         <is>
           <t>[26/10 croisement fichier propriétaire] Apporté par le fichier propriétaire du 26/10 (origine « Recherche 31 » de son côté). E-mail à re-vérifier sur site officiel avant envoi. NE RIEN ENVOYER — vrai From info@pierredegypte.online via Network Solutions à vérifier avant tout contact</t>
         </is>
       </c>
-      <c r="P312" t="inlineStr">
+      <c r="P312" s="12" t="inlineStr">
         <is>
           <t>5e liste — croisement (26/10)</t>
         </is>
       </c>
-      <c r="Q312" t="inlineStr">
+      <c r="Q312" s="12" t="inlineStr">
         <is>
           <t>contact@ildei.com</t>
         </is>
       </c>
     </row>
     <row r="313" ht="15" customHeight="1" s="13">
-      <c r="A313" t="n">
+      <c r="A313" s="12" t="n">
         <v>313</v>
       </c>
-      <c r="B313" t="inlineStr">
+      <c r="B313" s="12" t="inlineStr">
         <is>
           <t>Pro France</t>
         </is>
       </c>
-      <c r="C313" t="n">
+      <c r="C313" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="D313" t="inlineStr">
+      <c r="D313" s="12" t="inlineStr">
         <is>
           <t>Marbrerie</t>
         </is>
       </c>
-      <c r="E313" t="inlineStr">
+      <c r="E313" s="12" t="inlineStr">
         <is>
           <t>La Marbrerie Contemporaine</t>
         </is>
       </c>
-      <c r="F313" t="inlineStr">
+      <c r="F313" s="12" t="inlineStr">
         <is>
           <t>Bagnolet (93)</t>
         </is>
       </c>
-      <c r="G313" t="inlineStr">
+      <c r="G313" s="12" t="inlineStr">
         <is>
           <t>Île-de-France</t>
         </is>
       </c>
-      <c r="H313" t="inlineStr">
+      <c r="H313" s="12" t="inlineStr">
         <is>
           <t>Marbrerie</t>
         </is>
       </c>
-      <c r="J313" t="inlineStr">
+      <c r="J313" s="12" t="inlineStr">
         <is>
           <t>01 48 97 00 13</t>
         </is>
       </c>
-      <c r="K313" t="inlineStr">
+      <c r="K313" s="12" t="inlineStr">
         <is>
           <t>Croisement fichier (26/10)</t>
         </is>
@@ -22408,70 +22408,70 @@
           <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
         </is>
       </c>
-      <c r="N313" t="inlineStr">
+      <c r="N313" s="12" t="inlineStr">
         <is>
           <t>NE RIEN ENVOYER — vrai From info@pierredegypte.online via Network Solutions à vérifier avant tout contact</t>
         </is>
       </c>
-      <c r="O313" t="inlineStr">
+      <c r="O313" s="12" t="inlineStr">
         <is>
           <t>[26/10 croisement fichier propriétaire] Apporté par le fichier propriétaire du 26/10 (origine « Recherche 31 » de son côté). E-mail à re-vérifier sur site officiel avant envoi. NE RIEN ENVOYER — vrai From info@pierredegypte.online via Network Solutions à vérifier avant tout contact</t>
         </is>
       </c>
-      <c r="P313" t="inlineStr">
+      <c r="P313" s="12" t="inlineStr">
         <is>
           <t>5e liste — croisement (26/10)</t>
         </is>
       </c>
-      <c r="Q313" t="inlineStr">
+      <c r="Q313" s="12" t="inlineStr">
         <is>
           <t>contact@la-marbrerie-contemporaine.fr</t>
         </is>
       </c>
     </row>
     <row r="314" ht="15" customHeight="1" s="13">
-      <c r="A314" t="n">
+      <c r="A314" s="12" t="n">
         <v>314</v>
       </c>
-      <c r="B314" t="inlineStr">
+      <c r="B314" s="12" t="inlineStr">
         <is>
           <t>Pro France</t>
         </is>
       </c>
-      <c r="C314" t="n">
+      <c r="C314" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="D314" t="inlineStr">
+      <c r="D314" s="12" t="inlineStr">
         <is>
           <t>Marbrerie / négoce pierre</t>
         </is>
       </c>
-      <c r="E314" t="inlineStr">
+      <c r="E314" s="12" t="inlineStr">
         <is>
           <t>Paris Roches</t>
         </is>
       </c>
-      <c r="F314" t="inlineStr">
+      <c r="F314" s="12" t="inlineStr">
         <is>
           <t>Vitry-sur-Seine (94)</t>
         </is>
       </c>
-      <c r="G314" t="inlineStr">
+      <c r="G314" s="12" t="inlineStr">
         <is>
           <t>Île-de-France</t>
         </is>
       </c>
-      <c r="H314" t="inlineStr">
+      <c r="H314" s="12" t="inlineStr">
         <is>
           <t>Marbrerie / négoce pierre</t>
         </is>
       </c>
-      <c r="J314" t="inlineStr">
+      <c r="J314" s="12" t="inlineStr">
         <is>
           <t>01 47 26 00 99</t>
         </is>
       </c>
-      <c r="K314" t="inlineStr">
+      <c r="K314" s="12" t="inlineStr">
         <is>
           <t>Croisement fichier (26/10)</t>
         </is>
@@ -22481,70 +22481,70 @@
           <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
         </is>
       </c>
-      <c r="N314" t="inlineStr">
+      <c r="N314" s="12" t="inlineStr">
         <is>
           <t>NE RIEN ENVOYER — vrai From info@pierredegypte.online via Network Solutions à vérifier avant tout contact</t>
         </is>
       </c>
-      <c r="O314" t="inlineStr">
+      <c r="O314" s="12" t="inlineStr">
         <is>
           <t>[26/10 croisement fichier propriétaire] Apporté par le fichier propriétaire du 26/10 (origine « Recherche 31 » de son côté). E-mail à re-vérifier sur site officiel avant envoi. NE RIEN ENVOYER — vrai From info@pierredegypte.online via Network Solutions à vérifier avant tout contact</t>
         </is>
       </c>
-      <c r="P314" t="inlineStr">
+      <c r="P314" s="12" t="inlineStr">
         <is>
           <t>5e liste — croisement (26/10)</t>
         </is>
       </c>
-      <c r="Q314" t="inlineStr">
+      <c r="Q314" s="12" t="inlineStr">
         <is>
           <t>paris-roches@orange.fr</t>
         </is>
       </c>
     </row>
     <row r="315" ht="15" customHeight="1" s="13">
-      <c r="A315" t="n">
+      <c r="A315" s="12" t="n">
         <v>315</v>
       </c>
-      <c r="B315" t="inlineStr">
+      <c r="B315" s="12" t="inlineStr">
         <is>
           <t>Pro France</t>
         </is>
       </c>
-      <c r="C315" t="n">
+      <c r="C315" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="D315" t="inlineStr">
+      <c r="D315" s="12" t="inlineStr">
         <is>
           <t>Marbrerie</t>
         </is>
       </c>
-      <c r="E315" t="inlineStr">
+      <c r="E315" s="12" t="inlineStr">
         <is>
           <t>Alpha Marbre</t>
         </is>
       </c>
-      <c r="F315" t="inlineStr">
+      <c r="F315" s="12" t="inlineStr">
         <is>
           <t>Coubert (77)</t>
         </is>
       </c>
-      <c r="G315" t="inlineStr">
+      <c r="G315" s="12" t="inlineStr">
         <is>
           <t>Île-de-France</t>
         </is>
       </c>
-      <c r="H315" t="inlineStr">
+      <c r="H315" s="12" t="inlineStr">
         <is>
           <t>Marbrerie</t>
         </is>
       </c>
-      <c r="J315" t="inlineStr">
+      <c r="J315" s="12" t="inlineStr">
         <is>
           <t>01 64 16 03 69</t>
         </is>
       </c>
-      <c r="K315" t="inlineStr">
+      <c r="K315" s="12" t="inlineStr">
         <is>
           <t>Croisement fichier (26/10)</t>
         </is>
@@ -22554,70 +22554,70 @@
           <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
         </is>
       </c>
-      <c r="N315" t="inlineStr">
+      <c r="N315" s="12" t="inlineStr">
         <is>
           <t>NE RIEN ENVOYER — vrai From info@pierredegypte.online via Network Solutions à vérifier avant tout contact</t>
         </is>
       </c>
-      <c r="O315" t="inlineStr">
+      <c r="O315" s="12" t="inlineStr">
         <is>
           <t>[26/10 croisement fichier propriétaire] Apporté par le fichier propriétaire du 26/10 (origine « Recherche 31 » de son côté). E-mail à re-vérifier sur site officiel avant envoi. NE RIEN ENVOYER — vrai From info@pierredegypte.online via Network Solutions à vérifier avant tout contact</t>
         </is>
       </c>
-      <c r="P315" t="inlineStr">
+      <c r="P315" s="12" t="inlineStr">
         <is>
           <t>5e liste — croisement (26/10)</t>
         </is>
       </c>
-      <c r="Q315" t="inlineStr">
+      <c r="Q315" s="12" t="inlineStr">
         <is>
           <t>alpha.marbre@laposte.net</t>
         </is>
       </c>
     </row>
     <row r="316" ht="15" customHeight="1" s="13">
-      <c r="A316" t="n">
+      <c r="A316" s="12" t="n">
         <v>316</v>
       </c>
-      <c r="B316" t="inlineStr">
+      <c r="B316" s="12" t="inlineStr">
         <is>
           <t>Pro France</t>
         </is>
       </c>
-      <c r="C316" t="n">
+      <c r="C316" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="D316" t="inlineStr">
+      <c r="D316" s="12" t="inlineStr">
         <is>
           <t>Marbrerie</t>
         </is>
       </c>
-      <c r="E316" t="inlineStr">
+      <c r="E316" s="12" t="inlineStr">
         <is>
           <t>Marbrerie Christian Caudron</t>
         </is>
       </c>
-      <c r="F316" t="inlineStr">
+      <c r="F316" s="12" t="inlineStr">
         <is>
           <t>Noisy-le-Sec (93)</t>
         </is>
       </c>
-      <c r="G316" t="inlineStr">
+      <c r="G316" s="12" t="inlineStr">
         <is>
           <t>Île-de-France</t>
         </is>
       </c>
-      <c r="H316" t="inlineStr">
+      <c r="H316" s="12" t="inlineStr">
         <is>
           <t>Marbrerie</t>
         </is>
       </c>
-      <c r="J316" t="inlineStr">
+      <c r="J316" s="12" t="inlineStr">
         <is>
           <t>06 30 60 75 01</t>
         </is>
       </c>
-      <c r="K316" t="inlineStr">
+      <c r="K316" s="12" t="inlineStr">
         <is>
           <t>Croisement fichier (26/10)</t>
         </is>
@@ -22627,65 +22627,65 @@
           <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
         </is>
       </c>
-      <c r="N316" t="inlineStr">
+      <c r="N316" s="12" t="inlineStr">
         <is>
           <t>NE RIEN ENVOYER — vrai From info@pierredegypte.online via Network Solutions à vérifier avant tout contact</t>
         </is>
       </c>
-      <c r="O316" t="inlineStr">
+      <c r="O316" s="12" t="inlineStr">
         <is>
           <t>[26/10 croisement fichier propriétaire] Apporté par le fichier propriétaire du 26/10 (origine « Recherche 31 » de son côté). E-mail à re-vérifier sur site officiel avant envoi. NE RIEN ENVOYER — vrai From info@pierredegypte.online via Network Solutions à vérifier avant tout contact</t>
         </is>
       </c>
-      <c r="P316" t="inlineStr">
+      <c r="P316" s="12" t="inlineStr">
         <is>
           <t>5e liste — croisement (26/10)</t>
         </is>
       </c>
-      <c r="Q316" t="inlineStr">
+      <c r="Q316" s="12" t="inlineStr">
         <is>
           <t>atelier-marbre@orange.fr</t>
         </is>
       </c>
     </row>
     <row r="317" ht="15" customHeight="1" s="13">
-      <c r="A317" t="n">
+      <c r="A317" s="12" t="n">
         <v>317</v>
       </c>
-      <c r="B317" t="inlineStr">
+      <c r="B317" s="12" t="inlineStr">
         <is>
           <t>Pro France</t>
         </is>
       </c>
-      <c r="C317" t="n">
+      <c r="C317" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="D317" t="inlineStr">
+      <c r="D317" s="12" t="inlineStr">
         <is>
           <t>Négoce matériaux</t>
         </is>
       </c>
-      <c r="E317" t="inlineStr">
+      <c r="E317" s="12" t="inlineStr">
         <is>
           <t>Facomat</t>
         </is>
       </c>
-      <c r="F317" t="inlineStr">
+      <c r="F317" s="12" t="inlineStr">
         <is>
           <t>Buchy (76)</t>
         </is>
       </c>
-      <c r="G317" t="inlineStr">
+      <c r="G317" s="12" t="inlineStr">
         <is>
           <t>Normandie</t>
         </is>
       </c>
-      <c r="H317" t="inlineStr">
+      <c r="H317" s="12" t="inlineStr">
         <is>
           <t>Négoce matériaux</t>
         </is>
       </c>
-      <c r="K317" t="inlineStr">
+      <c r="K317" s="12" t="inlineStr">
         <is>
           <t>Croisement fichier (26/10)</t>
         </is>
@@ -22695,70 +22695,70 @@
           <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
         </is>
       </c>
-      <c r="N317" t="inlineStr">
+      <c r="N317" s="12" t="inlineStr">
         <is>
           <t>NE RIEN ENVOYER — vrai From info@pierredegypte.online via Network Solutions à vérifier avant tout contact</t>
         </is>
       </c>
-      <c r="O317" t="inlineStr">
+      <c r="O317" s="12" t="inlineStr">
         <is>
           <t>[26/10 croisement fichier propriétaire] Apporté par le fichier propriétaire du 26/10 (origine « Recherche 31 » de son côté). E-mail à re-vérifier sur site officiel avant envoi. NE RIEN ENVOYER — vrai From info@pierredegypte.online via Network Solutions à vérifier avant tout contact</t>
         </is>
       </c>
-      <c r="P317" t="inlineStr">
+      <c r="P317" s="12" t="inlineStr">
         <is>
           <t>5e liste — croisement (26/10)</t>
         </is>
       </c>
-      <c r="Q317" t="inlineStr">
+      <c r="Q317" s="12" t="inlineStr">
         <is>
           <t>facomat76@wanadoo.fr</t>
         </is>
       </c>
     </row>
     <row r="318" ht="15" customHeight="1" s="13">
-      <c r="A318" t="n">
+      <c r="A318" s="12" t="n">
         <v>318</v>
       </c>
-      <c r="B318" t="inlineStr">
+      <c r="B318" s="12" t="inlineStr">
         <is>
           <t>Pro France</t>
         </is>
       </c>
-      <c r="C318" t="n">
+      <c r="C318" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="D318" t="inlineStr">
+      <c r="D318" s="12" t="inlineStr">
         <is>
           <t>Négoce pierre</t>
         </is>
       </c>
-      <c r="E318" t="inlineStr">
+      <c r="E318" s="12" t="inlineStr">
         <is>
           <t>MasterPierre Caen</t>
         </is>
       </c>
-      <c r="F318" t="inlineStr">
+      <c r="F318" s="12" t="inlineStr">
         <is>
           <t>Mondeville (14)</t>
         </is>
       </c>
-      <c r="G318" t="inlineStr">
+      <c r="G318" s="12" t="inlineStr">
         <is>
           <t>Normandie</t>
         </is>
       </c>
-      <c r="H318" t="inlineStr">
+      <c r="H318" s="12" t="inlineStr">
         <is>
           <t>Négoce pierre</t>
         </is>
       </c>
-      <c r="J318" t="inlineStr">
+      <c r="J318" s="12" t="inlineStr">
         <is>
           <t>02 31 52 42 77</t>
         </is>
       </c>
-      <c r="K318" t="inlineStr">
+      <c r="K318" s="12" t="inlineStr">
         <is>
           <t>Croisement fichier (26/10)</t>
         </is>
@@ -22768,22 +22768,22 @@
           <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
         </is>
       </c>
-      <c r="N318" t="inlineStr">
+      <c r="N318" s="12" t="inlineStr">
         <is>
           <t>NE RIEN ENVOYER — vrai From info@pierredegypte.online via Network Solutions à vérifier avant tout contact</t>
         </is>
       </c>
-      <c r="O318" t="inlineStr">
+      <c r="O318" s="12" t="inlineStr">
         <is>
           <t>[26/10 croisement fichier propriétaire] Apporté par le fichier propriétaire du 26/10 (origine « Recherche 31 » de son côté). E-mail à re-vérifier sur site officiel avant envoi. ⚠️ Domaine masterpierre.com déjà croisé dans nos sources : vérifier l'historique avant envoi. NE RIEN ENVOYER — vrai From info@pierredegypte.online via Network Solutions à vérifier avant tout contact</t>
         </is>
       </c>
-      <c r="P318" t="inlineStr">
+      <c r="P318" s="12" t="inlineStr">
         <is>
           <t>5e liste — croisement (26/10)</t>
         </is>
       </c>
-      <c r="Q318" t="inlineStr">
+      <c r="Q318" s="12" t="inlineStr">
         <is>
           <t>caen@masterpierre.com</t>
         </is>

</xml_diff>

<commit_message>
Revendeurs à 35 € : 5 fiches vérifiées ajoutées, 1 fantôme écarté, brouillons
- Vérification web adversariale des 6 noms du relevé (26/10 soir) :
  C-Négoce (Gala 76,50 € confirmé), Thomas Sograma (Crema Sinai 55,57 €
  confirmé), Pierres & Décors (Sinaï 50-89 € confirmé) = P1 ;
  La Maison des Cailloux et Carrelage Market = P3 (marges contestées) ;
  Cubik Minéral Outdoor = ÉCARTÉ (société introuvable au registre national).
- Minéral Pierre Naturelle enrichie (Sinaï Pearl ~60,90 €, vraie piste
  derrière la fiche fantôme Cubik) ; Dalle Décor référencée dans l'onglet.
- Nouvel onglet « Revendeurs à 35 € » (marges chiffrées, verdicts, verrou).
- Brouillons des 5 messages Top 5 révisé (à valider, zéro envoi).
- CSV ré-exporté (garde-fou prix OK, 322 lignes).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xqm9tFtdvLdJdkiWw2VVp6
</commit_message>
<xml_diff>
--- a/minyala/clients-potentiels.xlsx
+++ b/minyala/clients-potentiels.xlsx
@@ -13,6 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plateformes pros" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Groupes Facebook" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contacts particuliers" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revendeurs à 35 €" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tous les clients'!$A$1:$P$250</definedName>
@@ -24,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -77,6 +78,9 @@
       <sz val="11"/>
       <u val="single"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -117,7 +121,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -182,6 +186,7 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -20120,7 +20125,7 @@
       </c>
       <c r="O283" s="12" t="inlineStr">
         <is>
-          <t>[26/10] Recherche vérifiée (segment importateurs). Confirmée : spécialiste pierre naturelle (travertin, calcaire, marbre, granit...), 7 magasins France/Allemagne dont Lyon, Strasbourg, Nancy, Beaune, Thionville. Mentions légales : Pierre de l'Est SAS, 44 Rue de Nancy, 57915 Woustviller — raison sociale et ville confirmées. AUCUN e-mail publié : vérifié sur l'accueil et les mentions légales (contact par téléphone ou formulaire uniquement). Repli téléphone VÉRIFIÉ : 03 60 12 33 53 affiché sur l'accueil (« Conseil d'expert ») et dans les mentions légales. Le produit Sinai Pearl n'était pas visible sur la portion d'accueil lue, mais l'activité calcaire/travertin est confirmée. Domaine hors liste d'exclusion. Source e-mail : aucune (pas d e-mail publié).  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi [26/10 croisement fichier propriétaire] 2e téléphone (fichier) : 03 87 98 67 37.</t>
+          <t>[26/10] Recherche vérifiée (segment importateurs). Confirmée : spécialiste pierre naturelle (travertin, calcaire, marbre, granit...), 7 magasins France/Allemagne dont Lyon, Strasbourg, Nancy, Beaune, Thionville. Mentions légales : Pierre de l'Est SAS, 44 Rue de Nancy, 57915 Woustviller — raison sociale et ville confirmées. AUCUN e-mail publié : vérifié sur l'accueil et les mentions légales (contact par téléphone ou formulaire uniquement). Repli téléphone VÉRIFIÉ : 03 60 12 33 53 affiché sur l'accueil (« Conseil d'expert ») et dans les mentions légales. Le produit Sinai Pearl n'était pas visible sur la portion d'accueil lue, mais l'activité calcaire/travertin est confirmée. Domaine hors liste d'exclusion. Source e-mail : aucune (pas d e-mail publié).  NE RIEN ENVOYER (ordre du 26/10) — vérification expéditeur info@pierredegypte.online préalable à tout envoi [26/10 croisement fichier propriétaire] 2e téléphone (fichier) : 03 87 98 67 37. [26/10 vérifié] Vend le Sinaï Pearl (calcaire égyptien) ~60,90 €/m² TTC → marge brute +25,90 €/m² à 35 €. Showrooms Est : Bischheim/Strasbourg, Thionville, Champigneulles, Givors, Ladoix-Serrigny, Woustviller. 3e tél relevé : 03 60 12 33 53. NB : la fiche « Cubik Minéral Outdoor » (Sélestat) du relevé est une société fantôme — introuvable au registre national ; le vrai vendeur de Sinaï Pearl dans l'Est, c'est cette fiche-ci.</t>
         </is>
       </c>
       <c r="P283" s="12" t="inlineStr">
@@ -22790,19 +22795,394 @@
       </c>
     </row>
     <row r="319" ht="15" customHeight="1" s="13">
-      <c r="L319" s="12" t="n"/>
+      <c r="A319" t="n">
+        <v>319</v>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C319" t="n">
+        <v>1</v>
+      </c>
+      <c r="D319" t="inlineStr">
+        <is>
+          <t>Négoce / revendeur pierre</t>
+        </is>
+      </c>
+      <c r="E319" t="inlineStr">
+        <is>
+          <t>C-Négoce (Centre Négoce SARL)</t>
+        </is>
+      </c>
+      <c r="F319" t="inlineStr">
+        <is>
+          <t>Saint-Priest (69800)</t>
+        </is>
+      </c>
+      <c r="G319" t="inlineStr">
+        <is>
+          <t>Auvergne-Rhône-Alpes</t>
+        </is>
+      </c>
+      <c r="H319" t="inlineStr">
+        <is>
+          <t>Revendeur vendant déjà une pierre comparable plus cher que 35 € TTC/m² — cible « Revendeurs à 35 € ».</t>
+        </is>
+      </c>
+      <c r="I319" t="inlineStr">
+        <is>
+          <t>https://www.c-negoce.com</t>
+        </is>
+      </c>
+      <c r="J319" t="inlineStr">
+        <is>
+          <t>04 72 51 77 70</t>
+        </is>
+      </c>
+      <c r="K319" t="inlineStr">
+        <is>
+          <t>Relevé revendeurs (26/10 soir), vérifié par nos soins</t>
+        </is>
+      </c>
+      <c r="L319" s="12" t="inlineStr">
+        <is>
+          <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
+        </is>
+      </c>
+      <c r="N319" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER — vrai From info@pierredegypte.online via Network Solutions à vérifier avant tout contact</t>
+        </is>
+      </c>
+      <c r="O319" t="inlineStr">
+        <is>
+          <t>[26/10 vérifié] Vend « marbre d'Égypte Gala » brossé 76,50 € TTC/m² (page produit officielle, réf. 005001) → marge brute +41,50 €/m² à 35 €. Importateur, NAF 46.90Z, 5 showrooms (Lyon Est, Dardilly, Dijon, Annemasse). Stock « 80 000 m² » = auto-déclaration marketing (fiche Leroy Merlin), non vérifiée. ⚠️ Site en maintenance (503) le 26/10 — prix lu sur version indexée récente, re-vérifier au retour en ligne. E-mails secondaires : contact94@ (Outdoor), dardilly@, dijon@, contact74@. NE RIEN ENVOYER — vrai From info@pierredegypte.online via Network Solutions à vérifier avant tout contact</t>
+        </is>
+      </c>
+      <c r="P319" t="inlineStr">
+        <is>
+          <t>Revendeurs à 35 € (26/10)</t>
+        </is>
+      </c>
+      <c r="Q319" t="inlineStr">
+        <is>
+          <t>contact@c-negoce.com</t>
+        </is>
+      </c>
     </row>
     <row r="320" ht="15" customHeight="1" s="13">
-      <c r="L320" s="12" t="n"/>
+      <c r="A320" t="n">
+        <v>320</v>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C320" t="n">
+        <v>1</v>
+      </c>
+      <c r="D320" t="inlineStr">
+        <is>
+          <t>Négoce matériaux multi-agences</t>
+        </is>
+      </c>
+      <c r="E320" t="inlineStr">
+        <is>
+          <t>Thomas Sograma Matériaux</t>
+        </is>
+      </c>
+      <c r="F320" t="inlineStr">
+        <is>
+          <t>Andrézieux-Bouthéon (42160)</t>
+        </is>
+      </c>
+      <c r="G320" t="inlineStr">
+        <is>
+          <t>Auvergne-Rhône-Alpes</t>
+        </is>
+      </c>
+      <c r="H320" t="inlineStr">
+        <is>
+          <t>Revendeur vendant déjà une pierre comparable plus cher que 35 € TTC/m² — cible « Revendeurs à 35 € ».</t>
+        </is>
+      </c>
+      <c r="I320" t="inlineStr">
+        <is>
+          <t>https://www.thomas-sograma.com</t>
+        </is>
+      </c>
+      <c r="J320" t="inlineStr">
+        <is>
+          <t>04 77 55 21 35</t>
+        </is>
+      </c>
+      <c r="K320" t="inlineStr">
+        <is>
+          <t>Relevé revendeurs (26/10 soir), vérifié par nos soins</t>
+        </is>
+      </c>
+      <c r="L320" s="12" t="inlineStr">
+        <is>
+          <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
+        </is>
+      </c>
+      <c r="N320" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER — vrai From info@pierredegypte.online via Network Solutions à vérifier avant tout contact</t>
+        </is>
+      </c>
+      <c r="O320" t="inlineStr">
+        <is>
+          <t>[26/10 vérifié] Vend Crema Sinai calcaire égyptien : opus romain 2 cm à 55,57 € TTC/m² (confirmé page officielle, réf. 510001), autres variantes 1,8 cm 60,65–75,10 €. Vend aussi pierre « Kemet » (provenance Égypte) 55,26 €. Marge brute +20,57 €/m² à 35 €. Groupe Thomas Peres et Fils, 8 établissements Loire. NE RIEN ENVOYER — vrai From info@pierredegypte.online via Network Solutions à vérifier avant tout contact</t>
+        </is>
+      </c>
+      <c r="P320" t="inlineStr">
+        <is>
+          <t>Revendeurs à 35 € (26/10)</t>
+        </is>
+      </c>
+      <c r="Q320" t="inlineStr">
+        <is>
+          <t>contact@thomas-sograma.com</t>
+        </is>
+      </c>
     </row>
     <row r="321" ht="15" customHeight="1" s="13">
-      <c r="L321" s="12" t="n"/>
+      <c r="A321" t="n">
+        <v>321</v>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C321" t="n">
+        <v>1</v>
+      </c>
+      <c r="D321" t="inlineStr">
+        <is>
+          <t>Revendeur pierre naturelle (showroom)</t>
+        </is>
+      </c>
+      <c r="E321" t="inlineStr">
+        <is>
+          <t>Pierres &amp; Décors (L'univers de la Pierre SASU)</t>
+        </is>
+      </c>
+      <c r="F321" t="inlineStr">
+        <is>
+          <t>Portet-sur-Garonne (31120)</t>
+        </is>
+      </c>
+      <c r="G321" t="inlineStr">
+        <is>
+          <t>Occitanie</t>
+        </is>
+      </c>
+      <c r="H321" t="inlineStr">
+        <is>
+          <t>Revendeur vendant déjà une pierre comparable plus cher que 35 € TTC/m² — cible « Revendeurs à 35 € ».</t>
+        </is>
+      </c>
+      <c r="I321" t="inlineStr">
+        <is>
+          <t>https://pierres-decors.com</t>
+        </is>
+      </c>
+      <c r="J321" t="inlineStr">
+        <is>
+          <t>09 84 40 18 41 / 07 67 89 52 78</t>
+        </is>
+      </c>
+      <c r="K321" t="inlineStr">
+        <is>
+          <t>Relevé revendeurs (26/10 soir), vérifié par nos soins</t>
+        </is>
+      </c>
+      <c r="L321" s="12" t="inlineStr">
+        <is>
+          <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
+        </is>
+      </c>
+      <c r="N321" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER — vrai From info@pierredegypte.online via Network Solutions à vérifier avant tout contact</t>
+        </is>
+      </c>
+      <c r="O321" t="inlineStr">
+        <is>
+          <t>[26/10 vérifié] Catégorie « Pierres d'Égypte » : dallages pierre du Sinaï (KEROS, SAHARA) à partir de 50 €/m², grands formats à partir de 89 €/m² (confirmé pages officielles). Marge brute +15 à +54 €/m² à 35 €. SIREN 799 580 188, Toulouse. ⚠️ Ne pas confondre avec « Pierres et Décors » de Royan (autre société). NE RIEN ENVOYER — vrai From info@pierredegypte.online via Network Solutions à vérifier avant tout contact</t>
+        </is>
+      </c>
+      <c r="P321" t="inlineStr">
+        <is>
+          <t>Revendeurs à 35 € (26/10)</t>
+        </is>
+      </c>
+      <c r="Q321" t="inlineStr">
+        <is>
+          <t>contact@pierres-decors.com</t>
+        </is>
+      </c>
     </row>
     <row r="322" ht="15" customHeight="1" s="13">
-      <c r="L322" s="12" t="n"/>
+      <c r="A322" t="n">
+        <v>322</v>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C322" t="n">
+        <v>3</v>
+      </c>
+      <c r="D322" t="inlineStr">
+        <is>
+          <t>Atelier-producteur pierre + boutique en ligne</t>
+        </is>
+      </c>
+      <c r="E322" t="inlineStr">
+        <is>
+          <t>La Maison des Cailloux</t>
+        </is>
+      </c>
+      <c r="F322" t="inlineStr">
+        <is>
+          <t>Capvern (65130)</t>
+        </is>
+      </c>
+      <c r="G322" t="inlineStr">
+        <is>
+          <t>Occitanie</t>
+        </is>
+      </c>
+      <c r="H322" t="inlineStr">
+        <is>
+          <t>Revendeur vendant déjà une pierre comparable plus cher que 35 € TTC/m² — cible « Revendeurs à 35 € ».</t>
+        </is>
+      </c>
+      <c r="I322" t="inlineStr">
+        <is>
+          <t>https://www.lamaisondescailloux.com</t>
+        </is>
+      </c>
+      <c r="J322" t="inlineStr">
+        <is>
+          <t>05 62 98 11 97</t>
+        </is>
+      </c>
+      <c r="K322" t="inlineStr">
+        <is>
+          <t>Relevé revendeurs (26/10 soir), vérifié par nos soins</t>
+        </is>
+      </c>
+      <c r="L322" s="12" t="inlineStr">
+        <is>
+          <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
+        </is>
+      </c>
+      <c r="N322" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER — vrai From info@pierredegypte.online via Network Solutions à vérifier avant tout contact</t>
+        </is>
+      </c>
+      <c r="O322" t="inlineStr">
+        <is>
+          <t>[26/10 vérifié] ⚠️ Angle marge FRAGILE : pas un pur revendeur (atelier-producteur pyrénéen, marbres Sarrancolin) ; son calcaire du Causse est à 60–80 €/m² mais son travertin import est à 29–30 €/m², DÉJÀ SOUS nos 35 €. Aucune pierre d'Égypte au catalogue. ~800 km de Gennevilliers, transport à chiffrer. SIREN 423 325 000. NE RIEN ENVOYER — vrai From info@pierredegypte.online via Network Solutions à vérifier avant tout contact</t>
+        </is>
+      </c>
+      <c r="P322" t="inlineStr">
+        <is>
+          <t>Revendeurs à 35 € (26/10)</t>
+        </is>
+      </c>
+      <c r="Q322" t="inlineStr">
+        <is>
+          <t>contact@lamaisondescailloux.com</t>
+        </is>
+      </c>
     </row>
     <row r="323" ht="15" customHeight="1" s="13">
-      <c r="L323" s="12" t="n"/>
+      <c r="A323" t="n">
+        <v>323</v>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>Pro France</t>
+        </is>
+      </c>
+      <c r="C323" t="n">
+        <v>3</v>
+      </c>
+      <c r="D323" t="inlineStr">
+        <is>
+          <t>Négoce gros matériaux / vente en ligne</t>
+        </is>
+      </c>
+      <c r="E323" t="inlineStr">
+        <is>
+          <t>Carrelage Market (Vente Pierre Naturelle.com SAS)</t>
+        </is>
+      </c>
+      <c r="F323" t="inlineStr">
+        <is>
+          <t>Puget-sur-Argens (83480)</t>
+        </is>
+      </c>
+      <c r="G323" t="inlineStr">
+        <is>
+          <t>PACA</t>
+        </is>
+      </c>
+      <c r="H323" t="inlineStr">
+        <is>
+          <t>Revendeur vendant déjà une pierre comparable plus cher que 35 € TTC/m² — cible « Revendeurs à 35 € ».</t>
+        </is>
+      </c>
+      <c r="I323" t="inlineStr">
+        <is>
+          <t>https://www.carrelage-market.com</t>
+        </is>
+      </c>
+      <c r="J323" t="inlineStr">
+        <is>
+          <t>06 51 49 72 78</t>
+        </is>
+      </c>
+      <c r="K323" t="inlineStr">
+        <is>
+          <t>Relevé revendeurs (26/10 soir), vérifié par nos soins</t>
+        </is>
+      </c>
+      <c r="L323" s="12" t="inlineStr">
+        <is>
+          <t>À contacter — EN ATTENTE (ne rien envoyer)</t>
+        </is>
+      </c>
+      <c r="N323" t="inlineStr">
+        <is>
+          <t>NE RIEN ENVOYER — vrai From info@pierredegypte.online via Network Solutions à vérifier avant tout contact</t>
+        </is>
+      </c>
+      <c r="O323" t="inlineStr">
+        <is>
+          <t>[26/10 vérifié] ⚠️ Marge annoncée (48 €/m²) NON retrouvée : leur seul Sinaï en ligne est un déstockage à ≈35,12 €/m² TTC (lot 41 m² à 1 440 €), quasiment notre prix. Argument marge inopérant tant que ce lot est affiché. SIREN 537 699 506, NAF 46.73A, siège Cannes, showroom Var. NE RIEN ENVOYER — vrai From info@pierredegypte.online via Network Solutions à vérifier avant tout contact</t>
+        </is>
+      </c>
+      <c r="P323" t="inlineStr">
+        <is>
+          <t>Revendeurs à 35 € (26/10)</t>
+        </is>
+      </c>
+      <c r="Q323" t="inlineStr">
+        <is>
+          <t>info@carrelage-market.com</t>
+        </is>
+      </c>
     </row>
     <row r="324" ht="15" customHeight="1" s="13">
       <c r="L324" s="12" t="n"/>
@@ -28686,4 +29066,537 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" style="13" min="1" max="1"/>
+    <col width="22" customWidth="1" style="13" min="2" max="2"/>
+    <col width="45" customWidth="1" style="13" min="3" max="3"/>
+    <col width="22" customWidth="1" style="13" min="4" max="4"/>
+    <col width="26" customWidth="1" style="13" min="5" max="5"/>
+    <col width="50" customWidth="1" style="13" min="6" max="6"/>
+    <col width="32" customWidth="1" style="13" min="7" max="7"/>
+    <col width="28" customWidth="1" style="13" min="8" max="8"/>
+    <col width="12" customWidth="1" style="13" min="9" max="9"/>
+    <col width="8" customWidth="1" style="13" min="10" max="10"/>
+    <col width="24" customWidth="1" style="13" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="22" t="inlineStr">
+        <is>
+          <t>REVENDEURS À 35 € — revendent déjà une pierre comparable plus cher (relevé 26/10 soir, vérifié le 26/10). 🔒 VERROU GLOBAL : ZÉRO ENVOI tant que l'expéditeur réel info@pierredegypte.online (Network Solutions) n'est pas vérifié. Jamais « prix le plus bas » ; prix public 35 €/m² TTC pierre seule, min 25 m².</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="22" t="inlineStr">
+        <is>
+          <t>Société</t>
+        </is>
+      </c>
+      <c r="B3" s="22" t="inlineStr">
+        <is>
+          <t>Ville</t>
+        </is>
+      </c>
+      <c r="C3" s="22" t="inlineStr">
+        <is>
+          <t>Produit comparable (leur catalogue)</t>
+        </is>
+      </c>
+      <c r="D3" s="22" t="inlineStr">
+        <is>
+          <t>Leur prix public TTC/m²</t>
+        </is>
+      </c>
+      <c r="E3" s="22" t="inlineStr">
+        <is>
+          <t>Marge brute à 35 €</t>
+        </is>
+      </c>
+      <c r="F3" s="22" t="inlineStr">
+        <is>
+          <t>Verdict vérif 26/10</t>
+        </is>
+      </c>
+      <c r="G3" s="22" t="inlineStr">
+        <is>
+          <t>E-mail</t>
+        </is>
+      </c>
+      <c r="H3" s="22" t="inlineStr">
+        <is>
+          <t>Tél</t>
+        </is>
+      </c>
+      <c r="I3" s="22" t="inlineStr">
+        <is>
+          <t>Ligne registre</t>
+        </is>
+      </c>
+      <c r="J3" s="22" t="inlineStr">
+        <is>
+          <t>Priorité</t>
+        </is>
+      </c>
+      <c r="K3" s="22" t="inlineStr">
+        <is>
+          <t>Statut</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>C-Négoce</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Saint-Priest (69)</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Marbre d'Égypte Gala brossé 60x90x1,5</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>76,50 €</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>+41,50 €/m²</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Confirmé (site en maintenance — prix via version indexée, à recontrôler)</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>contact@c-negoce.com</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>04 72 51 77 70</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>319</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>À contacter — EN ATTENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Thomas Sograma</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Andrézieux-Bouthéon (42)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Crema Sinai adouci vieilli opus romain 2 cm</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>55,57 €</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>+20,57 €/m²</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Confirmé (page produit officielle)</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>contact@thomas-sograma.com</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>04 77 55 21 35</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>320</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>À contacter — EN ATTENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Pierres &amp; Décors</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Portet-sur-Garonne (31)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Pierre du Sinaï KEROS/SAHARA dallages &amp; grands formats</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>50 à 89 €</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>+15 à +54 €/m²</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Confirmé (pages produit officielles)</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>contact@pierres-decors.com</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>09 84 40 18 41</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>321</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>À contacter — EN ATTENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Dalle Décor</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Galluis (78)</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Importateur pierre depuis 1972 (prix non affichés)</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Déjà en registre (5e liste) ; ~30 min du stock</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>(formulaire/tél)</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>01 34 86 41 72</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>271</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>À contacter — EN ATTENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Minéral Pierre Naturelle</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Est (Bischheim, Thionville…)</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Sinaï Pearl calcaire égyptien</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>≈60,90 €</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>+25,90 €/m²</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Confirmé — remplace la fiche fantôme « Cubik Minéral Outdoor »</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>(pas d'e-mail publié)</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>03 87 98 67 37 / 03 60 12 33 53</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>283</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>À contacter — EN ATTENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>La Maison des Cailloux</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Capvern (65)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Calcaire du Causse 60–80 € MAIS travertin import 29–30 €</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>60–80 € (Causse)</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>⚠️ fragile : son travertin est sous 35 €</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Existe, angle marge contesté ; ~800 km</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>contact@lamaisondescailloux.com</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>05 62 98 11 97</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>322</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>À contacter — EN ATTENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Carrelage Market</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Puget-sur-Argens (83)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Sinaï sablé/brossé 60x40x2 en déstockage</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>≈35,12 € (déstock) — 48 € non retrouvé</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>⚠️ ≈ 0 tant que le déstockage est en ligne</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Existe, marge annoncée réfutée</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>info@carrelage-market.com</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>06 51 49 72 78</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>323</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>À contacter — EN ATTENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Cubik Minéral Outdoor</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Sélestat (67) — annoncé</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Sinaï Pearl (annoncé)</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>ÉCARTÉ : société introuvable (registre national, web) — fiche fantôme</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>non ajouté</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>ÉCARTÉ</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>